<commit_message>
Make reviewer names optional for individual evaluation assignments
</commit_message>
<xml_diff>
--- a/Social Media Post Evaluation.xlsx
+++ b/Social Media Post Evaluation.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Ra8f9973531e949ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluation Log" sheetId="2" r:id="R72372df8de05405b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R604b3efd29854d58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compare Runs" sheetId="4" r:id="R39b83e11da83496d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failure Analysis" sheetId="5" r:id="R05f8f5add131422e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failure Traces" sheetId="6" r:id="R8139c5436fd44074"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worked Examples" sheetId="7" r:id="R8a697dfadd6448d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Ra60c74bccba444c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluation Log" sheetId="2" r:id="Rc25b9675dafc4da5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R3bffebb01c61495a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compare Runs" sheetId="4" r:id="Rd4c315767665471f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failure Analysis" sheetId="5" r:id="Rf416817ae9ee43a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failure Traces" sheetId="6" r:id="R9097a85faca04401"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worked Examples" sheetId="7" r:id="R03fa632cdea14416"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -435,7 +435,7 @@
         <x:v>3. Human review first</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>Write Human_Critique using an observable quote or omission and the decisive requirement. Then set Human_Decision to PASS or FAIL. Fill Human_Reviewer and Human_Policy_Version = social-publication-v2. Leave the decision blank while context is incomplete. Review revised posts independently.</x:v>
+        <x:v>Write Human_Critique using an observable quote or omission and the decisive requirement. Then set Human_Decision to PASS or FAIL and Human_Policy_Version = social-publication-v2. Human_Reviewer is optional. Leave the decision blank while context is incomplete. Review revised posts afresh.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="67.5" customHeight="1">
@@ -766,7 +766,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL2" s="9" t="str">
-        <x:f>IF(A2="","",IF(AND(AK2="OK",J2="READY",F2&lt;&gt;"",G2&lt;&gt;"",K2&lt;&gt;"",OR(L2="PASS",L2="FAIL"),M2&lt;&gt;"",O2&lt;&gt;"",P2="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A2="","",IF(AND(AK2="OK",J2="READY",F2&lt;&gt;"",G2&lt;&gt;"",K2&lt;&gt;"",OR(L2="PASS",L2="FAIL"),M2&lt;&gt;"",P2="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM2" s="9" t="str">
@@ -842,7 +842,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL3" s="9" t="str">
-        <x:f>IF(A3="","",IF(AND(AK3="OK",J3="READY",F3&lt;&gt;"",G3&lt;&gt;"",K3&lt;&gt;"",OR(L3="PASS",L3="FAIL"),M3&lt;&gt;"",O3&lt;&gt;"",P3="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A3="","",IF(AND(AK3="OK",J3="READY",F3&lt;&gt;"",G3&lt;&gt;"",K3&lt;&gt;"",OR(L3="PASS",L3="FAIL"),M3&lt;&gt;"",P3="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM3" s="9" t="str">
@@ -918,7 +918,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL4" s="9" t="str">
-        <x:f>IF(A4="","",IF(AND(AK4="OK",J4="READY",F4&lt;&gt;"",G4&lt;&gt;"",K4&lt;&gt;"",OR(L4="PASS",L4="FAIL"),M4&lt;&gt;"",O4&lt;&gt;"",P4="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A4="","",IF(AND(AK4="OK",J4="READY",F4&lt;&gt;"",G4&lt;&gt;"",K4&lt;&gt;"",OR(L4="PASS",L4="FAIL"),M4&lt;&gt;"",P4="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM4" s="9" t="str">
@@ -994,7 +994,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL5" s="9" t="str">
-        <x:f>IF(A5="","",IF(AND(AK5="OK",J5="READY",F5&lt;&gt;"",G5&lt;&gt;"",K5&lt;&gt;"",OR(L5="PASS",L5="FAIL"),M5&lt;&gt;"",O5&lt;&gt;"",P5="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A5="","",IF(AND(AK5="OK",J5="READY",F5&lt;&gt;"",G5&lt;&gt;"",K5&lt;&gt;"",OR(L5="PASS",L5="FAIL"),M5&lt;&gt;"",P5="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM5" s="9" t="str">
@@ -1070,7 +1070,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL6" s="9" t="str">
-        <x:f>IF(A6="","",IF(AND(AK6="OK",J6="READY",F6&lt;&gt;"",G6&lt;&gt;"",K6&lt;&gt;"",OR(L6="PASS",L6="FAIL"),M6&lt;&gt;"",O6&lt;&gt;"",P6="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A6="","",IF(AND(AK6="OK",J6="READY",F6&lt;&gt;"",G6&lt;&gt;"",K6&lt;&gt;"",OR(L6="PASS",L6="FAIL"),M6&lt;&gt;"",P6="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM6" s="9" t="str">
@@ -1146,7 +1146,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL7" s="9" t="str">
-        <x:f>IF(A7="","",IF(AND(AK7="OK",J7="READY",F7&lt;&gt;"",G7&lt;&gt;"",K7&lt;&gt;"",OR(L7="PASS",L7="FAIL"),M7&lt;&gt;"",O7&lt;&gt;"",P7="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A7="","",IF(AND(AK7="OK",J7="READY",F7&lt;&gt;"",G7&lt;&gt;"",K7&lt;&gt;"",OR(L7="PASS",L7="FAIL"),M7&lt;&gt;"",P7="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM7" s="9" t="str">
@@ -1222,7 +1222,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL8" s="9" t="str">
-        <x:f>IF(A8="","",IF(AND(AK8="OK",J8="READY",F8&lt;&gt;"",G8&lt;&gt;"",K8&lt;&gt;"",OR(L8="PASS",L8="FAIL"),M8&lt;&gt;"",O8&lt;&gt;"",P8="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A8="","",IF(AND(AK8="OK",J8="READY",F8&lt;&gt;"",G8&lt;&gt;"",K8&lt;&gt;"",OR(L8="PASS",L8="FAIL"),M8&lt;&gt;"",P8="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM8" s="9" t="str">
@@ -1298,7 +1298,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL9" s="9" t="str">
-        <x:f>IF(A9="","",IF(AND(AK9="OK",J9="READY",F9&lt;&gt;"",G9&lt;&gt;"",K9&lt;&gt;"",OR(L9="PASS",L9="FAIL"),M9&lt;&gt;"",O9&lt;&gt;"",P9="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A9="","",IF(AND(AK9="OK",J9="READY",F9&lt;&gt;"",G9&lt;&gt;"",K9&lt;&gt;"",OR(L9="PASS",L9="FAIL"),M9&lt;&gt;"",P9="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM9" s="9" t="str">
@@ -1374,7 +1374,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL10" s="9" t="str">
-        <x:f>IF(A10="","",IF(AND(AK10="OK",J10="READY",F10&lt;&gt;"",G10&lt;&gt;"",K10&lt;&gt;"",OR(L10="PASS",L10="FAIL"),M10&lt;&gt;"",O10&lt;&gt;"",P10="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A10="","",IF(AND(AK10="OK",J10="READY",F10&lt;&gt;"",G10&lt;&gt;"",K10&lt;&gt;"",OR(L10="PASS",L10="FAIL"),M10&lt;&gt;"",P10="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM10" s="9" t="str">
@@ -1450,7 +1450,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL11" s="9" t="str">
-        <x:f>IF(A11="","",IF(AND(AK11="OK",J11="READY",F11&lt;&gt;"",G11&lt;&gt;"",K11&lt;&gt;"",OR(L11="PASS",L11="FAIL"),M11&lt;&gt;"",O11&lt;&gt;"",P11="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A11="","",IF(AND(AK11="OK",J11="READY",F11&lt;&gt;"",G11&lt;&gt;"",K11&lt;&gt;"",OR(L11="PASS",L11="FAIL"),M11&lt;&gt;"",P11="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM11" s="9" t="str">
@@ -1526,7 +1526,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL12" s="9" t="str">
-        <x:f>IF(A12="","",IF(AND(AK12="OK",J12="READY",F12&lt;&gt;"",G12&lt;&gt;"",K12&lt;&gt;"",OR(L12="PASS",L12="FAIL"),M12&lt;&gt;"",O12&lt;&gt;"",P12="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A12="","",IF(AND(AK12="OK",J12="READY",F12&lt;&gt;"",G12&lt;&gt;"",K12&lt;&gt;"",OR(L12="PASS",L12="FAIL"),M12&lt;&gt;"",P12="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM12" s="9" t="str">
@@ -1602,7 +1602,7 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="AL13" s="9" t="str">
-        <x:f>IF(A13="","",IF(AND(AK13="OK",J13="READY",F13&lt;&gt;"",G13&lt;&gt;"",K13&lt;&gt;"",OR(L13="PASS",L13="FAIL"),M13&lt;&gt;"",O13&lt;&gt;"",P13="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A13="","",IF(AND(AK13="OK",J13="READY",F13&lt;&gt;"",G13&lt;&gt;"",K13&lt;&gt;"",OR(L13="PASS",L13="FAIL"),M13&lt;&gt;"",P13="social-publication-v2"),"YES","NO"))</x:f>
         <x:v>NO</x:v>
       </x:c>
       <x:c r="AM13" s="9" t="str">
@@ -1657,7 +1657,7 @@
         <x:f>IF(A14="",IF(B14="","","MISSING_TEST_ID"),IF(B14="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A14,$B$2:$B$501,B14)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL14" s="9" t="str">
-        <x:f>IF(A14="","",IF(AND(AK14="OK",J14="READY",F14&lt;&gt;"",G14&lt;&gt;"",K14&lt;&gt;"",OR(L14="PASS",L14="FAIL"),M14&lt;&gt;"",O14&lt;&gt;"",P14="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A14="","",IF(AND(AK14="OK",J14="READY",F14&lt;&gt;"",G14&lt;&gt;"",K14&lt;&gt;"",OR(L14="PASS",L14="FAIL"),M14&lt;&gt;"",P14="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM14" s="9" t="str">
         <x:f>IF(A14="","",IF(AND(AK14="OK",J14="READY",F14&lt;&gt;"",G14&lt;&gt;"",K14&lt;&gt;"",S14="OK",OR(R14="PASS",R14="FAIL")),"YES","NO"))</x:f>
@@ -1709,7 +1709,7 @@
         <x:f>IF(A15="",IF(B15="","","MISSING_TEST_ID"),IF(B15="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A15,$B$2:$B$501,B15)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL15" s="9" t="str">
-        <x:f>IF(A15="","",IF(AND(AK15="OK",J15="READY",F15&lt;&gt;"",G15&lt;&gt;"",K15&lt;&gt;"",OR(L15="PASS",L15="FAIL"),M15&lt;&gt;"",O15&lt;&gt;"",P15="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A15="","",IF(AND(AK15="OK",J15="READY",F15&lt;&gt;"",G15&lt;&gt;"",K15&lt;&gt;"",OR(L15="PASS",L15="FAIL"),M15&lt;&gt;"",P15="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM15" s="9" t="str">
         <x:f>IF(A15="","",IF(AND(AK15="OK",J15="READY",F15&lt;&gt;"",G15&lt;&gt;"",K15&lt;&gt;"",S15="OK",OR(R15="PASS",R15="FAIL")),"YES","NO"))</x:f>
@@ -1761,7 +1761,7 @@
         <x:f>IF(A16="",IF(B16="","","MISSING_TEST_ID"),IF(B16="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A16,$B$2:$B$501,B16)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL16" s="9" t="str">
-        <x:f>IF(A16="","",IF(AND(AK16="OK",J16="READY",F16&lt;&gt;"",G16&lt;&gt;"",K16&lt;&gt;"",OR(L16="PASS",L16="FAIL"),M16&lt;&gt;"",O16&lt;&gt;"",P16="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A16="","",IF(AND(AK16="OK",J16="READY",F16&lt;&gt;"",G16&lt;&gt;"",K16&lt;&gt;"",OR(L16="PASS",L16="FAIL"),M16&lt;&gt;"",P16="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM16" s="9" t="str">
         <x:f>IF(A16="","",IF(AND(AK16="OK",J16="READY",F16&lt;&gt;"",G16&lt;&gt;"",K16&lt;&gt;"",S16="OK",OR(R16="PASS",R16="FAIL")),"YES","NO"))</x:f>
@@ -1813,7 +1813,7 @@
         <x:f>IF(A17="",IF(B17="","","MISSING_TEST_ID"),IF(B17="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A17,$B$2:$B$501,B17)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL17" s="9" t="str">
-        <x:f>IF(A17="","",IF(AND(AK17="OK",J17="READY",F17&lt;&gt;"",G17&lt;&gt;"",K17&lt;&gt;"",OR(L17="PASS",L17="FAIL"),M17&lt;&gt;"",O17&lt;&gt;"",P17="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A17="","",IF(AND(AK17="OK",J17="READY",F17&lt;&gt;"",G17&lt;&gt;"",K17&lt;&gt;"",OR(L17="PASS",L17="FAIL"),M17&lt;&gt;"",P17="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM17" s="9" t="str">
         <x:f>IF(A17="","",IF(AND(AK17="OK",J17="READY",F17&lt;&gt;"",G17&lt;&gt;"",K17&lt;&gt;"",S17="OK",OR(R17="PASS",R17="FAIL")),"YES","NO"))</x:f>
@@ -1865,7 +1865,7 @@
         <x:f>IF(A18="",IF(B18="","","MISSING_TEST_ID"),IF(B18="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A18,$B$2:$B$501,B18)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL18" s="9" t="str">
-        <x:f>IF(A18="","",IF(AND(AK18="OK",J18="READY",F18&lt;&gt;"",G18&lt;&gt;"",K18&lt;&gt;"",OR(L18="PASS",L18="FAIL"),M18&lt;&gt;"",O18&lt;&gt;"",P18="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A18="","",IF(AND(AK18="OK",J18="READY",F18&lt;&gt;"",G18&lt;&gt;"",K18&lt;&gt;"",OR(L18="PASS",L18="FAIL"),M18&lt;&gt;"",P18="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM18" s="9" t="str">
         <x:f>IF(A18="","",IF(AND(AK18="OK",J18="READY",F18&lt;&gt;"",G18&lt;&gt;"",K18&lt;&gt;"",S18="OK",OR(R18="PASS",R18="FAIL")),"YES","NO"))</x:f>
@@ -1917,7 +1917,7 @@
         <x:f>IF(A19="",IF(B19="","","MISSING_TEST_ID"),IF(B19="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A19,$B$2:$B$501,B19)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL19" s="9" t="str">
-        <x:f>IF(A19="","",IF(AND(AK19="OK",J19="READY",F19&lt;&gt;"",G19&lt;&gt;"",K19&lt;&gt;"",OR(L19="PASS",L19="FAIL"),M19&lt;&gt;"",O19&lt;&gt;"",P19="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A19="","",IF(AND(AK19="OK",J19="READY",F19&lt;&gt;"",G19&lt;&gt;"",K19&lt;&gt;"",OR(L19="PASS",L19="FAIL"),M19&lt;&gt;"",P19="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM19" s="9" t="str">
         <x:f>IF(A19="","",IF(AND(AK19="OK",J19="READY",F19&lt;&gt;"",G19&lt;&gt;"",K19&lt;&gt;"",S19="OK",OR(R19="PASS",R19="FAIL")),"YES","NO"))</x:f>
@@ -1969,7 +1969,7 @@
         <x:f>IF(A20="",IF(B20="","","MISSING_TEST_ID"),IF(B20="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A20,$B$2:$B$501,B20)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL20" s="9" t="str">
-        <x:f>IF(A20="","",IF(AND(AK20="OK",J20="READY",F20&lt;&gt;"",G20&lt;&gt;"",K20&lt;&gt;"",OR(L20="PASS",L20="FAIL"),M20&lt;&gt;"",O20&lt;&gt;"",P20="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A20="","",IF(AND(AK20="OK",J20="READY",F20&lt;&gt;"",G20&lt;&gt;"",K20&lt;&gt;"",OR(L20="PASS",L20="FAIL"),M20&lt;&gt;"",P20="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM20" s="9" t="str">
         <x:f>IF(A20="","",IF(AND(AK20="OK",J20="READY",F20&lt;&gt;"",G20&lt;&gt;"",K20&lt;&gt;"",S20="OK",OR(R20="PASS",R20="FAIL")),"YES","NO"))</x:f>
@@ -2021,7 +2021,7 @@
         <x:f>IF(A21="",IF(B21="","","MISSING_TEST_ID"),IF(B21="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A21,$B$2:$B$501,B21)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL21" s="9" t="str">
-        <x:f>IF(A21="","",IF(AND(AK21="OK",J21="READY",F21&lt;&gt;"",G21&lt;&gt;"",K21&lt;&gt;"",OR(L21="PASS",L21="FAIL"),M21&lt;&gt;"",O21&lt;&gt;"",P21="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A21="","",IF(AND(AK21="OK",J21="READY",F21&lt;&gt;"",G21&lt;&gt;"",K21&lt;&gt;"",OR(L21="PASS",L21="FAIL"),M21&lt;&gt;"",P21="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM21" s="9" t="str">
         <x:f>IF(A21="","",IF(AND(AK21="OK",J21="READY",F21&lt;&gt;"",G21&lt;&gt;"",K21&lt;&gt;"",S21="OK",OR(R21="PASS",R21="FAIL")),"YES","NO"))</x:f>
@@ -2073,7 +2073,7 @@
         <x:f>IF(A22="",IF(B22="","","MISSING_TEST_ID"),IF(B22="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A22,$B$2:$B$501,B22)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL22" s="9" t="str">
-        <x:f>IF(A22="","",IF(AND(AK22="OK",J22="READY",F22&lt;&gt;"",G22&lt;&gt;"",K22&lt;&gt;"",OR(L22="PASS",L22="FAIL"),M22&lt;&gt;"",O22&lt;&gt;"",P22="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A22="","",IF(AND(AK22="OK",J22="READY",F22&lt;&gt;"",G22&lt;&gt;"",K22&lt;&gt;"",OR(L22="PASS",L22="FAIL"),M22&lt;&gt;"",P22="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM22" s="9" t="str">
         <x:f>IF(A22="","",IF(AND(AK22="OK",J22="READY",F22&lt;&gt;"",G22&lt;&gt;"",K22&lt;&gt;"",S22="OK",OR(R22="PASS",R22="FAIL")),"YES","NO"))</x:f>
@@ -2125,7 +2125,7 @@
         <x:f>IF(A23="",IF(B23="","","MISSING_TEST_ID"),IF(B23="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A23,$B$2:$B$501,B23)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL23" s="9" t="str">
-        <x:f>IF(A23="","",IF(AND(AK23="OK",J23="READY",F23&lt;&gt;"",G23&lt;&gt;"",K23&lt;&gt;"",OR(L23="PASS",L23="FAIL"),M23&lt;&gt;"",O23&lt;&gt;"",P23="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A23="","",IF(AND(AK23="OK",J23="READY",F23&lt;&gt;"",G23&lt;&gt;"",K23&lt;&gt;"",OR(L23="PASS",L23="FAIL"),M23&lt;&gt;"",P23="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM23" s="9" t="str">
         <x:f>IF(A23="","",IF(AND(AK23="OK",J23="READY",F23&lt;&gt;"",G23&lt;&gt;"",K23&lt;&gt;"",S23="OK",OR(R23="PASS",R23="FAIL")),"YES","NO"))</x:f>
@@ -2177,7 +2177,7 @@
         <x:f>IF(A24="",IF(B24="","","MISSING_TEST_ID"),IF(B24="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A24,$B$2:$B$501,B24)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL24" s="9" t="str">
-        <x:f>IF(A24="","",IF(AND(AK24="OK",J24="READY",F24&lt;&gt;"",G24&lt;&gt;"",K24&lt;&gt;"",OR(L24="PASS",L24="FAIL"),M24&lt;&gt;"",O24&lt;&gt;"",P24="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A24="","",IF(AND(AK24="OK",J24="READY",F24&lt;&gt;"",G24&lt;&gt;"",K24&lt;&gt;"",OR(L24="PASS",L24="FAIL"),M24&lt;&gt;"",P24="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM24" s="9" t="str">
         <x:f>IF(A24="","",IF(AND(AK24="OK",J24="READY",F24&lt;&gt;"",G24&lt;&gt;"",K24&lt;&gt;"",S24="OK",OR(R24="PASS",R24="FAIL")),"YES","NO"))</x:f>
@@ -2229,7 +2229,7 @@
         <x:f>IF(A25="",IF(B25="","","MISSING_TEST_ID"),IF(B25="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A25,$B$2:$B$501,B25)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL25" s="9" t="str">
-        <x:f>IF(A25="","",IF(AND(AK25="OK",J25="READY",F25&lt;&gt;"",G25&lt;&gt;"",K25&lt;&gt;"",OR(L25="PASS",L25="FAIL"),M25&lt;&gt;"",O25&lt;&gt;"",P25="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A25="","",IF(AND(AK25="OK",J25="READY",F25&lt;&gt;"",G25&lt;&gt;"",K25&lt;&gt;"",OR(L25="PASS",L25="FAIL"),M25&lt;&gt;"",P25="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM25" s="9" t="str">
         <x:f>IF(A25="","",IF(AND(AK25="OK",J25="READY",F25&lt;&gt;"",G25&lt;&gt;"",K25&lt;&gt;"",S25="OK",OR(R25="PASS",R25="FAIL")),"YES","NO"))</x:f>
@@ -2281,7 +2281,7 @@
         <x:f>IF(A26="",IF(B26="","","MISSING_TEST_ID"),IF(B26="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A26,$B$2:$B$501,B26)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL26" s="9" t="str">
-        <x:f>IF(A26="","",IF(AND(AK26="OK",J26="READY",F26&lt;&gt;"",G26&lt;&gt;"",K26&lt;&gt;"",OR(L26="PASS",L26="FAIL"),M26&lt;&gt;"",O26&lt;&gt;"",P26="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A26="","",IF(AND(AK26="OK",J26="READY",F26&lt;&gt;"",G26&lt;&gt;"",K26&lt;&gt;"",OR(L26="PASS",L26="FAIL"),M26&lt;&gt;"",P26="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM26" s="9" t="str">
         <x:f>IF(A26="","",IF(AND(AK26="OK",J26="READY",F26&lt;&gt;"",G26&lt;&gt;"",K26&lt;&gt;"",S26="OK",OR(R26="PASS",R26="FAIL")),"YES","NO"))</x:f>
@@ -2333,7 +2333,7 @@
         <x:f>IF(A27="",IF(B27="","","MISSING_TEST_ID"),IF(B27="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A27,$B$2:$B$501,B27)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL27" s="9" t="str">
-        <x:f>IF(A27="","",IF(AND(AK27="OK",J27="READY",F27&lt;&gt;"",G27&lt;&gt;"",K27&lt;&gt;"",OR(L27="PASS",L27="FAIL"),M27&lt;&gt;"",O27&lt;&gt;"",P27="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A27="","",IF(AND(AK27="OK",J27="READY",F27&lt;&gt;"",G27&lt;&gt;"",K27&lt;&gt;"",OR(L27="PASS",L27="FAIL"),M27&lt;&gt;"",P27="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM27" s="9" t="str">
         <x:f>IF(A27="","",IF(AND(AK27="OK",J27="READY",F27&lt;&gt;"",G27&lt;&gt;"",K27&lt;&gt;"",S27="OK",OR(R27="PASS",R27="FAIL")),"YES","NO"))</x:f>
@@ -2385,7 +2385,7 @@
         <x:f>IF(A28="",IF(B28="","","MISSING_TEST_ID"),IF(B28="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A28,$B$2:$B$501,B28)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL28" s="9" t="str">
-        <x:f>IF(A28="","",IF(AND(AK28="OK",J28="READY",F28&lt;&gt;"",G28&lt;&gt;"",K28&lt;&gt;"",OR(L28="PASS",L28="FAIL"),M28&lt;&gt;"",O28&lt;&gt;"",P28="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A28="","",IF(AND(AK28="OK",J28="READY",F28&lt;&gt;"",G28&lt;&gt;"",K28&lt;&gt;"",OR(L28="PASS",L28="FAIL"),M28&lt;&gt;"",P28="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM28" s="9" t="str">
         <x:f>IF(A28="","",IF(AND(AK28="OK",J28="READY",F28&lt;&gt;"",G28&lt;&gt;"",K28&lt;&gt;"",S28="OK",OR(R28="PASS",R28="FAIL")),"YES","NO"))</x:f>
@@ -2437,7 +2437,7 @@
         <x:f>IF(A29="",IF(B29="","","MISSING_TEST_ID"),IF(B29="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A29,$B$2:$B$501,B29)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL29" s="9" t="str">
-        <x:f>IF(A29="","",IF(AND(AK29="OK",J29="READY",F29&lt;&gt;"",G29&lt;&gt;"",K29&lt;&gt;"",OR(L29="PASS",L29="FAIL"),M29&lt;&gt;"",O29&lt;&gt;"",P29="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A29="","",IF(AND(AK29="OK",J29="READY",F29&lt;&gt;"",G29&lt;&gt;"",K29&lt;&gt;"",OR(L29="PASS",L29="FAIL"),M29&lt;&gt;"",P29="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM29" s="9" t="str">
         <x:f>IF(A29="","",IF(AND(AK29="OK",J29="READY",F29&lt;&gt;"",G29&lt;&gt;"",K29&lt;&gt;"",S29="OK",OR(R29="PASS",R29="FAIL")),"YES","NO"))</x:f>
@@ -2489,7 +2489,7 @@
         <x:f>IF(A30="",IF(B30="","","MISSING_TEST_ID"),IF(B30="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A30,$B$2:$B$501,B30)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL30" s="9" t="str">
-        <x:f>IF(A30="","",IF(AND(AK30="OK",J30="READY",F30&lt;&gt;"",G30&lt;&gt;"",K30&lt;&gt;"",OR(L30="PASS",L30="FAIL"),M30&lt;&gt;"",O30&lt;&gt;"",P30="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A30="","",IF(AND(AK30="OK",J30="READY",F30&lt;&gt;"",G30&lt;&gt;"",K30&lt;&gt;"",OR(L30="PASS",L30="FAIL"),M30&lt;&gt;"",P30="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM30" s="9" t="str">
         <x:f>IF(A30="","",IF(AND(AK30="OK",J30="READY",F30&lt;&gt;"",G30&lt;&gt;"",K30&lt;&gt;"",S30="OK",OR(R30="PASS",R30="FAIL")),"YES","NO"))</x:f>
@@ -2541,7 +2541,7 @@
         <x:f>IF(A31="",IF(B31="","","MISSING_TEST_ID"),IF(B31="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A31,$B$2:$B$501,B31)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL31" s="9" t="str">
-        <x:f>IF(A31="","",IF(AND(AK31="OK",J31="READY",F31&lt;&gt;"",G31&lt;&gt;"",K31&lt;&gt;"",OR(L31="PASS",L31="FAIL"),M31&lt;&gt;"",O31&lt;&gt;"",P31="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A31="","",IF(AND(AK31="OK",J31="READY",F31&lt;&gt;"",G31&lt;&gt;"",K31&lt;&gt;"",OR(L31="PASS",L31="FAIL"),M31&lt;&gt;"",P31="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM31" s="9" t="str">
         <x:f>IF(A31="","",IF(AND(AK31="OK",J31="READY",F31&lt;&gt;"",G31&lt;&gt;"",K31&lt;&gt;"",S31="OK",OR(R31="PASS",R31="FAIL")),"YES","NO"))</x:f>
@@ -2593,7 +2593,7 @@
         <x:f>IF(A32="",IF(B32="","","MISSING_TEST_ID"),IF(B32="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A32,$B$2:$B$501,B32)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL32" s="9" t="str">
-        <x:f>IF(A32="","",IF(AND(AK32="OK",J32="READY",F32&lt;&gt;"",G32&lt;&gt;"",K32&lt;&gt;"",OR(L32="PASS",L32="FAIL"),M32&lt;&gt;"",O32&lt;&gt;"",P32="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A32="","",IF(AND(AK32="OK",J32="READY",F32&lt;&gt;"",G32&lt;&gt;"",K32&lt;&gt;"",OR(L32="PASS",L32="FAIL"),M32&lt;&gt;"",P32="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM32" s="9" t="str">
         <x:f>IF(A32="","",IF(AND(AK32="OK",J32="READY",F32&lt;&gt;"",G32&lt;&gt;"",K32&lt;&gt;"",S32="OK",OR(R32="PASS",R32="FAIL")),"YES","NO"))</x:f>
@@ -2645,7 +2645,7 @@
         <x:f>IF(A33="",IF(B33="","","MISSING_TEST_ID"),IF(B33="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A33,$B$2:$B$501,B33)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL33" s="9" t="str">
-        <x:f>IF(A33="","",IF(AND(AK33="OK",J33="READY",F33&lt;&gt;"",G33&lt;&gt;"",K33&lt;&gt;"",OR(L33="PASS",L33="FAIL"),M33&lt;&gt;"",O33&lt;&gt;"",P33="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A33="","",IF(AND(AK33="OK",J33="READY",F33&lt;&gt;"",G33&lt;&gt;"",K33&lt;&gt;"",OR(L33="PASS",L33="FAIL"),M33&lt;&gt;"",P33="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM33" s="9" t="str">
         <x:f>IF(A33="","",IF(AND(AK33="OK",J33="READY",F33&lt;&gt;"",G33&lt;&gt;"",K33&lt;&gt;"",S33="OK",OR(R33="PASS",R33="FAIL")),"YES","NO"))</x:f>
@@ -2697,7 +2697,7 @@
         <x:f>IF(A34="",IF(B34="","","MISSING_TEST_ID"),IF(B34="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A34,$B$2:$B$501,B34)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL34" s="9" t="str">
-        <x:f>IF(A34="","",IF(AND(AK34="OK",J34="READY",F34&lt;&gt;"",G34&lt;&gt;"",K34&lt;&gt;"",OR(L34="PASS",L34="FAIL"),M34&lt;&gt;"",O34&lt;&gt;"",P34="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A34="","",IF(AND(AK34="OK",J34="READY",F34&lt;&gt;"",G34&lt;&gt;"",K34&lt;&gt;"",OR(L34="PASS",L34="FAIL"),M34&lt;&gt;"",P34="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM34" s="9" t="str">
         <x:f>IF(A34="","",IF(AND(AK34="OK",J34="READY",F34&lt;&gt;"",G34&lt;&gt;"",K34&lt;&gt;"",S34="OK",OR(R34="PASS",R34="FAIL")),"YES","NO"))</x:f>
@@ -2749,7 +2749,7 @@
         <x:f>IF(A35="",IF(B35="","","MISSING_TEST_ID"),IF(B35="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A35,$B$2:$B$501,B35)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL35" s="9" t="str">
-        <x:f>IF(A35="","",IF(AND(AK35="OK",J35="READY",F35&lt;&gt;"",G35&lt;&gt;"",K35&lt;&gt;"",OR(L35="PASS",L35="FAIL"),M35&lt;&gt;"",O35&lt;&gt;"",P35="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A35="","",IF(AND(AK35="OK",J35="READY",F35&lt;&gt;"",G35&lt;&gt;"",K35&lt;&gt;"",OR(L35="PASS",L35="FAIL"),M35&lt;&gt;"",P35="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM35" s="9" t="str">
         <x:f>IF(A35="","",IF(AND(AK35="OK",J35="READY",F35&lt;&gt;"",G35&lt;&gt;"",K35&lt;&gt;"",S35="OK",OR(R35="PASS",R35="FAIL")),"YES","NO"))</x:f>
@@ -2801,7 +2801,7 @@
         <x:f>IF(A36="",IF(B36="","","MISSING_TEST_ID"),IF(B36="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A36,$B$2:$B$501,B36)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL36" s="9" t="str">
-        <x:f>IF(A36="","",IF(AND(AK36="OK",J36="READY",F36&lt;&gt;"",G36&lt;&gt;"",K36&lt;&gt;"",OR(L36="PASS",L36="FAIL"),M36&lt;&gt;"",O36&lt;&gt;"",P36="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A36="","",IF(AND(AK36="OK",J36="READY",F36&lt;&gt;"",G36&lt;&gt;"",K36&lt;&gt;"",OR(L36="PASS",L36="FAIL"),M36&lt;&gt;"",P36="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM36" s="9" t="str">
         <x:f>IF(A36="","",IF(AND(AK36="OK",J36="READY",F36&lt;&gt;"",G36&lt;&gt;"",K36&lt;&gt;"",S36="OK",OR(R36="PASS",R36="FAIL")),"YES","NO"))</x:f>
@@ -2853,7 +2853,7 @@
         <x:f>IF(A37="",IF(B37="","","MISSING_TEST_ID"),IF(B37="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A37,$B$2:$B$501,B37)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL37" s="9" t="str">
-        <x:f>IF(A37="","",IF(AND(AK37="OK",J37="READY",F37&lt;&gt;"",G37&lt;&gt;"",K37&lt;&gt;"",OR(L37="PASS",L37="FAIL"),M37&lt;&gt;"",O37&lt;&gt;"",P37="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A37="","",IF(AND(AK37="OK",J37="READY",F37&lt;&gt;"",G37&lt;&gt;"",K37&lt;&gt;"",OR(L37="PASS",L37="FAIL"),M37&lt;&gt;"",P37="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM37" s="9" t="str">
         <x:f>IF(A37="","",IF(AND(AK37="OK",J37="READY",F37&lt;&gt;"",G37&lt;&gt;"",K37&lt;&gt;"",S37="OK",OR(R37="PASS",R37="FAIL")),"YES","NO"))</x:f>
@@ -2905,7 +2905,7 @@
         <x:f>IF(A38="",IF(B38="","","MISSING_TEST_ID"),IF(B38="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A38,$B$2:$B$501,B38)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL38" s="9" t="str">
-        <x:f>IF(A38="","",IF(AND(AK38="OK",J38="READY",F38&lt;&gt;"",G38&lt;&gt;"",K38&lt;&gt;"",OR(L38="PASS",L38="FAIL"),M38&lt;&gt;"",O38&lt;&gt;"",P38="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A38="","",IF(AND(AK38="OK",J38="READY",F38&lt;&gt;"",G38&lt;&gt;"",K38&lt;&gt;"",OR(L38="PASS",L38="FAIL"),M38&lt;&gt;"",P38="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM38" s="9" t="str">
         <x:f>IF(A38="","",IF(AND(AK38="OK",J38="READY",F38&lt;&gt;"",G38&lt;&gt;"",K38&lt;&gt;"",S38="OK",OR(R38="PASS",R38="FAIL")),"YES","NO"))</x:f>
@@ -2957,7 +2957,7 @@
         <x:f>IF(A39="",IF(B39="","","MISSING_TEST_ID"),IF(B39="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A39,$B$2:$B$501,B39)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL39" s="9" t="str">
-        <x:f>IF(A39="","",IF(AND(AK39="OK",J39="READY",F39&lt;&gt;"",G39&lt;&gt;"",K39&lt;&gt;"",OR(L39="PASS",L39="FAIL"),M39&lt;&gt;"",O39&lt;&gt;"",P39="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A39="","",IF(AND(AK39="OK",J39="READY",F39&lt;&gt;"",G39&lt;&gt;"",K39&lt;&gt;"",OR(L39="PASS",L39="FAIL"),M39&lt;&gt;"",P39="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM39" s="9" t="str">
         <x:f>IF(A39="","",IF(AND(AK39="OK",J39="READY",F39&lt;&gt;"",G39&lt;&gt;"",K39&lt;&gt;"",S39="OK",OR(R39="PASS",R39="FAIL")),"YES","NO"))</x:f>
@@ -3009,7 +3009,7 @@
         <x:f>IF(A40="",IF(B40="","","MISSING_TEST_ID"),IF(B40="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A40,$B$2:$B$501,B40)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL40" s="9" t="str">
-        <x:f>IF(A40="","",IF(AND(AK40="OK",J40="READY",F40&lt;&gt;"",G40&lt;&gt;"",K40&lt;&gt;"",OR(L40="PASS",L40="FAIL"),M40&lt;&gt;"",O40&lt;&gt;"",P40="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A40="","",IF(AND(AK40="OK",J40="READY",F40&lt;&gt;"",G40&lt;&gt;"",K40&lt;&gt;"",OR(L40="PASS",L40="FAIL"),M40&lt;&gt;"",P40="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM40" s="9" t="str">
         <x:f>IF(A40="","",IF(AND(AK40="OK",J40="READY",F40&lt;&gt;"",G40&lt;&gt;"",K40&lt;&gt;"",S40="OK",OR(R40="PASS",R40="FAIL")),"YES","NO"))</x:f>
@@ -3061,7 +3061,7 @@
         <x:f>IF(A41="",IF(B41="","","MISSING_TEST_ID"),IF(B41="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A41,$B$2:$B$501,B41)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL41" s="9" t="str">
-        <x:f>IF(A41="","",IF(AND(AK41="OK",J41="READY",F41&lt;&gt;"",G41&lt;&gt;"",K41&lt;&gt;"",OR(L41="PASS",L41="FAIL"),M41&lt;&gt;"",O41&lt;&gt;"",P41="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A41="","",IF(AND(AK41="OK",J41="READY",F41&lt;&gt;"",G41&lt;&gt;"",K41&lt;&gt;"",OR(L41="PASS",L41="FAIL"),M41&lt;&gt;"",P41="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM41" s="9" t="str">
         <x:f>IF(A41="","",IF(AND(AK41="OK",J41="READY",F41&lt;&gt;"",G41&lt;&gt;"",K41&lt;&gt;"",S41="OK",OR(R41="PASS",R41="FAIL")),"YES","NO"))</x:f>
@@ -3113,7 +3113,7 @@
         <x:f>IF(A42="",IF(B42="","","MISSING_TEST_ID"),IF(B42="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A42,$B$2:$B$501,B42)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL42" s="9" t="str">
-        <x:f>IF(A42="","",IF(AND(AK42="OK",J42="READY",F42&lt;&gt;"",G42&lt;&gt;"",K42&lt;&gt;"",OR(L42="PASS",L42="FAIL"),M42&lt;&gt;"",O42&lt;&gt;"",P42="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A42="","",IF(AND(AK42="OK",J42="READY",F42&lt;&gt;"",G42&lt;&gt;"",K42&lt;&gt;"",OR(L42="PASS",L42="FAIL"),M42&lt;&gt;"",P42="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM42" s="9" t="str">
         <x:f>IF(A42="","",IF(AND(AK42="OK",J42="READY",F42&lt;&gt;"",G42&lt;&gt;"",K42&lt;&gt;"",S42="OK",OR(R42="PASS",R42="FAIL")),"YES","NO"))</x:f>
@@ -3165,7 +3165,7 @@
         <x:f>IF(A43="",IF(B43="","","MISSING_TEST_ID"),IF(B43="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A43,$B$2:$B$501,B43)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL43" s="9" t="str">
-        <x:f>IF(A43="","",IF(AND(AK43="OK",J43="READY",F43&lt;&gt;"",G43&lt;&gt;"",K43&lt;&gt;"",OR(L43="PASS",L43="FAIL"),M43&lt;&gt;"",O43&lt;&gt;"",P43="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A43="","",IF(AND(AK43="OK",J43="READY",F43&lt;&gt;"",G43&lt;&gt;"",K43&lt;&gt;"",OR(L43="PASS",L43="FAIL"),M43&lt;&gt;"",P43="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM43" s="9" t="str">
         <x:f>IF(A43="","",IF(AND(AK43="OK",J43="READY",F43&lt;&gt;"",G43&lt;&gt;"",K43&lt;&gt;"",S43="OK",OR(R43="PASS",R43="FAIL")),"YES","NO"))</x:f>
@@ -3217,7 +3217,7 @@
         <x:f>IF(A44="",IF(B44="","","MISSING_TEST_ID"),IF(B44="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A44,$B$2:$B$501,B44)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL44" s="9" t="str">
-        <x:f>IF(A44="","",IF(AND(AK44="OK",J44="READY",F44&lt;&gt;"",G44&lt;&gt;"",K44&lt;&gt;"",OR(L44="PASS",L44="FAIL"),M44&lt;&gt;"",O44&lt;&gt;"",P44="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A44="","",IF(AND(AK44="OK",J44="READY",F44&lt;&gt;"",G44&lt;&gt;"",K44&lt;&gt;"",OR(L44="PASS",L44="FAIL"),M44&lt;&gt;"",P44="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM44" s="9" t="str">
         <x:f>IF(A44="","",IF(AND(AK44="OK",J44="READY",F44&lt;&gt;"",G44&lt;&gt;"",K44&lt;&gt;"",S44="OK",OR(R44="PASS",R44="FAIL")),"YES","NO"))</x:f>
@@ -3269,7 +3269,7 @@
         <x:f>IF(A45="",IF(B45="","","MISSING_TEST_ID"),IF(B45="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A45,$B$2:$B$501,B45)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL45" s="9" t="str">
-        <x:f>IF(A45="","",IF(AND(AK45="OK",J45="READY",F45&lt;&gt;"",G45&lt;&gt;"",K45&lt;&gt;"",OR(L45="PASS",L45="FAIL"),M45&lt;&gt;"",O45&lt;&gt;"",P45="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A45="","",IF(AND(AK45="OK",J45="READY",F45&lt;&gt;"",G45&lt;&gt;"",K45&lt;&gt;"",OR(L45="PASS",L45="FAIL"),M45&lt;&gt;"",P45="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM45" s="9" t="str">
         <x:f>IF(A45="","",IF(AND(AK45="OK",J45="READY",F45&lt;&gt;"",G45&lt;&gt;"",K45&lt;&gt;"",S45="OK",OR(R45="PASS",R45="FAIL")),"YES","NO"))</x:f>
@@ -3321,7 +3321,7 @@
         <x:f>IF(A46="",IF(B46="","","MISSING_TEST_ID"),IF(B46="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A46,$B$2:$B$501,B46)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL46" s="9" t="str">
-        <x:f>IF(A46="","",IF(AND(AK46="OK",J46="READY",F46&lt;&gt;"",G46&lt;&gt;"",K46&lt;&gt;"",OR(L46="PASS",L46="FAIL"),M46&lt;&gt;"",O46&lt;&gt;"",P46="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A46="","",IF(AND(AK46="OK",J46="READY",F46&lt;&gt;"",G46&lt;&gt;"",K46&lt;&gt;"",OR(L46="PASS",L46="FAIL"),M46&lt;&gt;"",P46="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM46" s="9" t="str">
         <x:f>IF(A46="","",IF(AND(AK46="OK",J46="READY",F46&lt;&gt;"",G46&lt;&gt;"",K46&lt;&gt;"",S46="OK",OR(R46="PASS",R46="FAIL")),"YES","NO"))</x:f>
@@ -3373,7 +3373,7 @@
         <x:f>IF(A47="",IF(B47="","","MISSING_TEST_ID"),IF(B47="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A47,$B$2:$B$501,B47)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL47" s="9" t="str">
-        <x:f>IF(A47="","",IF(AND(AK47="OK",J47="READY",F47&lt;&gt;"",G47&lt;&gt;"",K47&lt;&gt;"",OR(L47="PASS",L47="FAIL"),M47&lt;&gt;"",O47&lt;&gt;"",P47="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A47="","",IF(AND(AK47="OK",J47="READY",F47&lt;&gt;"",G47&lt;&gt;"",K47&lt;&gt;"",OR(L47="PASS",L47="FAIL"),M47&lt;&gt;"",P47="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM47" s="9" t="str">
         <x:f>IF(A47="","",IF(AND(AK47="OK",J47="READY",F47&lt;&gt;"",G47&lt;&gt;"",K47&lt;&gt;"",S47="OK",OR(R47="PASS",R47="FAIL")),"YES","NO"))</x:f>
@@ -3425,7 +3425,7 @@
         <x:f>IF(A48="",IF(B48="","","MISSING_TEST_ID"),IF(B48="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A48,$B$2:$B$501,B48)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL48" s="9" t="str">
-        <x:f>IF(A48="","",IF(AND(AK48="OK",J48="READY",F48&lt;&gt;"",G48&lt;&gt;"",K48&lt;&gt;"",OR(L48="PASS",L48="FAIL"),M48&lt;&gt;"",O48&lt;&gt;"",P48="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A48="","",IF(AND(AK48="OK",J48="READY",F48&lt;&gt;"",G48&lt;&gt;"",K48&lt;&gt;"",OR(L48="PASS",L48="FAIL"),M48&lt;&gt;"",P48="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM48" s="9" t="str">
         <x:f>IF(A48="","",IF(AND(AK48="OK",J48="READY",F48&lt;&gt;"",G48&lt;&gt;"",K48&lt;&gt;"",S48="OK",OR(R48="PASS",R48="FAIL")),"YES","NO"))</x:f>
@@ -3477,7 +3477,7 @@
         <x:f>IF(A49="",IF(B49="","","MISSING_TEST_ID"),IF(B49="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A49,$B$2:$B$501,B49)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL49" s="9" t="str">
-        <x:f>IF(A49="","",IF(AND(AK49="OK",J49="READY",F49&lt;&gt;"",G49&lt;&gt;"",K49&lt;&gt;"",OR(L49="PASS",L49="FAIL"),M49&lt;&gt;"",O49&lt;&gt;"",P49="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A49="","",IF(AND(AK49="OK",J49="READY",F49&lt;&gt;"",G49&lt;&gt;"",K49&lt;&gt;"",OR(L49="PASS",L49="FAIL"),M49&lt;&gt;"",P49="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM49" s="9" t="str">
         <x:f>IF(A49="","",IF(AND(AK49="OK",J49="READY",F49&lt;&gt;"",G49&lt;&gt;"",K49&lt;&gt;"",S49="OK",OR(R49="PASS",R49="FAIL")),"YES","NO"))</x:f>
@@ -3529,7 +3529,7 @@
         <x:f>IF(A50="",IF(B50="","","MISSING_TEST_ID"),IF(B50="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A50,$B$2:$B$501,B50)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL50" s="9" t="str">
-        <x:f>IF(A50="","",IF(AND(AK50="OK",J50="READY",F50&lt;&gt;"",G50&lt;&gt;"",K50&lt;&gt;"",OR(L50="PASS",L50="FAIL"),M50&lt;&gt;"",O50&lt;&gt;"",P50="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A50="","",IF(AND(AK50="OK",J50="READY",F50&lt;&gt;"",G50&lt;&gt;"",K50&lt;&gt;"",OR(L50="PASS",L50="FAIL"),M50&lt;&gt;"",P50="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM50" s="9" t="str">
         <x:f>IF(A50="","",IF(AND(AK50="OK",J50="READY",F50&lt;&gt;"",G50&lt;&gt;"",K50&lt;&gt;"",S50="OK",OR(R50="PASS",R50="FAIL")),"YES","NO"))</x:f>
@@ -3581,7 +3581,7 @@
         <x:f>IF(A51="",IF(B51="","","MISSING_TEST_ID"),IF(B51="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A51,$B$2:$B$501,B51)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL51" s="9" t="str">
-        <x:f>IF(A51="","",IF(AND(AK51="OK",J51="READY",F51&lt;&gt;"",G51&lt;&gt;"",K51&lt;&gt;"",OR(L51="PASS",L51="FAIL"),M51&lt;&gt;"",O51&lt;&gt;"",P51="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A51="","",IF(AND(AK51="OK",J51="READY",F51&lt;&gt;"",G51&lt;&gt;"",K51&lt;&gt;"",OR(L51="PASS",L51="FAIL"),M51&lt;&gt;"",P51="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM51" s="9" t="str">
         <x:f>IF(A51="","",IF(AND(AK51="OK",J51="READY",F51&lt;&gt;"",G51&lt;&gt;"",K51&lt;&gt;"",S51="OK",OR(R51="PASS",R51="FAIL")),"YES","NO"))</x:f>
@@ -3633,7 +3633,7 @@
         <x:f>IF(A52="",IF(B52="","","MISSING_TEST_ID"),IF(B52="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A52,$B$2:$B$501,B52)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL52" s="9" t="str">
-        <x:f>IF(A52="","",IF(AND(AK52="OK",J52="READY",F52&lt;&gt;"",G52&lt;&gt;"",K52&lt;&gt;"",OR(L52="PASS",L52="FAIL"),M52&lt;&gt;"",O52&lt;&gt;"",P52="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A52="","",IF(AND(AK52="OK",J52="READY",F52&lt;&gt;"",G52&lt;&gt;"",K52&lt;&gt;"",OR(L52="PASS",L52="FAIL"),M52&lt;&gt;"",P52="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM52" s="9" t="str">
         <x:f>IF(A52="","",IF(AND(AK52="OK",J52="READY",F52&lt;&gt;"",G52&lt;&gt;"",K52&lt;&gt;"",S52="OK",OR(R52="PASS",R52="FAIL")),"YES","NO"))</x:f>
@@ -3685,7 +3685,7 @@
         <x:f>IF(A53="",IF(B53="","","MISSING_TEST_ID"),IF(B53="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A53,$B$2:$B$501,B53)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL53" s="9" t="str">
-        <x:f>IF(A53="","",IF(AND(AK53="OK",J53="READY",F53&lt;&gt;"",G53&lt;&gt;"",K53&lt;&gt;"",OR(L53="PASS",L53="FAIL"),M53&lt;&gt;"",O53&lt;&gt;"",P53="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A53="","",IF(AND(AK53="OK",J53="READY",F53&lt;&gt;"",G53&lt;&gt;"",K53&lt;&gt;"",OR(L53="PASS",L53="FAIL"),M53&lt;&gt;"",P53="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM53" s="9" t="str">
         <x:f>IF(A53="","",IF(AND(AK53="OK",J53="READY",F53&lt;&gt;"",G53&lt;&gt;"",K53&lt;&gt;"",S53="OK",OR(R53="PASS",R53="FAIL")),"YES","NO"))</x:f>
@@ -3737,7 +3737,7 @@
         <x:f>IF(A54="",IF(B54="","","MISSING_TEST_ID"),IF(B54="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A54,$B$2:$B$501,B54)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL54" s="9" t="str">
-        <x:f>IF(A54="","",IF(AND(AK54="OK",J54="READY",F54&lt;&gt;"",G54&lt;&gt;"",K54&lt;&gt;"",OR(L54="PASS",L54="FAIL"),M54&lt;&gt;"",O54&lt;&gt;"",P54="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A54="","",IF(AND(AK54="OK",J54="READY",F54&lt;&gt;"",G54&lt;&gt;"",K54&lt;&gt;"",OR(L54="PASS",L54="FAIL"),M54&lt;&gt;"",P54="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM54" s="9" t="str">
         <x:f>IF(A54="","",IF(AND(AK54="OK",J54="READY",F54&lt;&gt;"",G54&lt;&gt;"",K54&lt;&gt;"",S54="OK",OR(R54="PASS",R54="FAIL")),"YES","NO"))</x:f>
@@ -3789,7 +3789,7 @@
         <x:f>IF(A55="",IF(B55="","","MISSING_TEST_ID"),IF(B55="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A55,$B$2:$B$501,B55)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL55" s="9" t="str">
-        <x:f>IF(A55="","",IF(AND(AK55="OK",J55="READY",F55&lt;&gt;"",G55&lt;&gt;"",K55&lt;&gt;"",OR(L55="PASS",L55="FAIL"),M55&lt;&gt;"",O55&lt;&gt;"",P55="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A55="","",IF(AND(AK55="OK",J55="READY",F55&lt;&gt;"",G55&lt;&gt;"",K55&lt;&gt;"",OR(L55="PASS",L55="FAIL"),M55&lt;&gt;"",P55="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM55" s="9" t="str">
         <x:f>IF(A55="","",IF(AND(AK55="OK",J55="READY",F55&lt;&gt;"",G55&lt;&gt;"",K55&lt;&gt;"",S55="OK",OR(R55="PASS",R55="FAIL")),"YES","NO"))</x:f>
@@ -3841,7 +3841,7 @@
         <x:f>IF(A56="",IF(B56="","","MISSING_TEST_ID"),IF(B56="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A56,$B$2:$B$501,B56)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL56" s="9" t="str">
-        <x:f>IF(A56="","",IF(AND(AK56="OK",J56="READY",F56&lt;&gt;"",G56&lt;&gt;"",K56&lt;&gt;"",OR(L56="PASS",L56="FAIL"),M56&lt;&gt;"",O56&lt;&gt;"",P56="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A56="","",IF(AND(AK56="OK",J56="READY",F56&lt;&gt;"",G56&lt;&gt;"",K56&lt;&gt;"",OR(L56="PASS",L56="FAIL"),M56&lt;&gt;"",P56="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM56" s="9" t="str">
         <x:f>IF(A56="","",IF(AND(AK56="OK",J56="READY",F56&lt;&gt;"",G56&lt;&gt;"",K56&lt;&gt;"",S56="OK",OR(R56="PASS",R56="FAIL")),"YES","NO"))</x:f>
@@ -3893,7 +3893,7 @@
         <x:f>IF(A57="",IF(B57="","","MISSING_TEST_ID"),IF(B57="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A57,$B$2:$B$501,B57)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL57" s="9" t="str">
-        <x:f>IF(A57="","",IF(AND(AK57="OK",J57="READY",F57&lt;&gt;"",G57&lt;&gt;"",K57&lt;&gt;"",OR(L57="PASS",L57="FAIL"),M57&lt;&gt;"",O57&lt;&gt;"",P57="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A57="","",IF(AND(AK57="OK",J57="READY",F57&lt;&gt;"",G57&lt;&gt;"",K57&lt;&gt;"",OR(L57="PASS",L57="FAIL"),M57&lt;&gt;"",P57="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM57" s="9" t="str">
         <x:f>IF(A57="","",IF(AND(AK57="OK",J57="READY",F57&lt;&gt;"",G57&lt;&gt;"",K57&lt;&gt;"",S57="OK",OR(R57="PASS",R57="FAIL")),"YES","NO"))</x:f>
@@ -3945,7 +3945,7 @@
         <x:f>IF(A58="",IF(B58="","","MISSING_TEST_ID"),IF(B58="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A58,$B$2:$B$501,B58)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL58" s="9" t="str">
-        <x:f>IF(A58="","",IF(AND(AK58="OK",J58="READY",F58&lt;&gt;"",G58&lt;&gt;"",K58&lt;&gt;"",OR(L58="PASS",L58="FAIL"),M58&lt;&gt;"",O58&lt;&gt;"",P58="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A58="","",IF(AND(AK58="OK",J58="READY",F58&lt;&gt;"",G58&lt;&gt;"",K58&lt;&gt;"",OR(L58="PASS",L58="FAIL"),M58&lt;&gt;"",P58="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM58" s="9" t="str">
         <x:f>IF(A58="","",IF(AND(AK58="OK",J58="READY",F58&lt;&gt;"",G58&lt;&gt;"",K58&lt;&gt;"",S58="OK",OR(R58="PASS",R58="FAIL")),"YES","NO"))</x:f>
@@ -3997,7 +3997,7 @@
         <x:f>IF(A59="",IF(B59="","","MISSING_TEST_ID"),IF(B59="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A59,$B$2:$B$501,B59)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL59" s="9" t="str">
-        <x:f>IF(A59="","",IF(AND(AK59="OK",J59="READY",F59&lt;&gt;"",G59&lt;&gt;"",K59&lt;&gt;"",OR(L59="PASS",L59="FAIL"),M59&lt;&gt;"",O59&lt;&gt;"",P59="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A59="","",IF(AND(AK59="OK",J59="READY",F59&lt;&gt;"",G59&lt;&gt;"",K59&lt;&gt;"",OR(L59="PASS",L59="FAIL"),M59&lt;&gt;"",P59="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM59" s="9" t="str">
         <x:f>IF(A59="","",IF(AND(AK59="OK",J59="READY",F59&lt;&gt;"",G59&lt;&gt;"",K59&lt;&gt;"",S59="OK",OR(R59="PASS",R59="FAIL")),"YES","NO"))</x:f>
@@ -4049,7 +4049,7 @@
         <x:f>IF(A60="",IF(B60="","","MISSING_TEST_ID"),IF(B60="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A60,$B$2:$B$501,B60)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL60" s="9" t="str">
-        <x:f>IF(A60="","",IF(AND(AK60="OK",J60="READY",F60&lt;&gt;"",G60&lt;&gt;"",K60&lt;&gt;"",OR(L60="PASS",L60="FAIL"),M60&lt;&gt;"",O60&lt;&gt;"",P60="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A60="","",IF(AND(AK60="OK",J60="READY",F60&lt;&gt;"",G60&lt;&gt;"",K60&lt;&gt;"",OR(L60="PASS",L60="FAIL"),M60&lt;&gt;"",P60="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM60" s="9" t="str">
         <x:f>IF(A60="","",IF(AND(AK60="OK",J60="READY",F60&lt;&gt;"",G60&lt;&gt;"",K60&lt;&gt;"",S60="OK",OR(R60="PASS",R60="FAIL")),"YES","NO"))</x:f>
@@ -4101,7 +4101,7 @@
         <x:f>IF(A61="",IF(B61="","","MISSING_TEST_ID"),IF(B61="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A61,$B$2:$B$501,B61)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL61" s="9" t="str">
-        <x:f>IF(A61="","",IF(AND(AK61="OK",J61="READY",F61&lt;&gt;"",G61&lt;&gt;"",K61&lt;&gt;"",OR(L61="PASS",L61="FAIL"),M61&lt;&gt;"",O61&lt;&gt;"",P61="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A61="","",IF(AND(AK61="OK",J61="READY",F61&lt;&gt;"",G61&lt;&gt;"",K61&lt;&gt;"",OR(L61="PASS",L61="FAIL"),M61&lt;&gt;"",P61="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM61" s="9" t="str">
         <x:f>IF(A61="","",IF(AND(AK61="OK",J61="READY",F61&lt;&gt;"",G61&lt;&gt;"",K61&lt;&gt;"",S61="OK",OR(R61="PASS",R61="FAIL")),"YES","NO"))</x:f>
@@ -4153,7 +4153,7 @@
         <x:f>IF(A62="",IF(B62="","","MISSING_TEST_ID"),IF(B62="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A62,$B$2:$B$501,B62)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL62" s="9" t="str">
-        <x:f>IF(A62="","",IF(AND(AK62="OK",J62="READY",F62&lt;&gt;"",G62&lt;&gt;"",K62&lt;&gt;"",OR(L62="PASS",L62="FAIL"),M62&lt;&gt;"",O62&lt;&gt;"",P62="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A62="","",IF(AND(AK62="OK",J62="READY",F62&lt;&gt;"",G62&lt;&gt;"",K62&lt;&gt;"",OR(L62="PASS",L62="FAIL"),M62&lt;&gt;"",P62="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM62" s="9" t="str">
         <x:f>IF(A62="","",IF(AND(AK62="OK",J62="READY",F62&lt;&gt;"",G62&lt;&gt;"",K62&lt;&gt;"",S62="OK",OR(R62="PASS",R62="FAIL")),"YES","NO"))</x:f>
@@ -4205,7 +4205,7 @@
         <x:f>IF(A63="",IF(B63="","","MISSING_TEST_ID"),IF(B63="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A63,$B$2:$B$501,B63)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL63" s="9" t="str">
-        <x:f>IF(A63="","",IF(AND(AK63="OK",J63="READY",F63&lt;&gt;"",G63&lt;&gt;"",K63&lt;&gt;"",OR(L63="PASS",L63="FAIL"),M63&lt;&gt;"",O63&lt;&gt;"",P63="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A63="","",IF(AND(AK63="OK",J63="READY",F63&lt;&gt;"",G63&lt;&gt;"",K63&lt;&gt;"",OR(L63="PASS",L63="FAIL"),M63&lt;&gt;"",P63="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM63" s="9" t="str">
         <x:f>IF(A63="","",IF(AND(AK63="OK",J63="READY",F63&lt;&gt;"",G63&lt;&gt;"",K63&lt;&gt;"",S63="OK",OR(R63="PASS",R63="FAIL")),"YES","NO"))</x:f>
@@ -4257,7 +4257,7 @@
         <x:f>IF(A64="",IF(B64="","","MISSING_TEST_ID"),IF(B64="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A64,$B$2:$B$501,B64)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL64" s="9" t="str">
-        <x:f>IF(A64="","",IF(AND(AK64="OK",J64="READY",F64&lt;&gt;"",G64&lt;&gt;"",K64&lt;&gt;"",OR(L64="PASS",L64="FAIL"),M64&lt;&gt;"",O64&lt;&gt;"",P64="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A64="","",IF(AND(AK64="OK",J64="READY",F64&lt;&gt;"",G64&lt;&gt;"",K64&lt;&gt;"",OR(L64="PASS",L64="FAIL"),M64&lt;&gt;"",P64="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM64" s="9" t="str">
         <x:f>IF(A64="","",IF(AND(AK64="OK",J64="READY",F64&lt;&gt;"",G64&lt;&gt;"",K64&lt;&gt;"",S64="OK",OR(R64="PASS",R64="FAIL")),"YES","NO"))</x:f>
@@ -4309,7 +4309,7 @@
         <x:f>IF(A65="",IF(B65="","","MISSING_TEST_ID"),IF(B65="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A65,$B$2:$B$501,B65)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL65" s="9" t="str">
-        <x:f>IF(A65="","",IF(AND(AK65="OK",J65="READY",F65&lt;&gt;"",G65&lt;&gt;"",K65&lt;&gt;"",OR(L65="PASS",L65="FAIL"),M65&lt;&gt;"",O65&lt;&gt;"",P65="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A65="","",IF(AND(AK65="OK",J65="READY",F65&lt;&gt;"",G65&lt;&gt;"",K65&lt;&gt;"",OR(L65="PASS",L65="FAIL"),M65&lt;&gt;"",P65="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM65" s="9" t="str">
         <x:f>IF(A65="","",IF(AND(AK65="OK",J65="READY",F65&lt;&gt;"",G65&lt;&gt;"",K65&lt;&gt;"",S65="OK",OR(R65="PASS",R65="FAIL")),"YES","NO"))</x:f>
@@ -4361,7 +4361,7 @@
         <x:f>IF(A66="",IF(B66="","","MISSING_TEST_ID"),IF(B66="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A66,$B$2:$B$501,B66)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL66" s="9" t="str">
-        <x:f>IF(A66="","",IF(AND(AK66="OK",J66="READY",F66&lt;&gt;"",G66&lt;&gt;"",K66&lt;&gt;"",OR(L66="PASS",L66="FAIL"),M66&lt;&gt;"",O66&lt;&gt;"",P66="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A66="","",IF(AND(AK66="OK",J66="READY",F66&lt;&gt;"",G66&lt;&gt;"",K66&lt;&gt;"",OR(L66="PASS",L66="FAIL"),M66&lt;&gt;"",P66="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM66" s="9" t="str">
         <x:f>IF(A66="","",IF(AND(AK66="OK",J66="READY",F66&lt;&gt;"",G66&lt;&gt;"",K66&lt;&gt;"",S66="OK",OR(R66="PASS",R66="FAIL")),"YES","NO"))</x:f>
@@ -4413,7 +4413,7 @@
         <x:f>IF(A67="",IF(B67="","","MISSING_TEST_ID"),IF(B67="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A67,$B$2:$B$501,B67)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL67" s="9" t="str">
-        <x:f>IF(A67="","",IF(AND(AK67="OK",J67="READY",F67&lt;&gt;"",G67&lt;&gt;"",K67&lt;&gt;"",OR(L67="PASS",L67="FAIL"),M67&lt;&gt;"",O67&lt;&gt;"",P67="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A67="","",IF(AND(AK67="OK",J67="READY",F67&lt;&gt;"",G67&lt;&gt;"",K67&lt;&gt;"",OR(L67="PASS",L67="FAIL"),M67&lt;&gt;"",P67="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM67" s="9" t="str">
         <x:f>IF(A67="","",IF(AND(AK67="OK",J67="READY",F67&lt;&gt;"",G67&lt;&gt;"",K67&lt;&gt;"",S67="OK",OR(R67="PASS",R67="FAIL")),"YES","NO"))</x:f>
@@ -4465,7 +4465,7 @@
         <x:f>IF(A68="",IF(B68="","","MISSING_TEST_ID"),IF(B68="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A68,$B$2:$B$501,B68)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL68" s="9" t="str">
-        <x:f>IF(A68="","",IF(AND(AK68="OK",J68="READY",F68&lt;&gt;"",G68&lt;&gt;"",K68&lt;&gt;"",OR(L68="PASS",L68="FAIL"),M68&lt;&gt;"",O68&lt;&gt;"",P68="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A68="","",IF(AND(AK68="OK",J68="READY",F68&lt;&gt;"",G68&lt;&gt;"",K68&lt;&gt;"",OR(L68="PASS",L68="FAIL"),M68&lt;&gt;"",P68="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM68" s="9" t="str">
         <x:f>IF(A68="","",IF(AND(AK68="OK",J68="READY",F68&lt;&gt;"",G68&lt;&gt;"",K68&lt;&gt;"",S68="OK",OR(R68="PASS",R68="FAIL")),"YES","NO"))</x:f>
@@ -4517,7 +4517,7 @@
         <x:f>IF(A69="",IF(B69="","","MISSING_TEST_ID"),IF(B69="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A69,$B$2:$B$501,B69)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL69" s="9" t="str">
-        <x:f>IF(A69="","",IF(AND(AK69="OK",J69="READY",F69&lt;&gt;"",G69&lt;&gt;"",K69&lt;&gt;"",OR(L69="PASS",L69="FAIL"),M69&lt;&gt;"",O69&lt;&gt;"",P69="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A69="","",IF(AND(AK69="OK",J69="READY",F69&lt;&gt;"",G69&lt;&gt;"",K69&lt;&gt;"",OR(L69="PASS",L69="FAIL"),M69&lt;&gt;"",P69="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM69" s="9" t="str">
         <x:f>IF(A69="","",IF(AND(AK69="OK",J69="READY",F69&lt;&gt;"",G69&lt;&gt;"",K69&lt;&gt;"",S69="OK",OR(R69="PASS",R69="FAIL")),"YES","NO"))</x:f>
@@ -4569,7 +4569,7 @@
         <x:f>IF(A70="",IF(B70="","","MISSING_TEST_ID"),IF(B70="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A70,$B$2:$B$501,B70)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL70" s="9" t="str">
-        <x:f>IF(A70="","",IF(AND(AK70="OK",J70="READY",F70&lt;&gt;"",G70&lt;&gt;"",K70&lt;&gt;"",OR(L70="PASS",L70="FAIL"),M70&lt;&gt;"",O70&lt;&gt;"",P70="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A70="","",IF(AND(AK70="OK",J70="READY",F70&lt;&gt;"",G70&lt;&gt;"",K70&lt;&gt;"",OR(L70="PASS",L70="FAIL"),M70&lt;&gt;"",P70="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM70" s="9" t="str">
         <x:f>IF(A70="","",IF(AND(AK70="OK",J70="READY",F70&lt;&gt;"",G70&lt;&gt;"",K70&lt;&gt;"",S70="OK",OR(R70="PASS",R70="FAIL")),"YES","NO"))</x:f>
@@ -4621,7 +4621,7 @@
         <x:f>IF(A71="",IF(B71="","","MISSING_TEST_ID"),IF(B71="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A71,$B$2:$B$501,B71)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL71" s="9" t="str">
-        <x:f>IF(A71="","",IF(AND(AK71="OK",J71="READY",F71&lt;&gt;"",G71&lt;&gt;"",K71&lt;&gt;"",OR(L71="PASS",L71="FAIL"),M71&lt;&gt;"",O71&lt;&gt;"",P71="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A71="","",IF(AND(AK71="OK",J71="READY",F71&lt;&gt;"",G71&lt;&gt;"",K71&lt;&gt;"",OR(L71="PASS",L71="FAIL"),M71&lt;&gt;"",P71="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM71" s="9" t="str">
         <x:f>IF(A71="","",IF(AND(AK71="OK",J71="READY",F71&lt;&gt;"",G71&lt;&gt;"",K71&lt;&gt;"",S71="OK",OR(R71="PASS",R71="FAIL")),"YES","NO"))</x:f>
@@ -4673,7 +4673,7 @@
         <x:f>IF(A72="",IF(B72="","","MISSING_TEST_ID"),IF(B72="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A72,$B$2:$B$501,B72)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL72" s="9" t="str">
-        <x:f>IF(A72="","",IF(AND(AK72="OK",J72="READY",F72&lt;&gt;"",G72&lt;&gt;"",K72&lt;&gt;"",OR(L72="PASS",L72="FAIL"),M72&lt;&gt;"",O72&lt;&gt;"",P72="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A72="","",IF(AND(AK72="OK",J72="READY",F72&lt;&gt;"",G72&lt;&gt;"",K72&lt;&gt;"",OR(L72="PASS",L72="FAIL"),M72&lt;&gt;"",P72="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM72" s="9" t="str">
         <x:f>IF(A72="","",IF(AND(AK72="OK",J72="READY",F72&lt;&gt;"",G72&lt;&gt;"",K72&lt;&gt;"",S72="OK",OR(R72="PASS",R72="FAIL")),"YES","NO"))</x:f>
@@ -4725,7 +4725,7 @@
         <x:f>IF(A73="",IF(B73="","","MISSING_TEST_ID"),IF(B73="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A73,$B$2:$B$501,B73)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL73" s="9" t="str">
-        <x:f>IF(A73="","",IF(AND(AK73="OK",J73="READY",F73&lt;&gt;"",G73&lt;&gt;"",K73&lt;&gt;"",OR(L73="PASS",L73="FAIL"),M73&lt;&gt;"",O73&lt;&gt;"",P73="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A73="","",IF(AND(AK73="OK",J73="READY",F73&lt;&gt;"",G73&lt;&gt;"",K73&lt;&gt;"",OR(L73="PASS",L73="FAIL"),M73&lt;&gt;"",P73="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM73" s="9" t="str">
         <x:f>IF(A73="","",IF(AND(AK73="OK",J73="READY",F73&lt;&gt;"",G73&lt;&gt;"",K73&lt;&gt;"",S73="OK",OR(R73="PASS",R73="FAIL")),"YES","NO"))</x:f>
@@ -4777,7 +4777,7 @@
         <x:f>IF(A74="",IF(B74="","","MISSING_TEST_ID"),IF(B74="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A74,$B$2:$B$501,B74)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL74" s="9" t="str">
-        <x:f>IF(A74="","",IF(AND(AK74="OK",J74="READY",F74&lt;&gt;"",G74&lt;&gt;"",K74&lt;&gt;"",OR(L74="PASS",L74="FAIL"),M74&lt;&gt;"",O74&lt;&gt;"",P74="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A74="","",IF(AND(AK74="OK",J74="READY",F74&lt;&gt;"",G74&lt;&gt;"",K74&lt;&gt;"",OR(L74="PASS",L74="FAIL"),M74&lt;&gt;"",P74="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM74" s="9" t="str">
         <x:f>IF(A74="","",IF(AND(AK74="OK",J74="READY",F74&lt;&gt;"",G74&lt;&gt;"",K74&lt;&gt;"",S74="OK",OR(R74="PASS",R74="FAIL")),"YES","NO"))</x:f>
@@ -4829,7 +4829,7 @@
         <x:f>IF(A75="",IF(B75="","","MISSING_TEST_ID"),IF(B75="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A75,$B$2:$B$501,B75)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL75" s="9" t="str">
-        <x:f>IF(A75="","",IF(AND(AK75="OK",J75="READY",F75&lt;&gt;"",G75&lt;&gt;"",K75&lt;&gt;"",OR(L75="PASS",L75="FAIL"),M75&lt;&gt;"",O75&lt;&gt;"",P75="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A75="","",IF(AND(AK75="OK",J75="READY",F75&lt;&gt;"",G75&lt;&gt;"",K75&lt;&gt;"",OR(L75="PASS",L75="FAIL"),M75&lt;&gt;"",P75="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM75" s="9" t="str">
         <x:f>IF(A75="","",IF(AND(AK75="OK",J75="READY",F75&lt;&gt;"",G75&lt;&gt;"",K75&lt;&gt;"",S75="OK",OR(R75="PASS",R75="FAIL")),"YES","NO"))</x:f>
@@ -4881,7 +4881,7 @@
         <x:f>IF(A76="",IF(B76="","","MISSING_TEST_ID"),IF(B76="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A76,$B$2:$B$501,B76)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL76" s="9" t="str">
-        <x:f>IF(A76="","",IF(AND(AK76="OK",J76="READY",F76&lt;&gt;"",G76&lt;&gt;"",K76&lt;&gt;"",OR(L76="PASS",L76="FAIL"),M76&lt;&gt;"",O76&lt;&gt;"",P76="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A76="","",IF(AND(AK76="OK",J76="READY",F76&lt;&gt;"",G76&lt;&gt;"",K76&lt;&gt;"",OR(L76="PASS",L76="FAIL"),M76&lt;&gt;"",P76="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM76" s="9" t="str">
         <x:f>IF(A76="","",IF(AND(AK76="OK",J76="READY",F76&lt;&gt;"",G76&lt;&gt;"",K76&lt;&gt;"",S76="OK",OR(R76="PASS",R76="FAIL")),"YES","NO"))</x:f>
@@ -4933,7 +4933,7 @@
         <x:f>IF(A77="",IF(B77="","","MISSING_TEST_ID"),IF(B77="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A77,$B$2:$B$501,B77)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL77" s="9" t="str">
-        <x:f>IF(A77="","",IF(AND(AK77="OK",J77="READY",F77&lt;&gt;"",G77&lt;&gt;"",K77&lt;&gt;"",OR(L77="PASS",L77="FAIL"),M77&lt;&gt;"",O77&lt;&gt;"",P77="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A77="","",IF(AND(AK77="OK",J77="READY",F77&lt;&gt;"",G77&lt;&gt;"",K77&lt;&gt;"",OR(L77="PASS",L77="FAIL"),M77&lt;&gt;"",P77="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM77" s="9" t="str">
         <x:f>IF(A77="","",IF(AND(AK77="OK",J77="READY",F77&lt;&gt;"",G77&lt;&gt;"",K77&lt;&gt;"",S77="OK",OR(R77="PASS",R77="FAIL")),"YES","NO"))</x:f>
@@ -4985,7 +4985,7 @@
         <x:f>IF(A78="",IF(B78="","","MISSING_TEST_ID"),IF(B78="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A78,$B$2:$B$501,B78)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL78" s="9" t="str">
-        <x:f>IF(A78="","",IF(AND(AK78="OK",J78="READY",F78&lt;&gt;"",G78&lt;&gt;"",K78&lt;&gt;"",OR(L78="PASS",L78="FAIL"),M78&lt;&gt;"",O78&lt;&gt;"",P78="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A78="","",IF(AND(AK78="OK",J78="READY",F78&lt;&gt;"",G78&lt;&gt;"",K78&lt;&gt;"",OR(L78="PASS",L78="FAIL"),M78&lt;&gt;"",P78="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM78" s="9" t="str">
         <x:f>IF(A78="","",IF(AND(AK78="OK",J78="READY",F78&lt;&gt;"",G78&lt;&gt;"",K78&lt;&gt;"",S78="OK",OR(R78="PASS",R78="FAIL")),"YES","NO"))</x:f>
@@ -5037,7 +5037,7 @@
         <x:f>IF(A79="",IF(B79="","","MISSING_TEST_ID"),IF(B79="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A79,$B$2:$B$501,B79)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL79" s="9" t="str">
-        <x:f>IF(A79="","",IF(AND(AK79="OK",J79="READY",F79&lt;&gt;"",G79&lt;&gt;"",K79&lt;&gt;"",OR(L79="PASS",L79="FAIL"),M79&lt;&gt;"",O79&lt;&gt;"",P79="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A79="","",IF(AND(AK79="OK",J79="READY",F79&lt;&gt;"",G79&lt;&gt;"",K79&lt;&gt;"",OR(L79="PASS",L79="FAIL"),M79&lt;&gt;"",P79="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM79" s="9" t="str">
         <x:f>IF(A79="","",IF(AND(AK79="OK",J79="READY",F79&lt;&gt;"",G79&lt;&gt;"",K79&lt;&gt;"",S79="OK",OR(R79="PASS",R79="FAIL")),"YES","NO"))</x:f>
@@ -5089,7 +5089,7 @@
         <x:f>IF(A80="",IF(B80="","","MISSING_TEST_ID"),IF(B80="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A80,$B$2:$B$501,B80)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL80" s="9" t="str">
-        <x:f>IF(A80="","",IF(AND(AK80="OK",J80="READY",F80&lt;&gt;"",G80&lt;&gt;"",K80&lt;&gt;"",OR(L80="PASS",L80="FAIL"),M80&lt;&gt;"",O80&lt;&gt;"",P80="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A80="","",IF(AND(AK80="OK",J80="READY",F80&lt;&gt;"",G80&lt;&gt;"",K80&lt;&gt;"",OR(L80="PASS",L80="FAIL"),M80&lt;&gt;"",P80="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM80" s="9" t="str">
         <x:f>IF(A80="","",IF(AND(AK80="OK",J80="READY",F80&lt;&gt;"",G80&lt;&gt;"",K80&lt;&gt;"",S80="OK",OR(R80="PASS",R80="FAIL")),"YES","NO"))</x:f>
@@ -5141,7 +5141,7 @@
         <x:f>IF(A81="",IF(B81="","","MISSING_TEST_ID"),IF(B81="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A81,$B$2:$B$501,B81)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL81" s="9" t="str">
-        <x:f>IF(A81="","",IF(AND(AK81="OK",J81="READY",F81&lt;&gt;"",G81&lt;&gt;"",K81&lt;&gt;"",OR(L81="PASS",L81="FAIL"),M81&lt;&gt;"",O81&lt;&gt;"",P81="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A81="","",IF(AND(AK81="OK",J81="READY",F81&lt;&gt;"",G81&lt;&gt;"",K81&lt;&gt;"",OR(L81="PASS",L81="FAIL"),M81&lt;&gt;"",P81="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM81" s="9" t="str">
         <x:f>IF(A81="","",IF(AND(AK81="OK",J81="READY",F81&lt;&gt;"",G81&lt;&gt;"",K81&lt;&gt;"",S81="OK",OR(R81="PASS",R81="FAIL")),"YES","NO"))</x:f>
@@ -5193,7 +5193,7 @@
         <x:f>IF(A82="",IF(B82="","","MISSING_TEST_ID"),IF(B82="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A82,$B$2:$B$501,B82)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL82" s="9" t="str">
-        <x:f>IF(A82="","",IF(AND(AK82="OK",J82="READY",F82&lt;&gt;"",G82&lt;&gt;"",K82&lt;&gt;"",OR(L82="PASS",L82="FAIL"),M82&lt;&gt;"",O82&lt;&gt;"",P82="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A82="","",IF(AND(AK82="OK",J82="READY",F82&lt;&gt;"",G82&lt;&gt;"",K82&lt;&gt;"",OR(L82="PASS",L82="FAIL"),M82&lt;&gt;"",P82="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM82" s="9" t="str">
         <x:f>IF(A82="","",IF(AND(AK82="OK",J82="READY",F82&lt;&gt;"",G82&lt;&gt;"",K82&lt;&gt;"",S82="OK",OR(R82="PASS",R82="FAIL")),"YES","NO"))</x:f>
@@ -5245,7 +5245,7 @@
         <x:f>IF(A83="",IF(B83="","","MISSING_TEST_ID"),IF(B83="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A83,$B$2:$B$501,B83)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL83" s="9" t="str">
-        <x:f>IF(A83="","",IF(AND(AK83="OK",J83="READY",F83&lt;&gt;"",G83&lt;&gt;"",K83&lt;&gt;"",OR(L83="PASS",L83="FAIL"),M83&lt;&gt;"",O83&lt;&gt;"",P83="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A83="","",IF(AND(AK83="OK",J83="READY",F83&lt;&gt;"",G83&lt;&gt;"",K83&lt;&gt;"",OR(L83="PASS",L83="FAIL"),M83&lt;&gt;"",P83="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM83" s="9" t="str">
         <x:f>IF(A83="","",IF(AND(AK83="OK",J83="READY",F83&lt;&gt;"",G83&lt;&gt;"",K83&lt;&gt;"",S83="OK",OR(R83="PASS",R83="FAIL")),"YES","NO"))</x:f>
@@ -5297,7 +5297,7 @@
         <x:f>IF(A84="",IF(B84="","","MISSING_TEST_ID"),IF(B84="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A84,$B$2:$B$501,B84)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL84" s="9" t="str">
-        <x:f>IF(A84="","",IF(AND(AK84="OK",J84="READY",F84&lt;&gt;"",G84&lt;&gt;"",K84&lt;&gt;"",OR(L84="PASS",L84="FAIL"),M84&lt;&gt;"",O84&lt;&gt;"",P84="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A84="","",IF(AND(AK84="OK",J84="READY",F84&lt;&gt;"",G84&lt;&gt;"",K84&lt;&gt;"",OR(L84="PASS",L84="FAIL"),M84&lt;&gt;"",P84="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM84" s="9" t="str">
         <x:f>IF(A84="","",IF(AND(AK84="OK",J84="READY",F84&lt;&gt;"",G84&lt;&gt;"",K84&lt;&gt;"",S84="OK",OR(R84="PASS",R84="FAIL")),"YES","NO"))</x:f>
@@ -5349,7 +5349,7 @@
         <x:f>IF(A85="",IF(B85="","","MISSING_TEST_ID"),IF(B85="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A85,$B$2:$B$501,B85)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL85" s="9" t="str">
-        <x:f>IF(A85="","",IF(AND(AK85="OK",J85="READY",F85&lt;&gt;"",G85&lt;&gt;"",K85&lt;&gt;"",OR(L85="PASS",L85="FAIL"),M85&lt;&gt;"",O85&lt;&gt;"",P85="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A85="","",IF(AND(AK85="OK",J85="READY",F85&lt;&gt;"",G85&lt;&gt;"",K85&lt;&gt;"",OR(L85="PASS",L85="FAIL"),M85&lt;&gt;"",P85="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM85" s="9" t="str">
         <x:f>IF(A85="","",IF(AND(AK85="OK",J85="READY",F85&lt;&gt;"",G85&lt;&gt;"",K85&lt;&gt;"",S85="OK",OR(R85="PASS",R85="FAIL")),"YES","NO"))</x:f>
@@ -5401,7 +5401,7 @@
         <x:f>IF(A86="",IF(B86="","","MISSING_TEST_ID"),IF(B86="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A86,$B$2:$B$501,B86)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL86" s="9" t="str">
-        <x:f>IF(A86="","",IF(AND(AK86="OK",J86="READY",F86&lt;&gt;"",G86&lt;&gt;"",K86&lt;&gt;"",OR(L86="PASS",L86="FAIL"),M86&lt;&gt;"",O86&lt;&gt;"",P86="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A86="","",IF(AND(AK86="OK",J86="READY",F86&lt;&gt;"",G86&lt;&gt;"",K86&lt;&gt;"",OR(L86="PASS",L86="FAIL"),M86&lt;&gt;"",P86="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM86" s="9" t="str">
         <x:f>IF(A86="","",IF(AND(AK86="OK",J86="READY",F86&lt;&gt;"",G86&lt;&gt;"",K86&lt;&gt;"",S86="OK",OR(R86="PASS",R86="FAIL")),"YES","NO"))</x:f>
@@ -5453,7 +5453,7 @@
         <x:f>IF(A87="",IF(B87="","","MISSING_TEST_ID"),IF(B87="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A87,$B$2:$B$501,B87)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL87" s="9" t="str">
-        <x:f>IF(A87="","",IF(AND(AK87="OK",J87="READY",F87&lt;&gt;"",G87&lt;&gt;"",K87&lt;&gt;"",OR(L87="PASS",L87="FAIL"),M87&lt;&gt;"",O87&lt;&gt;"",P87="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A87="","",IF(AND(AK87="OK",J87="READY",F87&lt;&gt;"",G87&lt;&gt;"",K87&lt;&gt;"",OR(L87="PASS",L87="FAIL"),M87&lt;&gt;"",P87="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM87" s="9" t="str">
         <x:f>IF(A87="","",IF(AND(AK87="OK",J87="READY",F87&lt;&gt;"",G87&lt;&gt;"",K87&lt;&gt;"",S87="OK",OR(R87="PASS",R87="FAIL")),"YES","NO"))</x:f>
@@ -5505,7 +5505,7 @@
         <x:f>IF(A88="",IF(B88="","","MISSING_TEST_ID"),IF(B88="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A88,$B$2:$B$501,B88)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL88" s="9" t="str">
-        <x:f>IF(A88="","",IF(AND(AK88="OK",J88="READY",F88&lt;&gt;"",G88&lt;&gt;"",K88&lt;&gt;"",OR(L88="PASS",L88="FAIL"),M88&lt;&gt;"",O88&lt;&gt;"",P88="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A88="","",IF(AND(AK88="OK",J88="READY",F88&lt;&gt;"",G88&lt;&gt;"",K88&lt;&gt;"",OR(L88="PASS",L88="FAIL"),M88&lt;&gt;"",P88="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM88" s="9" t="str">
         <x:f>IF(A88="","",IF(AND(AK88="OK",J88="READY",F88&lt;&gt;"",G88&lt;&gt;"",K88&lt;&gt;"",S88="OK",OR(R88="PASS",R88="FAIL")),"YES","NO"))</x:f>
@@ -5557,7 +5557,7 @@
         <x:f>IF(A89="",IF(B89="","","MISSING_TEST_ID"),IF(B89="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A89,$B$2:$B$501,B89)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL89" s="9" t="str">
-        <x:f>IF(A89="","",IF(AND(AK89="OK",J89="READY",F89&lt;&gt;"",G89&lt;&gt;"",K89&lt;&gt;"",OR(L89="PASS",L89="FAIL"),M89&lt;&gt;"",O89&lt;&gt;"",P89="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A89="","",IF(AND(AK89="OK",J89="READY",F89&lt;&gt;"",G89&lt;&gt;"",K89&lt;&gt;"",OR(L89="PASS",L89="FAIL"),M89&lt;&gt;"",P89="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM89" s="9" t="str">
         <x:f>IF(A89="","",IF(AND(AK89="OK",J89="READY",F89&lt;&gt;"",G89&lt;&gt;"",K89&lt;&gt;"",S89="OK",OR(R89="PASS",R89="FAIL")),"YES","NO"))</x:f>
@@ -5609,7 +5609,7 @@
         <x:f>IF(A90="",IF(B90="","","MISSING_TEST_ID"),IF(B90="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A90,$B$2:$B$501,B90)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL90" s="9" t="str">
-        <x:f>IF(A90="","",IF(AND(AK90="OK",J90="READY",F90&lt;&gt;"",G90&lt;&gt;"",K90&lt;&gt;"",OR(L90="PASS",L90="FAIL"),M90&lt;&gt;"",O90&lt;&gt;"",P90="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A90="","",IF(AND(AK90="OK",J90="READY",F90&lt;&gt;"",G90&lt;&gt;"",K90&lt;&gt;"",OR(L90="PASS",L90="FAIL"),M90&lt;&gt;"",P90="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM90" s="9" t="str">
         <x:f>IF(A90="","",IF(AND(AK90="OK",J90="READY",F90&lt;&gt;"",G90&lt;&gt;"",K90&lt;&gt;"",S90="OK",OR(R90="PASS",R90="FAIL")),"YES","NO"))</x:f>
@@ -5661,7 +5661,7 @@
         <x:f>IF(A91="",IF(B91="","","MISSING_TEST_ID"),IF(B91="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A91,$B$2:$B$501,B91)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL91" s="9" t="str">
-        <x:f>IF(A91="","",IF(AND(AK91="OK",J91="READY",F91&lt;&gt;"",G91&lt;&gt;"",K91&lt;&gt;"",OR(L91="PASS",L91="FAIL"),M91&lt;&gt;"",O91&lt;&gt;"",P91="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A91="","",IF(AND(AK91="OK",J91="READY",F91&lt;&gt;"",G91&lt;&gt;"",K91&lt;&gt;"",OR(L91="PASS",L91="FAIL"),M91&lt;&gt;"",P91="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM91" s="9" t="str">
         <x:f>IF(A91="","",IF(AND(AK91="OK",J91="READY",F91&lt;&gt;"",G91&lt;&gt;"",K91&lt;&gt;"",S91="OK",OR(R91="PASS",R91="FAIL")),"YES","NO"))</x:f>
@@ -5713,7 +5713,7 @@
         <x:f>IF(A92="",IF(B92="","","MISSING_TEST_ID"),IF(B92="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A92,$B$2:$B$501,B92)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL92" s="9" t="str">
-        <x:f>IF(A92="","",IF(AND(AK92="OK",J92="READY",F92&lt;&gt;"",G92&lt;&gt;"",K92&lt;&gt;"",OR(L92="PASS",L92="FAIL"),M92&lt;&gt;"",O92&lt;&gt;"",P92="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A92="","",IF(AND(AK92="OK",J92="READY",F92&lt;&gt;"",G92&lt;&gt;"",K92&lt;&gt;"",OR(L92="PASS",L92="FAIL"),M92&lt;&gt;"",P92="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM92" s="9" t="str">
         <x:f>IF(A92="","",IF(AND(AK92="OK",J92="READY",F92&lt;&gt;"",G92&lt;&gt;"",K92&lt;&gt;"",S92="OK",OR(R92="PASS",R92="FAIL")),"YES","NO"))</x:f>
@@ -5765,7 +5765,7 @@
         <x:f>IF(A93="",IF(B93="","","MISSING_TEST_ID"),IF(B93="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A93,$B$2:$B$501,B93)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL93" s="9" t="str">
-        <x:f>IF(A93="","",IF(AND(AK93="OK",J93="READY",F93&lt;&gt;"",G93&lt;&gt;"",K93&lt;&gt;"",OR(L93="PASS",L93="FAIL"),M93&lt;&gt;"",O93&lt;&gt;"",P93="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A93="","",IF(AND(AK93="OK",J93="READY",F93&lt;&gt;"",G93&lt;&gt;"",K93&lt;&gt;"",OR(L93="PASS",L93="FAIL"),M93&lt;&gt;"",P93="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM93" s="9" t="str">
         <x:f>IF(A93="","",IF(AND(AK93="OK",J93="READY",F93&lt;&gt;"",G93&lt;&gt;"",K93&lt;&gt;"",S93="OK",OR(R93="PASS",R93="FAIL")),"YES","NO"))</x:f>
@@ -5817,7 +5817,7 @@
         <x:f>IF(A94="",IF(B94="","","MISSING_TEST_ID"),IF(B94="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A94,$B$2:$B$501,B94)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL94" s="9" t="str">
-        <x:f>IF(A94="","",IF(AND(AK94="OK",J94="READY",F94&lt;&gt;"",G94&lt;&gt;"",K94&lt;&gt;"",OR(L94="PASS",L94="FAIL"),M94&lt;&gt;"",O94&lt;&gt;"",P94="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A94="","",IF(AND(AK94="OK",J94="READY",F94&lt;&gt;"",G94&lt;&gt;"",K94&lt;&gt;"",OR(L94="PASS",L94="FAIL"),M94&lt;&gt;"",P94="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM94" s="9" t="str">
         <x:f>IF(A94="","",IF(AND(AK94="OK",J94="READY",F94&lt;&gt;"",G94&lt;&gt;"",K94&lt;&gt;"",S94="OK",OR(R94="PASS",R94="FAIL")),"YES","NO"))</x:f>
@@ -5869,7 +5869,7 @@
         <x:f>IF(A95="",IF(B95="","","MISSING_TEST_ID"),IF(B95="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A95,$B$2:$B$501,B95)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL95" s="9" t="str">
-        <x:f>IF(A95="","",IF(AND(AK95="OK",J95="READY",F95&lt;&gt;"",G95&lt;&gt;"",K95&lt;&gt;"",OR(L95="PASS",L95="FAIL"),M95&lt;&gt;"",O95&lt;&gt;"",P95="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A95="","",IF(AND(AK95="OK",J95="READY",F95&lt;&gt;"",G95&lt;&gt;"",K95&lt;&gt;"",OR(L95="PASS",L95="FAIL"),M95&lt;&gt;"",P95="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM95" s="9" t="str">
         <x:f>IF(A95="","",IF(AND(AK95="OK",J95="READY",F95&lt;&gt;"",G95&lt;&gt;"",K95&lt;&gt;"",S95="OK",OR(R95="PASS",R95="FAIL")),"YES","NO"))</x:f>
@@ -5921,7 +5921,7 @@
         <x:f>IF(A96="",IF(B96="","","MISSING_TEST_ID"),IF(B96="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A96,$B$2:$B$501,B96)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL96" s="9" t="str">
-        <x:f>IF(A96="","",IF(AND(AK96="OK",J96="READY",F96&lt;&gt;"",G96&lt;&gt;"",K96&lt;&gt;"",OR(L96="PASS",L96="FAIL"),M96&lt;&gt;"",O96&lt;&gt;"",P96="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A96="","",IF(AND(AK96="OK",J96="READY",F96&lt;&gt;"",G96&lt;&gt;"",K96&lt;&gt;"",OR(L96="PASS",L96="FAIL"),M96&lt;&gt;"",P96="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM96" s="9" t="str">
         <x:f>IF(A96="","",IF(AND(AK96="OK",J96="READY",F96&lt;&gt;"",G96&lt;&gt;"",K96&lt;&gt;"",S96="OK",OR(R96="PASS",R96="FAIL")),"YES","NO"))</x:f>
@@ -5973,7 +5973,7 @@
         <x:f>IF(A97="",IF(B97="","","MISSING_TEST_ID"),IF(B97="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A97,$B$2:$B$501,B97)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL97" s="9" t="str">
-        <x:f>IF(A97="","",IF(AND(AK97="OK",J97="READY",F97&lt;&gt;"",G97&lt;&gt;"",K97&lt;&gt;"",OR(L97="PASS",L97="FAIL"),M97&lt;&gt;"",O97&lt;&gt;"",P97="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A97="","",IF(AND(AK97="OK",J97="READY",F97&lt;&gt;"",G97&lt;&gt;"",K97&lt;&gt;"",OR(L97="PASS",L97="FAIL"),M97&lt;&gt;"",P97="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM97" s="9" t="str">
         <x:f>IF(A97="","",IF(AND(AK97="OK",J97="READY",F97&lt;&gt;"",G97&lt;&gt;"",K97&lt;&gt;"",S97="OK",OR(R97="PASS",R97="FAIL")),"YES","NO"))</x:f>
@@ -6025,7 +6025,7 @@
         <x:f>IF(A98="",IF(B98="","","MISSING_TEST_ID"),IF(B98="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A98,$B$2:$B$501,B98)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL98" s="9" t="str">
-        <x:f>IF(A98="","",IF(AND(AK98="OK",J98="READY",F98&lt;&gt;"",G98&lt;&gt;"",K98&lt;&gt;"",OR(L98="PASS",L98="FAIL"),M98&lt;&gt;"",O98&lt;&gt;"",P98="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A98="","",IF(AND(AK98="OK",J98="READY",F98&lt;&gt;"",G98&lt;&gt;"",K98&lt;&gt;"",OR(L98="PASS",L98="FAIL"),M98&lt;&gt;"",P98="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM98" s="9" t="str">
         <x:f>IF(A98="","",IF(AND(AK98="OK",J98="READY",F98&lt;&gt;"",G98&lt;&gt;"",K98&lt;&gt;"",S98="OK",OR(R98="PASS",R98="FAIL")),"YES","NO"))</x:f>
@@ -6077,7 +6077,7 @@
         <x:f>IF(A99="",IF(B99="","","MISSING_TEST_ID"),IF(B99="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A99,$B$2:$B$501,B99)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL99" s="9" t="str">
-        <x:f>IF(A99="","",IF(AND(AK99="OK",J99="READY",F99&lt;&gt;"",G99&lt;&gt;"",K99&lt;&gt;"",OR(L99="PASS",L99="FAIL"),M99&lt;&gt;"",O99&lt;&gt;"",P99="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A99="","",IF(AND(AK99="OK",J99="READY",F99&lt;&gt;"",G99&lt;&gt;"",K99&lt;&gt;"",OR(L99="PASS",L99="FAIL"),M99&lt;&gt;"",P99="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM99" s="9" t="str">
         <x:f>IF(A99="","",IF(AND(AK99="OK",J99="READY",F99&lt;&gt;"",G99&lt;&gt;"",K99&lt;&gt;"",S99="OK",OR(R99="PASS",R99="FAIL")),"YES","NO"))</x:f>
@@ -6129,7 +6129,7 @@
         <x:f>IF(A100="",IF(B100="","","MISSING_TEST_ID"),IF(B100="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A100,$B$2:$B$501,B100)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL100" s="9" t="str">
-        <x:f>IF(A100="","",IF(AND(AK100="OK",J100="READY",F100&lt;&gt;"",G100&lt;&gt;"",K100&lt;&gt;"",OR(L100="PASS",L100="FAIL"),M100&lt;&gt;"",O100&lt;&gt;"",P100="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A100="","",IF(AND(AK100="OK",J100="READY",F100&lt;&gt;"",G100&lt;&gt;"",K100&lt;&gt;"",OR(L100="PASS",L100="FAIL"),M100&lt;&gt;"",P100="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM100" s="9" t="str">
         <x:f>IF(A100="","",IF(AND(AK100="OK",J100="READY",F100&lt;&gt;"",G100&lt;&gt;"",K100&lt;&gt;"",S100="OK",OR(R100="PASS",R100="FAIL")),"YES","NO"))</x:f>
@@ -6181,7 +6181,7 @@
         <x:f>IF(A101="",IF(B101="","","MISSING_TEST_ID"),IF(B101="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A101,$B$2:$B$501,B101)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL101" s="9" t="str">
-        <x:f>IF(A101="","",IF(AND(AK101="OK",J101="READY",F101&lt;&gt;"",G101&lt;&gt;"",K101&lt;&gt;"",OR(L101="PASS",L101="FAIL"),M101&lt;&gt;"",O101&lt;&gt;"",P101="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A101="","",IF(AND(AK101="OK",J101="READY",F101&lt;&gt;"",G101&lt;&gt;"",K101&lt;&gt;"",OR(L101="PASS",L101="FAIL"),M101&lt;&gt;"",P101="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM101" s="9" t="str">
         <x:f>IF(A101="","",IF(AND(AK101="OK",J101="READY",F101&lt;&gt;"",G101&lt;&gt;"",K101&lt;&gt;"",S101="OK",OR(R101="PASS",R101="FAIL")),"YES","NO"))</x:f>
@@ -6233,7 +6233,7 @@
         <x:f>IF(A102="",IF(B102="","","MISSING_TEST_ID"),IF(B102="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A102,$B$2:$B$501,B102)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL102" s="9" t="str">
-        <x:f>IF(A102="","",IF(AND(AK102="OK",J102="READY",F102&lt;&gt;"",G102&lt;&gt;"",K102&lt;&gt;"",OR(L102="PASS",L102="FAIL"),M102&lt;&gt;"",O102&lt;&gt;"",P102="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A102="","",IF(AND(AK102="OK",J102="READY",F102&lt;&gt;"",G102&lt;&gt;"",K102&lt;&gt;"",OR(L102="PASS",L102="FAIL"),M102&lt;&gt;"",P102="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM102" s="9" t="str">
         <x:f>IF(A102="","",IF(AND(AK102="OK",J102="READY",F102&lt;&gt;"",G102&lt;&gt;"",K102&lt;&gt;"",S102="OK",OR(R102="PASS",R102="FAIL")),"YES","NO"))</x:f>
@@ -6285,7 +6285,7 @@
         <x:f>IF(A103="",IF(B103="","","MISSING_TEST_ID"),IF(B103="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A103,$B$2:$B$501,B103)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL103" s="9" t="str">
-        <x:f>IF(A103="","",IF(AND(AK103="OK",J103="READY",F103&lt;&gt;"",G103&lt;&gt;"",K103&lt;&gt;"",OR(L103="PASS",L103="FAIL"),M103&lt;&gt;"",O103&lt;&gt;"",P103="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A103="","",IF(AND(AK103="OK",J103="READY",F103&lt;&gt;"",G103&lt;&gt;"",K103&lt;&gt;"",OR(L103="PASS",L103="FAIL"),M103&lt;&gt;"",P103="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM103" s="9" t="str">
         <x:f>IF(A103="","",IF(AND(AK103="OK",J103="READY",F103&lt;&gt;"",G103&lt;&gt;"",K103&lt;&gt;"",S103="OK",OR(R103="PASS",R103="FAIL")),"YES","NO"))</x:f>
@@ -6337,7 +6337,7 @@
         <x:f>IF(A104="",IF(B104="","","MISSING_TEST_ID"),IF(B104="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A104,$B$2:$B$501,B104)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL104" s="9" t="str">
-        <x:f>IF(A104="","",IF(AND(AK104="OK",J104="READY",F104&lt;&gt;"",G104&lt;&gt;"",K104&lt;&gt;"",OR(L104="PASS",L104="FAIL"),M104&lt;&gt;"",O104&lt;&gt;"",P104="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A104="","",IF(AND(AK104="OK",J104="READY",F104&lt;&gt;"",G104&lt;&gt;"",K104&lt;&gt;"",OR(L104="PASS",L104="FAIL"),M104&lt;&gt;"",P104="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM104" s="9" t="str">
         <x:f>IF(A104="","",IF(AND(AK104="OK",J104="READY",F104&lt;&gt;"",G104&lt;&gt;"",K104&lt;&gt;"",S104="OK",OR(R104="PASS",R104="FAIL")),"YES","NO"))</x:f>
@@ -6389,7 +6389,7 @@
         <x:f>IF(A105="",IF(B105="","","MISSING_TEST_ID"),IF(B105="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A105,$B$2:$B$501,B105)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL105" s="9" t="str">
-        <x:f>IF(A105="","",IF(AND(AK105="OK",J105="READY",F105&lt;&gt;"",G105&lt;&gt;"",K105&lt;&gt;"",OR(L105="PASS",L105="FAIL"),M105&lt;&gt;"",O105&lt;&gt;"",P105="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A105="","",IF(AND(AK105="OK",J105="READY",F105&lt;&gt;"",G105&lt;&gt;"",K105&lt;&gt;"",OR(L105="PASS",L105="FAIL"),M105&lt;&gt;"",P105="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM105" s="9" t="str">
         <x:f>IF(A105="","",IF(AND(AK105="OK",J105="READY",F105&lt;&gt;"",G105&lt;&gt;"",K105&lt;&gt;"",S105="OK",OR(R105="PASS",R105="FAIL")),"YES","NO"))</x:f>
@@ -6441,7 +6441,7 @@
         <x:f>IF(A106="",IF(B106="","","MISSING_TEST_ID"),IF(B106="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A106,$B$2:$B$501,B106)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL106" s="9" t="str">
-        <x:f>IF(A106="","",IF(AND(AK106="OK",J106="READY",F106&lt;&gt;"",G106&lt;&gt;"",K106&lt;&gt;"",OR(L106="PASS",L106="FAIL"),M106&lt;&gt;"",O106&lt;&gt;"",P106="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A106="","",IF(AND(AK106="OK",J106="READY",F106&lt;&gt;"",G106&lt;&gt;"",K106&lt;&gt;"",OR(L106="PASS",L106="FAIL"),M106&lt;&gt;"",P106="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM106" s="9" t="str">
         <x:f>IF(A106="","",IF(AND(AK106="OK",J106="READY",F106&lt;&gt;"",G106&lt;&gt;"",K106&lt;&gt;"",S106="OK",OR(R106="PASS",R106="FAIL")),"YES","NO"))</x:f>
@@ -6493,7 +6493,7 @@
         <x:f>IF(A107="",IF(B107="","","MISSING_TEST_ID"),IF(B107="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A107,$B$2:$B$501,B107)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL107" s="9" t="str">
-        <x:f>IF(A107="","",IF(AND(AK107="OK",J107="READY",F107&lt;&gt;"",G107&lt;&gt;"",K107&lt;&gt;"",OR(L107="PASS",L107="FAIL"),M107&lt;&gt;"",O107&lt;&gt;"",P107="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A107="","",IF(AND(AK107="OK",J107="READY",F107&lt;&gt;"",G107&lt;&gt;"",K107&lt;&gt;"",OR(L107="PASS",L107="FAIL"),M107&lt;&gt;"",P107="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM107" s="9" t="str">
         <x:f>IF(A107="","",IF(AND(AK107="OK",J107="READY",F107&lt;&gt;"",G107&lt;&gt;"",K107&lt;&gt;"",S107="OK",OR(R107="PASS",R107="FAIL")),"YES","NO"))</x:f>
@@ -6545,7 +6545,7 @@
         <x:f>IF(A108="",IF(B108="","","MISSING_TEST_ID"),IF(B108="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A108,$B$2:$B$501,B108)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL108" s="9" t="str">
-        <x:f>IF(A108="","",IF(AND(AK108="OK",J108="READY",F108&lt;&gt;"",G108&lt;&gt;"",K108&lt;&gt;"",OR(L108="PASS",L108="FAIL"),M108&lt;&gt;"",O108&lt;&gt;"",P108="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A108="","",IF(AND(AK108="OK",J108="READY",F108&lt;&gt;"",G108&lt;&gt;"",K108&lt;&gt;"",OR(L108="PASS",L108="FAIL"),M108&lt;&gt;"",P108="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM108" s="9" t="str">
         <x:f>IF(A108="","",IF(AND(AK108="OK",J108="READY",F108&lt;&gt;"",G108&lt;&gt;"",K108&lt;&gt;"",S108="OK",OR(R108="PASS",R108="FAIL")),"YES","NO"))</x:f>
@@ -6597,7 +6597,7 @@
         <x:f>IF(A109="",IF(B109="","","MISSING_TEST_ID"),IF(B109="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A109,$B$2:$B$501,B109)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL109" s="9" t="str">
-        <x:f>IF(A109="","",IF(AND(AK109="OK",J109="READY",F109&lt;&gt;"",G109&lt;&gt;"",K109&lt;&gt;"",OR(L109="PASS",L109="FAIL"),M109&lt;&gt;"",O109&lt;&gt;"",P109="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A109="","",IF(AND(AK109="OK",J109="READY",F109&lt;&gt;"",G109&lt;&gt;"",K109&lt;&gt;"",OR(L109="PASS",L109="FAIL"),M109&lt;&gt;"",P109="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM109" s="9" t="str">
         <x:f>IF(A109="","",IF(AND(AK109="OK",J109="READY",F109&lt;&gt;"",G109&lt;&gt;"",K109&lt;&gt;"",S109="OK",OR(R109="PASS",R109="FAIL")),"YES","NO"))</x:f>
@@ -6649,7 +6649,7 @@
         <x:f>IF(A110="",IF(B110="","","MISSING_TEST_ID"),IF(B110="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A110,$B$2:$B$501,B110)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL110" s="9" t="str">
-        <x:f>IF(A110="","",IF(AND(AK110="OK",J110="READY",F110&lt;&gt;"",G110&lt;&gt;"",K110&lt;&gt;"",OR(L110="PASS",L110="FAIL"),M110&lt;&gt;"",O110&lt;&gt;"",P110="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A110="","",IF(AND(AK110="OK",J110="READY",F110&lt;&gt;"",G110&lt;&gt;"",K110&lt;&gt;"",OR(L110="PASS",L110="FAIL"),M110&lt;&gt;"",P110="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM110" s="9" t="str">
         <x:f>IF(A110="","",IF(AND(AK110="OK",J110="READY",F110&lt;&gt;"",G110&lt;&gt;"",K110&lt;&gt;"",S110="OK",OR(R110="PASS",R110="FAIL")),"YES","NO"))</x:f>
@@ -6701,7 +6701,7 @@
         <x:f>IF(A111="",IF(B111="","","MISSING_TEST_ID"),IF(B111="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A111,$B$2:$B$501,B111)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL111" s="9" t="str">
-        <x:f>IF(A111="","",IF(AND(AK111="OK",J111="READY",F111&lt;&gt;"",G111&lt;&gt;"",K111&lt;&gt;"",OR(L111="PASS",L111="FAIL"),M111&lt;&gt;"",O111&lt;&gt;"",P111="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A111="","",IF(AND(AK111="OK",J111="READY",F111&lt;&gt;"",G111&lt;&gt;"",K111&lt;&gt;"",OR(L111="PASS",L111="FAIL"),M111&lt;&gt;"",P111="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM111" s="9" t="str">
         <x:f>IF(A111="","",IF(AND(AK111="OK",J111="READY",F111&lt;&gt;"",G111&lt;&gt;"",K111&lt;&gt;"",S111="OK",OR(R111="PASS",R111="FAIL")),"YES","NO"))</x:f>
@@ -6753,7 +6753,7 @@
         <x:f>IF(A112="",IF(B112="","","MISSING_TEST_ID"),IF(B112="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A112,$B$2:$B$501,B112)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL112" s="9" t="str">
-        <x:f>IF(A112="","",IF(AND(AK112="OK",J112="READY",F112&lt;&gt;"",G112&lt;&gt;"",K112&lt;&gt;"",OR(L112="PASS",L112="FAIL"),M112&lt;&gt;"",O112&lt;&gt;"",P112="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A112="","",IF(AND(AK112="OK",J112="READY",F112&lt;&gt;"",G112&lt;&gt;"",K112&lt;&gt;"",OR(L112="PASS",L112="FAIL"),M112&lt;&gt;"",P112="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM112" s="9" t="str">
         <x:f>IF(A112="","",IF(AND(AK112="OK",J112="READY",F112&lt;&gt;"",G112&lt;&gt;"",K112&lt;&gt;"",S112="OK",OR(R112="PASS",R112="FAIL")),"YES","NO"))</x:f>
@@ -6805,7 +6805,7 @@
         <x:f>IF(A113="",IF(B113="","","MISSING_TEST_ID"),IF(B113="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A113,$B$2:$B$501,B113)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL113" s="9" t="str">
-        <x:f>IF(A113="","",IF(AND(AK113="OK",J113="READY",F113&lt;&gt;"",G113&lt;&gt;"",K113&lt;&gt;"",OR(L113="PASS",L113="FAIL"),M113&lt;&gt;"",O113&lt;&gt;"",P113="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A113="","",IF(AND(AK113="OK",J113="READY",F113&lt;&gt;"",G113&lt;&gt;"",K113&lt;&gt;"",OR(L113="PASS",L113="FAIL"),M113&lt;&gt;"",P113="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM113" s="9" t="str">
         <x:f>IF(A113="","",IF(AND(AK113="OK",J113="READY",F113&lt;&gt;"",G113&lt;&gt;"",K113&lt;&gt;"",S113="OK",OR(R113="PASS",R113="FAIL")),"YES","NO"))</x:f>
@@ -6857,7 +6857,7 @@
         <x:f>IF(A114="",IF(B114="","","MISSING_TEST_ID"),IF(B114="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A114,$B$2:$B$501,B114)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL114" s="9" t="str">
-        <x:f>IF(A114="","",IF(AND(AK114="OK",J114="READY",F114&lt;&gt;"",G114&lt;&gt;"",K114&lt;&gt;"",OR(L114="PASS",L114="FAIL"),M114&lt;&gt;"",O114&lt;&gt;"",P114="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A114="","",IF(AND(AK114="OK",J114="READY",F114&lt;&gt;"",G114&lt;&gt;"",K114&lt;&gt;"",OR(L114="PASS",L114="FAIL"),M114&lt;&gt;"",P114="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM114" s="9" t="str">
         <x:f>IF(A114="","",IF(AND(AK114="OK",J114="READY",F114&lt;&gt;"",G114&lt;&gt;"",K114&lt;&gt;"",S114="OK",OR(R114="PASS",R114="FAIL")),"YES","NO"))</x:f>
@@ -6909,7 +6909,7 @@
         <x:f>IF(A115="",IF(B115="","","MISSING_TEST_ID"),IF(B115="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A115,$B$2:$B$501,B115)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL115" s="9" t="str">
-        <x:f>IF(A115="","",IF(AND(AK115="OK",J115="READY",F115&lt;&gt;"",G115&lt;&gt;"",K115&lt;&gt;"",OR(L115="PASS",L115="FAIL"),M115&lt;&gt;"",O115&lt;&gt;"",P115="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A115="","",IF(AND(AK115="OK",J115="READY",F115&lt;&gt;"",G115&lt;&gt;"",K115&lt;&gt;"",OR(L115="PASS",L115="FAIL"),M115&lt;&gt;"",P115="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM115" s="9" t="str">
         <x:f>IF(A115="","",IF(AND(AK115="OK",J115="READY",F115&lt;&gt;"",G115&lt;&gt;"",K115&lt;&gt;"",S115="OK",OR(R115="PASS",R115="FAIL")),"YES","NO"))</x:f>
@@ -6961,7 +6961,7 @@
         <x:f>IF(A116="",IF(B116="","","MISSING_TEST_ID"),IF(B116="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A116,$B$2:$B$501,B116)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL116" s="9" t="str">
-        <x:f>IF(A116="","",IF(AND(AK116="OK",J116="READY",F116&lt;&gt;"",G116&lt;&gt;"",K116&lt;&gt;"",OR(L116="PASS",L116="FAIL"),M116&lt;&gt;"",O116&lt;&gt;"",P116="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A116="","",IF(AND(AK116="OK",J116="READY",F116&lt;&gt;"",G116&lt;&gt;"",K116&lt;&gt;"",OR(L116="PASS",L116="FAIL"),M116&lt;&gt;"",P116="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM116" s="9" t="str">
         <x:f>IF(A116="","",IF(AND(AK116="OK",J116="READY",F116&lt;&gt;"",G116&lt;&gt;"",K116&lt;&gt;"",S116="OK",OR(R116="PASS",R116="FAIL")),"YES","NO"))</x:f>
@@ -7013,7 +7013,7 @@
         <x:f>IF(A117="",IF(B117="","","MISSING_TEST_ID"),IF(B117="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A117,$B$2:$B$501,B117)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL117" s="9" t="str">
-        <x:f>IF(A117="","",IF(AND(AK117="OK",J117="READY",F117&lt;&gt;"",G117&lt;&gt;"",K117&lt;&gt;"",OR(L117="PASS",L117="FAIL"),M117&lt;&gt;"",O117&lt;&gt;"",P117="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A117="","",IF(AND(AK117="OK",J117="READY",F117&lt;&gt;"",G117&lt;&gt;"",K117&lt;&gt;"",OR(L117="PASS",L117="FAIL"),M117&lt;&gt;"",P117="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM117" s="9" t="str">
         <x:f>IF(A117="","",IF(AND(AK117="OK",J117="READY",F117&lt;&gt;"",G117&lt;&gt;"",K117&lt;&gt;"",S117="OK",OR(R117="PASS",R117="FAIL")),"YES","NO"))</x:f>
@@ -7065,7 +7065,7 @@
         <x:f>IF(A118="",IF(B118="","","MISSING_TEST_ID"),IF(B118="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A118,$B$2:$B$501,B118)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL118" s="9" t="str">
-        <x:f>IF(A118="","",IF(AND(AK118="OK",J118="READY",F118&lt;&gt;"",G118&lt;&gt;"",K118&lt;&gt;"",OR(L118="PASS",L118="FAIL"),M118&lt;&gt;"",O118&lt;&gt;"",P118="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A118="","",IF(AND(AK118="OK",J118="READY",F118&lt;&gt;"",G118&lt;&gt;"",K118&lt;&gt;"",OR(L118="PASS",L118="FAIL"),M118&lt;&gt;"",P118="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM118" s="9" t="str">
         <x:f>IF(A118="","",IF(AND(AK118="OK",J118="READY",F118&lt;&gt;"",G118&lt;&gt;"",K118&lt;&gt;"",S118="OK",OR(R118="PASS",R118="FAIL")),"YES","NO"))</x:f>
@@ -7117,7 +7117,7 @@
         <x:f>IF(A119="",IF(B119="","","MISSING_TEST_ID"),IF(B119="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A119,$B$2:$B$501,B119)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL119" s="9" t="str">
-        <x:f>IF(A119="","",IF(AND(AK119="OK",J119="READY",F119&lt;&gt;"",G119&lt;&gt;"",K119&lt;&gt;"",OR(L119="PASS",L119="FAIL"),M119&lt;&gt;"",O119&lt;&gt;"",P119="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A119="","",IF(AND(AK119="OK",J119="READY",F119&lt;&gt;"",G119&lt;&gt;"",K119&lt;&gt;"",OR(L119="PASS",L119="FAIL"),M119&lt;&gt;"",P119="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM119" s="9" t="str">
         <x:f>IF(A119="","",IF(AND(AK119="OK",J119="READY",F119&lt;&gt;"",G119&lt;&gt;"",K119&lt;&gt;"",S119="OK",OR(R119="PASS",R119="FAIL")),"YES","NO"))</x:f>
@@ -7169,7 +7169,7 @@
         <x:f>IF(A120="",IF(B120="","","MISSING_TEST_ID"),IF(B120="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A120,$B$2:$B$501,B120)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL120" s="9" t="str">
-        <x:f>IF(A120="","",IF(AND(AK120="OK",J120="READY",F120&lt;&gt;"",G120&lt;&gt;"",K120&lt;&gt;"",OR(L120="PASS",L120="FAIL"),M120&lt;&gt;"",O120&lt;&gt;"",P120="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A120="","",IF(AND(AK120="OK",J120="READY",F120&lt;&gt;"",G120&lt;&gt;"",K120&lt;&gt;"",OR(L120="PASS",L120="FAIL"),M120&lt;&gt;"",P120="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM120" s="9" t="str">
         <x:f>IF(A120="","",IF(AND(AK120="OK",J120="READY",F120&lt;&gt;"",G120&lt;&gt;"",K120&lt;&gt;"",S120="OK",OR(R120="PASS",R120="FAIL")),"YES","NO"))</x:f>
@@ -7221,7 +7221,7 @@
         <x:f>IF(A121="",IF(B121="","","MISSING_TEST_ID"),IF(B121="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A121,$B$2:$B$501,B121)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL121" s="9" t="str">
-        <x:f>IF(A121="","",IF(AND(AK121="OK",J121="READY",F121&lt;&gt;"",G121&lt;&gt;"",K121&lt;&gt;"",OR(L121="PASS",L121="FAIL"),M121&lt;&gt;"",O121&lt;&gt;"",P121="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A121="","",IF(AND(AK121="OK",J121="READY",F121&lt;&gt;"",G121&lt;&gt;"",K121&lt;&gt;"",OR(L121="PASS",L121="FAIL"),M121&lt;&gt;"",P121="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM121" s="9" t="str">
         <x:f>IF(A121="","",IF(AND(AK121="OK",J121="READY",F121&lt;&gt;"",G121&lt;&gt;"",K121&lt;&gt;"",S121="OK",OR(R121="PASS",R121="FAIL")),"YES","NO"))</x:f>
@@ -7273,7 +7273,7 @@
         <x:f>IF(A122="",IF(B122="","","MISSING_TEST_ID"),IF(B122="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A122,$B$2:$B$501,B122)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL122" s="9" t="str">
-        <x:f>IF(A122="","",IF(AND(AK122="OK",J122="READY",F122&lt;&gt;"",G122&lt;&gt;"",K122&lt;&gt;"",OR(L122="PASS",L122="FAIL"),M122&lt;&gt;"",O122&lt;&gt;"",P122="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A122="","",IF(AND(AK122="OK",J122="READY",F122&lt;&gt;"",G122&lt;&gt;"",K122&lt;&gt;"",OR(L122="PASS",L122="FAIL"),M122&lt;&gt;"",P122="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM122" s="9" t="str">
         <x:f>IF(A122="","",IF(AND(AK122="OK",J122="READY",F122&lt;&gt;"",G122&lt;&gt;"",K122&lt;&gt;"",S122="OK",OR(R122="PASS",R122="FAIL")),"YES","NO"))</x:f>
@@ -7325,7 +7325,7 @@
         <x:f>IF(A123="",IF(B123="","","MISSING_TEST_ID"),IF(B123="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A123,$B$2:$B$501,B123)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL123" s="9" t="str">
-        <x:f>IF(A123="","",IF(AND(AK123="OK",J123="READY",F123&lt;&gt;"",G123&lt;&gt;"",K123&lt;&gt;"",OR(L123="PASS",L123="FAIL"),M123&lt;&gt;"",O123&lt;&gt;"",P123="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A123="","",IF(AND(AK123="OK",J123="READY",F123&lt;&gt;"",G123&lt;&gt;"",K123&lt;&gt;"",OR(L123="PASS",L123="FAIL"),M123&lt;&gt;"",P123="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM123" s="9" t="str">
         <x:f>IF(A123="","",IF(AND(AK123="OK",J123="READY",F123&lt;&gt;"",G123&lt;&gt;"",K123&lt;&gt;"",S123="OK",OR(R123="PASS",R123="FAIL")),"YES","NO"))</x:f>
@@ -7377,7 +7377,7 @@
         <x:f>IF(A124="",IF(B124="","","MISSING_TEST_ID"),IF(B124="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A124,$B$2:$B$501,B124)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL124" s="9" t="str">
-        <x:f>IF(A124="","",IF(AND(AK124="OK",J124="READY",F124&lt;&gt;"",G124&lt;&gt;"",K124&lt;&gt;"",OR(L124="PASS",L124="FAIL"),M124&lt;&gt;"",O124&lt;&gt;"",P124="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A124="","",IF(AND(AK124="OK",J124="READY",F124&lt;&gt;"",G124&lt;&gt;"",K124&lt;&gt;"",OR(L124="PASS",L124="FAIL"),M124&lt;&gt;"",P124="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM124" s="9" t="str">
         <x:f>IF(A124="","",IF(AND(AK124="OK",J124="READY",F124&lt;&gt;"",G124&lt;&gt;"",K124&lt;&gt;"",S124="OK",OR(R124="PASS",R124="FAIL")),"YES","NO"))</x:f>
@@ -7429,7 +7429,7 @@
         <x:f>IF(A125="",IF(B125="","","MISSING_TEST_ID"),IF(B125="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A125,$B$2:$B$501,B125)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL125" s="9" t="str">
-        <x:f>IF(A125="","",IF(AND(AK125="OK",J125="READY",F125&lt;&gt;"",G125&lt;&gt;"",K125&lt;&gt;"",OR(L125="PASS",L125="FAIL"),M125&lt;&gt;"",O125&lt;&gt;"",P125="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A125="","",IF(AND(AK125="OK",J125="READY",F125&lt;&gt;"",G125&lt;&gt;"",K125&lt;&gt;"",OR(L125="PASS",L125="FAIL"),M125&lt;&gt;"",P125="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM125" s="9" t="str">
         <x:f>IF(A125="","",IF(AND(AK125="OK",J125="READY",F125&lt;&gt;"",G125&lt;&gt;"",K125&lt;&gt;"",S125="OK",OR(R125="PASS",R125="FAIL")),"YES","NO"))</x:f>
@@ -7481,7 +7481,7 @@
         <x:f>IF(A126="",IF(B126="","","MISSING_TEST_ID"),IF(B126="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A126,$B$2:$B$501,B126)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL126" s="9" t="str">
-        <x:f>IF(A126="","",IF(AND(AK126="OK",J126="READY",F126&lt;&gt;"",G126&lt;&gt;"",K126&lt;&gt;"",OR(L126="PASS",L126="FAIL"),M126&lt;&gt;"",O126&lt;&gt;"",P126="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A126="","",IF(AND(AK126="OK",J126="READY",F126&lt;&gt;"",G126&lt;&gt;"",K126&lt;&gt;"",OR(L126="PASS",L126="FAIL"),M126&lt;&gt;"",P126="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM126" s="9" t="str">
         <x:f>IF(A126="","",IF(AND(AK126="OK",J126="READY",F126&lt;&gt;"",G126&lt;&gt;"",K126&lt;&gt;"",S126="OK",OR(R126="PASS",R126="FAIL")),"YES","NO"))</x:f>
@@ -7533,7 +7533,7 @@
         <x:f>IF(A127="",IF(B127="","","MISSING_TEST_ID"),IF(B127="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A127,$B$2:$B$501,B127)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL127" s="9" t="str">
-        <x:f>IF(A127="","",IF(AND(AK127="OK",J127="READY",F127&lt;&gt;"",G127&lt;&gt;"",K127&lt;&gt;"",OR(L127="PASS",L127="FAIL"),M127&lt;&gt;"",O127&lt;&gt;"",P127="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A127="","",IF(AND(AK127="OK",J127="READY",F127&lt;&gt;"",G127&lt;&gt;"",K127&lt;&gt;"",OR(L127="PASS",L127="FAIL"),M127&lt;&gt;"",P127="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM127" s="9" t="str">
         <x:f>IF(A127="","",IF(AND(AK127="OK",J127="READY",F127&lt;&gt;"",G127&lt;&gt;"",K127&lt;&gt;"",S127="OK",OR(R127="PASS",R127="FAIL")),"YES","NO"))</x:f>
@@ -7585,7 +7585,7 @@
         <x:f>IF(A128="",IF(B128="","","MISSING_TEST_ID"),IF(B128="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A128,$B$2:$B$501,B128)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL128" s="9" t="str">
-        <x:f>IF(A128="","",IF(AND(AK128="OK",J128="READY",F128&lt;&gt;"",G128&lt;&gt;"",K128&lt;&gt;"",OR(L128="PASS",L128="FAIL"),M128&lt;&gt;"",O128&lt;&gt;"",P128="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A128="","",IF(AND(AK128="OK",J128="READY",F128&lt;&gt;"",G128&lt;&gt;"",K128&lt;&gt;"",OR(L128="PASS",L128="FAIL"),M128&lt;&gt;"",P128="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM128" s="9" t="str">
         <x:f>IF(A128="","",IF(AND(AK128="OK",J128="READY",F128&lt;&gt;"",G128&lt;&gt;"",K128&lt;&gt;"",S128="OK",OR(R128="PASS",R128="FAIL")),"YES","NO"))</x:f>
@@ -7637,7 +7637,7 @@
         <x:f>IF(A129="",IF(B129="","","MISSING_TEST_ID"),IF(B129="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A129,$B$2:$B$501,B129)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL129" s="9" t="str">
-        <x:f>IF(A129="","",IF(AND(AK129="OK",J129="READY",F129&lt;&gt;"",G129&lt;&gt;"",K129&lt;&gt;"",OR(L129="PASS",L129="FAIL"),M129&lt;&gt;"",O129&lt;&gt;"",P129="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A129="","",IF(AND(AK129="OK",J129="READY",F129&lt;&gt;"",G129&lt;&gt;"",K129&lt;&gt;"",OR(L129="PASS",L129="FAIL"),M129&lt;&gt;"",P129="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM129" s="9" t="str">
         <x:f>IF(A129="","",IF(AND(AK129="OK",J129="READY",F129&lt;&gt;"",G129&lt;&gt;"",K129&lt;&gt;"",S129="OK",OR(R129="PASS",R129="FAIL")),"YES","NO"))</x:f>
@@ -7689,7 +7689,7 @@
         <x:f>IF(A130="",IF(B130="","","MISSING_TEST_ID"),IF(B130="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A130,$B$2:$B$501,B130)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL130" s="9" t="str">
-        <x:f>IF(A130="","",IF(AND(AK130="OK",J130="READY",F130&lt;&gt;"",G130&lt;&gt;"",K130&lt;&gt;"",OR(L130="PASS",L130="FAIL"),M130&lt;&gt;"",O130&lt;&gt;"",P130="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A130="","",IF(AND(AK130="OK",J130="READY",F130&lt;&gt;"",G130&lt;&gt;"",K130&lt;&gt;"",OR(L130="PASS",L130="FAIL"),M130&lt;&gt;"",P130="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM130" s="9" t="str">
         <x:f>IF(A130="","",IF(AND(AK130="OK",J130="READY",F130&lt;&gt;"",G130&lt;&gt;"",K130&lt;&gt;"",S130="OK",OR(R130="PASS",R130="FAIL")),"YES","NO"))</x:f>
@@ -7741,7 +7741,7 @@
         <x:f>IF(A131="",IF(B131="","","MISSING_TEST_ID"),IF(B131="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A131,$B$2:$B$501,B131)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL131" s="9" t="str">
-        <x:f>IF(A131="","",IF(AND(AK131="OK",J131="READY",F131&lt;&gt;"",G131&lt;&gt;"",K131&lt;&gt;"",OR(L131="PASS",L131="FAIL"),M131&lt;&gt;"",O131&lt;&gt;"",P131="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A131="","",IF(AND(AK131="OK",J131="READY",F131&lt;&gt;"",G131&lt;&gt;"",K131&lt;&gt;"",OR(L131="PASS",L131="FAIL"),M131&lt;&gt;"",P131="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM131" s="9" t="str">
         <x:f>IF(A131="","",IF(AND(AK131="OK",J131="READY",F131&lt;&gt;"",G131&lt;&gt;"",K131&lt;&gt;"",S131="OK",OR(R131="PASS",R131="FAIL")),"YES","NO"))</x:f>
@@ -7793,7 +7793,7 @@
         <x:f>IF(A132="",IF(B132="","","MISSING_TEST_ID"),IF(B132="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A132,$B$2:$B$501,B132)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL132" s="9" t="str">
-        <x:f>IF(A132="","",IF(AND(AK132="OK",J132="READY",F132&lt;&gt;"",G132&lt;&gt;"",K132&lt;&gt;"",OR(L132="PASS",L132="FAIL"),M132&lt;&gt;"",O132&lt;&gt;"",P132="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A132="","",IF(AND(AK132="OK",J132="READY",F132&lt;&gt;"",G132&lt;&gt;"",K132&lt;&gt;"",OR(L132="PASS",L132="FAIL"),M132&lt;&gt;"",P132="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM132" s="9" t="str">
         <x:f>IF(A132="","",IF(AND(AK132="OK",J132="READY",F132&lt;&gt;"",G132&lt;&gt;"",K132&lt;&gt;"",S132="OK",OR(R132="PASS",R132="FAIL")),"YES","NO"))</x:f>
@@ -7845,7 +7845,7 @@
         <x:f>IF(A133="",IF(B133="","","MISSING_TEST_ID"),IF(B133="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A133,$B$2:$B$501,B133)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL133" s="9" t="str">
-        <x:f>IF(A133="","",IF(AND(AK133="OK",J133="READY",F133&lt;&gt;"",G133&lt;&gt;"",K133&lt;&gt;"",OR(L133="PASS",L133="FAIL"),M133&lt;&gt;"",O133&lt;&gt;"",P133="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A133="","",IF(AND(AK133="OK",J133="READY",F133&lt;&gt;"",G133&lt;&gt;"",K133&lt;&gt;"",OR(L133="PASS",L133="FAIL"),M133&lt;&gt;"",P133="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM133" s="9" t="str">
         <x:f>IF(A133="","",IF(AND(AK133="OK",J133="READY",F133&lt;&gt;"",G133&lt;&gt;"",K133&lt;&gt;"",S133="OK",OR(R133="PASS",R133="FAIL")),"YES","NO"))</x:f>
@@ -7897,7 +7897,7 @@
         <x:f>IF(A134="",IF(B134="","","MISSING_TEST_ID"),IF(B134="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A134,$B$2:$B$501,B134)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL134" s="9" t="str">
-        <x:f>IF(A134="","",IF(AND(AK134="OK",J134="READY",F134&lt;&gt;"",G134&lt;&gt;"",K134&lt;&gt;"",OR(L134="PASS",L134="FAIL"),M134&lt;&gt;"",O134&lt;&gt;"",P134="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A134="","",IF(AND(AK134="OK",J134="READY",F134&lt;&gt;"",G134&lt;&gt;"",K134&lt;&gt;"",OR(L134="PASS",L134="FAIL"),M134&lt;&gt;"",P134="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM134" s="9" t="str">
         <x:f>IF(A134="","",IF(AND(AK134="OK",J134="READY",F134&lt;&gt;"",G134&lt;&gt;"",K134&lt;&gt;"",S134="OK",OR(R134="PASS",R134="FAIL")),"YES","NO"))</x:f>
@@ -7949,7 +7949,7 @@
         <x:f>IF(A135="",IF(B135="","","MISSING_TEST_ID"),IF(B135="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A135,$B$2:$B$501,B135)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL135" s="9" t="str">
-        <x:f>IF(A135="","",IF(AND(AK135="OK",J135="READY",F135&lt;&gt;"",G135&lt;&gt;"",K135&lt;&gt;"",OR(L135="PASS",L135="FAIL"),M135&lt;&gt;"",O135&lt;&gt;"",P135="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A135="","",IF(AND(AK135="OK",J135="READY",F135&lt;&gt;"",G135&lt;&gt;"",K135&lt;&gt;"",OR(L135="PASS",L135="FAIL"),M135&lt;&gt;"",P135="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM135" s="9" t="str">
         <x:f>IF(A135="","",IF(AND(AK135="OK",J135="READY",F135&lt;&gt;"",G135&lt;&gt;"",K135&lt;&gt;"",S135="OK",OR(R135="PASS",R135="FAIL")),"YES","NO"))</x:f>
@@ -8001,7 +8001,7 @@
         <x:f>IF(A136="",IF(B136="","","MISSING_TEST_ID"),IF(B136="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A136,$B$2:$B$501,B136)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL136" s="9" t="str">
-        <x:f>IF(A136="","",IF(AND(AK136="OK",J136="READY",F136&lt;&gt;"",G136&lt;&gt;"",K136&lt;&gt;"",OR(L136="PASS",L136="FAIL"),M136&lt;&gt;"",O136&lt;&gt;"",P136="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A136="","",IF(AND(AK136="OK",J136="READY",F136&lt;&gt;"",G136&lt;&gt;"",K136&lt;&gt;"",OR(L136="PASS",L136="FAIL"),M136&lt;&gt;"",P136="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM136" s="9" t="str">
         <x:f>IF(A136="","",IF(AND(AK136="OK",J136="READY",F136&lt;&gt;"",G136&lt;&gt;"",K136&lt;&gt;"",S136="OK",OR(R136="PASS",R136="FAIL")),"YES","NO"))</x:f>
@@ -8053,7 +8053,7 @@
         <x:f>IF(A137="",IF(B137="","","MISSING_TEST_ID"),IF(B137="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A137,$B$2:$B$501,B137)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL137" s="9" t="str">
-        <x:f>IF(A137="","",IF(AND(AK137="OK",J137="READY",F137&lt;&gt;"",G137&lt;&gt;"",K137&lt;&gt;"",OR(L137="PASS",L137="FAIL"),M137&lt;&gt;"",O137&lt;&gt;"",P137="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A137="","",IF(AND(AK137="OK",J137="READY",F137&lt;&gt;"",G137&lt;&gt;"",K137&lt;&gt;"",OR(L137="PASS",L137="FAIL"),M137&lt;&gt;"",P137="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM137" s="9" t="str">
         <x:f>IF(A137="","",IF(AND(AK137="OK",J137="READY",F137&lt;&gt;"",G137&lt;&gt;"",K137&lt;&gt;"",S137="OK",OR(R137="PASS",R137="FAIL")),"YES","NO"))</x:f>
@@ -8105,7 +8105,7 @@
         <x:f>IF(A138="",IF(B138="","","MISSING_TEST_ID"),IF(B138="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A138,$B$2:$B$501,B138)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL138" s="9" t="str">
-        <x:f>IF(A138="","",IF(AND(AK138="OK",J138="READY",F138&lt;&gt;"",G138&lt;&gt;"",K138&lt;&gt;"",OR(L138="PASS",L138="FAIL"),M138&lt;&gt;"",O138&lt;&gt;"",P138="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A138="","",IF(AND(AK138="OK",J138="READY",F138&lt;&gt;"",G138&lt;&gt;"",K138&lt;&gt;"",OR(L138="PASS",L138="FAIL"),M138&lt;&gt;"",P138="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM138" s="9" t="str">
         <x:f>IF(A138="","",IF(AND(AK138="OK",J138="READY",F138&lt;&gt;"",G138&lt;&gt;"",K138&lt;&gt;"",S138="OK",OR(R138="PASS",R138="FAIL")),"YES","NO"))</x:f>
@@ -8157,7 +8157,7 @@
         <x:f>IF(A139="",IF(B139="","","MISSING_TEST_ID"),IF(B139="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A139,$B$2:$B$501,B139)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL139" s="9" t="str">
-        <x:f>IF(A139="","",IF(AND(AK139="OK",J139="READY",F139&lt;&gt;"",G139&lt;&gt;"",K139&lt;&gt;"",OR(L139="PASS",L139="FAIL"),M139&lt;&gt;"",O139&lt;&gt;"",P139="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A139="","",IF(AND(AK139="OK",J139="READY",F139&lt;&gt;"",G139&lt;&gt;"",K139&lt;&gt;"",OR(L139="PASS",L139="FAIL"),M139&lt;&gt;"",P139="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM139" s="9" t="str">
         <x:f>IF(A139="","",IF(AND(AK139="OK",J139="READY",F139&lt;&gt;"",G139&lt;&gt;"",K139&lt;&gt;"",S139="OK",OR(R139="PASS",R139="FAIL")),"YES","NO"))</x:f>
@@ -8209,7 +8209,7 @@
         <x:f>IF(A140="",IF(B140="","","MISSING_TEST_ID"),IF(B140="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A140,$B$2:$B$501,B140)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL140" s="9" t="str">
-        <x:f>IF(A140="","",IF(AND(AK140="OK",J140="READY",F140&lt;&gt;"",G140&lt;&gt;"",K140&lt;&gt;"",OR(L140="PASS",L140="FAIL"),M140&lt;&gt;"",O140&lt;&gt;"",P140="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A140="","",IF(AND(AK140="OK",J140="READY",F140&lt;&gt;"",G140&lt;&gt;"",K140&lt;&gt;"",OR(L140="PASS",L140="FAIL"),M140&lt;&gt;"",P140="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM140" s="9" t="str">
         <x:f>IF(A140="","",IF(AND(AK140="OK",J140="READY",F140&lt;&gt;"",G140&lt;&gt;"",K140&lt;&gt;"",S140="OK",OR(R140="PASS",R140="FAIL")),"YES","NO"))</x:f>
@@ -8261,7 +8261,7 @@
         <x:f>IF(A141="",IF(B141="","","MISSING_TEST_ID"),IF(B141="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A141,$B$2:$B$501,B141)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL141" s="9" t="str">
-        <x:f>IF(A141="","",IF(AND(AK141="OK",J141="READY",F141&lt;&gt;"",G141&lt;&gt;"",K141&lt;&gt;"",OR(L141="PASS",L141="FAIL"),M141&lt;&gt;"",O141&lt;&gt;"",P141="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A141="","",IF(AND(AK141="OK",J141="READY",F141&lt;&gt;"",G141&lt;&gt;"",K141&lt;&gt;"",OR(L141="PASS",L141="FAIL"),M141&lt;&gt;"",P141="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM141" s="9" t="str">
         <x:f>IF(A141="","",IF(AND(AK141="OK",J141="READY",F141&lt;&gt;"",G141&lt;&gt;"",K141&lt;&gt;"",S141="OK",OR(R141="PASS",R141="FAIL")),"YES","NO"))</x:f>
@@ -8313,7 +8313,7 @@
         <x:f>IF(A142="",IF(B142="","","MISSING_TEST_ID"),IF(B142="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A142,$B$2:$B$501,B142)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL142" s="9" t="str">
-        <x:f>IF(A142="","",IF(AND(AK142="OK",J142="READY",F142&lt;&gt;"",G142&lt;&gt;"",K142&lt;&gt;"",OR(L142="PASS",L142="FAIL"),M142&lt;&gt;"",O142&lt;&gt;"",P142="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A142="","",IF(AND(AK142="OK",J142="READY",F142&lt;&gt;"",G142&lt;&gt;"",K142&lt;&gt;"",OR(L142="PASS",L142="FAIL"),M142&lt;&gt;"",P142="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM142" s="9" t="str">
         <x:f>IF(A142="","",IF(AND(AK142="OK",J142="READY",F142&lt;&gt;"",G142&lt;&gt;"",K142&lt;&gt;"",S142="OK",OR(R142="PASS",R142="FAIL")),"YES","NO"))</x:f>
@@ -8365,7 +8365,7 @@
         <x:f>IF(A143="",IF(B143="","","MISSING_TEST_ID"),IF(B143="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A143,$B$2:$B$501,B143)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL143" s="9" t="str">
-        <x:f>IF(A143="","",IF(AND(AK143="OK",J143="READY",F143&lt;&gt;"",G143&lt;&gt;"",K143&lt;&gt;"",OR(L143="PASS",L143="FAIL"),M143&lt;&gt;"",O143&lt;&gt;"",P143="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A143="","",IF(AND(AK143="OK",J143="READY",F143&lt;&gt;"",G143&lt;&gt;"",K143&lt;&gt;"",OR(L143="PASS",L143="FAIL"),M143&lt;&gt;"",P143="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM143" s="9" t="str">
         <x:f>IF(A143="","",IF(AND(AK143="OK",J143="READY",F143&lt;&gt;"",G143&lt;&gt;"",K143&lt;&gt;"",S143="OK",OR(R143="PASS",R143="FAIL")),"YES","NO"))</x:f>
@@ -8417,7 +8417,7 @@
         <x:f>IF(A144="",IF(B144="","","MISSING_TEST_ID"),IF(B144="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A144,$B$2:$B$501,B144)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL144" s="9" t="str">
-        <x:f>IF(A144="","",IF(AND(AK144="OK",J144="READY",F144&lt;&gt;"",G144&lt;&gt;"",K144&lt;&gt;"",OR(L144="PASS",L144="FAIL"),M144&lt;&gt;"",O144&lt;&gt;"",P144="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A144="","",IF(AND(AK144="OK",J144="READY",F144&lt;&gt;"",G144&lt;&gt;"",K144&lt;&gt;"",OR(L144="PASS",L144="FAIL"),M144&lt;&gt;"",P144="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM144" s="9" t="str">
         <x:f>IF(A144="","",IF(AND(AK144="OK",J144="READY",F144&lt;&gt;"",G144&lt;&gt;"",K144&lt;&gt;"",S144="OK",OR(R144="PASS",R144="FAIL")),"YES","NO"))</x:f>
@@ -8469,7 +8469,7 @@
         <x:f>IF(A145="",IF(B145="","","MISSING_TEST_ID"),IF(B145="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A145,$B$2:$B$501,B145)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL145" s="9" t="str">
-        <x:f>IF(A145="","",IF(AND(AK145="OK",J145="READY",F145&lt;&gt;"",G145&lt;&gt;"",K145&lt;&gt;"",OR(L145="PASS",L145="FAIL"),M145&lt;&gt;"",O145&lt;&gt;"",P145="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A145="","",IF(AND(AK145="OK",J145="READY",F145&lt;&gt;"",G145&lt;&gt;"",K145&lt;&gt;"",OR(L145="PASS",L145="FAIL"),M145&lt;&gt;"",P145="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM145" s="9" t="str">
         <x:f>IF(A145="","",IF(AND(AK145="OK",J145="READY",F145&lt;&gt;"",G145&lt;&gt;"",K145&lt;&gt;"",S145="OK",OR(R145="PASS",R145="FAIL")),"YES","NO"))</x:f>
@@ -8521,7 +8521,7 @@
         <x:f>IF(A146="",IF(B146="","","MISSING_TEST_ID"),IF(B146="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A146,$B$2:$B$501,B146)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL146" s="9" t="str">
-        <x:f>IF(A146="","",IF(AND(AK146="OK",J146="READY",F146&lt;&gt;"",G146&lt;&gt;"",K146&lt;&gt;"",OR(L146="PASS",L146="FAIL"),M146&lt;&gt;"",O146&lt;&gt;"",P146="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A146="","",IF(AND(AK146="OK",J146="READY",F146&lt;&gt;"",G146&lt;&gt;"",K146&lt;&gt;"",OR(L146="PASS",L146="FAIL"),M146&lt;&gt;"",P146="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM146" s="9" t="str">
         <x:f>IF(A146="","",IF(AND(AK146="OK",J146="READY",F146&lt;&gt;"",G146&lt;&gt;"",K146&lt;&gt;"",S146="OK",OR(R146="PASS",R146="FAIL")),"YES","NO"))</x:f>
@@ -8573,7 +8573,7 @@
         <x:f>IF(A147="",IF(B147="","","MISSING_TEST_ID"),IF(B147="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A147,$B$2:$B$501,B147)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL147" s="9" t="str">
-        <x:f>IF(A147="","",IF(AND(AK147="OK",J147="READY",F147&lt;&gt;"",G147&lt;&gt;"",K147&lt;&gt;"",OR(L147="PASS",L147="FAIL"),M147&lt;&gt;"",O147&lt;&gt;"",P147="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A147="","",IF(AND(AK147="OK",J147="READY",F147&lt;&gt;"",G147&lt;&gt;"",K147&lt;&gt;"",OR(L147="PASS",L147="FAIL"),M147&lt;&gt;"",P147="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM147" s="9" t="str">
         <x:f>IF(A147="","",IF(AND(AK147="OK",J147="READY",F147&lt;&gt;"",G147&lt;&gt;"",K147&lt;&gt;"",S147="OK",OR(R147="PASS",R147="FAIL")),"YES","NO"))</x:f>
@@ -8625,7 +8625,7 @@
         <x:f>IF(A148="",IF(B148="","","MISSING_TEST_ID"),IF(B148="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A148,$B$2:$B$501,B148)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL148" s="9" t="str">
-        <x:f>IF(A148="","",IF(AND(AK148="OK",J148="READY",F148&lt;&gt;"",G148&lt;&gt;"",K148&lt;&gt;"",OR(L148="PASS",L148="FAIL"),M148&lt;&gt;"",O148&lt;&gt;"",P148="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A148="","",IF(AND(AK148="OK",J148="READY",F148&lt;&gt;"",G148&lt;&gt;"",K148&lt;&gt;"",OR(L148="PASS",L148="FAIL"),M148&lt;&gt;"",P148="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM148" s="9" t="str">
         <x:f>IF(A148="","",IF(AND(AK148="OK",J148="READY",F148&lt;&gt;"",G148&lt;&gt;"",K148&lt;&gt;"",S148="OK",OR(R148="PASS",R148="FAIL")),"YES","NO"))</x:f>
@@ -8677,7 +8677,7 @@
         <x:f>IF(A149="",IF(B149="","","MISSING_TEST_ID"),IF(B149="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A149,$B$2:$B$501,B149)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL149" s="9" t="str">
-        <x:f>IF(A149="","",IF(AND(AK149="OK",J149="READY",F149&lt;&gt;"",G149&lt;&gt;"",K149&lt;&gt;"",OR(L149="PASS",L149="FAIL"),M149&lt;&gt;"",O149&lt;&gt;"",P149="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A149="","",IF(AND(AK149="OK",J149="READY",F149&lt;&gt;"",G149&lt;&gt;"",K149&lt;&gt;"",OR(L149="PASS",L149="FAIL"),M149&lt;&gt;"",P149="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM149" s="9" t="str">
         <x:f>IF(A149="","",IF(AND(AK149="OK",J149="READY",F149&lt;&gt;"",G149&lt;&gt;"",K149&lt;&gt;"",S149="OK",OR(R149="PASS",R149="FAIL")),"YES","NO"))</x:f>
@@ -8729,7 +8729,7 @@
         <x:f>IF(A150="",IF(B150="","","MISSING_TEST_ID"),IF(B150="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A150,$B$2:$B$501,B150)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL150" s="9" t="str">
-        <x:f>IF(A150="","",IF(AND(AK150="OK",J150="READY",F150&lt;&gt;"",G150&lt;&gt;"",K150&lt;&gt;"",OR(L150="PASS",L150="FAIL"),M150&lt;&gt;"",O150&lt;&gt;"",P150="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A150="","",IF(AND(AK150="OK",J150="READY",F150&lt;&gt;"",G150&lt;&gt;"",K150&lt;&gt;"",OR(L150="PASS",L150="FAIL"),M150&lt;&gt;"",P150="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM150" s="9" t="str">
         <x:f>IF(A150="","",IF(AND(AK150="OK",J150="READY",F150&lt;&gt;"",G150&lt;&gt;"",K150&lt;&gt;"",S150="OK",OR(R150="PASS",R150="FAIL")),"YES","NO"))</x:f>
@@ -8781,7 +8781,7 @@
         <x:f>IF(A151="",IF(B151="","","MISSING_TEST_ID"),IF(B151="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A151,$B$2:$B$501,B151)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL151" s="9" t="str">
-        <x:f>IF(A151="","",IF(AND(AK151="OK",J151="READY",F151&lt;&gt;"",G151&lt;&gt;"",K151&lt;&gt;"",OR(L151="PASS",L151="FAIL"),M151&lt;&gt;"",O151&lt;&gt;"",P151="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A151="","",IF(AND(AK151="OK",J151="READY",F151&lt;&gt;"",G151&lt;&gt;"",K151&lt;&gt;"",OR(L151="PASS",L151="FAIL"),M151&lt;&gt;"",P151="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM151" s="9" t="str">
         <x:f>IF(A151="","",IF(AND(AK151="OK",J151="READY",F151&lt;&gt;"",G151&lt;&gt;"",K151&lt;&gt;"",S151="OK",OR(R151="PASS",R151="FAIL")),"YES","NO"))</x:f>
@@ -8833,7 +8833,7 @@
         <x:f>IF(A152="",IF(B152="","","MISSING_TEST_ID"),IF(B152="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A152,$B$2:$B$501,B152)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL152" s="9" t="str">
-        <x:f>IF(A152="","",IF(AND(AK152="OK",J152="READY",F152&lt;&gt;"",G152&lt;&gt;"",K152&lt;&gt;"",OR(L152="PASS",L152="FAIL"),M152&lt;&gt;"",O152&lt;&gt;"",P152="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A152="","",IF(AND(AK152="OK",J152="READY",F152&lt;&gt;"",G152&lt;&gt;"",K152&lt;&gt;"",OR(L152="PASS",L152="FAIL"),M152&lt;&gt;"",P152="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM152" s="9" t="str">
         <x:f>IF(A152="","",IF(AND(AK152="OK",J152="READY",F152&lt;&gt;"",G152&lt;&gt;"",K152&lt;&gt;"",S152="OK",OR(R152="PASS",R152="FAIL")),"YES","NO"))</x:f>
@@ -8885,7 +8885,7 @@
         <x:f>IF(A153="",IF(B153="","","MISSING_TEST_ID"),IF(B153="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A153,$B$2:$B$501,B153)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL153" s="9" t="str">
-        <x:f>IF(A153="","",IF(AND(AK153="OK",J153="READY",F153&lt;&gt;"",G153&lt;&gt;"",K153&lt;&gt;"",OR(L153="PASS",L153="FAIL"),M153&lt;&gt;"",O153&lt;&gt;"",P153="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A153="","",IF(AND(AK153="OK",J153="READY",F153&lt;&gt;"",G153&lt;&gt;"",K153&lt;&gt;"",OR(L153="PASS",L153="FAIL"),M153&lt;&gt;"",P153="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM153" s="9" t="str">
         <x:f>IF(A153="","",IF(AND(AK153="OK",J153="READY",F153&lt;&gt;"",G153&lt;&gt;"",K153&lt;&gt;"",S153="OK",OR(R153="PASS",R153="FAIL")),"YES","NO"))</x:f>
@@ -8937,7 +8937,7 @@
         <x:f>IF(A154="",IF(B154="","","MISSING_TEST_ID"),IF(B154="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A154,$B$2:$B$501,B154)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL154" s="9" t="str">
-        <x:f>IF(A154="","",IF(AND(AK154="OK",J154="READY",F154&lt;&gt;"",G154&lt;&gt;"",K154&lt;&gt;"",OR(L154="PASS",L154="FAIL"),M154&lt;&gt;"",O154&lt;&gt;"",P154="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A154="","",IF(AND(AK154="OK",J154="READY",F154&lt;&gt;"",G154&lt;&gt;"",K154&lt;&gt;"",OR(L154="PASS",L154="FAIL"),M154&lt;&gt;"",P154="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM154" s="9" t="str">
         <x:f>IF(A154="","",IF(AND(AK154="OK",J154="READY",F154&lt;&gt;"",G154&lt;&gt;"",K154&lt;&gt;"",S154="OK",OR(R154="PASS",R154="FAIL")),"YES","NO"))</x:f>
@@ -8989,7 +8989,7 @@
         <x:f>IF(A155="",IF(B155="","","MISSING_TEST_ID"),IF(B155="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A155,$B$2:$B$501,B155)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL155" s="9" t="str">
-        <x:f>IF(A155="","",IF(AND(AK155="OK",J155="READY",F155&lt;&gt;"",G155&lt;&gt;"",K155&lt;&gt;"",OR(L155="PASS",L155="FAIL"),M155&lt;&gt;"",O155&lt;&gt;"",P155="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A155="","",IF(AND(AK155="OK",J155="READY",F155&lt;&gt;"",G155&lt;&gt;"",K155&lt;&gt;"",OR(L155="PASS",L155="FAIL"),M155&lt;&gt;"",P155="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM155" s="9" t="str">
         <x:f>IF(A155="","",IF(AND(AK155="OK",J155="READY",F155&lt;&gt;"",G155&lt;&gt;"",K155&lt;&gt;"",S155="OK",OR(R155="PASS",R155="FAIL")),"YES","NO"))</x:f>
@@ -9041,7 +9041,7 @@
         <x:f>IF(A156="",IF(B156="","","MISSING_TEST_ID"),IF(B156="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A156,$B$2:$B$501,B156)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL156" s="9" t="str">
-        <x:f>IF(A156="","",IF(AND(AK156="OK",J156="READY",F156&lt;&gt;"",G156&lt;&gt;"",K156&lt;&gt;"",OR(L156="PASS",L156="FAIL"),M156&lt;&gt;"",O156&lt;&gt;"",P156="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A156="","",IF(AND(AK156="OK",J156="READY",F156&lt;&gt;"",G156&lt;&gt;"",K156&lt;&gt;"",OR(L156="PASS",L156="FAIL"),M156&lt;&gt;"",P156="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM156" s="9" t="str">
         <x:f>IF(A156="","",IF(AND(AK156="OK",J156="READY",F156&lt;&gt;"",G156&lt;&gt;"",K156&lt;&gt;"",S156="OK",OR(R156="PASS",R156="FAIL")),"YES","NO"))</x:f>
@@ -9093,7 +9093,7 @@
         <x:f>IF(A157="",IF(B157="","","MISSING_TEST_ID"),IF(B157="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A157,$B$2:$B$501,B157)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL157" s="9" t="str">
-        <x:f>IF(A157="","",IF(AND(AK157="OK",J157="READY",F157&lt;&gt;"",G157&lt;&gt;"",K157&lt;&gt;"",OR(L157="PASS",L157="FAIL"),M157&lt;&gt;"",O157&lt;&gt;"",P157="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A157="","",IF(AND(AK157="OK",J157="READY",F157&lt;&gt;"",G157&lt;&gt;"",K157&lt;&gt;"",OR(L157="PASS",L157="FAIL"),M157&lt;&gt;"",P157="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM157" s="9" t="str">
         <x:f>IF(A157="","",IF(AND(AK157="OK",J157="READY",F157&lt;&gt;"",G157&lt;&gt;"",K157&lt;&gt;"",S157="OK",OR(R157="PASS",R157="FAIL")),"YES","NO"))</x:f>
@@ -9145,7 +9145,7 @@
         <x:f>IF(A158="",IF(B158="","","MISSING_TEST_ID"),IF(B158="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A158,$B$2:$B$501,B158)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL158" s="9" t="str">
-        <x:f>IF(A158="","",IF(AND(AK158="OK",J158="READY",F158&lt;&gt;"",G158&lt;&gt;"",K158&lt;&gt;"",OR(L158="PASS",L158="FAIL"),M158&lt;&gt;"",O158&lt;&gt;"",P158="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A158="","",IF(AND(AK158="OK",J158="READY",F158&lt;&gt;"",G158&lt;&gt;"",K158&lt;&gt;"",OR(L158="PASS",L158="FAIL"),M158&lt;&gt;"",P158="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM158" s="9" t="str">
         <x:f>IF(A158="","",IF(AND(AK158="OK",J158="READY",F158&lt;&gt;"",G158&lt;&gt;"",K158&lt;&gt;"",S158="OK",OR(R158="PASS",R158="FAIL")),"YES","NO"))</x:f>
@@ -9197,7 +9197,7 @@
         <x:f>IF(A159="",IF(B159="","","MISSING_TEST_ID"),IF(B159="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A159,$B$2:$B$501,B159)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL159" s="9" t="str">
-        <x:f>IF(A159="","",IF(AND(AK159="OK",J159="READY",F159&lt;&gt;"",G159&lt;&gt;"",K159&lt;&gt;"",OR(L159="PASS",L159="FAIL"),M159&lt;&gt;"",O159&lt;&gt;"",P159="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A159="","",IF(AND(AK159="OK",J159="READY",F159&lt;&gt;"",G159&lt;&gt;"",K159&lt;&gt;"",OR(L159="PASS",L159="FAIL"),M159&lt;&gt;"",P159="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM159" s="9" t="str">
         <x:f>IF(A159="","",IF(AND(AK159="OK",J159="READY",F159&lt;&gt;"",G159&lt;&gt;"",K159&lt;&gt;"",S159="OK",OR(R159="PASS",R159="FAIL")),"YES","NO"))</x:f>
@@ -9249,7 +9249,7 @@
         <x:f>IF(A160="",IF(B160="","","MISSING_TEST_ID"),IF(B160="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A160,$B$2:$B$501,B160)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL160" s="9" t="str">
-        <x:f>IF(A160="","",IF(AND(AK160="OK",J160="READY",F160&lt;&gt;"",G160&lt;&gt;"",K160&lt;&gt;"",OR(L160="PASS",L160="FAIL"),M160&lt;&gt;"",O160&lt;&gt;"",P160="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A160="","",IF(AND(AK160="OK",J160="READY",F160&lt;&gt;"",G160&lt;&gt;"",K160&lt;&gt;"",OR(L160="PASS",L160="FAIL"),M160&lt;&gt;"",P160="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM160" s="9" t="str">
         <x:f>IF(A160="","",IF(AND(AK160="OK",J160="READY",F160&lt;&gt;"",G160&lt;&gt;"",K160&lt;&gt;"",S160="OK",OR(R160="PASS",R160="FAIL")),"YES","NO"))</x:f>
@@ -9301,7 +9301,7 @@
         <x:f>IF(A161="",IF(B161="","","MISSING_TEST_ID"),IF(B161="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A161,$B$2:$B$501,B161)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL161" s="9" t="str">
-        <x:f>IF(A161="","",IF(AND(AK161="OK",J161="READY",F161&lt;&gt;"",G161&lt;&gt;"",K161&lt;&gt;"",OR(L161="PASS",L161="FAIL"),M161&lt;&gt;"",O161&lt;&gt;"",P161="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A161="","",IF(AND(AK161="OK",J161="READY",F161&lt;&gt;"",G161&lt;&gt;"",K161&lt;&gt;"",OR(L161="PASS",L161="FAIL"),M161&lt;&gt;"",P161="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM161" s="9" t="str">
         <x:f>IF(A161="","",IF(AND(AK161="OK",J161="READY",F161&lt;&gt;"",G161&lt;&gt;"",K161&lt;&gt;"",S161="OK",OR(R161="PASS",R161="FAIL")),"YES","NO"))</x:f>
@@ -9353,7 +9353,7 @@
         <x:f>IF(A162="",IF(B162="","","MISSING_TEST_ID"),IF(B162="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A162,$B$2:$B$501,B162)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL162" s="9" t="str">
-        <x:f>IF(A162="","",IF(AND(AK162="OK",J162="READY",F162&lt;&gt;"",G162&lt;&gt;"",K162&lt;&gt;"",OR(L162="PASS",L162="FAIL"),M162&lt;&gt;"",O162&lt;&gt;"",P162="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A162="","",IF(AND(AK162="OK",J162="READY",F162&lt;&gt;"",G162&lt;&gt;"",K162&lt;&gt;"",OR(L162="PASS",L162="FAIL"),M162&lt;&gt;"",P162="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM162" s="9" t="str">
         <x:f>IF(A162="","",IF(AND(AK162="OK",J162="READY",F162&lt;&gt;"",G162&lt;&gt;"",K162&lt;&gt;"",S162="OK",OR(R162="PASS",R162="FAIL")),"YES","NO"))</x:f>
@@ -9405,7 +9405,7 @@
         <x:f>IF(A163="",IF(B163="","","MISSING_TEST_ID"),IF(B163="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A163,$B$2:$B$501,B163)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL163" s="9" t="str">
-        <x:f>IF(A163="","",IF(AND(AK163="OK",J163="READY",F163&lt;&gt;"",G163&lt;&gt;"",K163&lt;&gt;"",OR(L163="PASS",L163="FAIL"),M163&lt;&gt;"",O163&lt;&gt;"",P163="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A163="","",IF(AND(AK163="OK",J163="READY",F163&lt;&gt;"",G163&lt;&gt;"",K163&lt;&gt;"",OR(L163="PASS",L163="FAIL"),M163&lt;&gt;"",P163="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM163" s="9" t="str">
         <x:f>IF(A163="","",IF(AND(AK163="OK",J163="READY",F163&lt;&gt;"",G163&lt;&gt;"",K163&lt;&gt;"",S163="OK",OR(R163="PASS",R163="FAIL")),"YES","NO"))</x:f>
@@ -9457,7 +9457,7 @@
         <x:f>IF(A164="",IF(B164="","","MISSING_TEST_ID"),IF(B164="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A164,$B$2:$B$501,B164)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL164" s="9" t="str">
-        <x:f>IF(A164="","",IF(AND(AK164="OK",J164="READY",F164&lt;&gt;"",G164&lt;&gt;"",K164&lt;&gt;"",OR(L164="PASS",L164="FAIL"),M164&lt;&gt;"",O164&lt;&gt;"",P164="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A164="","",IF(AND(AK164="OK",J164="READY",F164&lt;&gt;"",G164&lt;&gt;"",K164&lt;&gt;"",OR(L164="PASS",L164="FAIL"),M164&lt;&gt;"",P164="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM164" s="9" t="str">
         <x:f>IF(A164="","",IF(AND(AK164="OK",J164="READY",F164&lt;&gt;"",G164&lt;&gt;"",K164&lt;&gt;"",S164="OK",OR(R164="PASS",R164="FAIL")),"YES","NO"))</x:f>
@@ -9509,7 +9509,7 @@
         <x:f>IF(A165="",IF(B165="","","MISSING_TEST_ID"),IF(B165="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A165,$B$2:$B$501,B165)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL165" s="9" t="str">
-        <x:f>IF(A165="","",IF(AND(AK165="OK",J165="READY",F165&lt;&gt;"",G165&lt;&gt;"",K165&lt;&gt;"",OR(L165="PASS",L165="FAIL"),M165&lt;&gt;"",O165&lt;&gt;"",P165="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A165="","",IF(AND(AK165="OK",J165="READY",F165&lt;&gt;"",G165&lt;&gt;"",K165&lt;&gt;"",OR(L165="PASS",L165="FAIL"),M165&lt;&gt;"",P165="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM165" s="9" t="str">
         <x:f>IF(A165="","",IF(AND(AK165="OK",J165="READY",F165&lt;&gt;"",G165&lt;&gt;"",K165&lt;&gt;"",S165="OK",OR(R165="PASS",R165="FAIL")),"YES","NO"))</x:f>
@@ -9561,7 +9561,7 @@
         <x:f>IF(A166="",IF(B166="","","MISSING_TEST_ID"),IF(B166="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A166,$B$2:$B$501,B166)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL166" s="9" t="str">
-        <x:f>IF(A166="","",IF(AND(AK166="OK",J166="READY",F166&lt;&gt;"",G166&lt;&gt;"",K166&lt;&gt;"",OR(L166="PASS",L166="FAIL"),M166&lt;&gt;"",O166&lt;&gt;"",P166="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A166="","",IF(AND(AK166="OK",J166="READY",F166&lt;&gt;"",G166&lt;&gt;"",K166&lt;&gt;"",OR(L166="PASS",L166="FAIL"),M166&lt;&gt;"",P166="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM166" s="9" t="str">
         <x:f>IF(A166="","",IF(AND(AK166="OK",J166="READY",F166&lt;&gt;"",G166&lt;&gt;"",K166&lt;&gt;"",S166="OK",OR(R166="PASS",R166="FAIL")),"YES","NO"))</x:f>
@@ -9613,7 +9613,7 @@
         <x:f>IF(A167="",IF(B167="","","MISSING_TEST_ID"),IF(B167="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A167,$B$2:$B$501,B167)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL167" s="9" t="str">
-        <x:f>IF(A167="","",IF(AND(AK167="OK",J167="READY",F167&lt;&gt;"",G167&lt;&gt;"",K167&lt;&gt;"",OR(L167="PASS",L167="FAIL"),M167&lt;&gt;"",O167&lt;&gt;"",P167="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A167="","",IF(AND(AK167="OK",J167="READY",F167&lt;&gt;"",G167&lt;&gt;"",K167&lt;&gt;"",OR(L167="PASS",L167="FAIL"),M167&lt;&gt;"",P167="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM167" s="9" t="str">
         <x:f>IF(A167="","",IF(AND(AK167="OK",J167="READY",F167&lt;&gt;"",G167&lt;&gt;"",K167&lt;&gt;"",S167="OK",OR(R167="PASS",R167="FAIL")),"YES","NO"))</x:f>
@@ -9665,7 +9665,7 @@
         <x:f>IF(A168="",IF(B168="","","MISSING_TEST_ID"),IF(B168="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A168,$B$2:$B$501,B168)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL168" s="9" t="str">
-        <x:f>IF(A168="","",IF(AND(AK168="OK",J168="READY",F168&lt;&gt;"",G168&lt;&gt;"",K168&lt;&gt;"",OR(L168="PASS",L168="FAIL"),M168&lt;&gt;"",O168&lt;&gt;"",P168="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A168="","",IF(AND(AK168="OK",J168="READY",F168&lt;&gt;"",G168&lt;&gt;"",K168&lt;&gt;"",OR(L168="PASS",L168="FAIL"),M168&lt;&gt;"",P168="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM168" s="9" t="str">
         <x:f>IF(A168="","",IF(AND(AK168="OK",J168="READY",F168&lt;&gt;"",G168&lt;&gt;"",K168&lt;&gt;"",S168="OK",OR(R168="PASS",R168="FAIL")),"YES","NO"))</x:f>
@@ -9717,7 +9717,7 @@
         <x:f>IF(A169="",IF(B169="","","MISSING_TEST_ID"),IF(B169="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A169,$B$2:$B$501,B169)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL169" s="9" t="str">
-        <x:f>IF(A169="","",IF(AND(AK169="OK",J169="READY",F169&lt;&gt;"",G169&lt;&gt;"",K169&lt;&gt;"",OR(L169="PASS",L169="FAIL"),M169&lt;&gt;"",O169&lt;&gt;"",P169="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A169="","",IF(AND(AK169="OK",J169="READY",F169&lt;&gt;"",G169&lt;&gt;"",K169&lt;&gt;"",OR(L169="PASS",L169="FAIL"),M169&lt;&gt;"",P169="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM169" s="9" t="str">
         <x:f>IF(A169="","",IF(AND(AK169="OK",J169="READY",F169&lt;&gt;"",G169&lt;&gt;"",K169&lt;&gt;"",S169="OK",OR(R169="PASS",R169="FAIL")),"YES","NO"))</x:f>
@@ -9769,7 +9769,7 @@
         <x:f>IF(A170="",IF(B170="","","MISSING_TEST_ID"),IF(B170="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A170,$B$2:$B$501,B170)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL170" s="9" t="str">
-        <x:f>IF(A170="","",IF(AND(AK170="OK",J170="READY",F170&lt;&gt;"",G170&lt;&gt;"",K170&lt;&gt;"",OR(L170="PASS",L170="FAIL"),M170&lt;&gt;"",O170&lt;&gt;"",P170="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A170="","",IF(AND(AK170="OK",J170="READY",F170&lt;&gt;"",G170&lt;&gt;"",K170&lt;&gt;"",OR(L170="PASS",L170="FAIL"),M170&lt;&gt;"",P170="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM170" s="9" t="str">
         <x:f>IF(A170="","",IF(AND(AK170="OK",J170="READY",F170&lt;&gt;"",G170&lt;&gt;"",K170&lt;&gt;"",S170="OK",OR(R170="PASS",R170="FAIL")),"YES","NO"))</x:f>
@@ -9821,7 +9821,7 @@
         <x:f>IF(A171="",IF(B171="","","MISSING_TEST_ID"),IF(B171="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A171,$B$2:$B$501,B171)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL171" s="9" t="str">
-        <x:f>IF(A171="","",IF(AND(AK171="OK",J171="READY",F171&lt;&gt;"",G171&lt;&gt;"",K171&lt;&gt;"",OR(L171="PASS",L171="FAIL"),M171&lt;&gt;"",O171&lt;&gt;"",P171="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A171="","",IF(AND(AK171="OK",J171="READY",F171&lt;&gt;"",G171&lt;&gt;"",K171&lt;&gt;"",OR(L171="PASS",L171="FAIL"),M171&lt;&gt;"",P171="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM171" s="9" t="str">
         <x:f>IF(A171="","",IF(AND(AK171="OK",J171="READY",F171&lt;&gt;"",G171&lt;&gt;"",K171&lt;&gt;"",S171="OK",OR(R171="PASS",R171="FAIL")),"YES","NO"))</x:f>
@@ -9873,7 +9873,7 @@
         <x:f>IF(A172="",IF(B172="","","MISSING_TEST_ID"),IF(B172="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A172,$B$2:$B$501,B172)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL172" s="9" t="str">
-        <x:f>IF(A172="","",IF(AND(AK172="OK",J172="READY",F172&lt;&gt;"",G172&lt;&gt;"",K172&lt;&gt;"",OR(L172="PASS",L172="FAIL"),M172&lt;&gt;"",O172&lt;&gt;"",P172="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A172="","",IF(AND(AK172="OK",J172="READY",F172&lt;&gt;"",G172&lt;&gt;"",K172&lt;&gt;"",OR(L172="PASS",L172="FAIL"),M172&lt;&gt;"",P172="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM172" s="9" t="str">
         <x:f>IF(A172="","",IF(AND(AK172="OK",J172="READY",F172&lt;&gt;"",G172&lt;&gt;"",K172&lt;&gt;"",S172="OK",OR(R172="PASS",R172="FAIL")),"YES","NO"))</x:f>
@@ -9925,7 +9925,7 @@
         <x:f>IF(A173="",IF(B173="","","MISSING_TEST_ID"),IF(B173="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A173,$B$2:$B$501,B173)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL173" s="9" t="str">
-        <x:f>IF(A173="","",IF(AND(AK173="OK",J173="READY",F173&lt;&gt;"",G173&lt;&gt;"",K173&lt;&gt;"",OR(L173="PASS",L173="FAIL"),M173&lt;&gt;"",O173&lt;&gt;"",P173="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A173="","",IF(AND(AK173="OK",J173="READY",F173&lt;&gt;"",G173&lt;&gt;"",K173&lt;&gt;"",OR(L173="PASS",L173="FAIL"),M173&lt;&gt;"",P173="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM173" s="9" t="str">
         <x:f>IF(A173="","",IF(AND(AK173="OK",J173="READY",F173&lt;&gt;"",G173&lt;&gt;"",K173&lt;&gt;"",S173="OK",OR(R173="PASS",R173="FAIL")),"YES","NO"))</x:f>
@@ -9977,7 +9977,7 @@
         <x:f>IF(A174="",IF(B174="","","MISSING_TEST_ID"),IF(B174="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A174,$B$2:$B$501,B174)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL174" s="9" t="str">
-        <x:f>IF(A174="","",IF(AND(AK174="OK",J174="READY",F174&lt;&gt;"",G174&lt;&gt;"",K174&lt;&gt;"",OR(L174="PASS",L174="FAIL"),M174&lt;&gt;"",O174&lt;&gt;"",P174="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A174="","",IF(AND(AK174="OK",J174="READY",F174&lt;&gt;"",G174&lt;&gt;"",K174&lt;&gt;"",OR(L174="PASS",L174="FAIL"),M174&lt;&gt;"",P174="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM174" s="9" t="str">
         <x:f>IF(A174="","",IF(AND(AK174="OK",J174="READY",F174&lt;&gt;"",G174&lt;&gt;"",K174&lt;&gt;"",S174="OK",OR(R174="PASS",R174="FAIL")),"YES","NO"))</x:f>
@@ -10029,7 +10029,7 @@
         <x:f>IF(A175="",IF(B175="","","MISSING_TEST_ID"),IF(B175="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A175,$B$2:$B$501,B175)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL175" s="9" t="str">
-        <x:f>IF(A175="","",IF(AND(AK175="OK",J175="READY",F175&lt;&gt;"",G175&lt;&gt;"",K175&lt;&gt;"",OR(L175="PASS",L175="FAIL"),M175&lt;&gt;"",O175&lt;&gt;"",P175="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A175="","",IF(AND(AK175="OK",J175="READY",F175&lt;&gt;"",G175&lt;&gt;"",K175&lt;&gt;"",OR(L175="PASS",L175="FAIL"),M175&lt;&gt;"",P175="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM175" s="9" t="str">
         <x:f>IF(A175="","",IF(AND(AK175="OK",J175="READY",F175&lt;&gt;"",G175&lt;&gt;"",K175&lt;&gt;"",S175="OK",OR(R175="PASS",R175="FAIL")),"YES","NO"))</x:f>
@@ -10081,7 +10081,7 @@
         <x:f>IF(A176="",IF(B176="","","MISSING_TEST_ID"),IF(B176="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A176,$B$2:$B$501,B176)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL176" s="9" t="str">
-        <x:f>IF(A176="","",IF(AND(AK176="OK",J176="READY",F176&lt;&gt;"",G176&lt;&gt;"",K176&lt;&gt;"",OR(L176="PASS",L176="FAIL"),M176&lt;&gt;"",O176&lt;&gt;"",P176="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A176="","",IF(AND(AK176="OK",J176="READY",F176&lt;&gt;"",G176&lt;&gt;"",K176&lt;&gt;"",OR(L176="PASS",L176="FAIL"),M176&lt;&gt;"",P176="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM176" s="9" t="str">
         <x:f>IF(A176="","",IF(AND(AK176="OK",J176="READY",F176&lt;&gt;"",G176&lt;&gt;"",K176&lt;&gt;"",S176="OK",OR(R176="PASS",R176="FAIL")),"YES","NO"))</x:f>
@@ -10133,7 +10133,7 @@
         <x:f>IF(A177="",IF(B177="","","MISSING_TEST_ID"),IF(B177="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A177,$B$2:$B$501,B177)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL177" s="9" t="str">
-        <x:f>IF(A177="","",IF(AND(AK177="OK",J177="READY",F177&lt;&gt;"",G177&lt;&gt;"",K177&lt;&gt;"",OR(L177="PASS",L177="FAIL"),M177&lt;&gt;"",O177&lt;&gt;"",P177="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A177="","",IF(AND(AK177="OK",J177="READY",F177&lt;&gt;"",G177&lt;&gt;"",K177&lt;&gt;"",OR(L177="PASS",L177="FAIL"),M177&lt;&gt;"",P177="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM177" s="9" t="str">
         <x:f>IF(A177="","",IF(AND(AK177="OK",J177="READY",F177&lt;&gt;"",G177&lt;&gt;"",K177&lt;&gt;"",S177="OK",OR(R177="PASS",R177="FAIL")),"YES","NO"))</x:f>
@@ -10185,7 +10185,7 @@
         <x:f>IF(A178="",IF(B178="","","MISSING_TEST_ID"),IF(B178="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A178,$B$2:$B$501,B178)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL178" s="9" t="str">
-        <x:f>IF(A178="","",IF(AND(AK178="OK",J178="READY",F178&lt;&gt;"",G178&lt;&gt;"",K178&lt;&gt;"",OR(L178="PASS",L178="FAIL"),M178&lt;&gt;"",O178&lt;&gt;"",P178="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A178="","",IF(AND(AK178="OK",J178="READY",F178&lt;&gt;"",G178&lt;&gt;"",K178&lt;&gt;"",OR(L178="PASS",L178="FAIL"),M178&lt;&gt;"",P178="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM178" s="9" t="str">
         <x:f>IF(A178="","",IF(AND(AK178="OK",J178="READY",F178&lt;&gt;"",G178&lt;&gt;"",K178&lt;&gt;"",S178="OK",OR(R178="PASS",R178="FAIL")),"YES","NO"))</x:f>
@@ -10237,7 +10237,7 @@
         <x:f>IF(A179="",IF(B179="","","MISSING_TEST_ID"),IF(B179="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A179,$B$2:$B$501,B179)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL179" s="9" t="str">
-        <x:f>IF(A179="","",IF(AND(AK179="OK",J179="READY",F179&lt;&gt;"",G179&lt;&gt;"",K179&lt;&gt;"",OR(L179="PASS",L179="FAIL"),M179&lt;&gt;"",O179&lt;&gt;"",P179="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A179="","",IF(AND(AK179="OK",J179="READY",F179&lt;&gt;"",G179&lt;&gt;"",K179&lt;&gt;"",OR(L179="PASS",L179="FAIL"),M179&lt;&gt;"",P179="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM179" s="9" t="str">
         <x:f>IF(A179="","",IF(AND(AK179="OK",J179="READY",F179&lt;&gt;"",G179&lt;&gt;"",K179&lt;&gt;"",S179="OK",OR(R179="PASS",R179="FAIL")),"YES","NO"))</x:f>
@@ -10289,7 +10289,7 @@
         <x:f>IF(A180="",IF(B180="","","MISSING_TEST_ID"),IF(B180="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A180,$B$2:$B$501,B180)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL180" s="9" t="str">
-        <x:f>IF(A180="","",IF(AND(AK180="OK",J180="READY",F180&lt;&gt;"",G180&lt;&gt;"",K180&lt;&gt;"",OR(L180="PASS",L180="FAIL"),M180&lt;&gt;"",O180&lt;&gt;"",P180="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A180="","",IF(AND(AK180="OK",J180="READY",F180&lt;&gt;"",G180&lt;&gt;"",K180&lt;&gt;"",OR(L180="PASS",L180="FAIL"),M180&lt;&gt;"",P180="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM180" s="9" t="str">
         <x:f>IF(A180="","",IF(AND(AK180="OK",J180="READY",F180&lt;&gt;"",G180&lt;&gt;"",K180&lt;&gt;"",S180="OK",OR(R180="PASS",R180="FAIL")),"YES","NO"))</x:f>
@@ -10341,7 +10341,7 @@
         <x:f>IF(A181="",IF(B181="","","MISSING_TEST_ID"),IF(B181="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A181,$B$2:$B$501,B181)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL181" s="9" t="str">
-        <x:f>IF(A181="","",IF(AND(AK181="OK",J181="READY",F181&lt;&gt;"",G181&lt;&gt;"",K181&lt;&gt;"",OR(L181="PASS",L181="FAIL"),M181&lt;&gt;"",O181&lt;&gt;"",P181="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A181="","",IF(AND(AK181="OK",J181="READY",F181&lt;&gt;"",G181&lt;&gt;"",K181&lt;&gt;"",OR(L181="PASS",L181="FAIL"),M181&lt;&gt;"",P181="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM181" s="9" t="str">
         <x:f>IF(A181="","",IF(AND(AK181="OK",J181="READY",F181&lt;&gt;"",G181&lt;&gt;"",K181&lt;&gt;"",S181="OK",OR(R181="PASS",R181="FAIL")),"YES","NO"))</x:f>
@@ -10393,7 +10393,7 @@
         <x:f>IF(A182="",IF(B182="","","MISSING_TEST_ID"),IF(B182="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A182,$B$2:$B$501,B182)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL182" s="9" t="str">
-        <x:f>IF(A182="","",IF(AND(AK182="OK",J182="READY",F182&lt;&gt;"",G182&lt;&gt;"",K182&lt;&gt;"",OR(L182="PASS",L182="FAIL"),M182&lt;&gt;"",O182&lt;&gt;"",P182="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A182="","",IF(AND(AK182="OK",J182="READY",F182&lt;&gt;"",G182&lt;&gt;"",K182&lt;&gt;"",OR(L182="PASS",L182="FAIL"),M182&lt;&gt;"",P182="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM182" s="9" t="str">
         <x:f>IF(A182="","",IF(AND(AK182="OK",J182="READY",F182&lt;&gt;"",G182&lt;&gt;"",K182&lt;&gt;"",S182="OK",OR(R182="PASS",R182="FAIL")),"YES","NO"))</x:f>
@@ -10445,7 +10445,7 @@
         <x:f>IF(A183="",IF(B183="","","MISSING_TEST_ID"),IF(B183="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A183,$B$2:$B$501,B183)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL183" s="9" t="str">
-        <x:f>IF(A183="","",IF(AND(AK183="OK",J183="READY",F183&lt;&gt;"",G183&lt;&gt;"",K183&lt;&gt;"",OR(L183="PASS",L183="FAIL"),M183&lt;&gt;"",O183&lt;&gt;"",P183="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A183="","",IF(AND(AK183="OK",J183="READY",F183&lt;&gt;"",G183&lt;&gt;"",K183&lt;&gt;"",OR(L183="PASS",L183="FAIL"),M183&lt;&gt;"",P183="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM183" s="9" t="str">
         <x:f>IF(A183="","",IF(AND(AK183="OK",J183="READY",F183&lt;&gt;"",G183&lt;&gt;"",K183&lt;&gt;"",S183="OK",OR(R183="PASS",R183="FAIL")),"YES","NO"))</x:f>
@@ -10497,7 +10497,7 @@
         <x:f>IF(A184="",IF(B184="","","MISSING_TEST_ID"),IF(B184="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A184,$B$2:$B$501,B184)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL184" s="9" t="str">
-        <x:f>IF(A184="","",IF(AND(AK184="OK",J184="READY",F184&lt;&gt;"",G184&lt;&gt;"",K184&lt;&gt;"",OR(L184="PASS",L184="FAIL"),M184&lt;&gt;"",O184&lt;&gt;"",P184="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A184="","",IF(AND(AK184="OK",J184="READY",F184&lt;&gt;"",G184&lt;&gt;"",K184&lt;&gt;"",OR(L184="PASS",L184="FAIL"),M184&lt;&gt;"",P184="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM184" s="9" t="str">
         <x:f>IF(A184="","",IF(AND(AK184="OK",J184="READY",F184&lt;&gt;"",G184&lt;&gt;"",K184&lt;&gt;"",S184="OK",OR(R184="PASS",R184="FAIL")),"YES","NO"))</x:f>
@@ -10549,7 +10549,7 @@
         <x:f>IF(A185="",IF(B185="","","MISSING_TEST_ID"),IF(B185="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A185,$B$2:$B$501,B185)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL185" s="9" t="str">
-        <x:f>IF(A185="","",IF(AND(AK185="OK",J185="READY",F185&lt;&gt;"",G185&lt;&gt;"",K185&lt;&gt;"",OR(L185="PASS",L185="FAIL"),M185&lt;&gt;"",O185&lt;&gt;"",P185="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A185="","",IF(AND(AK185="OK",J185="READY",F185&lt;&gt;"",G185&lt;&gt;"",K185&lt;&gt;"",OR(L185="PASS",L185="FAIL"),M185&lt;&gt;"",P185="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM185" s="9" t="str">
         <x:f>IF(A185="","",IF(AND(AK185="OK",J185="READY",F185&lt;&gt;"",G185&lt;&gt;"",K185&lt;&gt;"",S185="OK",OR(R185="PASS",R185="FAIL")),"YES","NO"))</x:f>
@@ -10601,7 +10601,7 @@
         <x:f>IF(A186="",IF(B186="","","MISSING_TEST_ID"),IF(B186="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A186,$B$2:$B$501,B186)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL186" s="9" t="str">
-        <x:f>IF(A186="","",IF(AND(AK186="OK",J186="READY",F186&lt;&gt;"",G186&lt;&gt;"",K186&lt;&gt;"",OR(L186="PASS",L186="FAIL"),M186&lt;&gt;"",O186&lt;&gt;"",P186="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A186="","",IF(AND(AK186="OK",J186="READY",F186&lt;&gt;"",G186&lt;&gt;"",K186&lt;&gt;"",OR(L186="PASS",L186="FAIL"),M186&lt;&gt;"",P186="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM186" s="9" t="str">
         <x:f>IF(A186="","",IF(AND(AK186="OK",J186="READY",F186&lt;&gt;"",G186&lt;&gt;"",K186&lt;&gt;"",S186="OK",OR(R186="PASS",R186="FAIL")),"YES","NO"))</x:f>
@@ -10653,7 +10653,7 @@
         <x:f>IF(A187="",IF(B187="","","MISSING_TEST_ID"),IF(B187="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A187,$B$2:$B$501,B187)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL187" s="9" t="str">
-        <x:f>IF(A187="","",IF(AND(AK187="OK",J187="READY",F187&lt;&gt;"",G187&lt;&gt;"",K187&lt;&gt;"",OR(L187="PASS",L187="FAIL"),M187&lt;&gt;"",O187&lt;&gt;"",P187="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A187="","",IF(AND(AK187="OK",J187="READY",F187&lt;&gt;"",G187&lt;&gt;"",K187&lt;&gt;"",OR(L187="PASS",L187="FAIL"),M187&lt;&gt;"",P187="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM187" s="9" t="str">
         <x:f>IF(A187="","",IF(AND(AK187="OK",J187="READY",F187&lt;&gt;"",G187&lt;&gt;"",K187&lt;&gt;"",S187="OK",OR(R187="PASS",R187="FAIL")),"YES","NO"))</x:f>
@@ -10705,7 +10705,7 @@
         <x:f>IF(A188="",IF(B188="","","MISSING_TEST_ID"),IF(B188="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A188,$B$2:$B$501,B188)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL188" s="9" t="str">
-        <x:f>IF(A188="","",IF(AND(AK188="OK",J188="READY",F188&lt;&gt;"",G188&lt;&gt;"",K188&lt;&gt;"",OR(L188="PASS",L188="FAIL"),M188&lt;&gt;"",O188&lt;&gt;"",P188="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A188="","",IF(AND(AK188="OK",J188="READY",F188&lt;&gt;"",G188&lt;&gt;"",K188&lt;&gt;"",OR(L188="PASS",L188="FAIL"),M188&lt;&gt;"",P188="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM188" s="9" t="str">
         <x:f>IF(A188="","",IF(AND(AK188="OK",J188="READY",F188&lt;&gt;"",G188&lt;&gt;"",K188&lt;&gt;"",S188="OK",OR(R188="PASS",R188="FAIL")),"YES","NO"))</x:f>
@@ -10757,7 +10757,7 @@
         <x:f>IF(A189="",IF(B189="","","MISSING_TEST_ID"),IF(B189="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A189,$B$2:$B$501,B189)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL189" s="9" t="str">
-        <x:f>IF(A189="","",IF(AND(AK189="OK",J189="READY",F189&lt;&gt;"",G189&lt;&gt;"",K189&lt;&gt;"",OR(L189="PASS",L189="FAIL"),M189&lt;&gt;"",O189&lt;&gt;"",P189="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A189="","",IF(AND(AK189="OK",J189="READY",F189&lt;&gt;"",G189&lt;&gt;"",K189&lt;&gt;"",OR(L189="PASS",L189="FAIL"),M189&lt;&gt;"",P189="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM189" s="9" t="str">
         <x:f>IF(A189="","",IF(AND(AK189="OK",J189="READY",F189&lt;&gt;"",G189&lt;&gt;"",K189&lt;&gt;"",S189="OK",OR(R189="PASS",R189="FAIL")),"YES","NO"))</x:f>
@@ -10809,7 +10809,7 @@
         <x:f>IF(A190="",IF(B190="","","MISSING_TEST_ID"),IF(B190="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A190,$B$2:$B$501,B190)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL190" s="9" t="str">
-        <x:f>IF(A190="","",IF(AND(AK190="OK",J190="READY",F190&lt;&gt;"",G190&lt;&gt;"",K190&lt;&gt;"",OR(L190="PASS",L190="FAIL"),M190&lt;&gt;"",O190&lt;&gt;"",P190="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A190="","",IF(AND(AK190="OK",J190="READY",F190&lt;&gt;"",G190&lt;&gt;"",K190&lt;&gt;"",OR(L190="PASS",L190="FAIL"),M190&lt;&gt;"",P190="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM190" s="9" t="str">
         <x:f>IF(A190="","",IF(AND(AK190="OK",J190="READY",F190&lt;&gt;"",G190&lt;&gt;"",K190&lt;&gt;"",S190="OK",OR(R190="PASS",R190="FAIL")),"YES","NO"))</x:f>
@@ -10861,7 +10861,7 @@
         <x:f>IF(A191="",IF(B191="","","MISSING_TEST_ID"),IF(B191="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A191,$B$2:$B$501,B191)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL191" s="9" t="str">
-        <x:f>IF(A191="","",IF(AND(AK191="OK",J191="READY",F191&lt;&gt;"",G191&lt;&gt;"",K191&lt;&gt;"",OR(L191="PASS",L191="FAIL"),M191&lt;&gt;"",O191&lt;&gt;"",P191="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A191="","",IF(AND(AK191="OK",J191="READY",F191&lt;&gt;"",G191&lt;&gt;"",K191&lt;&gt;"",OR(L191="PASS",L191="FAIL"),M191&lt;&gt;"",P191="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM191" s="9" t="str">
         <x:f>IF(A191="","",IF(AND(AK191="OK",J191="READY",F191&lt;&gt;"",G191&lt;&gt;"",K191&lt;&gt;"",S191="OK",OR(R191="PASS",R191="FAIL")),"YES","NO"))</x:f>
@@ -10913,7 +10913,7 @@
         <x:f>IF(A192="",IF(B192="","","MISSING_TEST_ID"),IF(B192="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A192,$B$2:$B$501,B192)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL192" s="9" t="str">
-        <x:f>IF(A192="","",IF(AND(AK192="OK",J192="READY",F192&lt;&gt;"",G192&lt;&gt;"",K192&lt;&gt;"",OR(L192="PASS",L192="FAIL"),M192&lt;&gt;"",O192&lt;&gt;"",P192="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A192="","",IF(AND(AK192="OK",J192="READY",F192&lt;&gt;"",G192&lt;&gt;"",K192&lt;&gt;"",OR(L192="PASS",L192="FAIL"),M192&lt;&gt;"",P192="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM192" s="9" t="str">
         <x:f>IF(A192="","",IF(AND(AK192="OK",J192="READY",F192&lt;&gt;"",G192&lt;&gt;"",K192&lt;&gt;"",S192="OK",OR(R192="PASS",R192="FAIL")),"YES","NO"))</x:f>
@@ -10965,7 +10965,7 @@
         <x:f>IF(A193="",IF(B193="","","MISSING_TEST_ID"),IF(B193="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A193,$B$2:$B$501,B193)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL193" s="9" t="str">
-        <x:f>IF(A193="","",IF(AND(AK193="OK",J193="READY",F193&lt;&gt;"",G193&lt;&gt;"",K193&lt;&gt;"",OR(L193="PASS",L193="FAIL"),M193&lt;&gt;"",O193&lt;&gt;"",P193="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A193="","",IF(AND(AK193="OK",J193="READY",F193&lt;&gt;"",G193&lt;&gt;"",K193&lt;&gt;"",OR(L193="PASS",L193="FAIL"),M193&lt;&gt;"",P193="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM193" s="9" t="str">
         <x:f>IF(A193="","",IF(AND(AK193="OK",J193="READY",F193&lt;&gt;"",G193&lt;&gt;"",K193&lt;&gt;"",S193="OK",OR(R193="PASS",R193="FAIL")),"YES","NO"))</x:f>
@@ -11017,7 +11017,7 @@
         <x:f>IF(A194="",IF(B194="","","MISSING_TEST_ID"),IF(B194="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A194,$B$2:$B$501,B194)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL194" s="9" t="str">
-        <x:f>IF(A194="","",IF(AND(AK194="OK",J194="READY",F194&lt;&gt;"",G194&lt;&gt;"",K194&lt;&gt;"",OR(L194="PASS",L194="FAIL"),M194&lt;&gt;"",O194&lt;&gt;"",P194="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A194="","",IF(AND(AK194="OK",J194="READY",F194&lt;&gt;"",G194&lt;&gt;"",K194&lt;&gt;"",OR(L194="PASS",L194="FAIL"),M194&lt;&gt;"",P194="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM194" s="9" t="str">
         <x:f>IF(A194="","",IF(AND(AK194="OK",J194="READY",F194&lt;&gt;"",G194&lt;&gt;"",K194&lt;&gt;"",S194="OK",OR(R194="PASS",R194="FAIL")),"YES","NO"))</x:f>
@@ -11069,7 +11069,7 @@
         <x:f>IF(A195="",IF(B195="","","MISSING_TEST_ID"),IF(B195="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A195,$B$2:$B$501,B195)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL195" s="9" t="str">
-        <x:f>IF(A195="","",IF(AND(AK195="OK",J195="READY",F195&lt;&gt;"",G195&lt;&gt;"",K195&lt;&gt;"",OR(L195="PASS",L195="FAIL"),M195&lt;&gt;"",O195&lt;&gt;"",P195="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A195="","",IF(AND(AK195="OK",J195="READY",F195&lt;&gt;"",G195&lt;&gt;"",K195&lt;&gt;"",OR(L195="PASS",L195="FAIL"),M195&lt;&gt;"",P195="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM195" s="9" t="str">
         <x:f>IF(A195="","",IF(AND(AK195="OK",J195="READY",F195&lt;&gt;"",G195&lt;&gt;"",K195&lt;&gt;"",S195="OK",OR(R195="PASS",R195="FAIL")),"YES","NO"))</x:f>
@@ -11121,7 +11121,7 @@
         <x:f>IF(A196="",IF(B196="","","MISSING_TEST_ID"),IF(B196="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A196,$B$2:$B$501,B196)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL196" s="9" t="str">
-        <x:f>IF(A196="","",IF(AND(AK196="OK",J196="READY",F196&lt;&gt;"",G196&lt;&gt;"",K196&lt;&gt;"",OR(L196="PASS",L196="FAIL"),M196&lt;&gt;"",O196&lt;&gt;"",P196="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A196="","",IF(AND(AK196="OK",J196="READY",F196&lt;&gt;"",G196&lt;&gt;"",K196&lt;&gt;"",OR(L196="PASS",L196="FAIL"),M196&lt;&gt;"",P196="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM196" s="9" t="str">
         <x:f>IF(A196="","",IF(AND(AK196="OK",J196="READY",F196&lt;&gt;"",G196&lt;&gt;"",K196&lt;&gt;"",S196="OK",OR(R196="PASS",R196="FAIL")),"YES","NO"))</x:f>
@@ -11173,7 +11173,7 @@
         <x:f>IF(A197="",IF(B197="","","MISSING_TEST_ID"),IF(B197="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A197,$B$2:$B$501,B197)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL197" s="9" t="str">
-        <x:f>IF(A197="","",IF(AND(AK197="OK",J197="READY",F197&lt;&gt;"",G197&lt;&gt;"",K197&lt;&gt;"",OR(L197="PASS",L197="FAIL"),M197&lt;&gt;"",O197&lt;&gt;"",P197="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A197="","",IF(AND(AK197="OK",J197="READY",F197&lt;&gt;"",G197&lt;&gt;"",K197&lt;&gt;"",OR(L197="PASS",L197="FAIL"),M197&lt;&gt;"",P197="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM197" s="9" t="str">
         <x:f>IF(A197="","",IF(AND(AK197="OK",J197="READY",F197&lt;&gt;"",G197&lt;&gt;"",K197&lt;&gt;"",S197="OK",OR(R197="PASS",R197="FAIL")),"YES","NO"))</x:f>
@@ -11225,7 +11225,7 @@
         <x:f>IF(A198="",IF(B198="","","MISSING_TEST_ID"),IF(B198="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A198,$B$2:$B$501,B198)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL198" s="9" t="str">
-        <x:f>IF(A198="","",IF(AND(AK198="OK",J198="READY",F198&lt;&gt;"",G198&lt;&gt;"",K198&lt;&gt;"",OR(L198="PASS",L198="FAIL"),M198&lt;&gt;"",O198&lt;&gt;"",P198="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A198="","",IF(AND(AK198="OK",J198="READY",F198&lt;&gt;"",G198&lt;&gt;"",K198&lt;&gt;"",OR(L198="PASS",L198="FAIL"),M198&lt;&gt;"",P198="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM198" s="9" t="str">
         <x:f>IF(A198="","",IF(AND(AK198="OK",J198="READY",F198&lt;&gt;"",G198&lt;&gt;"",K198&lt;&gt;"",S198="OK",OR(R198="PASS",R198="FAIL")),"YES","NO"))</x:f>
@@ -11277,7 +11277,7 @@
         <x:f>IF(A199="",IF(B199="","","MISSING_TEST_ID"),IF(B199="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A199,$B$2:$B$501,B199)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL199" s="9" t="str">
-        <x:f>IF(A199="","",IF(AND(AK199="OK",J199="READY",F199&lt;&gt;"",G199&lt;&gt;"",K199&lt;&gt;"",OR(L199="PASS",L199="FAIL"),M199&lt;&gt;"",O199&lt;&gt;"",P199="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A199="","",IF(AND(AK199="OK",J199="READY",F199&lt;&gt;"",G199&lt;&gt;"",K199&lt;&gt;"",OR(L199="PASS",L199="FAIL"),M199&lt;&gt;"",P199="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM199" s="9" t="str">
         <x:f>IF(A199="","",IF(AND(AK199="OK",J199="READY",F199&lt;&gt;"",G199&lt;&gt;"",K199&lt;&gt;"",S199="OK",OR(R199="PASS",R199="FAIL")),"YES","NO"))</x:f>
@@ -11329,7 +11329,7 @@
         <x:f>IF(A200="",IF(B200="","","MISSING_TEST_ID"),IF(B200="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A200,$B$2:$B$501,B200)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL200" s="9" t="str">
-        <x:f>IF(A200="","",IF(AND(AK200="OK",J200="READY",F200&lt;&gt;"",G200&lt;&gt;"",K200&lt;&gt;"",OR(L200="PASS",L200="FAIL"),M200&lt;&gt;"",O200&lt;&gt;"",P200="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A200="","",IF(AND(AK200="OK",J200="READY",F200&lt;&gt;"",G200&lt;&gt;"",K200&lt;&gt;"",OR(L200="PASS",L200="FAIL"),M200&lt;&gt;"",P200="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM200" s="9" t="str">
         <x:f>IF(A200="","",IF(AND(AK200="OK",J200="READY",F200&lt;&gt;"",G200&lt;&gt;"",K200&lt;&gt;"",S200="OK",OR(R200="PASS",R200="FAIL")),"YES","NO"))</x:f>
@@ -11381,7 +11381,7 @@
         <x:f>IF(A201="",IF(B201="","","MISSING_TEST_ID"),IF(B201="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A201,$B$2:$B$501,B201)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL201" s="9" t="str">
-        <x:f>IF(A201="","",IF(AND(AK201="OK",J201="READY",F201&lt;&gt;"",G201&lt;&gt;"",K201&lt;&gt;"",OR(L201="PASS",L201="FAIL"),M201&lt;&gt;"",O201&lt;&gt;"",P201="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A201="","",IF(AND(AK201="OK",J201="READY",F201&lt;&gt;"",G201&lt;&gt;"",K201&lt;&gt;"",OR(L201="PASS",L201="FAIL"),M201&lt;&gt;"",P201="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM201" s="9" t="str">
         <x:f>IF(A201="","",IF(AND(AK201="OK",J201="READY",F201&lt;&gt;"",G201&lt;&gt;"",K201&lt;&gt;"",S201="OK",OR(R201="PASS",R201="FAIL")),"YES","NO"))</x:f>
@@ -11433,7 +11433,7 @@
         <x:f>IF(A202="",IF(B202="","","MISSING_TEST_ID"),IF(B202="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A202,$B$2:$B$501,B202)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL202" s="9" t="str">
-        <x:f>IF(A202="","",IF(AND(AK202="OK",J202="READY",F202&lt;&gt;"",G202&lt;&gt;"",K202&lt;&gt;"",OR(L202="PASS",L202="FAIL"),M202&lt;&gt;"",O202&lt;&gt;"",P202="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A202="","",IF(AND(AK202="OK",J202="READY",F202&lt;&gt;"",G202&lt;&gt;"",K202&lt;&gt;"",OR(L202="PASS",L202="FAIL"),M202&lt;&gt;"",P202="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM202" s="9" t="str">
         <x:f>IF(A202="","",IF(AND(AK202="OK",J202="READY",F202&lt;&gt;"",G202&lt;&gt;"",K202&lt;&gt;"",S202="OK",OR(R202="PASS",R202="FAIL")),"YES","NO"))</x:f>
@@ -11485,7 +11485,7 @@
         <x:f>IF(A203="",IF(B203="","","MISSING_TEST_ID"),IF(B203="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A203,$B$2:$B$501,B203)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL203" s="9" t="str">
-        <x:f>IF(A203="","",IF(AND(AK203="OK",J203="READY",F203&lt;&gt;"",G203&lt;&gt;"",K203&lt;&gt;"",OR(L203="PASS",L203="FAIL"),M203&lt;&gt;"",O203&lt;&gt;"",P203="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A203="","",IF(AND(AK203="OK",J203="READY",F203&lt;&gt;"",G203&lt;&gt;"",K203&lt;&gt;"",OR(L203="PASS",L203="FAIL"),M203&lt;&gt;"",P203="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM203" s="9" t="str">
         <x:f>IF(A203="","",IF(AND(AK203="OK",J203="READY",F203&lt;&gt;"",G203&lt;&gt;"",K203&lt;&gt;"",S203="OK",OR(R203="PASS",R203="FAIL")),"YES","NO"))</x:f>
@@ -11537,7 +11537,7 @@
         <x:f>IF(A204="",IF(B204="","","MISSING_TEST_ID"),IF(B204="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A204,$B$2:$B$501,B204)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL204" s="9" t="str">
-        <x:f>IF(A204="","",IF(AND(AK204="OK",J204="READY",F204&lt;&gt;"",G204&lt;&gt;"",K204&lt;&gt;"",OR(L204="PASS",L204="FAIL"),M204&lt;&gt;"",O204&lt;&gt;"",P204="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A204="","",IF(AND(AK204="OK",J204="READY",F204&lt;&gt;"",G204&lt;&gt;"",K204&lt;&gt;"",OR(L204="PASS",L204="FAIL"),M204&lt;&gt;"",P204="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM204" s="9" t="str">
         <x:f>IF(A204="","",IF(AND(AK204="OK",J204="READY",F204&lt;&gt;"",G204&lt;&gt;"",K204&lt;&gt;"",S204="OK",OR(R204="PASS",R204="FAIL")),"YES","NO"))</x:f>
@@ -11589,7 +11589,7 @@
         <x:f>IF(A205="",IF(B205="","","MISSING_TEST_ID"),IF(B205="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A205,$B$2:$B$501,B205)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL205" s="9" t="str">
-        <x:f>IF(A205="","",IF(AND(AK205="OK",J205="READY",F205&lt;&gt;"",G205&lt;&gt;"",K205&lt;&gt;"",OR(L205="PASS",L205="FAIL"),M205&lt;&gt;"",O205&lt;&gt;"",P205="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A205="","",IF(AND(AK205="OK",J205="READY",F205&lt;&gt;"",G205&lt;&gt;"",K205&lt;&gt;"",OR(L205="PASS",L205="FAIL"),M205&lt;&gt;"",P205="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM205" s="9" t="str">
         <x:f>IF(A205="","",IF(AND(AK205="OK",J205="READY",F205&lt;&gt;"",G205&lt;&gt;"",K205&lt;&gt;"",S205="OK",OR(R205="PASS",R205="FAIL")),"YES","NO"))</x:f>
@@ -11641,7 +11641,7 @@
         <x:f>IF(A206="",IF(B206="","","MISSING_TEST_ID"),IF(B206="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A206,$B$2:$B$501,B206)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL206" s="9" t="str">
-        <x:f>IF(A206="","",IF(AND(AK206="OK",J206="READY",F206&lt;&gt;"",G206&lt;&gt;"",K206&lt;&gt;"",OR(L206="PASS",L206="FAIL"),M206&lt;&gt;"",O206&lt;&gt;"",P206="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A206="","",IF(AND(AK206="OK",J206="READY",F206&lt;&gt;"",G206&lt;&gt;"",K206&lt;&gt;"",OR(L206="PASS",L206="FAIL"),M206&lt;&gt;"",P206="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM206" s="9" t="str">
         <x:f>IF(A206="","",IF(AND(AK206="OK",J206="READY",F206&lt;&gt;"",G206&lt;&gt;"",K206&lt;&gt;"",S206="OK",OR(R206="PASS",R206="FAIL")),"YES","NO"))</x:f>
@@ -11693,7 +11693,7 @@
         <x:f>IF(A207="",IF(B207="","","MISSING_TEST_ID"),IF(B207="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A207,$B$2:$B$501,B207)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL207" s="9" t="str">
-        <x:f>IF(A207="","",IF(AND(AK207="OK",J207="READY",F207&lt;&gt;"",G207&lt;&gt;"",K207&lt;&gt;"",OR(L207="PASS",L207="FAIL"),M207&lt;&gt;"",O207&lt;&gt;"",P207="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A207="","",IF(AND(AK207="OK",J207="READY",F207&lt;&gt;"",G207&lt;&gt;"",K207&lt;&gt;"",OR(L207="PASS",L207="FAIL"),M207&lt;&gt;"",P207="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM207" s="9" t="str">
         <x:f>IF(A207="","",IF(AND(AK207="OK",J207="READY",F207&lt;&gt;"",G207&lt;&gt;"",K207&lt;&gt;"",S207="OK",OR(R207="PASS",R207="FAIL")),"YES","NO"))</x:f>
@@ -11745,7 +11745,7 @@
         <x:f>IF(A208="",IF(B208="","","MISSING_TEST_ID"),IF(B208="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A208,$B$2:$B$501,B208)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL208" s="9" t="str">
-        <x:f>IF(A208="","",IF(AND(AK208="OK",J208="READY",F208&lt;&gt;"",G208&lt;&gt;"",K208&lt;&gt;"",OR(L208="PASS",L208="FAIL"),M208&lt;&gt;"",O208&lt;&gt;"",P208="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A208="","",IF(AND(AK208="OK",J208="READY",F208&lt;&gt;"",G208&lt;&gt;"",K208&lt;&gt;"",OR(L208="PASS",L208="FAIL"),M208&lt;&gt;"",P208="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM208" s="9" t="str">
         <x:f>IF(A208="","",IF(AND(AK208="OK",J208="READY",F208&lt;&gt;"",G208&lt;&gt;"",K208&lt;&gt;"",S208="OK",OR(R208="PASS",R208="FAIL")),"YES","NO"))</x:f>
@@ -11797,7 +11797,7 @@
         <x:f>IF(A209="",IF(B209="","","MISSING_TEST_ID"),IF(B209="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A209,$B$2:$B$501,B209)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL209" s="9" t="str">
-        <x:f>IF(A209="","",IF(AND(AK209="OK",J209="READY",F209&lt;&gt;"",G209&lt;&gt;"",K209&lt;&gt;"",OR(L209="PASS",L209="FAIL"),M209&lt;&gt;"",O209&lt;&gt;"",P209="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A209="","",IF(AND(AK209="OK",J209="READY",F209&lt;&gt;"",G209&lt;&gt;"",K209&lt;&gt;"",OR(L209="PASS",L209="FAIL"),M209&lt;&gt;"",P209="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM209" s="9" t="str">
         <x:f>IF(A209="","",IF(AND(AK209="OK",J209="READY",F209&lt;&gt;"",G209&lt;&gt;"",K209&lt;&gt;"",S209="OK",OR(R209="PASS",R209="FAIL")),"YES","NO"))</x:f>
@@ -11849,7 +11849,7 @@
         <x:f>IF(A210="",IF(B210="","","MISSING_TEST_ID"),IF(B210="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A210,$B$2:$B$501,B210)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL210" s="9" t="str">
-        <x:f>IF(A210="","",IF(AND(AK210="OK",J210="READY",F210&lt;&gt;"",G210&lt;&gt;"",K210&lt;&gt;"",OR(L210="PASS",L210="FAIL"),M210&lt;&gt;"",O210&lt;&gt;"",P210="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A210="","",IF(AND(AK210="OK",J210="READY",F210&lt;&gt;"",G210&lt;&gt;"",K210&lt;&gt;"",OR(L210="PASS",L210="FAIL"),M210&lt;&gt;"",P210="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM210" s="9" t="str">
         <x:f>IF(A210="","",IF(AND(AK210="OK",J210="READY",F210&lt;&gt;"",G210&lt;&gt;"",K210&lt;&gt;"",S210="OK",OR(R210="PASS",R210="FAIL")),"YES","NO"))</x:f>
@@ -11901,7 +11901,7 @@
         <x:f>IF(A211="",IF(B211="","","MISSING_TEST_ID"),IF(B211="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A211,$B$2:$B$501,B211)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL211" s="9" t="str">
-        <x:f>IF(A211="","",IF(AND(AK211="OK",J211="READY",F211&lt;&gt;"",G211&lt;&gt;"",K211&lt;&gt;"",OR(L211="PASS",L211="FAIL"),M211&lt;&gt;"",O211&lt;&gt;"",P211="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A211="","",IF(AND(AK211="OK",J211="READY",F211&lt;&gt;"",G211&lt;&gt;"",K211&lt;&gt;"",OR(L211="PASS",L211="FAIL"),M211&lt;&gt;"",P211="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM211" s="9" t="str">
         <x:f>IF(A211="","",IF(AND(AK211="OK",J211="READY",F211&lt;&gt;"",G211&lt;&gt;"",K211&lt;&gt;"",S211="OK",OR(R211="PASS",R211="FAIL")),"YES","NO"))</x:f>
@@ -11953,7 +11953,7 @@
         <x:f>IF(A212="",IF(B212="","","MISSING_TEST_ID"),IF(B212="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A212,$B$2:$B$501,B212)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL212" s="9" t="str">
-        <x:f>IF(A212="","",IF(AND(AK212="OK",J212="READY",F212&lt;&gt;"",G212&lt;&gt;"",K212&lt;&gt;"",OR(L212="PASS",L212="FAIL"),M212&lt;&gt;"",O212&lt;&gt;"",P212="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A212="","",IF(AND(AK212="OK",J212="READY",F212&lt;&gt;"",G212&lt;&gt;"",K212&lt;&gt;"",OR(L212="PASS",L212="FAIL"),M212&lt;&gt;"",P212="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM212" s="9" t="str">
         <x:f>IF(A212="","",IF(AND(AK212="OK",J212="READY",F212&lt;&gt;"",G212&lt;&gt;"",K212&lt;&gt;"",S212="OK",OR(R212="PASS",R212="FAIL")),"YES","NO"))</x:f>
@@ -12005,7 +12005,7 @@
         <x:f>IF(A213="",IF(B213="","","MISSING_TEST_ID"),IF(B213="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A213,$B$2:$B$501,B213)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL213" s="9" t="str">
-        <x:f>IF(A213="","",IF(AND(AK213="OK",J213="READY",F213&lt;&gt;"",G213&lt;&gt;"",K213&lt;&gt;"",OR(L213="PASS",L213="FAIL"),M213&lt;&gt;"",O213&lt;&gt;"",P213="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A213="","",IF(AND(AK213="OK",J213="READY",F213&lt;&gt;"",G213&lt;&gt;"",K213&lt;&gt;"",OR(L213="PASS",L213="FAIL"),M213&lt;&gt;"",P213="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM213" s="9" t="str">
         <x:f>IF(A213="","",IF(AND(AK213="OK",J213="READY",F213&lt;&gt;"",G213&lt;&gt;"",K213&lt;&gt;"",S213="OK",OR(R213="PASS",R213="FAIL")),"YES","NO"))</x:f>
@@ -12057,7 +12057,7 @@
         <x:f>IF(A214="",IF(B214="","","MISSING_TEST_ID"),IF(B214="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A214,$B$2:$B$501,B214)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL214" s="9" t="str">
-        <x:f>IF(A214="","",IF(AND(AK214="OK",J214="READY",F214&lt;&gt;"",G214&lt;&gt;"",K214&lt;&gt;"",OR(L214="PASS",L214="FAIL"),M214&lt;&gt;"",O214&lt;&gt;"",P214="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A214="","",IF(AND(AK214="OK",J214="READY",F214&lt;&gt;"",G214&lt;&gt;"",K214&lt;&gt;"",OR(L214="PASS",L214="FAIL"),M214&lt;&gt;"",P214="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM214" s="9" t="str">
         <x:f>IF(A214="","",IF(AND(AK214="OK",J214="READY",F214&lt;&gt;"",G214&lt;&gt;"",K214&lt;&gt;"",S214="OK",OR(R214="PASS",R214="FAIL")),"YES","NO"))</x:f>
@@ -12109,7 +12109,7 @@
         <x:f>IF(A215="",IF(B215="","","MISSING_TEST_ID"),IF(B215="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A215,$B$2:$B$501,B215)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL215" s="9" t="str">
-        <x:f>IF(A215="","",IF(AND(AK215="OK",J215="READY",F215&lt;&gt;"",G215&lt;&gt;"",K215&lt;&gt;"",OR(L215="PASS",L215="FAIL"),M215&lt;&gt;"",O215&lt;&gt;"",P215="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A215="","",IF(AND(AK215="OK",J215="READY",F215&lt;&gt;"",G215&lt;&gt;"",K215&lt;&gt;"",OR(L215="PASS",L215="FAIL"),M215&lt;&gt;"",P215="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM215" s="9" t="str">
         <x:f>IF(A215="","",IF(AND(AK215="OK",J215="READY",F215&lt;&gt;"",G215&lt;&gt;"",K215&lt;&gt;"",S215="OK",OR(R215="PASS",R215="FAIL")),"YES","NO"))</x:f>
@@ -12161,7 +12161,7 @@
         <x:f>IF(A216="",IF(B216="","","MISSING_TEST_ID"),IF(B216="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A216,$B$2:$B$501,B216)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL216" s="9" t="str">
-        <x:f>IF(A216="","",IF(AND(AK216="OK",J216="READY",F216&lt;&gt;"",G216&lt;&gt;"",K216&lt;&gt;"",OR(L216="PASS",L216="FAIL"),M216&lt;&gt;"",O216&lt;&gt;"",P216="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A216="","",IF(AND(AK216="OK",J216="READY",F216&lt;&gt;"",G216&lt;&gt;"",K216&lt;&gt;"",OR(L216="PASS",L216="FAIL"),M216&lt;&gt;"",P216="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM216" s="9" t="str">
         <x:f>IF(A216="","",IF(AND(AK216="OK",J216="READY",F216&lt;&gt;"",G216&lt;&gt;"",K216&lt;&gt;"",S216="OK",OR(R216="PASS",R216="FAIL")),"YES","NO"))</x:f>
@@ -12213,7 +12213,7 @@
         <x:f>IF(A217="",IF(B217="","","MISSING_TEST_ID"),IF(B217="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A217,$B$2:$B$501,B217)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL217" s="9" t="str">
-        <x:f>IF(A217="","",IF(AND(AK217="OK",J217="READY",F217&lt;&gt;"",G217&lt;&gt;"",K217&lt;&gt;"",OR(L217="PASS",L217="FAIL"),M217&lt;&gt;"",O217&lt;&gt;"",P217="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A217="","",IF(AND(AK217="OK",J217="READY",F217&lt;&gt;"",G217&lt;&gt;"",K217&lt;&gt;"",OR(L217="PASS",L217="FAIL"),M217&lt;&gt;"",P217="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM217" s="9" t="str">
         <x:f>IF(A217="","",IF(AND(AK217="OK",J217="READY",F217&lt;&gt;"",G217&lt;&gt;"",K217&lt;&gt;"",S217="OK",OR(R217="PASS",R217="FAIL")),"YES","NO"))</x:f>
@@ -12265,7 +12265,7 @@
         <x:f>IF(A218="",IF(B218="","","MISSING_TEST_ID"),IF(B218="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A218,$B$2:$B$501,B218)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL218" s="9" t="str">
-        <x:f>IF(A218="","",IF(AND(AK218="OK",J218="READY",F218&lt;&gt;"",G218&lt;&gt;"",K218&lt;&gt;"",OR(L218="PASS",L218="FAIL"),M218&lt;&gt;"",O218&lt;&gt;"",P218="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A218="","",IF(AND(AK218="OK",J218="READY",F218&lt;&gt;"",G218&lt;&gt;"",K218&lt;&gt;"",OR(L218="PASS",L218="FAIL"),M218&lt;&gt;"",P218="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM218" s="9" t="str">
         <x:f>IF(A218="","",IF(AND(AK218="OK",J218="READY",F218&lt;&gt;"",G218&lt;&gt;"",K218&lt;&gt;"",S218="OK",OR(R218="PASS",R218="FAIL")),"YES","NO"))</x:f>
@@ -12317,7 +12317,7 @@
         <x:f>IF(A219="",IF(B219="","","MISSING_TEST_ID"),IF(B219="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A219,$B$2:$B$501,B219)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL219" s="9" t="str">
-        <x:f>IF(A219="","",IF(AND(AK219="OK",J219="READY",F219&lt;&gt;"",G219&lt;&gt;"",K219&lt;&gt;"",OR(L219="PASS",L219="FAIL"),M219&lt;&gt;"",O219&lt;&gt;"",P219="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A219="","",IF(AND(AK219="OK",J219="READY",F219&lt;&gt;"",G219&lt;&gt;"",K219&lt;&gt;"",OR(L219="PASS",L219="FAIL"),M219&lt;&gt;"",P219="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM219" s="9" t="str">
         <x:f>IF(A219="","",IF(AND(AK219="OK",J219="READY",F219&lt;&gt;"",G219&lt;&gt;"",K219&lt;&gt;"",S219="OK",OR(R219="PASS",R219="FAIL")),"YES","NO"))</x:f>
@@ -12369,7 +12369,7 @@
         <x:f>IF(A220="",IF(B220="","","MISSING_TEST_ID"),IF(B220="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A220,$B$2:$B$501,B220)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL220" s="9" t="str">
-        <x:f>IF(A220="","",IF(AND(AK220="OK",J220="READY",F220&lt;&gt;"",G220&lt;&gt;"",K220&lt;&gt;"",OR(L220="PASS",L220="FAIL"),M220&lt;&gt;"",O220&lt;&gt;"",P220="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A220="","",IF(AND(AK220="OK",J220="READY",F220&lt;&gt;"",G220&lt;&gt;"",K220&lt;&gt;"",OR(L220="PASS",L220="FAIL"),M220&lt;&gt;"",P220="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM220" s="9" t="str">
         <x:f>IF(A220="","",IF(AND(AK220="OK",J220="READY",F220&lt;&gt;"",G220&lt;&gt;"",K220&lt;&gt;"",S220="OK",OR(R220="PASS",R220="FAIL")),"YES","NO"))</x:f>
@@ -12421,7 +12421,7 @@
         <x:f>IF(A221="",IF(B221="","","MISSING_TEST_ID"),IF(B221="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A221,$B$2:$B$501,B221)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL221" s="9" t="str">
-        <x:f>IF(A221="","",IF(AND(AK221="OK",J221="READY",F221&lt;&gt;"",G221&lt;&gt;"",K221&lt;&gt;"",OR(L221="PASS",L221="FAIL"),M221&lt;&gt;"",O221&lt;&gt;"",P221="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A221="","",IF(AND(AK221="OK",J221="READY",F221&lt;&gt;"",G221&lt;&gt;"",K221&lt;&gt;"",OR(L221="PASS",L221="FAIL"),M221&lt;&gt;"",P221="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM221" s="9" t="str">
         <x:f>IF(A221="","",IF(AND(AK221="OK",J221="READY",F221&lt;&gt;"",G221&lt;&gt;"",K221&lt;&gt;"",S221="OK",OR(R221="PASS",R221="FAIL")),"YES","NO"))</x:f>
@@ -12473,7 +12473,7 @@
         <x:f>IF(A222="",IF(B222="","","MISSING_TEST_ID"),IF(B222="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A222,$B$2:$B$501,B222)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL222" s="9" t="str">
-        <x:f>IF(A222="","",IF(AND(AK222="OK",J222="READY",F222&lt;&gt;"",G222&lt;&gt;"",K222&lt;&gt;"",OR(L222="PASS",L222="FAIL"),M222&lt;&gt;"",O222&lt;&gt;"",P222="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A222="","",IF(AND(AK222="OK",J222="READY",F222&lt;&gt;"",G222&lt;&gt;"",K222&lt;&gt;"",OR(L222="PASS",L222="FAIL"),M222&lt;&gt;"",P222="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM222" s="9" t="str">
         <x:f>IF(A222="","",IF(AND(AK222="OK",J222="READY",F222&lt;&gt;"",G222&lt;&gt;"",K222&lt;&gt;"",S222="OK",OR(R222="PASS",R222="FAIL")),"YES","NO"))</x:f>
@@ -12525,7 +12525,7 @@
         <x:f>IF(A223="",IF(B223="","","MISSING_TEST_ID"),IF(B223="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A223,$B$2:$B$501,B223)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL223" s="9" t="str">
-        <x:f>IF(A223="","",IF(AND(AK223="OK",J223="READY",F223&lt;&gt;"",G223&lt;&gt;"",K223&lt;&gt;"",OR(L223="PASS",L223="FAIL"),M223&lt;&gt;"",O223&lt;&gt;"",P223="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A223="","",IF(AND(AK223="OK",J223="READY",F223&lt;&gt;"",G223&lt;&gt;"",K223&lt;&gt;"",OR(L223="PASS",L223="FAIL"),M223&lt;&gt;"",P223="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM223" s="9" t="str">
         <x:f>IF(A223="","",IF(AND(AK223="OK",J223="READY",F223&lt;&gt;"",G223&lt;&gt;"",K223&lt;&gt;"",S223="OK",OR(R223="PASS",R223="FAIL")),"YES","NO"))</x:f>
@@ -12577,7 +12577,7 @@
         <x:f>IF(A224="",IF(B224="","","MISSING_TEST_ID"),IF(B224="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A224,$B$2:$B$501,B224)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL224" s="9" t="str">
-        <x:f>IF(A224="","",IF(AND(AK224="OK",J224="READY",F224&lt;&gt;"",G224&lt;&gt;"",K224&lt;&gt;"",OR(L224="PASS",L224="FAIL"),M224&lt;&gt;"",O224&lt;&gt;"",P224="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A224="","",IF(AND(AK224="OK",J224="READY",F224&lt;&gt;"",G224&lt;&gt;"",K224&lt;&gt;"",OR(L224="PASS",L224="FAIL"),M224&lt;&gt;"",P224="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM224" s="9" t="str">
         <x:f>IF(A224="","",IF(AND(AK224="OK",J224="READY",F224&lt;&gt;"",G224&lt;&gt;"",K224&lt;&gt;"",S224="OK",OR(R224="PASS",R224="FAIL")),"YES","NO"))</x:f>
@@ -12629,7 +12629,7 @@
         <x:f>IF(A225="",IF(B225="","","MISSING_TEST_ID"),IF(B225="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A225,$B$2:$B$501,B225)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL225" s="9" t="str">
-        <x:f>IF(A225="","",IF(AND(AK225="OK",J225="READY",F225&lt;&gt;"",G225&lt;&gt;"",K225&lt;&gt;"",OR(L225="PASS",L225="FAIL"),M225&lt;&gt;"",O225&lt;&gt;"",P225="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A225="","",IF(AND(AK225="OK",J225="READY",F225&lt;&gt;"",G225&lt;&gt;"",K225&lt;&gt;"",OR(L225="PASS",L225="FAIL"),M225&lt;&gt;"",P225="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM225" s="9" t="str">
         <x:f>IF(A225="","",IF(AND(AK225="OK",J225="READY",F225&lt;&gt;"",G225&lt;&gt;"",K225&lt;&gt;"",S225="OK",OR(R225="PASS",R225="FAIL")),"YES","NO"))</x:f>
@@ -12681,7 +12681,7 @@
         <x:f>IF(A226="",IF(B226="","","MISSING_TEST_ID"),IF(B226="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A226,$B$2:$B$501,B226)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL226" s="9" t="str">
-        <x:f>IF(A226="","",IF(AND(AK226="OK",J226="READY",F226&lt;&gt;"",G226&lt;&gt;"",K226&lt;&gt;"",OR(L226="PASS",L226="FAIL"),M226&lt;&gt;"",O226&lt;&gt;"",P226="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A226="","",IF(AND(AK226="OK",J226="READY",F226&lt;&gt;"",G226&lt;&gt;"",K226&lt;&gt;"",OR(L226="PASS",L226="FAIL"),M226&lt;&gt;"",P226="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM226" s="9" t="str">
         <x:f>IF(A226="","",IF(AND(AK226="OK",J226="READY",F226&lt;&gt;"",G226&lt;&gt;"",K226&lt;&gt;"",S226="OK",OR(R226="PASS",R226="FAIL")),"YES","NO"))</x:f>
@@ -12733,7 +12733,7 @@
         <x:f>IF(A227="",IF(B227="","","MISSING_TEST_ID"),IF(B227="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A227,$B$2:$B$501,B227)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL227" s="9" t="str">
-        <x:f>IF(A227="","",IF(AND(AK227="OK",J227="READY",F227&lt;&gt;"",G227&lt;&gt;"",K227&lt;&gt;"",OR(L227="PASS",L227="FAIL"),M227&lt;&gt;"",O227&lt;&gt;"",P227="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A227="","",IF(AND(AK227="OK",J227="READY",F227&lt;&gt;"",G227&lt;&gt;"",K227&lt;&gt;"",OR(L227="PASS",L227="FAIL"),M227&lt;&gt;"",P227="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM227" s="9" t="str">
         <x:f>IF(A227="","",IF(AND(AK227="OK",J227="READY",F227&lt;&gt;"",G227&lt;&gt;"",K227&lt;&gt;"",S227="OK",OR(R227="PASS",R227="FAIL")),"YES","NO"))</x:f>
@@ -12785,7 +12785,7 @@
         <x:f>IF(A228="",IF(B228="","","MISSING_TEST_ID"),IF(B228="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A228,$B$2:$B$501,B228)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL228" s="9" t="str">
-        <x:f>IF(A228="","",IF(AND(AK228="OK",J228="READY",F228&lt;&gt;"",G228&lt;&gt;"",K228&lt;&gt;"",OR(L228="PASS",L228="FAIL"),M228&lt;&gt;"",O228&lt;&gt;"",P228="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A228="","",IF(AND(AK228="OK",J228="READY",F228&lt;&gt;"",G228&lt;&gt;"",K228&lt;&gt;"",OR(L228="PASS",L228="FAIL"),M228&lt;&gt;"",P228="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM228" s="9" t="str">
         <x:f>IF(A228="","",IF(AND(AK228="OK",J228="READY",F228&lt;&gt;"",G228&lt;&gt;"",K228&lt;&gt;"",S228="OK",OR(R228="PASS",R228="FAIL")),"YES","NO"))</x:f>
@@ -12837,7 +12837,7 @@
         <x:f>IF(A229="",IF(B229="","","MISSING_TEST_ID"),IF(B229="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A229,$B$2:$B$501,B229)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL229" s="9" t="str">
-        <x:f>IF(A229="","",IF(AND(AK229="OK",J229="READY",F229&lt;&gt;"",G229&lt;&gt;"",K229&lt;&gt;"",OR(L229="PASS",L229="FAIL"),M229&lt;&gt;"",O229&lt;&gt;"",P229="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A229="","",IF(AND(AK229="OK",J229="READY",F229&lt;&gt;"",G229&lt;&gt;"",K229&lt;&gt;"",OR(L229="PASS",L229="FAIL"),M229&lt;&gt;"",P229="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM229" s="9" t="str">
         <x:f>IF(A229="","",IF(AND(AK229="OK",J229="READY",F229&lt;&gt;"",G229&lt;&gt;"",K229&lt;&gt;"",S229="OK",OR(R229="PASS",R229="FAIL")),"YES","NO"))</x:f>
@@ -12889,7 +12889,7 @@
         <x:f>IF(A230="",IF(B230="","","MISSING_TEST_ID"),IF(B230="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A230,$B$2:$B$501,B230)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL230" s="9" t="str">
-        <x:f>IF(A230="","",IF(AND(AK230="OK",J230="READY",F230&lt;&gt;"",G230&lt;&gt;"",K230&lt;&gt;"",OR(L230="PASS",L230="FAIL"),M230&lt;&gt;"",O230&lt;&gt;"",P230="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A230="","",IF(AND(AK230="OK",J230="READY",F230&lt;&gt;"",G230&lt;&gt;"",K230&lt;&gt;"",OR(L230="PASS",L230="FAIL"),M230&lt;&gt;"",P230="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM230" s="9" t="str">
         <x:f>IF(A230="","",IF(AND(AK230="OK",J230="READY",F230&lt;&gt;"",G230&lt;&gt;"",K230&lt;&gt;"",S230="OK",OR(R230="PASS",R230="FAIL")),"YES","NO"))</x:f>
@@ -12941,7 +12941,7 @@
         <x:f>IF(A231="",IF(B231="","","MISSING_TEST_ID"),IF(B231="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A231,$B$2:$B$501,B231)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL231" s="9" t="str">
-        <x:f>IF(A231="","",IF(AND(AK231="OK",J231="READY",F231&lt;&gt;"",G231&lt;&gt;"",K231&lt;&gt;"",OR(L231="PASS",L231="FAIL"),M231&lt;&gt;"",O231&lt;&gt;"",P231="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A231="","",IF(AND(AK231="OK",J231="READY",F231&lt;&gt;"",G231&lt;&gt;"",K231&lt;&gt;"",OR(L231="PASS",L231="FAIL"),M231&lt;&gt;"",P231="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM231" s="9" t="str">
         <x:f>IF(A231="","",IF(AND(AK231="OK",J231="READY",F231&lt;&gt;"",G231&lt;&gt;"",K231&lt;&gt;"",S231="OK",OR(R231="PASS",R231="FAIL")),"YES","NO"))</x:f>
@@ -12993,7 +12993,7 @@
         <x:f>IF(A232="",IF(B232="","","MISSING_TEST_ID"),IF(B232="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A232,$B$2:$B$501,B232)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL232" s="9" t="str">
-        <x:f>IF(A232="","",IF(AND(AK232="OK",J232="READY",F232&lt;&gt;"",G232&lt;&gt;"",K232&lt;&gt;"",OR(L232="PASS",L232="FAIL"),M232&lt;&gt;"",O232&lt;&gt;"",P232="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A232="","",IF(AND(AK232="OK",J232="READY",F232&lt;&gt;"",G232&lt;&gt;"",K232&lt;&gt;"",OR(L232="PASS",L232="FAIL"),M232&lt;&gt;"",P232="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM232" s="9" t="str">
         <x:f>IF(A232="","",IF(AND(AK232="OK",J232="READY",F232&lt;&gt;"",G232&lt;&gt;"",K232&lt;&gt;"",S232="OK",OR(R232="PASS",R232="FAIL")),"YES","NO"))</x:f>
@@ -13045,7 +13045,7 @@
         <x:f>IF(A233="",IF(B233="","","MISSING_TEST_ID"),IF(B233="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A233,$B$2:$B$501,B233)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL233" s="9" t="str">
-        <x:f>IF(A233="","",IF(AND(AK233="OK",J233="READY",F233&lt;&gt;"",G233&lt;&gt;"",K233&lt;&gt;"",OR(L233="PASS",L233="FAIL"),M233&lt;&gt;"",O233&lt;&gt;"",P233="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A233="","",IF(AND(AK233="OK",J233="READY",F233&lt;&gt;"",G233&lt;&gt;"",K233&lt;&gt;"",OR(L233="PASS",L233="FAIL"),M233&lt;&gt;"",P233="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM233" s="9" t="str">
         <x:f>IF(A233="","",IF(AND(AK233="OK",J233="READY",F233&lt;&gt;"",G233&lt;&gt;"",K233&lt;&gt;"",S233="OK",OR(R233="PASS",R233="FAIL")),"YES","NO"))</x:f>
@@ -13097,7 +13097,7 @@
         <x:f>IF(A234="",IF(B234="","","MISSING_TEST_ID"),IF(B234="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A234,$B$2:$B$501,B234)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL234" s="9" t="str">
-        <x:f>IF(A234="","",IF(AND(AK234="OK",J234="READY",F234&lt;&gt;"",G234&lt;&gt;"",K234&lt;&gt;"",OR(L234="PASS",L234="FAIL"),M234&lt;&gt;"",O234&lt;&gt;"",P234="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A234="","",IF(AND(AK234="OK",J234="READY",F234&lt;&gt;"",G234&lt;&gt;"",K234&lt;&gt;"",OR(L234="PASS",L234="FAIL"),M234&lt;&gt;"",P234="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM234" s="9" t="str">
         <x:f>IF(A234="","",IF(AND(AK234="OK",J234="READY",F234&lt;&gt;"",G234&lt;&gt;"",K234&lt;&gt;"",S234="OK",OR(R234="PASS",R234="FAIL")),"YES","NO"))</x:f>
@@ -13149,7 +13149,7 @@
         <x:f>IF(A235="",IF(B235="","","MISSING_TEST_ID"),IF(B235="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A235,$B$2:$B$501,B235)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL235" s="9" t="str">
-        <x:f>IF(A235="","",IF(AND(AK235="OK",J235="READY",F235&lt;&gt;"",G235&lt;&gt;"",K235&lt;&gt;"",OR(L235="PASS",L235="FAIL"),M235&lt;&gt;"",O235&lt;&gt;"",P235="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A235="","",IF(AND(AK235="OK",J235="READY",F235&lt;&gt;"",G235&lt;&gt;"",K235&lt;&gt;"",OR(L235="PASS",L235="FAIL"),M235&lt;&gt;"",P235="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM235" s="9" t="str">
         <x:f>IF(A235="","",IF(AND(AK235="OK",J235="READY",F235&lt;&gt;"",G235&lt;&gt;"",K235&lt;&gt;"",S235="OK",OR(R235="PASS",R235="FAIL")),"YES","NO"))</x:f>
@@ -13201,7 +13201,7 @@
         <x:f>IF(A236="",IF(B236="","","MISSING_TEST_ID"),IF(B236="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A236,$B$2:$B$501,B236)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL236" s="9" t="str">
-        <x:f>IF(A236="","",IF(AND(AK236="OK",J236="READY",F236&lt;&gt;"",G236&lt;&gt;"",K236&lt;&gt;"",OR(L236="PASS",L236="FAIL"),M236&lt;&gt;"",O236&lt;&gt;"",P236="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A236="","",IF(AND(AK236="OK",J236="READY",F236&lt;&gt;"",G236&lt;&gt;"",K236&lt;&gt;"",OR(L236="PASS",L236="FAIL"),M236&lt;&gt;"",P236="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM236" s="9" t="str">
         <x:f>IF(A236="","",IF(AND(AK236="OK",J236="READY",F236&lt;&gt;"",G236&lt;&gt;"",K236&lt;&gt;"",S236="OK",OR(R236="PASS",R236="FAIL")),"YES","NO"))</x:f>
@@ -13253,7 +13253,7 @@
         <x:f>IF(A237="",IF(B237="","","MISSING_TEST_ID"),IF(B237="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A237,$B$2:$B$501,B237)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL237" s="9" t="str">
-        <x:f>IF(A237="","",IF(AND(AK237="OK",J237="READY",F237&lt;&gt;"",G237&lt;&gt;"",K237&lt;&gt;"",OR(L237="PASS",L237="FAIL"),M237&lt;&gt;"",O237&lt;&gt;"",P237="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A237="","",IF(AND(AK237="OK",J237="READY",F237&lt;&gt;"",G237&lt;&gt;"",K237&lt;&gt;"",OR(L237="PASS",L237="FAIL"),M237&lt;&gt;"",P237="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM237" s="9" t="str">
         <x:f>IF(A237="","",IF(AND(AK237="OK",J237="READY",F237&lt;&gt;"",G237&lt;&gt;"",K237&lt;&gt;"",S237="OK",OR(R237="PASS",R237="FAIL")),"YES","NO"))</x:f>
@@ -13305,7 +13305,7 @@
         <x:f>IF(A238="",IF(B238="","","MISSING_TEST_ID"),IF(B238="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A238,$B$2:$B$501,B238)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL238" s="9" t="str">
-        <x:f>IF(A238="","",IF(AND(AK238="OK",J238="READY",F238&lt;&gt;"",G238&lt;&gt;"",K238&lt;&gt;"",OR(L238="PASS",L238="FAIL"),M238&lt;&gt;"",O238&lt;&gt;"",P238="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A238="","",IF(AND(AK238="OK",J238="READY",F238&lt;&gt;"",G238&lt;&gt;"",K238&lt;&gt;"",OR(L238="PASS",L238="FAIL"),M238&lt;&gt;"",P238="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM238" s="9" t="str">
         <x:f>IF(A238="","",IF(AND(AK238="OK",J238="READY",F238&lt;&gt;"",G238&lt;&gt;"",K238&lt;&gt;"",S238="OK",OR(R238="PASS",R238="FAIL")),"YES","NO"))</x:f>
@@ -13357,7 +13357,7 @@
         <x:f>IF(A239="",IF(B239="","","MISSING_TEST_ID"),IF(B239="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A239,$B$2:$B$501,B239)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL239" s="9" t="str">
-        <x:f>IF(A239="","",IF(AND(AK239="OK",J239="READY",F239&lt;&gt;"",G239&lt;&gt;"",K239&lt;&gt;"",OR(L239="PASS",L239="FAIL"),M239&lt;&gt;"",O239&lt;&gt;"",P239="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A239="","",IF(AND(AK239="OK",J239="READY",F239&lt;&gt;"",G239&lt;&gt;"",K239&lt;&gt;"",OR(L239="PASS",L239="FAIL"),M239&lt;&gt;"",P239="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM239" s="9" t="str">
         <x:f>IF(A239="","",IF(AND(AK239="OK",J239="READY",F239&lt;&gt;"",G239&lt;&gt;"",K239&lt;&gt;"",S239="OK",OR(R239="PASS",R239="FAIL")),"YES","NO"))</x:f>
@@ -13409,7 +13409,7 @@
         <x:f>IF(A240="",IF(B240="","","MISSING_TEST_ID"),IF(B240="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A240,$B$2:$B$501,B240)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL240" s="9" t="str">
-        <x:f>IF(A240="","",IF(AND(AK240="OK",J240="READY",F240&lt;&gt;"",G240&lt;&gt;"",K240&lt;&gt;"",OR(L240="PASS",L240="FAIL"),M240&lt;&gt;"",O240&lt;&gt;"",P240="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A240="","",IF(AND(AK240="OK",J240="READY",F240&lt;&gt;"",G240&lt;&gt;"",K240&lt;&gt;"",OR(L240="PASS",L240="FAIL"),M240&lt;&gt;"",P240="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM240" s="9" t="str">
         <x:f>IF(A240="","",IF(AND(AK240="OK",J240="READY",F240&lt;&gt;"",G240&lt;&gt;"",K240&lt;&gt;"",S240="OK",OR(R240="PASS",R240="FAIL")),"YES","NO"))</x:f>
@@ -13461,7 +13461,7 @@
         <x:f>IF(A241="",IF(B241="","","MISSING_TEST_ID"),IF(B241="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A241,$B$2:$B$501,B241)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL241" s="9" t="str">
-        <x:f>IF(A241="","",IF(AND(AK241="OK",J241="READY",F241&lt;&gt;"",G241&lt;&gt;"",K241&lt;&gt;"",OR(L241="PASS",L241="FAIL"),M241&lt;&gt;"",O241&lt;&gt;"",P241="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A241="","",IF(AND(AK241="OK",J241="READY",F241&lt;&gt;"",G241&lt;&gt;"",K241&lt;&gt;"",OR(L241="PASS",L241="FAIL"),M241&lt;&gt;"",P241="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM241" s="9" t="str">
         <x:f>IF(A241="","",IF(AND(AK241="OK",J241="READY",F241&lt;&gt;"",G241&lt;&gt;"",K241&lt;&gt;"",S241="OK",OR(R241="PASS",R241="FAIL")),"YES","NO"))</x:f>
@@ -13513,7 +13513,7 @@
         <x:f>IF(A242="",IF(B242="","","MISSING_TEST_ID"),IF(B242="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A242,$B$2:$B$501,B242)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL242" s="9" t="str">
-        <x:f>IF(A242="","",IF(AND(AK242="OK",J242="READY",F242&lt;&gt;"",G242&lt;&gt;"",K242&lt;&gt;"",OR(L242="PASS",L242="FAIL"),M242&lt;&gt;"",O242&lt;&gt;"",P242="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A242="","",IF(AND(AK242="OK",J242="READY",F242&lt;&gt;"",G242&lt;&gt;"",K242&lt;&gt;"",OR(L242="PASS",L242="FAIL"),M242&lt;&gt;"",P242="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM242" s="9" t="str">
         <x:f>IF(A242="","",IF(AND(AK242="OK",J242="READY",F242&lt;&gt;"",G242&lt;&gt;"",K242&lt;&gt;"",S242="OK",OR(R242="PASS",R242="FAIL")),"YES","NO"))</x:f>
@@ -13565,7 +13565,7 @@
         <x:f>IF(A243="",IF(B243="","","MISSING_TEST_ID"),IF(B243="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A243,$B$2:$B$501,B243)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL243" s="9" t="str">
-        <x:f>IF(A243="","",IF(AND(AK243="OK",J243="READY",F243&lt;&gt;"",G243&lt;&gt;"",K243&lt;&gt;"",OR(L243="PASS",L243="FAIL"),M243&lt;&gt;"",O243&lt;&gt;"",P243="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A243="","",IF(AND(AK243="OK",J243="READY",F243&lt;&gt;"",G243&lt;&gt;"",K243&lt;&gt;"",OR(L243="PASS",L243="FAIL"),M243&lt;&gt;"",P243="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM243" s="9" t="str">
         <x:f>IF(A243="","",IF(AND(AK243="OK",J243="READY",F243&lt;&gt;"",G243&lt;&gt;"",K243&lt;&gt;"",S243="OK",OR(R243="PASS",R243="FAIL")),"YES","NO"))</x:f>
@@ -13617,7 +13617,7 @@
         <x:f>IF(A244="",IF(B244="","","MISSING_TEST_ID"),IF(B244="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A244,$B$2:$B$501,B244)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL244" s="9" t="str">
-        <x:f>IF(A244="","",IF(AND(AK244="OK",J244="READY",F244&lt;&gt;"",G244&lt;&gt;"",K244&lt;&gt;"",OR(L244="PASS",L244="FAIL"),M244&lt;&gt;"",O244&lt;&gt;"",P244="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A244="","",IF(AND(AK244="OK",J244="READY",F244&lt;&gt;"",G244&lt;&gt;"",K244&lt;&gt;"",OR(L244="PASS",L244="FAIL"),M244&lt;&gt;"",P244="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM244" s="9" t="str">
         <x:f>IF(A244="","",IF(AND(AK244="OK",J244="READY",F244&lt;&gt;"",G244&lt;&gt;"",K244&lt;&gt;"",S244="OK",OR(R244="PASS",R244="FAIL")),"YES","NO"))</x:f>
@@ -13669,7 +13669,7 @@
         <x:f>IF(A245="",IF(B245="","","MISSING_TEST_ID"),IF(B245="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A245,$B$2:$B$501,B245)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL245" s="9" t="str">
-        <x:f>IF(A245="","",IF(AND(AK245="OK",J245="READY",F245&lt;&gt;"",G245&lt;&gt;"",K245&lt;&gt;"",OR(L245="PASS",L245="FAIL"),M245&lt;&gt;"",O245&lt;&gt;"",P245="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A245="","",IF(AND(AK245="OK",J245="READY",F245&lt;&gt;"",G245&lt;&gt;"",K245&lt;&gt;"",OR(L245="PASS",L245="FAIL"),M245&lt;&gt;"",P245="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM245" s="9" t="str">
         <x:f>IF(A245="","",IF(AND(AK245="OK",J245="READY",F245&lt;&gt;"",G245&lt;&gt;"",K245&lt;&gt;"",S245="OK",OR(R245="PASS",R245="FAIL")),"YES","NO"))</x:f>
@@ -13721,7 +13721,7 @@
         <x:f>IF(A246="",IF(B246="","","MISSING_TEST_ID"),IF(B246="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A246,$B$2:$B$501,B246)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL246" s="9" t="str">
-        <x:f>IF(A246="","",IF(AND(AK246="OK",J246="READY",F246&lt;&gt;"",G246&lt;&gt;"",K246&lt;&gt;"",OR(L246="PASS",L246="FAIL"),M246&lt;&gt;"",O246&lt;&gt;"",P246="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A246="","",IF(AND(AK246="OK",J246="READY",F246&lt;&gt;"",G246&lt;&gt;"",K246&lt;&gt;"",OR(L246="PASS",L246="FAIL"),M246&lt;&gt;"",P246="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM246" s="9" t="str">
         <x:f>IF(A246="","",IF(AND(AK246="OK",J246="READY",F246&lt;&gt;"",G246&lt;&gt;"",K246&lt;&gt;"",S246="OK",OR(R246="PASS",R246="FAIL")),"YES","NO"))</x:f>
@@ -13773,7 +13773,7 @@
         <x:f>IF(A247="",IF(B247="","","MISSING_TEST_ID"),IF(B247="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A247,$B$2:$B$501,B247)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL247" s="9" t="str">
-        <x:f>IF(A247="","",IF(AND(AK247="OK",J247="READY",F247&lt;&gt;"",G247&lt;&gt;"",K247&lt;&gt;"",OR(L247="PASS",L247="FAIL"),M247&lt;&gt;"",O247&lt;&gt;"",P247="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A247="","",IF(AND(AK247="OK",J247="READY",F247&lt;&gt;"",G247&lt;&gt;"",K247&lt;&gt;"",OR(L247="PASS",L247="FAIL"),M247&lt;&gt;"",P247="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM247" s="9" t="str">
         <x:f>IF(A247="","",IF(AND(AK247="OK",J247="READY",F247&lt;&gt;"",G247&lt;&gt;"",K247&lt;&gt;"",S247="OK",OR(R247="PASS",R247="FAIL")),"YES","NO"))</x:f>
@@ -13825,7 +13825,7 @@
         <x:f>IF(A248="",IF(B248="","","MISSING_TEST_ID"),IF(B248="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A248,$B$2:$B$501,B248)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL248" s="9" t="str">
-        <x:f>IF(A248="","",IF(AND(AK248="OK",J248="READY",F248&lt;&gt;"",G248&lt;&gt;"",K248&lt;&gt;"",OR(L248="PASS",L248="FAIL"),M248&lt;&gt;"",O248&lt;&gt;"",P248="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A248="","",IF(AND(AK248="OK",J248="READY",F248&lt;&gt;"",G248&lt;&gt;"",K248&lt;&gt;"",OR(L248="PASS",L248="FAIL"),M248&lt;&gt;"",P248="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM248" s="9" t="str">
         <x:f>IF(A248="","",IF(AND(AK248="OK",J248="READY",F248&lt;&gt;"",G248&lt;&gt;"",K248&lt;&gt;"",S248="OK",OR(R248="PASS",R248="FAIL")),"YES","NO"))</x:f>
@@ -13877,7 +13877,7 @@
         <x:f>IF(A249="",IF(B249="","","MISSING_TEST_ID"),IF(B249="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A249,$B$2:$B$501,B249)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL249" s="9" t="str">
-        <x:f>IF(A249="","",IF(AND(AK249="OK",J249="READY",F249&lt;&gt;"",G249&lt;&gt;"",K249&lt;&gt;"",OR(L249="PASS",L249="FAIL"),M249&lt;&gt;"",O249&lt;&gt;"",P249="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A249="","",IF(AND(AK249="OK",J249="READY",F249&lt;&gt;"",G249&lt;&gt;"",K249&lt;&gt;"",OR(L249="PASS",L249="FAIL"),M249&lt;&gt;"",P249="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM249" s="9" t="str">
         <x:f>IF(A249="","",IF(AND(AK249="OK",J249="READY",F249&lt;&gt;"",G249&lt;&gt;"",K249&lt;&gt;"",S249="OK",OR(R249="PASS",R249="FAIL")),"YES","NO"))</x:f>
@@ -13929,7 +13929,7 @@
         <x:f>IF(A250="",IF(B250="","","MISSING_TEST_ID"),IF(B250="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A250,$B$2:$B$501,B250)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL250" s="9" t="str">
-        <x:f>IF(A250="","",IF(AND(AK250="OK",J250="READY",F250&lt;&gt;"",G250&lt;&gt;"",K250&lt;&gt;"",OR(L250="PASS",L250="FAIL"),M250&lt;&gt;"",O250&lt;&gt;"",P250="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A250="","",IF(AND(AK250="OK",J250="READY",F250&lt;&gt;"",G250&lt;&gt;"",K250&lt;&gt;"",OR(L250="PASS",L250="FAIL"),M250&lt;&gt;"",P250="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM250" s="9" t="str">
         <x:f>IF(A250="","",IF(AND(AK250="OK",J250="READY",F250&lt;&gt;"",G250&lt;&gt;"",K250&lt;&gt;"",S250="OK",OR(R250="PASS",R250="FAIL")),"YES","NO"))</x:f>
@@ -13981,7 +13981,7 @@
         <x:f>IF(A251="",IF(B251="","","MISSING_TEST_ID"),IF(B251="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A251,$B$2:$B$501,B251)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL251" s="9" t="str">
-        <x:f>IF(A251="","",IF(AND(AK251="OK",J251="READY",F251&lt;&gt;"",G251&lt;&gt;"",K251&lt;&gt;"",OR(L251="PASS",L251="FAIL"),M251&lt;&gt;"",O251&lt;&gt;"",P251="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A251="","",IF(AND(AK251="OK",J251="READY",F251&lt;&gt;"",G251&lt;&gt;"",K251&lt;&gt;"",OR(L251="PASS",L251="FAIL"),M251&lt;&gt;"",P251="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM251" s="9" t="str">
         <x:f>IF(A251="","",IF(AND(AK251="OK",J251="READY",F251&lt;&gt;"",G251&lt;&gt;"",K251&lt;&gt;"",S251="OK",OR(R251="PASS",R251="FAIL")),"YES","NO"))</x:f>
@@ -14033,7 +14033,7 @@
         <x:f>IF(A252="",IF(B252="","","MISSING_TEST_ID"),IF(B252="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A252,$B$2:$B$501,B252)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL252" s="9" t="str">
-        <x:f>IF(A252="","",IF(AND(AK252="OK",J252="READY",F252&lt;&gt;"",G252&lt;&gt;"",K252&lt;&gt;"",OR(L252="PASS",L252="FAIL"),M252&lt;&gt;"",O252&lt;&gt;"",P252="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A252="","",IF(AND(AK252="OK",J252="READY",F252&lt;&gt;"",G252&lt;&gt;"",K252&lt;&gt;"",OR(L252="PASS",L252="FAIL"),M252&lt;&gt;"",P252="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM252" s="9" t="str">
         <x:f>IF(A252="","",IF(AND(AK252="OK",J252="READY",F252&lt;&gt;"",G252&lt;&gt;"",K252&lt;&gt;"",S252="OK",OR(R252="PASS",R252="FAIL")),"YES","NO"))</x:f>
@@ -14085,7 +14085,7 @@
         <x:f>IF(A253="",IF(B253="","","MISSING_TEST_ID"),IF(B253="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A253,$B$2:$B$501,B253)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL253" s="9" t="str">
-        <x:f>IF(A253="","",IF(AND(AK253="OK",J253="READY",F253&lt;&gt;"",G253&lt;&gt;"",K253&lt;&gt;"",OR(L253="PASS",L253="FAIL"),M253&lt;&gt;"",O253&lt;&gt;"",P253="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A253="","",IF(AND(AK253="OK",J253="READY",F253&lt;&gt;"",G253&lt;&gt;"",K253&lt;&gt;"",OR(L253="PASS",L253="FAIL"),M253&lt;&gt;"",P253="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM253" s="9" t="str">
         <x:f>IF(A253="","",IF(AND(AK253="OK",J253="READY",F253&lt;&gt;"",G253&lt;&gt;"",K253&lt;&gt;"",S253="OK",OR(R253="PASS",R253="FAIL")),"YES","NO"))</x:f>
@@ -14137,7 +14137,7 @@
         <x:f>IF(A254="",IF(B254="","","MISSING_TEST_ID"),IF(B254="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A254,$B$2:$B$501,B254)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL254" s="9" t="str">
-        <x:f>IF(A254="","",IF(AND(AK254="OK",J254="READY",F254&lt;&gt;"",G254&lt;&gt;"",K254&lt;&gt;"",OR(L254="PASS",L254="FAIL"),M254&lt;&gt;"",O254&lt;&gt;"",P254="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A254="","",IF(AND(AK254="OK",J254="READY",F254&lt;&gt;"",G254&lt;&gt;"",K254&lt;&gt;"",OR(L254="PASS",L254="FAIL"),M254&lt;&gt;"",P254="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM254" s="9" t="str">
         <x:f>IF(A254="","",IF(AND(AK254="OK",J254="READY",F254&lt;&gt;"",G254&lt;&gt;"",K254&lt;&gt;"",S254="OK",OR(R254="PASS",R254="FAIL")),"YES","NO"))</x:f>
@@ -14189,7 +14189,7 @@
         <x:f>IF(A255="",IF(B255="","","MISSING_TEST_ID"),IF(B255="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A255,$B$2:$B$501,B255)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL255" s="9" t="str">
-        <x:f>IF(A255="","",IF(AND(AK255="OK",J255="READY",F255&lt;&gt;"",G255&lt;&gt;"",K255&lt;&gt;"",OR(L255="PASS",L255="FAIL"),M255&lt;&gt;"",O255&lt;&gt;"",P255="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A255="","",IF(AND(AK255="OK",J255="READY",F255&lt;&gt;"",G255&lt;&gt;"",K255&lt;&gt;"",OR(L255="PASS",L255="FAIL"),M255&lt;&gt;"",P255="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM255" s="9" t="str">
         <x:f>IF(A255="","",IF(AND(AK255="OK",J255="READY",F255&lt;&gt;"",G255&lt;&gt;"",K255&lt;&gt;"",S255="OK",OR(R255="PASS",R255="FAIL")),"YES","NO"))</x:f>
@@ -14241,7 +14241,7 @@
         <x:f>IF(A256="",IF(B256="","","MISSING_TEST_ID"),IF(B256="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A256,$B$2:$B$501,B256)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL256" s="9" t="str">
-        <x:f>IF(A256="","",IF(AND(AK256="OK",J256="READY",F256&lt;&gt;"",G256&lt;&gt;"",K256&lt;&gt;"",OR(L256="PASS",L256="FAIL"),M256&lt;&gt;"",O256&lt;&gt;"",P256="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A256="","",IF(AND(AK256="OK",J256="READY",F256&lt;&gt;"",G256&lt;&gt;"",K256&lt;&gt;"",OR(L256="PASS",L256="FAIL"),M256&lt;&gt;"",P256="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM256" s="9" t="str">
         <x:f>IF(A256="","",IF(AND(AK256="OK",J256="READY",F256&lt;&gt;"",G256&lt;&gt;"",K256&lt;&gt;"",S256="OK",OR(R256="PASS",R256="FAIL")),"YES","NO"))</x:f>
@@ -14293,7 +14293,7 @@
         <x:f>IF(A257="",IF(B257="","","MISSING_TEST_ID"),IF(B257="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A257,$B$2:$B$501,B257)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL257" s="9" t="str">
-        <x:f>IF(A257="","",IF(AND(AK257="OK",J257="READY",F257&lt;&gt;"",G257&lt;&gt;"",K257&lt;&gt;"",OR(L257="PASS",L257="FAIL"),M257&lt;&gt;"",O257&lt;&gt;"",P257="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A257="","",IF(AND(AK257="OK",J257="READY",F257&lt;&gt;"",G257&lt;&gt;"",K257&lt;&gt;"",OR(L257="PASS",L257="FAIL"),M257&lt;&gt;"",P257="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM257" s="9" t="str">
         <x:f>IF(A257="","",IF(AND(AK257="OK",J257="READY",F257&lt;&gt;"",G257&lt;&gt;"",K257&lt;&gt;"",S257="OK",OR(R257="PASS",R257="FAIL")),"YES","NO"))</x:f>
@@ -14345,7 +14345,7 @@
         <x:f>IF(A258="",IF(B258="","","MISSING_TEST_ID"),IF(B258="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A258,$B$2:$B$501,B258)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL258" s="9" t="str">
-        <x:f>IF(A258="","",IF(AND(AK258="OK",J258="READY",F258&lt;&gt;"",G258&lt;&gt;"",K258&lt;&gt;"",OR(L258="PASS",L258="FAIL"),M258&lt;&gt;"",O258&lt;&gt;"",P258="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A258="","",IF(AND(AK258="OK",J258="READY",F258&lt;&gt;"",G258&lt;&gt;"",K258&lt;&gt;"",OR(L258="PASS",L258="FAIL"),M258&lt;&gt;"",P258="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM258" s="9" t="str">
         <x:f>IF(A258="","",IF(AND(AK258="OK",J258="READY",F258&lt;&gt;"",G258&lt;&gt;"",K258&lt;&gt;"",S258="OK",OR(R258="PASS",R258="FAIL")),"YES","NO"))</x:f>
@@ -14397,7 +14397,7 @@
         <x:f>IF(A259="",IF(B259="","","MISSING_TEST_ID"),IF(B259="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A259,$B$2:$B$501,B259)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL259" s="9" t="str">
-        <x:f>IF(A259="","",IF(AND(AK259="OK",J259="READY",F259&lt;&gt;"",G259&lt;&gt;"",K259&lt;&gt;"",OR(L259="PASS",L259="FAIL"),M259&lt;&gt;"",O259&lt;&gt;"",P259="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A259="","",IF(AND(AK259="OK",J259="READY",F259&lt;&gt;"",G259&lt;&gt;"",K259&lt;&gt;"",OR(L259="PASS",L259="FAIL"),M259&lt;&gt;"",P259="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM259" s="9" t="str">
         <x:f>IF(A259="","",IF(AND(AK259="OK",J259="READY",F259&lt;&gt;"",G259&lt;&gt;"",K259&lt;&gt;"",S259="OK",OR(R259="PASS",R259="FAIL")),"YES","NO"))</x:f>
@@ -14449,7 +14449,7 @@
         <x:f>IF(A260="",IF(B260="","","MISSING_TEST_ID"),IF(B260="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A260,$B$2:$B$501,B260)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL260" s="9" t="str">
-        <x:f>IF(A260="","",IF(AND(AK260="OK",J260="READY",F260&lt;&gt;"",G260&lt;&gt;"",K260&lt;&gt;"",OR(L260="PASS",L260="FAIL"),M260&lt;&gt;"",O260&lt;&gt;"",P260="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A260="","",IF(AND(AK260="OK",J260="READY",F260&lt;&gt;"",G260&lt;&gt;"",K260&lt;&gt;"",OR(L260="PASS",L260="FAIL"),M260&lt;&gt;"",P260="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM260" s="9" t="str">
         <x:f>IF(A260="","",IF(AND(AK260="OK",J260="READY",F260&lt;&gt;"",G260&lt;&gt;"",K260&lt;&gt;"",S260="OK",OR(R260="PASS",R260="FAIL")),"YES","NO"))</x:f>
@@ -14501,7 +14501,7 @@
         <x:f>IF(A261="",IF(B261="","","MISSING_TEST_ID"),IF(B261="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A261,$B$2:$B$501,B261)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL261" s="9" t="str">
-        <x:f>IF(A261="","",IF(AND(AK261="OK",J261="READY",F261&lt;&gt;"",G261&lt;&gt;"",K261&lt;&gt;"",OR(L261="PASS",L261="FAIL"),M261&lt;&gt;"",O261&lt;&gt;"",P261="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A261="","",IF(AND(AK261="OK",J261="READY",F261&lt;&gt;"",G261&lt;&gt;"",K261&lt;&gt;"",OR(L261="PASS",L261="FAIL"),M261&lt;&gt;"",P261="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM261" s="9" t="str">
         <x:f>IF(A261="","",IF(AND(AK261="OK",J261="READY",F261&lt;&gt;"",G261&lt;&gt;"",K261&lt;&gt;"",S261="OK",OR(R261="PASS",R261="FAIL")),"YES","NO"))</x:f>
@@ -14553,7 +14553,7 @@
         <x:f>IF(A262="",IF(B262="","","MISSING_TEST_ID"),IF(B262="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A262,$B$2:$B$501,B262)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL262" s="9" t="str">
-        <x:f>IF(A262="","",IF(AND(AK262="OK",J262="READY",F262&lt;&gt;"",G262&lt;&gt;"",K262&lt;&gt;"",OR(L262="PASS",L262="FAIL"),M262&lt;&gt;"",O262&lt;&gt;"",P262="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A262="","",IF(AND(AK262="OK",J262="READY",F262&lt;&gt;"",G262&lt;&gt;"",K262&lt;&gt;"",OR(L262="PASS",L262="FAIL"),M262&lt;&gt;"",P262="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM262" s="9" t="str">
         <x:f>IF(A262="","",IF(AND(AK262="OK",J262="READY",F262&lt;&gt;"",G262&lt;&gt;"",K262&lt;&gt;"",S262="OK",OR(R262="PASS",R262="FAIL")),"YES","NO"))</x:f>
@@ -14605,7 +14605,7 @@
         <x:f>IF(A263="",IF(B263="","","MISSING_TEST_ID"),IF(B263="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A263,$B$2:$B$501,B263)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL263" s="9" t="str">
-        <x:f>IF(A263="","",IF(AND(AK263="OK",J263="READY",F263&lt;&gt;"",G263&lt;&gt;"",K263&lt;&gt;"",OR(L263="PASS",L263="FAIL"),M263&lt;&gt;"",O263&lt;&gt;"",P263="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A263="","",IF(AND(AK263="OK",J263="READY",F263&lt;&gt;"",G263&lt;&gt;"",K263&lt;&gt;"",OR(L263="PASS",L263="FAIL"),M263&lt;&gt;"",P263="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM263" s="9" t="str">
         <x:f>IF(A263="","",IF(AND(AK263="OK",J263="READY",F263&lt;&gt;"",G263&lt;&gt;"",K263&lt;&gt;"",S263="OK",OR(R263="PASS",R263="FAIL")),"YES","NO"))</x:f>
@@ -14657,7 +14657,7 @@
         <x:f>IF(A264="",IF(B264="","","MISSING_TEST_ID"),IF(B264="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A264,$B$2:$B$501,B264)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL264" s="9" t="str">
-        <x:f>IF(A264="","",IF(AND(AK264="OK",J264="READY",F264&lt;&gt;"",G264&lt;&gt;"",K264&lt;&gt;"",OR(L264="PASS",L264="FAIL"),M264&lt;&gt;"",O264&lt;&gt;"",P264="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A264="","",IF(AND(AK264="OK",J264="READY",F264&lt;&gt;"",G264&lt;&gt;"",K264&lt;&gt;"",OR(L264="PASS",L264="FAIL"),M264&lt;&gt;"",P264="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM264" s="9" t="str">
         <x:f>IF(A264="","",IF(AND(AK264="OK",J264="READY",F264&lt;&gt;"",G264&lt;&gt;"",K264&lt;&gt;"",S264="OK",OR(R264="PASS",R264="FAIL")),"YES","NO"))</x:f>
@@ -14709,7 +14709,7 @@
         <x:f>IF(A265="",IF(B265="","","MISSING_TEST_ID"),IF(B265="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A265,$B$2:$B$501,B265)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL265" s="9" t="str">
-        <x:f>IF(A265="","",IF(AND(AK265="OK",J265="READY",F265&lt;&gt;"",G265&lt;&gt;"",K265&lt;&gt;"",OR(L265="PASS",L265="FAIL"),M265&lt;&gt;"",O265&lt;&gt;"",P265="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A265="","",IF(AND(AK265="OK",J265="READY",F265&lt;&gt;"",G265&lt;&gt;"",K265&lt;&gt;"",OR(L265="PASS",L265="FAIL"),M265&lt;&gt;"",P265="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM265" s="9" t="str">
         <x:f>IF(A265="","",IF(AND(AK265="OK",J265="READY",F265&lt;&gt;"",G265&lt;&gt;"",K265&lt;&gt;"",S265="OK",OR(R265="PASS",R265="FAIL")),"YES","NO"))</x:f>
@@ -14761,7 +14761,7 @@
         <x:f>IF(A266="",IF(B266="","","MISSING_TEST_ID"),IF(B266="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A266,$B$2:$B$501,B266)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL266" s="9" t="str">
-        <x:f>IF(A266="","",IF(AND(AK266="OK",J266="READY",F266&lt;&gt;"",G266&lt;&gt;"",K266&lt;&gt;"",OR(L266="PASS",L266="FAIL"),M266&lt;&gt;"",O266&lt;&gt;"",P266="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A266="","",IF(AND(AK266="OK",J266="READY",F266&lt;&gt;"",G266&lt;&gt;"",K266&lt;&gt;"",OR(L266="PASS",L266="FAIL"),M266&lt;&gt;"",P266="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM266" s="9" t="str">
         <x:f>IF(A266="","",IF(AND(AK266="OK",J266="READY",F266&lt;&gt;"",G266&lt;&gt;"",K266&lt;&gt;"",S266="OK",OR(R266="PASS",R266="FAIL")),"YES","NO"))</x:f>
@@ -14813,7 +14813,7 @@
         <x:f>IF(A267="",IF(B267="","","MISSING_TEST_ID"),IF(B267="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A267,$B$2:$B$501,B267)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL267" s="9" t="str">
-        <x:f>IF(A267="","",IF(AND(AK267="OK",J267="READY",F267&lt;&gt;"",G267&lt;&gt;"",K267&lt;&gt;"",OR(L267="PASS",L267="FAIL"),M267&lt;&gt;"",O267&lt;&gt;"",P267="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A267="","",IF(AND(AK267="OK",J267="READY",F267&lt;&gt;"",G267&lt;&gt;"",K267&lt;&gt;"",OR(L267="PASS",L267="FAIL"),M267&lt;&gt;"",P267="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM267" s="9" t="str">
         <x:f>IF(A267="","",IF(AND(AK267="OK",J267="READY",F267&lt;&gt;"",G267&lt;&gt;"",K267&lt;&gt;"",S267="OK",OR(R267="PASS",R267="FAIL")),"YES","NO"))</x:f>
@@ -14865,7 +14865,7 @@
         <x:f>IF(A268="",IF(B268="","","MISSING_TEST_ID"),IF(B268="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A268,$B$2:$B$501,B268)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL268" s="9" t="str">
-        <x:f>IF(A268="","",IF(AND(AK268="OK",J268="READY",F268&lt;&gt;"",G268&lt;&gt;"",K268&lt;&gt;"",OR(L268="PASS",L268="FAIL"),M268&lt;&gt;"",O268&lt;&gt;"",P268="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A268="","",IF(AND(AK268="OK",J268="READY",F268&lt;&gt;"",G268&lt;&gt;"",K268&lt;&gt;"",OR(L268="PASS",L268="FAIL"),M268&lt;&gt;"",P268="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM268" s="9" t="str">
         <x:f>IF(A268="","",IF(AND(AK268="OK",J268="READY",F268&lt;&gt;"",G268&lt;&gt;"",K268&lt;&gt;"",S268="OK",OR(R268="PASS",R268="FAIL")),"YES","NO"))</x:f>
@@ -14917,7 +14917,7 @@
         <x:f>IF(A269="",IF(B269="","","MISSING_TEST_ID"),IF(B269="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A269,$B$2:$B$501,B269)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL269" s="9" t="str">
-        <x:f>IF(A269="","",IF(AND(AK269="OK",J269="READY",F269&lt;&gt;"",G269&lt;&gt;"",K269&lt;&gt;"",OR(L269="PASS",L269="FAIL"),M269&lt;&gt;"",O269&lt;&gt;"",P269="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A269="","",IF(AND(AK269="OK",J269="READY",F269&lt;&gt;"",G269&lt;&gt;"",K269&lt;&gt;"",OR(L269="PASS",L269="FAIL"),M269&lt;&gt;"",P269="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM269" s="9" t="str">
         <x:f>IF(A269="","",IF(AND(AK269="OK",J269="READY",F269&lt;&gt;"",G269&lt;&gt;"",K269&lt;&gt;"",S269="OK",OR(R269="PASS",R269="FAIL")),"YES","NO"))</x:f>
@@ -14969,7 +14969,7 @@
         <x:f>IF(A270="",IF(B270="","","MISSING_TEST_ID"),IF(B270="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A270,$B$2:$B$501,B270)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL270" s="9" t="str">
-        <x:f>IF(A270="","",IF(AND(AK270="OK",J270="READY",F270&lt;&gt;"",G270&lt;&gt;"",K270&lt;&gt;"",OR(L270="PASS",L270="FAIL"),M270&lt;&gt;"",O270&lt;&gt;"",P270="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A270="","",IF(AND(AK270="OK",J270="READY",F270&lt;&gt;"",G270&lt;&gt;"",K270&lt;&gt;"",OR(L270="PASS",L270="FAIL"),M270&lt;&gt;"",P270="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM270" s="9" t="str">
         <x:f>IF(A270="","",IF(AND(AK270="OK",J270="READY",F270&lt;&gt;"",G270&lt;&gt;"",K270&lt;&gt;"",S270="OK",OR(R270="PASS",R270="FAIL")),"YES","NO"))</x:f>
@@ -15021,7 +15021,7 @@
         <x:f>IF(A271="",IF(B271="","","MISSING_TEST_ID"),IF(B271="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A271,$B$2:$B$501,B271)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL271" s="9" t="str">
-        <x:f>IF(A271="","",IF(AND(AK271="OK",J271="READY",F271&lt;&gt;"",G271&lt;&gt;"",K271&lt;&gt;"",OR(L271="PASS",L271="FAIL"),M271&lt;&gt;"",O271&lt;&gt;"",P271="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A271="","",IF(AND(AK271="OK",J271="READY",F271&lt;&gt;"",G271&lt;&gt;"",K271&lt;&gt;"",OR(L271="PASS",L271="FAIL"),M271&lt;&gt;"",P271="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM271" s="9" t="str">
         <x:f>IF(A271="","",IF(AND(AK271="OK",J271="READY",F271&lt;&gt;"",G271&lt;&gt;"",K271&lt;&gt;"",S271="OK",OR(R271="PASS",R271="FAIL")),"YES","NO"))</x:f>
@@ -15073,7 +15073,7 @@
         <x:f>IF(A272="",IF(B272="","","MISSING_TEST_ID"),IF(B272="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A272,$B$2:$B$501,B272)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL272" s="9" t="str">
-        <x:f>IF(A272="","",IF(AND(AK272="OK",J272="READY",F272&lt;&gt;"",G272&lt;&gt;"",K272&lt;&gt;"",OR(L272="PASS",L272="FAIL"),M272&lt;&gt;"",O272&lt;&gt;"",P272="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A272="","",IF(AND(AK272="OK",J272="READY",F272&lt;&gt;"",G272&lt;&gt;"",K272&lt;&gt;"",OR(L272="PASS",L272="FAIL"),M272&lt;&gt;"",P272="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM272" s="9" t="str">
         <x:f>IF(A272="","",IF(AND(AK272="OK",J272="READY",F272&lt;&gt;"",G272&lt;&gt;"",K272&lt;&gt;"",S272="OK",OR(R272="PASS",R272="FAIL")),"YES","NO"))</x:f>
@@ -15125,7 +15125,7 @@
         <x:f>IF(A273="",IF(B273="","","MISSING_TEST_ID"),IF(B273="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A273,$B$2:$B$501,B273)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL273" s="9" t="str">
-        <x:f>IF(A273="","",IF(AND(AK273="OK",J273="READY",F273&lt;&gt;"",G273&lt;&gt;"",K273&lt;&gt;"",OR(L273="PASS",L273="FAIL"),M273&lt;&gt;"",O273&lt;&gt;"",P273="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A273="","",IF(AND(AK273="OK",J273="READY",F273&lt;&gt;"",G273&lt;&gt;"",K273&lt;&gt;"",OR(L273="PASS",L273="FAIL"),M273&lt;&gt;"",P273="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM273" s="9" t="str">
         <x:f>IF(A273="","",IF(AND(AK273="OK",J273="READY",F273&lt;&gt;"",G273&lt;&gt;"",K273&lt;&gt;"",S273="OK",OR(R273="PASS",R273="FAIL")),"YES","NO"))</x:f>
@@ -15177,7 +15177,7 @@
         <x:f>IF(A274="",IF(B274="","","MISSING_TEST_ID"),IF(B274="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A274,$B$2:$B$501,B274)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL274" s="9" t="str">
-        <x:f>IF(A274="","",IF(AND(AK274="OK",J274="READY",F274&lt;&gt;"",G274&lt;&gt;"",K274&lt;&gt;"",OR(L274="PASS",L274="FAIL"),M274&lt;&gt;"",O274&lt;&gt;"",P274="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A274="","",IF(AND(AK274="OK",J274="READY",F274&lt;&gt;"",G274&lt;&gt;"",K274&lt;&gt;"",OR(L274="PASS",L274="FAIL"),M274&lt;&gt;"",P274="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM274" s="9" t="str">
         <x:f>IF(A274="","",IF(AND(AK274="OK",J274="READY",F274&lt;&gt;"",G274&lt;&gt;"",K274&lt;&gt;"",S274="OK",OR(R274="PASS",R274="FAIL")),"YES","NO"))</x:f>
@@ -15229,7 +15229,7 @@
         <x:f>IF(A275="",IF(B275="","","MISSING_TEST_ID"),IF(B275="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A275,$B$2:$B$501,B275)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL275" s="9" t="str">
-        <x:f>IF(A275="","",IF(AND(AK275="OK",J275="READY",F275&lt;&gt;"",G275&lt;&gt;"",K275&lt;&gt;"",OR(L275="PASS",L275="FAIL"),M275&lt;&gt;"",O275&lt;&gt;"",P275="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A275="","",IF(AND(AK275="OK",J275="READY",F275&lt;&gt;"",G275&lt;&gt;"",K275&lt;&gt;"",OR(L275="PASS",L275="FAIL"),M275&lt;&gt;"",P275="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM275" s="9" t="str">
         <x:f>IF(A275="","",IF(AND(AK275="OK",J275="READY",F275&lt;&gt;"",G275&lt;&gt;"",K275&lt;&gt;"",S275="OK",OR(R275="PASS",R275="FAIL")),"YES","NO"))</x:f>
@@ -15281,7 +15281,7 @@
         <x:f>IF(A276="",IF(B276="","","MISSING_TEST_ID"),IF(B276="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A276,$B$2:$B$501,B276)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL276" s="9" t="str">
-        <x:f>IF(A276="","",IF(AND(AK276="OK",J276="READY",F276&lt;&gt;"",G276&lt;&gt;"",K276&lt;&gt;"",OR(L276="PASS",L276="FAIL"),M276&lt;&gt;"",O276&lt;&gt;"",P276="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A276="","",IF(AND(AK276="OK",J276="READY",F276&lt;&gt;"",G276&lt;&gt;"",K276&lt;&gt;"",OR(L276="PASS",L276="FAIL"),M276&lt;&gt;"",P276="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM276" s="9" t="str">
         <x:f>IF(A276="","",IF(AND(AK276="OK",J276="READY",F276&lt;&gt;"",G276&lt;&gt;"",K276&lt;&gt;"",S276="OK",OR(R276="PASS",R276="FAIL")),"YES","NO"))</x:f>
@@ -15333,7 +15333,7 @@
         <x:f>IF(A277="",IF(B277="","","MISSING_TEST_ID"),IF(B277="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A277,$B$2:$B$501,B277)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL277" s="9" t="str">
-        <x:f>IF(A277="","",IF(AND(AK277="OK",J277="READY",F277&lt;&gt;"",G277&lt;&gt;"",K277&lt;&gt;"",OR(L277="PASS",L277="FAIL"),M277&lt;&gt;"",O277&lt;&gt;"",P277="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A277="","",IF(AND(AK277="OK",J277="READY",F277&lt;&gt;"",G277&lt;&gt;"",K277&lt;&gt;"",OR(L277="PASS",L277="FAIL"),M277&lt;&gt;"",P277="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM277" s="9" t="str">
         <x:f>IF(A277="","",IF(AND(AK277="OK",J277="READY",F277&lt;&gt;"",G277&lt;&gt;"",K277&lt;&gt;"",S277="OK",OR(R277="PASS",R277="FAIL")),"YES","NO"))</x:f>
@@ -15385,7 +15385,7 @@
         <x:f>IF(A278="",IF(B278="","","MISSING_TEST_ID"),IF(B278="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A278,$B$2:$B$501,B278)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL278" s="9" t="str">
-        <x:f>IF(A278="","",IF(AND(AK278="OK",J278="READY",F278&lt;&gt;"",G278&lt;&gt;"",K278&lt;&gt;"",OR(L278="PASS",L278="FAIL"),M278&lt;&gt;"",O278&lt;&gt;"",P278="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A278="","",IF(AND(AK278="OK",J278="READY",F278&lt;&gt;"",G278&lt;&gt;"",K278&lt;&gt;"",OR(L278="PASS",L278="FAIL"),M278&lt;&gt;"",P278="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM278" s="9" t="str">
         <x:f>IF(A278="","",IF(AND(AK278="OK",J278="READY",F278&lt;&gt;"",G278&lt;&gt;"",K278&lt;&gt;"",S278="OK",OR(R278="PASS",R278="FAIL")),"YES","NO"))</x:f>
@@ -15437,7 +15437,7 @@
         <x:f>IF(A279="",IF(B279="","","MISSING_TEST_ID"),IF(B279="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A279,$B$2:$B$501,B279)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL279" s="9" t="str">
-        <x:f>IF(A279="","",IF(AND(AK279="OK",J279="READY",F279&lt;&gt;"",G279&lt;&gt;"",K279&lt;&gt;"",OR(L279="PASS",L279="FAIL"),M279&lt;&gt;"",O279&lt;&gt;"",P279="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A279="","",IF(AND(AK279="OK",J279="READY",F279&lt;&gt;"",G279&lt;&gt;"",K279&lt;&gt;"",OR(L279="PASS",L279="FAIL"),M279&lt;&gt;"",P279="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM279" s="9" t="str">
         <x:f>IF(A279="","",IF(AND(AK279="OK",J279="READY",F279&lt;&gt;"",G279&lt;&gt;"",K279&lt;&gt;"",S279="OK",OR(R279="PASS",R279="FAIL")),"YES","NO"))</x:f>
@@ -15489,7 +15489,7 @@
         <x:f>IF(A280="",IF(B280="","","MISSING_TEST_ID"),IF(B280="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A280,$B$2:$B$501,B280)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL280" s="9" t="str">
-        <x:f>IF(A280="","",IF(AND(AK280="OK",J280="READY",F280&lt;&gt;"",G280&lt;&gt;"",K280&lt;&gt;"",OR(L280="PASS",L280="FAIL"),M280&lt;&gt;"",O280&lt;&gt;"",P280="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A280="","",IF(AND(AK280="OK",J280="READY",F280&lt;&gt;"",G280&lt;&gt;"",K280&lt;&gt;"",OR(L280="PASS",L280="FAIL"),M280&lt;&gt;"",P280="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM280" s="9" t="str">
         <x:f>IF(A280="","",IF(AND(AK280="OK",J280="READY",F280&lt;&gt;"",G280&lt;&gt;"",K280&lt;&gt;"",S280="OK",OR(R280="PASS",R280="FAIL")),"YES","NO"))</x:f>
@@ -15541,7 +15541,7 @@
         <x:f>IF(A281="",IF(B281="","","MISSING_TEST_ID"),IF(B281="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A281,$B$2:$B$501,B281)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL281" s="9" t="str">
-        <x:f>IF(A281="","",IF(AND(AK281="OK",J281="READY",F281&lt;&gt;"",G281&lt;&gt;"",K281&lt;&gt;"",OR(L281="PASS",L281="FAIL"),M281&lt;&gt;"",O281&lt;&gt;"",P281="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A281="","",IF(AND(AK281="OK",J281="READY",F281&lt;&gt;"",G281&lt;&gt;"",K281&lt;&gt;"",OR(L281="PASS",L281="FAIL"),M281&lt;&gt;"",P281="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM281" s="9" t="str">
         <x:f>IF(A281="","",IF(AND(AK281="OK",J281="READY",F281&lt;&gt;"",G281&lt;&gt;"",K281&lt;&gt;"",S281="OK",OR(R281="PASS",R281="FAIL")),"YES","NO"))</x:f>
@@ -15593,7 +15593,7 @@
         <x:f>IF(A282="",IF(B282="","","MISSING_TEST_ID"),IF(B282="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A282,$B$2:$B$501,B282)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL282" s="9" t="str">
-        <x:f>IF(A282="","",IF(AND(AK282="OK",J282="READY",F282&lt;&gt;"",G282&lt;&gt;"",K282&lt;&gt;"",OR(L282="PASS",L282="FAIL"),M282&lt;&gt;"",O282&lt;&gt;"",P282="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A282="","",IF(AND(AK282="OK",J282="READY",F282&lt;&gt;"",G282&lt;&gt;"",K282&lt;&gt;"",OR(L282="PASS",L282="FAIL"),M282&lt;&gt;"",P282="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM282" s="9" t="str">
         <x:f>IF(A282="","",IF(AND(AK282="OK",J282="READY",F282&lt;&gt;"",G282&lt;&gt;"",K282&lt;&gt;"",S282="OK",OR(R282="PASS",R282="FAIL")),"YES","NO"))</x:f>
@@ -15645,7 +15645,7 @@
         <x:f>IF(A283="",IF(B283="","","MISSING_TEST_ID"),IF(B283="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A283,$B$2:$B$501,B283)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL283" s="9" t="str">
-        <x:f>IF(A283="","",IF(AND(AK283="OK",J283="READY",F283&lt;&gt;"",G283&lt;&gt;"",K283&lt;&gt;"",OR(L283="PASS",L283="FAIL"),M283&lt;&gt;"",O283&lt;&gt;"",P283="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A283="","",IF(AND(AK283="OK",J283="READY",F283&lt;&gt;"",G283&lt;&gt;"",K283&lt;&gt;"",OR(L283="PASS",L283="FAIL"),M283&lt;&gt;"",P283="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM283" s="9" t="str">
         <x:f>IF(A283="","",IF(AND(AK283="OK",J283="READY",F283&lt;&gt;"",G283&lt;&gt;"",K283&lt;&gt;"",S283="OK",OR(R283="PASS",R283="FAIL")),"YES","NO"))</x:f>
@@ -15697,7 +15697,7 @@
         <x:f>IF(A284="",IF(B284="","","MISSING_TEST_ID"),IF(B284="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A284,$B$2:$B$501,B284)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL284" s="9" t="str">
-        <x:f>IF(A284="","",IF(AND(AK284="OK",J284="READY",F284&lt;&gt;"",G284&lt;&gt;"",K284&lt;&gt;"",OR(L284="PASS",L284="FAIL"),M284&lt;&gt;"",O284&lt;&gt;"",P284="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A284="","",IF(AND(AK284="OK",J284="READY",F284&lt;&gt;"",G284&lt;&gt;"",K284&lt;&gt;"",OR(L284="PASS",L284="FAIL"),M284&lt;&gt;"",P284="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM284" s="9" t="str">
         <x:f>IF(A284="","",IF(AND(AK284="OK",J284="READY",F284&lt;&gt;"",G284&lt;&gt;"",K284&lt;&gt;"",S284="OK",OR(R284="PASS",R284="FAIL")),"YES","NO"))</x:f>
@@ -15749,7 +15749,7 @@
         <x:f>IF(A285="",IF(B285="","","MISSING_TEST_ID"),IF(B285="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A285,$B$2:$B$501,B285)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL285" s="9" t="str">
-        <x:f>IF(A285="","",IF(AND(AK285="OK",J285="READY",F285&lt;&gt;"",G285&lt;&gt;"",K285&lt;&gt;"",OR(L285="PASS",L285="FAIL"),M285&lt;&gt;"",O285&lt;&gt;"",P285="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A285="","",IF(AND(AK285="OK",J285="READY",F285&lt;&gt;"",G285&lt;&gt;"",K285&lt;&gt;"",OR(L285="PASS",L285="FAIL"),M285&lt;&gt;"",P285="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM285" s="9" t="str">
         <x:f>IF(A285="","",IF(AND(AK285="OK",J285="READY",F285&lt;&gt;"",G285&lt;&gt;"",K285&lt;&gt;"",S285="OK",OR(R285="PASS",R285="FAIL")),"YES","NO"))</x:f>
@@ -15801,7 +15801,7 @@
         <x:f>IF(A286="",IF(B286="","","MISSING_TEST_ID"),IF(B286="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A286,$B$2:$B$501,B286)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL286" s="9" t="str">
-        <x:f>IF(A286="","",IF(AND(AK286="OK",J286="READY",F286&lt;&gt;"",G286&lt;&gt;"",K286&lt;&gt;"",OR(L286="PASS",L286="FAIL"),M286&lt;&gt;"",O286&lt;&gt;"",P286="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A286="","",IF(AND(AK286="OK",J286="READY",F286&lt;&gt;"",G286&lt;&gt;"",K286&lt;&gt;"",OR(L286="PASS",L286="FAIL"),M286&lt;&gt;"",P286="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM286" s="9" t="str">
         <x:f>IF(A286="","",IF(AND(AK286="OK",J286="READY",F286&lt;&gt;"",G286&lt;&gt;"",K286&lt;&gt;"",S286="OK",OR(R286="PASS",R286="FAIL")),"YES","NO"))</x:f>
@@ -15853,7 +15853,7 @@
         <x:f>IF(A287="",IF(B287="","","MISSING_TEST_ID"),IF(B287="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A287,$B$2:$B$501,B287)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL287" s="9" t="str">
-        <x:f>IF(A287="","",IF(AND(AK287="OK",J287="READY",F287&lt;&gt;"",G287&lt;&gt;"",K287&lt;&gt;"",OR(L287="PASS",L287="FAIL"),M287&lt;&gt;"",O287&lt;&gt;"",P287="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A287="","",IF(AND(AK287="OK",J287="READY",F287&lt;&gt;"",G287&lt;&gt;"",K287&lt;&gt;"",OR(L287="PASS",L287="FAIL"),M287&lt;&gt;"",P287="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM287" s="9" t="str">
         <x:f>IF(A287="","",IF(AND(AK287="OK",J287="READY",F287&lt;&gt;"",G287&lt;&gt;"",K287&lt;&gt;"",S287="OK",OR(R287="PASS",R287="FAIL")),"YES","NO"))</x:f>
@@ -15905,7 +15905,7 @@
         <x:f>IF(A288="",IF(B288="","","MISSING_TEST_ID"),IF(B288="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A288,$B$2:$B$501,B288)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL288" s="9" t="str">
-        <x:f>IF(A288="","",IF(AND(AK288="OK",J288="READY",F288&lt;&gt;"",G288&lt;&gt;"",K288&lt;&gt;"",OR(L288="PASS",L288="FAIL"),M288&lt;&gt;"",O288&lt;&gt;"",P288="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A288="","",IF(AND(AK288="OK",J288="READY",F288&lt;&gt;"",G288&lt;&gt;"",K288&lt;&gt;"",OR(L288="PASS",L288="FAIL"),M288&lt;&gt;"",P288="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM288" s="9" t="str">
         <x:f>IF(A288="","",IF(AND(AK288="OK",J288="READY",F288&lt;&gt;"",G288&lt;&gt;"",K288&lt;&gt;"",S288="OK",OR(R288="PASS",R288="FAIL")),"YES","NO"))</x:f>
@@ -15957,7 +15957,7 @@
         <x:f>IF(A289="",IF(B289="","","MISSING_TEST_ID"),IF(B289="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A289,$B$2:$B$501,B289)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL289" s="9" t="str">
-        <x:f>IF(A289="","",IF(AND(AK289="OK",J289="READY",F289&lt;&gt;"",G289&lt;&gt;"",K289&lt;&gt;"",OR(L289="PASS",L289="FAIL"),M289&lt;&gt;"",O289&lt;&gt;"",P289="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A289="","",IF(AND(AK289="OK",J289="READY",F289&lt;&gt;"",G289&lt;&gt;"",K289&lt;&gt;"",OR(L289="PASS",L289="FAIL"),M289&lt;&gt;"",P289="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM289" s="9" t="str">
         <x:f>IF(A289="","",IF(AND(AK289="OK",J289="READY",F289&lt;&gt;"",G289&lt;&gt;"",K289&lt;&gt;"",S289="OK",OR(R289="PASS",R289="FAIL")),"YES","NO"))</x:f>
@@ -16009,7 +16009,7 @@
         <x:f>IF(A290="",IF(B290="","","MISSING_TEST_ID"),IF(B290="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A290,$B$2:$B$501,B290)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL290" s="9" t="str">
-        <x:f>IF(A290="","",IF(AND(AK290="OK",J290="READY",F290&lt;&gt;"",G290&lt;&gt;"",K290&lt;&gt;"",OR(L290="PASS",L290="FAIL"),M290&lt;&gt;"",O290&lt;&gt;"",P290="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A290="","",IF(AND(AK290="OK",J290="READY",F290&lt;&gt;"",G290&lt;&gt;"",K290&lt;&gt;"",OR(L290="PASS",L290="FAIL"),M290&lt;&gt;"",P290="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM290" s="9" t="str">
         <x:f>IF(A290="","",IF(AND(AK290="OK",J290="READY",F290&lt;&gt;"",G290&lt;&gt;"",K290&lt;&gt;"",S290="OK",OR(R290="PASS",R290="FAIL")),"YES","NO"))</x:f>
@@ -16061,7 +16061,7 @@
         <x:f>IF(A291="",IF(B291="","","MISSING_TEST_ID"),IF(B291="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A291,$B$2:$B$501,B291)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL291" s="9" t="str">
-        <x:f>IF(A291="","",IF(AND(AK291="OK",J291="READY",F291&lt;&gt;"",G291&lt;&gt;"",K291&lt;&gt;"",OR(L291="PASS",L291="FAIL"),M291&lt;&gt;"",O291&lt;&gt;"",P291="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A291="","",IF(AND(AK291="OK",J291="READY",F291&lt;&gt;"",G291&lt;&gt;"",K291&lt;&gt;"",OR(L291="PASS",L291="FAIL"),M291&lt;&gt;"",P291="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM291" s="9" t="str">
         <x:f>IF(A291="","",IF(AND(AK291="OK",J291="READY",F291&lt;&gt;"",G291&lt;&gt;"",K291&lt;&gt;"",S291="OK",OR(R291="PASS",R291="FAIL")),"YES","NO"))</x:f>
@@ -16113,7 +16113,7 @@
         <x:f>IF(A292="",IF(B292="","","MISSING_TEST_ID"),IF(B292="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A292,$B$2:$B$501,B292)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL292" s="9" t="str">
-        <x:f>IF(A292="","",IF(AND(AK292="OK",J292="READY",F292&lt;&gt;"",G292&lt;&gt;"",K292&lt;&gt;"",OR(L292="PASS",L292="FAIL"),M292&lt;&gt;"",O292&lt;&gt;"",P292="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A292="","",IF(AND(AK292="OK",J292="READY",F292&lt;&gt;"",G292&lt;&gt;"",K292&lt;&gt;"",OR(L292="PASS",L292="FAIL"),M292&lt;&gt;"",P292="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM292" s="9" t="str">
         <x:f>IF(A292="","",IF(AND(AK292="OK",J292="READY",F292&lt;&gt;"",G292&lt;&gt;"",K292&lt;&gt;"",S292="OK",OR(R292="PASS",R292="FAIL")),"YES","NO"))</x:f>
@@ -16165,7 +16165,7 @@
         <x:f>IF(A293="",IF(B293="","","MISSING_TEST_ID"),IF(B293="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A293,$B$2:$B$501,B293)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL293" s="9" t="str">
-        <x:f>IF(A293="","",IF(AND(AK293="OK",J293="READY",F293&lt;&gt;"",G293&lt;&gt;"",K293&lt;&gt;"",OR(L293="PASS",L293="FAIL"),M293&lt;&gt;"",O293&lt;&gt;"",P293="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A293="","",IF(AND(AK293="OK",J293="READY",F293&lt;&gt;"",G293&lt;&gt;"",K293&lt;&gt;"",OR(L293="PASS",L293="FAIL"),M293&lt;&gt;"",P293="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM293" s="9" t="str">
         <x:f>IF(A293="","",IF(AND(AK293="OK",J293="READY",F293&lt;&gt;"",G293&lt;&gt;"",K293&lt;&gt;"",S293="OK",OR(R293="PASS",R293="FAIL")),"YES","NO"))</x:f>
@@ -16217,7 +16217,7 @@
         <x:f>IF(A294="",IF(B294="","","MISSING_TEST_ID"),IF(B294="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A294,$B$2:$B$501,B294)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL294" s="9" t="str">
-        <x:f>IF(A294="","",IF(AND(AK294="OK",J294="READY",F294&lt;&gt;"",G294&lt;&gt;"",K294&lt;&gt;"",OR(L294="PASS",L294="FAIL"),M294&lt;&gt;"",O294&lt;&gt;"",P294="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A294="","",IF(AND(AK294="OK",J294="READY",F294&lt;&gt;"",G294&lt;&gt;"",K294&lt;&gt;"",OR(L294="PASS",L294="FAIL"),M294&lt;&gt;"",P294="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM294" s="9" t="str">
         <x:f>IF(A294="","",IF(AND(AK294="OK",J294="READY",F294&lt;&gt;"",G294&lt;&gt;"",K294&lt;&gt;"",S294="OK",OR(R294="PASS",R294="FAIL")),"YES","NO"))</x:f>
@@ -16269,7 +16269,7 @@
         <x:f>IF(A295="",IF(B295="","","MISSING_TEST_ID"),IF(B295="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A295,$B$2:$B$501,B295)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL295" s="9" t="str">
-        <x:f>IF(A295="","",IF(AND(AK295="OK",J295="READY",F295&lt;&gt;"",G295&lt;&gt;"",K295&lt;&gt;"",OR(L295="PASS",L295="FAIL"),M295&lt;&gt;"",O295&lt;&gt;"",P295="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A295="","",IF(AND(AK295="OK",J295="READY",F295&lt;&gt;"",G295&lt;&gt;"",K295&lt;&gt;"",OR(L295="PASS",L295="FAIL"),M295&lt;&gt;"",P295="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM295" s="9" t="str">
         <x:f>IF(A295="","",IF(AND(AK295="OK",J295="READY",F295&lt;&gt;"",G295&lt;&gt;"",K295&lt;&gt;"",S295="OK",OR(R295="PASS",R295="FAIL")),"YES","NO"))</x:f>
@@ -16321,7 +16321,7 @@
         <x:f>IF(A296="",IF(B296="","","MISSING_TEST_ID"),IF(B296="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A296,$B$2:$B$501,B296)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL296" s="9" t="str">
-        <x:f>IF(A296="","",IF(AND(AK296="OK",J296="READY",F296&lt;&gt;"",G296&lt;&gt;"",K296&lt;&gt;"",OR(L296="PASS",L296="FAIL"),M296&lt;&gt;"",O296&lt;&gt;"",P296="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A296="","",IF(AND(AK296="OK",J296="READY",F296&lt;&gt;"",G296&lt;&gt;"",K296&lt;&gt;"",OR(L296="PASS",L296="FAIL"),M296&lt;&gt;"",P296="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM296" s="9" t="str">
         <x:f>IF(A296="","",IF(AND(AK296="OK",J296="READY",F296&lt;&gt;"",G296&lt;&gt;"",K296&lt;&gt;"",S296="OK",OR(R296="PASS",R296="FAIL")),"YES","NO"))</x:f>
@@ -16373,7 +16373,7 @@
         <x:f>IF(A297="",IF(B297="","","MISSING_TEST_ID"),IF(B297="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A297,$B$2:$B$501,B297)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL297" s="9" t="str">
-        <x:f>IF(A297="","",IF(AND(AK297="OK",J297="READY",F297&lt;&gt;"",G297&lt;&gt;"",K297&lt;&gt;"",OR(L297="PASS",L297="FAIL"),M297&lt;&gt;"",O297&lt;&gt;"",P297="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A297="","",IF(AND(AK297="OK",J297="READY",F297&lt;&gt;"",G297&lt;&gt;"",K297&lt;&gt;"",OR(L297="PASS",L297="FAIL"),M297&lt;&gt;"",P297="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM297" s="9" t="str">
         <x:f>IF(A297="","",IF(AND(AK297="OK",J297="READY",F297&lt;&gt;"",G297&lt;&gt;"",K297&lt;&gt;"",S297="OK",OR(R297="PASS",R297="FAIL")),"YES","NO"))</x:f>
@@ -16425,7 +16425,7 @@
         <x:f>IF(A298="",IF(B298="","","MISSING_TEST_ID"),IF(B298="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A298,$B$2:$B$501,B298)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL298" s="9" t="str">
-        <x:f>IF(A298="","",IF(AND(AK298="OK",J298="READY",F298&lt;&gt;"",G298&lt;&gt;"",K298&lt;&gt;"",OR(L298="PASS",L298="FAIL"),M298&lt;&gt;"",O298&lt;&gt;"",P298="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A298="","",IF(AND(AK298="OK",J298="READY",F298&lt;&gt;"",G298&lt;&gt;"",K298&lt;&gt;"",OR(L298="PASS",L298="FAIL"),M298&lt;&gt;"",P298="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM298" s="9" t="str">
         <x:f>IF(A298="","",IF(AND(AK298="OK",J298="READY",F298&lt;&gt;"",G298&lt;&gt;"",K298&lt;&gt;"",S298="OK",OR(R298="PASS",R298="FAIL")),"YES","NO"))</x:f>
@@ -16477,7 +16477,7 @@
         <x:f>IF(A299="",IF(B299="","","MISSING_TEST_ID"),IF(B299="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A299,$B$2:$B$501,B299)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL299" s="9" t="str">
-        <x:f>IF(A299="","",IF(AND(AK299="OK",J299="READY",F299&lt;&gt;"",G299&lt;&gt;"",K299&lt;&gt;"",OR(L299="PASS",L299="FAIL"),M299&lt;&gt;"",O299&lt;&gt;"",P299="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A299="","",IF(AND(AK299="OK",J299="READY",F299&lt;&gt;"",G299&lt;&gt;"",K299&lt;&gt;"",OR(L299="PASS",L299="FAIL"),M299&lt;&gt;"",P299="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM299" s="9" t="str">
         <x:f>IF(A299="","",IF(AND(AK299="OK",J299="READY",F299&lt;&gt;"",G299&lt;&gt;"",K299&lt;&gt;"",S299="OK",OR(R299="PASS",R299="FAIL")),"YES","NO"))</x:f>
@@ -16529,7 +16529,7 @@
         <x:f>IF(A300="",IF(B300="","","MISSING_TEST_ID"),IF(B300="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A300,$B$2:$B$501,B300)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL300" s="9" t="str">
-        <x:f>IF(A300="","",IF(AND(AK300="OK",J300="READY",F300&lt;&gt;"",G300&lt;&gt;"",K300&lt;&gt;"",OR(L300="PASS",L300="FAIL"),M300&lt;&gt;"",O300&lt;&gt;"",P300="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A300="","",IF(AND(AK300="OK",J300="READY",F300&lt;&gt;"",G300&lt;&gt;"",K300&lt;&gt;"",OR(L300="PASS",L300="FAIL"),M300&lt;&gt;"",P300="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM300" s="9" t="str">
         <x:f>IF(A300="","",IF(AND(AK300="OK",J300="READY",F300&lt;&gt;"",G300&lt;&gt;"",K300&lt;&gt;"",S300="OK",OR(R300="PASS",R300="FAIL")),"YES","NO"))</x:f>
@@ -16581,7 +16581,7 @@
         <x:f>IF(A301="",IF(B301="","","MISSING_TEST_ID"),IF(B301="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A301,$B$2:$B$501,B301)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL301" s="9" t="str">
-        <x:f>IF(A301="","",IF(AND(AK301="OK",J301="READY",F301&lt;&gt;"",G301&lt;&gt;"",K301&lt;&gt;"",OR(L301="PASS",L301="FAIL"),M301&lt;&gt;"",O301&lt;&gt;"",P301="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A301="","",IF(AND(AK301="OK",J301="READY",F301&lt;&gt;"",G301&lt;&gt;"",K301&lt;&gt;"",OR(L301="PASS",L301="FAIL"),M301&lt;&gt;"",P301="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM301" s="9" t="str">
         <x:f>IF(A301="","",IF(AND(AK301="OK",J301="READY",F301&lt;&gt;"",G301&lt;&gt;"",K301&lt;&gt;"",S301="OK",OR(R301="PASS",R301="FAIL")),"YES","NO"))</x:f>
@@ -16633,7 +16633,7 @@
         <x:f>IF(A302="",IF(B302="","","MISSING_TEST_ID"),IF(B302="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A302,$B$2:$B$501,B302)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL302" s="9" t="str">
-        <x:f>IF(A302="","",IF(AND(AK302="OK",J302="READY",F302&lt;&gt;"",G302&lt;&gt;"",K302&lt;&gt;"",OR(L302="PASS",L302="FAIL"),M302&lt;&gt;"",O302&lt;&gt;"",P302="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A302="","",IF(AND(AK302="OK",J302="READY",F302&lt;&gt;"",G302&lt;&gt;"",K302&lt;&gt;"",OR(L302="PASS",L302="FAIL"),M302&lt;&gt;"",P302="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM302" s="9" t="str">
         <x:f>IF(A302="","",IF(AND(AK302="OK",J302="READY",F302&lt;&gt;"",G302&lt;&gt;"",K302&lt;&gt;"",S302="OK",OR(R302="PASS",R302="FAIL")),"YES","NO"))</x:f>
@@ -16685,7 +16685,7 @@
         <x:f>IF(A303="",IF(B303="","","MISSING_TEST_ID"),IF(B303="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A303,$B$2:$B$501,B303)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL303" s="9" t="str">
-        <x:f>IF(A303="","",IF(AND(AK303="OK",J303="READY",F303&lt;&gt;"",G303&lt;&gt;"",K303&lt;&gt;"",OR(L303="PASS",L303="FAIL"),M303&lt;&gt;"",O303&lt;&gt;"",P303="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A303="","",IF(AND(AK303="OK",J303="READY",F303&lt;&gt;"",G303&lt;&gt;"",K303&lt;&gt;"",OR(L303="PASS",L303="FAIL"),M303&lt;&gt;"",P303="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM303" s="9" t="str">
         <x:f>IF(A303="","",IF(AND(AK303="OK",J303="READY",F303&lt;&gt;"",G303&lt;&gt;"",K303&lt;&gt;"",S303="OK",OR(R303="PASS",R303="FAIL")),"YES","NO"))</x:f>
@@ -16737,7 +16737,7 @@
         <x:f>IF(A304="",IF(B304="","","MISSING_TEST_ID"),IF(B304="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A304,$B$2:$B$501,B304)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL304" s="9" t="str">
-        <x:f>IF(A304="","",IF(AND(AK304="OK",J304="READY",F304&lt;&gt;"",G304&lt;&gt;"",K304&lt;&gt;"",OR(L304="PASS",L304="FAIL"),M304&lt;&gt;"",O304&lt;&gt;"",P304="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A304="","",IF(AND(AK304="OK",J304="READY",F304&lt;&gt;"",G304&lt;&gt;"",K304&lt;&gt;"",OR(L304="PASS",L304="FAIL"),M304&lt;&gt;"",P304="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM304" s="9" t="str">
         <x:f>IF(A304="","",IF(AND(AK304="OK",J304="READY",F304&lt;&gt;"",G304&lt;&gt;"",K304&lt;&gt;"",S304="OK",OR(R304="PASS",R304="FAIL")),"YES","NO"))</x:f>
@@ -16789,7 +16789,7 @@
         <x:f>IF(A305="",IF(B305="","","MISSING_TEST_ID"),IF(B305="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A305,$B$2:$B$501,B305)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL305" s="9" t="str">
-        <x:f>IF(A305="","",IF(AND(AK305="OK",J305="READY",F305&lt;&gt;"",G305&lt;&gt;"",K305&lt;&gt;"",OR(L305="PASS",L305="FAIL"),M305&lt;&gt;"",O305&lt;&gt;"",P305="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A305="","",IF(AND(AK305="OK",J305="READY",F305&lt;&gt;"",G305&lt;&gt;"",K305&lt;&gt;"",OR(L305="PASS",L305="FAIL"),M305&lt;&gt;"",P305="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM305" s="9" t="str">
         <x:f>IF(A305="","",IF(AND(AK305="OK",J305="READY",F305&lt;&gt;"",G305&lt;&gt;"",K305&lt;&gt;"",S305="OK",OR(R305="PASS",R305="FAIL")),"YES","NO"))</x:f>
@@ -16841,7 +16841,7 @@
         <x:f>IF(A306="",IF(B306="","","MISSING_TEST_ID"),IF(B306="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A306,$B$2:$B$501,B306)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL306" s="9" t="str">
-        <x:f>IF(A306="","",IF(AND(AK306="OK",J306="READY",F306&lt;&gt;"",G306&lt;&gt;"",K306&lt;&gt;"",OR(L306="PASS",L306="FAIL"),M306&lt;&gt;"",O306&lt;&gt;"",P306="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A306="","",IF(AND(AK306="OK",J306="READY",F306&lt;&gt;"",G306&lt;&gt;"",K306&lt;&gt;"",OR(L306="PASS",L306="FAIL"),M306&lt;&gt;"",P306="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM306" s="9" t="str">
         <x:f>IF(A306="","",IF(AND(AK306="OK",J306="READY",F306&lt;&gt;"",G306&lt;&gt;"",K306&lt;&gt;"",S306="OK",OR(R306="PASS",R306="FAIL")),"YES","NO"))</x:f>
@@ -16893,7 +16893,7 @@
         <x:f>IF(A307="",IF(B307="","","MISSING_TEST_ID"),IF(B307="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A307,$B$2:$B$501,B307)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL307" s="9" t="str">
-        <x:f>IF(A307="","",IF(AND(AK307="OK",J307="READY",F307&lt;&gt;"",G307&lt;&gt;"",K307&lt;&gt;"",OR(L307="PASS",L307="FAIL"),M307&lt;&gt;"",O307&lt;&gt;"",P307="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A307="","",IF(AND(AK307="OK",J307="READY",F307&lt;&gt;"",G307&lt;&gt;"",K307&lt;&gt;"",OR(L307="PASS",L307="FAIL"),M307&lt;&gt;"",P307="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM307" s="9" t="str">
         <x:f>IF(A307="","",IF(AND(AK307="OK",J307="READY",F307&lt;&gt;"",G307&lt;&gt;"",K307&lt;&gt;"",S307="OK",OR(R307="PASS",R307="FAIL")),"YES","NO"))</x:f>
@@ -16945,7 +16945,7 @@
         <x:f>IF(A308="",IF(B308="","","MISSING_TEST_ID"),IF(B308="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A308,$B$2:$B$501,B308)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL308" s="9" t="str">
-        <x:f>IF(A308="","",IF(AND(AK308="OK",J308="READY",F308&lt;&gt;"",G308&lt;&gt;"",K308&lt;&gt;"",OR(L308="PASS",L308="FAIL"),M308&lt;&gt;"",O308&lt;&gt;"",P308="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A308="","",IF(AND(AK308="OK",J308="READY",F308&lt;&gt;"",G308&lt;&gt;"",K308&lt;&gt;"",OR(L308="PASS",L308="FAIL"),M308&lt;&gt;"",P308="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM308" s="9" t="str">
         <x:f>IF(A308="","",IF(AND(AK308="OK",J308="READY",F308&lt;&gt;"",G308&lt;&gt;"",K308&lt;&gt;"",S308="OK",OR(R308="PASS",R308="FAIL")),"YES","NO"))</x:f>
@@ -16997,7 +16997,7 @@
         <x:f>IF(A309="",IF(B309="","","MISSING_TEST_ID"),IF(B309="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A309,$B$2:$B$501,B309)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL309" s="9" t="str">
-        <x:f>IF(A309="","",IF(AND(AK309="OK",J309="READY",F309&lt;&gt;"",G309&lt;&gt;"",K309&lt;&gt;"",OR(L309="PASS",L309="FAIL"),M309&lt;&gt;"",O309&lt;&gt;"",P309="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A309="","",IF(AND(AK309="OK",J309="READY",F309&lt;&gt;"",G309&lt;&gt;"",K309&lt;&gt;"",OR(L309="PASS",L309="FAIL"),M309&lt;&gt;"",P309="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM309" s="9" t="str">
         <x:f>IF(A309="","",IF(AND(AK309="OK",J309="READY",F309&lt;&gt;"",G309&lt;&gt;"",K309&lt;&gt;"",S309="OK",OR(R309="PASS",R309="FAIL")),"YES","NO"))</x:f>
@@ -17049,7 +17049,7 @@
         <x:f>IF(A310="",IF(B310="","","MISSING_TEST_ID"),IF(B310="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A310,$B$2:$B$501,B310)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL310" s="9" t="str">
-        <x:f>IF(A310="","",IF(AND(AK310="OK",J310="READY",F310&lt;&gt;"",G310&lt;&gt;"",K310&lt;&gt;"",OR(L310="PASS",L310="FAIL"),M310&lt;&gt;"",O310&lt;&gt;"",P310="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A310="","",IF(AND(AK310="OK",J310="READY",F310&lt;&gt;"",G310&lt;&gt;"",K310&lt;&gt;"",OR(L310="PASS",L310="FAIL"),M310&lt;&gt;"",P310="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM310" s="9" t="str">
         <x:f>IF(A310="","",IF(AND(AK310="OK",J310="READY",F310&lt;&gt;"",G310&lt;&gt;"",K310&lt;&gt;"",S310="OK",OR(R310="PASS",R310="FAIL")),"YES","NO"))</x:f>
@@ -17101,7 +17101,7 @@
         <x:f>IF(A311="",IF(B311="","","MISSING_TEST_ID"),IF(B311="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A311,$B$2:$B$501,B311)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL311" s="9" t="str">
-        <x:f>IF(A311="","",IF(AND(AK311="OK",J311="READY",F311&lt;&gt;"",G311&lt;&gt;"",K311&lt;&gt;"",OR(L311="PASS",L311="FAIL"),M311&lt;&gt;"",O311&lt;&gt;"",P311="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A311="","",IF(AND(AK311="OK",J311="READY",F311&lt;&gt;"",G311&lt;&gt;"",K311&lt;&gt;"",OR(L311="PASS",L311="FAIL"),M311&lt;&gt;"",P311="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM311" s="9" t="str">
         <x:f>IF(A311="","",IF(AND(AK311="OK",J311="READY",F311&lt;&gt;"",G311&lt;&gt;"",K311&lt;&gt;"",S311="OK",OR(R311="PASS",R311="FAIL")),"YES","NO"))</x:f>
@@ -17153,7 +17153,7 @@
         <x:f>IF(A312="",IF(B312="","","MISSING_TEST_ID"),IF(B312="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A312,$B$2:$B$501,B312)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL312" s="9" t="str">
-        <x:f>IF(A312="","",IF(AND(AK312="OK",J312="READY",F312&lt;&gt;"",G312&lt;&gt;"",K312&lt;&gt;"",OR(L312="PASS",L312="FAIL"),M312&lt;&gt;"",O312&lt;&gt;"",P312="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A312="","",IF(AND(AK312="OK",J312="READY",F312&lt;&gt;"",G312&lt;&gt;"",K312&lt;&gt;"",OR(L312="PASS",L312="FAIL"),M312&lt;&gt;"",P312="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM312" s="9" t="str">
         <x:f>IF(A312="","",IF(AND(AK312="OK",J312="READY",F312&lt;&gt;"",G312&lt;&gt;"",K312&lt;&gt;"",S312="OK",OR(R312="PASS",R312="FAIL")),"YES","NO"))</x:f>
@@ -17205,7 +17205,7 @@
         <x:f>IF(A313="",IF(B313="","","MISSING_TEST_ID"),IF(B313="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A313,$B$2:$B$501,B313)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL313" s="9" t="str">
-        <x:f>IF(A313="","",IF(AND(AK313="OK",J313="READY",F313&lt;&gt;"",G313&lt;&gt;"",K313&lt;&gt;"",OR(L313="PASS",L313="FAIL"),M313&lt;&gt;"",O313&lt;&gt;"",P313="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A313="","",IF(AND(AK313="OK",J313="READY",F313&lt;&gt;"",G313&lt;&gt;"",K313&lt;&gt;"",OR(L313="PASS",L313="FAIL"),M313&lt;&gt;"",P313="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM313" s="9" t="str">
         <x:f>IF(A313="","",IF(AND(AK313="OK",J313="READY",F313&lt;&gt;"",G313&lt;&gt;"",K313&lt;&gt;"",S313="OK",OR(R313="PASS",R313="FAIL")),"YES","NO"))</x:f>
@@ -17257,7 +17257,7 @@
         <x:f>IF(A314="",IF(B314="","","MISSING_TEST_ID"),IF(B314="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A314,$B$2:$B$501,B314)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL314" s="9" t="str">
-        <x:f>IF(A314="","",IF(AND(AK314="OK",J314="READY",F314&lt;&gt;"",G314&lt;&gt;"",K314&lt;&gt;"",OR(L314="PASS",L314="FAIL"),M314&lt;&gt;"",O314&lt;&gt;"",P314="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A314="","",IF(AND(AK314="OK",J314="READY",F314&lt;&gt;"",G314&lt;&gt;"",K314&lt;&gt;"",OR(L314="PASS",L314="FAIL"),M314&lt;&gt;"",P314="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM314" s="9" t="str">
         <x:f>IF(A314="","",IF(AND(AK314="OK",J314="READY",F314&lt;&gt;"",G314&lt;&gt;"",K314&lt;&gt;"",S314="OK",OR(R314="PASS",R314="FAIL")),"YES","NO"))</x:f>
@@ -17309,7 +17309,7 @@
         <x:f>IF(A315="",IF(B315="","","MISSING_TEST_ID"),IF(B315="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A315,$B$2:$B$501,B315)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL315" s="9" t="str">
-        <x:f>IF(A315="","",IF(AND(AK315="OK",J315="READY",F315&lt;&gt;"",G315&lt;&gt;"",K315&lt;&gt;"",OR(L315="PASS",L315="FAIL"),M315&lt;&gt;"",O315&lt;&gt;"",P315="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A315="","",IF(AND(AK315="OK",J315="READY",F315&lt;&gt;"",G315&lt;&gt;"",K315&lt;&gt;"",OR(L315="PASS",L315="FAIL"),M315&lt;&gt;"",P315="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM315" s="9" t="str">
         <x:f>IF(A315="","",IF(AND(AK315="OK",J315="READY",F315&lt;&gt;"",G315&lt;&gt;"",K315&lt;&gt;"",S315="OK",OR(R315="PASS",R315="FAIL")),"YES","NO"))</x:f>
@@ -17361,7 +17361,7 @@
         <x:f>IF(A316="",IF(B316="","","MISSING_TEST_ID"),IF(B316="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A316,$B$2:$B$501,B316)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL316" s="9" t="str">
-        <x:f>IF(A316="","",IF(AND(AK316="OK",J316="READY",F316&lt;&gt;"",G316&lt;&gt;"",K316&lt;&gt;"",OR(L316="PASS",L316="FAIL"),M316&lt;&gt;"",O316&lt;&gt;"",P316="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A316="","",IF(AND(AK316="OK",J316="READY",F316&lt;&gt;"",G316&lt;&gt;"",K316&lt;&gt;"",OR(L316="PASS",L316="FAIL"),M316&lt;&gt;"",P316="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM316" s="9" t="str">
         <x:f>IF(A316="","",IF(AND(AK316="OK",J316="READY",F316&lt;&gt;"",G316&lt;&gt;"",K316&lt;&gt;"",S316="OK",OR(R316="PASS",R316="FAIL")),"YES","NO"))</x:f>
@@ -17413,7 +17413,7 @@
         <x:f>IF(A317="",IF(B317="","","MISSING_TEST_ID"),IF(B317="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A317,$B$2:$B$501,B317)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL317" s="9" t="str">
-        <x:f>IF(A317="","",IF(AND(AK317="OK",J317="READY",F317&lt;&gt;"",G317&lt;&gt;"",K317&lt;&gt;"",OR(L317="PASS",L317="FAIL"),M317&lt;&gt;"",O317&lt;&gt;"",P317="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A317="","",IF(AND(AK317="OK",J317="READY",F317&lt;&gt;"",G317&lt;&gt;"",K317&lt;&gt;"",OR(L317="PASS",L317="FAIL"),M317&lt;&gt;"",P317="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM317" s="9" t="str">
         <x:f>IF(A317="","",IF(AND(AK317="OK",J317="READY",F317&lt;&gt;"",G317&lt;&gt;"",K317&lt;&gt;"",S317="OK",OR(R317="PASS",R317="FAIL")),"YES","NO"))</x:f>
@@ -17465,7 +17465,7 @@
         <x:f>IF(A318="",IF(B318="","","MISSING_TEST_ID"),IF(B318="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A318,$B$2:$B$501,B318)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL318" s="9" t="str">
-        <x:f>IF(A318="","",IF(AND(AK318="OK",J318="READY",F318&lt;&gt;"",G318&lt;&gt;"",K318&lt;&gt;"",OR(L318="PASS",L318="FAIL"),M318&lt;&gt;"",O318&lt;&gt;"",P318="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A318="","",IF(AND(AK318="OK",J318="READY",F318&lt;&gt;"",G318&lt;&gt;"",K318&lt;&gt;"",OR(L318="PASS",L318="FAIL"),M318&lt;&gt;"",P318="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM318" s="9" t="str">
         <x:f>IF(A318="","",IF(AND(AK318="OK",J318="READY",F318&lt;&gt;"",G318&lt;&gt;"",K318&lt;&gt;"",S318="OK",OR(R318="PASS",R318="FAIL")),"YES","NO"))</x:f>
@@ -17517,7 +17517,7 @@
         <x:f>IF(A319="",IF(B319="","","MISSING_TEST_ID"),IF(B319="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A319,$B$2:$B$501,B319)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL319" s="9" t="str">
-        <x:f>IF(A319="","",IF(AND(AK319="OK",J319="READY",F319&lt;&gt;"",G319&lt;&gt;"",K319&lt;&gt;"",OR(L319="PASS",L319="FAIL"),M319&lt;&gt;"",O319&lt;&gt;"",P319="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A319="","",IF(AND(AK319="OK",J319="READY",F319&lt;&gt;"",G319&lt;&gt;"",K319&lt;&gt;"",OR(L319="PASS",L319="FAIL"),M319&lt;&gt;"",P319="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM319" s="9" t="str">
         <x:f>IF(A319="","",IF(AND(AK319="OK",J319="READY",F319&lt;&gt;"",G319&lt;&gt;"",K319&lt;&gt;"",S319="OK",OR(R319="PASS",R319="FAIL")),"YES","NO"))</x:f>
@@ -17569,7 +17569,7 @@
         <x:f>IF(A320="",IF(B320="","","MISSING_TEST_ID"),IF(B320="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A320,$B$2:$B$501,B320)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL320" s="9" t="str">
-        <x:f>IF(A320="","",IF(AND(AK320="OK",J320="READY",F320&lt;&gt;"",G320&lt;&gt;"",K320&lt;&gt;"",OR(L320="PASS",L320="FAIL"),M320&lt;&gt;"",O320&lt;&gt;"",P320="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A320="","",IF(AND(AK320="OK",J320="READY",F320&lt;&gt;"",G320&lt;&gt;"",K320&lt;&gt;"",OR(L320="PASS",L320="FAIL"),M320&lt;&gt;"",P320="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM320" s="9" t="str">
         <x:f>IF(A320="","",IF(AND(AK320="OK",J320="READY",F320&lt;&gt;"",G320&lt;&gt;"",K320&lt;&gt;"",S320="OK",OR(R320="PASS",R320="FAIL")),"YES","NO"))</x:f>
@@ -17621,7 +17621,7 @@
         <x:f>IF(A321="",IF(B321="","","MISSING_TEST_ID"),IF(B321="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A321,$B$2:$B$501,B321)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL321" s="9" t="str">
-        <x:f>IF(A321="","",IF(AND(AK321="OK",J321="READY",F321&lt;&gt;"",G321&lt;&gt;"",K321&lt;&gt;"",OR(L321="PASS",L321="FAIL"),M321&lt;&gt;"",O321&lt;&gt;"",P321="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A321="","",IF(AND(AK321="OK",J321="READY",F321&lt;&gt;"",G321&lt;&gt;"",K321&lt;&gt;"",OR(L321="PASS",L321="FAIL"),M321&lt;&gt;"",P321="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM321" s="9" t="str">
         <x:f>IF(A321="","",IF(AND(AK321="OK",J321="READY",F321&lt;&gt;"",G321&lt;&gt;"",K321&lt;&gt;"",S321="OK",OR(R321="PASS",R321="FAIL")),"YES","NO"))</x:f>
@@ -17673,7 +17673,7 @@
         <x:f>IF(A322="",IF(B322="","","MISSING_TEST_ID"),IF(B322="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A322,$B$2:$B$501,B322)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL322" s="9" t="str">
-        <x:f>IF(A322="","",IF(AND(AK322="OK",J322="READY",F322&lt;&gt;"",G322&lt;&gt;"",K322&lt;&gt;"",OR(L322="PASS",L322="FAIL"),M322&lt;&gt;"",O322&lt;&gt;"",P322="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A322="","",IF(AND(AK322="OK",J322="READY",F322&lt;&gt;"",G322&lt;&gt;"",K322&lt;&gt;"",OR(L322="PASS",L322="FAIL"),M322&lt;&gt;"",P322="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM322" s="9" t="str">
         <x:f>IF(A322="","",IF(AND(AK322="OK",J322="READY",F322&lt;&gt;"",G322&lt;&gt;"",K322&lt;&gt;"",S322="OK",OR(R322="PASS",R322="FAIL")),"YES","NO"))</x:f>
@@ -17725,7 +17725,7 @@
         <x:f>IF(A323="",IF(B323="","","MISSING_TEST_ID"),IF(B323="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A323,$B$2:$B$501,B323)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL323" s="9" t="str">
-        <x:f>IF(A323="","",IF(AND(AK323="OK",J323="READY",F323&lt;&gt;"",G323&lt;&gt;"",K323&lt;&gt;"",OR(L323="PASS",L323="FAIL"),M323&lt;&gt;"",O323&lt;&gt;"",P323="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A323="","",IF(AND(AK323="OK",J323="READY",F323&lt;&gt;"",G323&lt;&gt;"",K323&lt;&gt;"",OR(L323="PASS",L323="FAIL"),M323&lt;&gt;"",P323="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM323" s="9" t="str">
         <x:f>IF(A323="","",IF(AND(AK323="OK",J323="READY",F323&lt;&gt;"",G323&lt;&gt;"",K323&lt;&gt;"",S323="OK",OR(R323="PASS",R323="FAIL")),"YES","NO"))</x:f>
@@ -17777,7 +17777,7 @@
         <x:f>IF(A324="",IF(B324="","","MISSING_TEST_ID"),IF(B324="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A324,$B$2:$B$501,B324)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL324" s="9" t="str">
-        <x:f>IF(A324="","",IF(AND(AK324="OK",J324="READY",F324&lt;&gt;"",G324&lt;&gt;"",K324&lt;&gt;"",OR(L324="PASS",L324="FAIL"),M324&lt;&gt;"",O324&lt;&gt;"",P324="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A324="","",IF(AND(AK324="OK",J324="READY",F324&lt;&gt;"",G324&lt;&gt;"",K324&lt;&gt;"",OR(L324="PASS",L324="FAIL"),M324&lt;&gt;"",P324="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM324" s="9" t="str">
         <x:f>IF(A324="","",IF(AND(AK324="OK",J324="READY",F324&lt;&gt;"",G324&lt;&gt;"",K324&lt;&gt;"",S324="OK",OR(R324="PASS",R324="FAIL")),"YES","NO"))</x:f>
@@ -17829,7 +17829,7 @@
         <x:f>IF(A325="",IF(B325="","","MISSING_TEST_ID"),IF(B325="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A325,$B$2:$B$501,B325)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL325" s="9" t="str">
-        <x:f>IF(A325="","",IF(AND(AK325="OK",J325="READY",F325&lt;&gt;"",G325&lt;&gt;"",K325&lt;&gt;"",OR(L325="PASS",L325="FAIL"),M325&lt;&gt;"",O325&lt;&gt;"",P325="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A325="","",IF(AND(AK325="OK",J325="READY",F325&lt;&gt;"",G325&lt;&gt;"",K325&lt;&gt;"",OR(L325="PASS",L325="FAIL"),M325&lt;&gt;"",P325="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM325" s="9" t="str">
         <x:f>IF(A325="","",IF(AND(AK325="OK",J325="READY",F325&lt;&gt;"",G325&lt;&gt;"",K325&lt;&gt;"",S325="OK",OR(R325="PASS",R325="FAIL")),"YES","NO"))</x:f>
@@ -17881,7 +17881,7 @@
         <x:f>IF(A326="",IF(B326="","","MISSING_TEST_ID"),IF(B326="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A326,$B$2:$B$501,B326)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL326" s="9" t="str">
-        <x:f>IF(A326="","",IF(AND(AK326="OK",J326="READY",F326&lt;&gt;"",G326&lt;&gt;"",K326&lt;&gt;"",OR(L326="PASS",L326="FAIL"),M326&lt;&gt;"",O326&lt;&gt;"",P326="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A326="","",IF(AND(AK326="OK",J326="READY",F326&lt;&gt;"",G326&lt;&gt;"",K326&lt;&gt;"",OR(L326="PASS",L326="FAIL"),M326&lt;&gt;"",P326="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM326" s="9" t="str">
         <x:f>IF(A326="","",IF(AND(AK326="OK",J326="READY",F326&lt;&gt;"",G326&lt;&gt;"",K326&lt;&gt;"",S326="OK",OR(R326="PASS",R326="FAIL")),"YES","NO"))</x:f>
@@ -17933,7 +17933,7 @@
         <x:f>IF(A327="",IF(B327="","","MISSING_TEST_ID"),IF(B327="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A327,$B$2:$B$501,B327)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL327" s="9" t="str">
-        <x:f>IF(A327="","",IF(AND(AK327="OK",J327="READY",F327&lt;&gt;"",G327&lt;&gt;"",K327&lt;&gt;"",OR(L327="PASS",L327="FAIL"),M327&lt;&gt;"",O327&lt;&gt;"",P327="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A327="","",IF(AND(AK327="OK",J327="READY",F327&lt;&gt;"",G327&lt;&gt;"",K327&lt;&gt;"",OR(L327="PASS",L327="FAIL"),M327&lt;&gt;"",P327="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM327" s="9" t="str">
         <x:f>IF(A327="","",IF(AND(AK327="OK",J327="READY",F327&lt;&gt;"",G327&lt;&gt;"",K327&lt;&gt;"",S327="OK",OR(R327="PASS",R327="FAIL")),"YES","NO"))</x:f>
@@ -17985,7 +17985,7 @@
         <x:f>IF(A328="",IF(B328="","","MISSING_TEST_ID"),IF(B328="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A328,$B$2:$B$501,B328)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL328" s="9" t="str">
-        <x:f>IF(A328="","",IF(AND(AK328="OK",J328="READY",F328&lt;&gt;"",G328&lt;&gt;"",K328&lt;&gt;"",OR(L328="PASS",L328="FAIL"),M328&lt;&gt;"",O328&lt;&gt;"",P328="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A328="","",IF(AND(AK328="OK",J328="READY",F328&lt;&gt;"",G328&lt;&gt;"",K328&lt;&gt;"",OR(L328="PASS",L328="FAIL"),M328&lt;&gt;"",P328="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM328" s="9" t="str">
         <x:f>IF(A328="","",IF(AND(AK328="OK",J328="READY",F328&lt;&gt;"",G328&lt;&gt;"",K328&lt;&gt;"",S328="OK",OR(R328="PASS",R328="FAIL")),"YES","NO"))</x:f>
@@ -18037,7 +18037,7 @@
         <x:f>IF(A329="",IF(B329="","","MISSING_TEST_ID"),IF(B329="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A329,$B$2:$B$501,B329)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL329" s="9" t="str">
-        <x:f>IF(A329="","",IF(AND(AK329="OK",J329="READY",F329&lt;&gt;"",G329&lt;&gt;"",K329&lt;&gt;"",OR(L329="PASS",L329="FAIL"),M329&lt;&gt;"",O329&lt;&gt;"",P329="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A329="","",IF(AND(AK329="OK",J329="READY",F329&lt;&gt;"",G329&lt;&gt;"",K329&lt;&gt;"",OR(L329="PASS",L329="FAIL"),M329&lt;&gt;"",P329="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM329" s="9" t="str">
         <x:f>IF(A329="","",IF(AND(AK329="OK",J329="READY",F329&lt;&gt;"",G329&lt;&gt;"",K329&lt;&gt;"",S329="OK",OR(R329="PASS",R329="FAIL")),"YES","NO"))</x:f>
@@ -18089,7 +18089,7 @@
         <x:f>IF(A330="",IF(B330="","","MISSING_TEST_ID"),IF(B330="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A330,$B$2:$B$501,B330)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL330" s="9" t="str">
-        <x:f>IF(A330="","",IF(AND(AK330="OK",J330="READY",F330&lt;&gt;"",G330&lt;&gt;"",K330&lt;&gt;"",OR(L330="PASS",L330="FAIL"),M330&lt;&gt;"",O330&lt;&gt;"",P330="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A330="","",IF(AND(AK330="OK",J330="READY",F330&lt;&gt;"",G330&lt;&gt;"",K330&lt;&gt;"",OR(L330="PASS",L330="FAIL"),M330&lt;&gt;"",P330="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM330" s="9" t="str">
         <x:f>IF(A330="","",IF(AND(AK330="OK",J330="READY",F330&lt;&gt;"",G330&lt;&gt;"",K330&lt;&gt;"",S330="OK",OR(R330="PASS",R330="FAIL")),"YES","NO"))</x:f>
@@ -18141,7 +18141,7 @@
         <x:f>IF(A331="",IF(B331="","","MISSING_TEST_ID"),IF(B331="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A331,$B$2:$B$501,B331)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL331" s="9" t="str">
-        <x:f>IF(A331="","",IF(AND(AK331="OK",J331="READY",F331&lt;&gt;"",G331&lt;&gt;"",K331&lt;&gt;"",OR(L331="PASS",L331="FAIL"),M331&lt;&gt;"",O331&lt;&gt;"",P331="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A331="","",IF(AND(AK331="OK",J331="READY",F331&lt;&gt;"",G331&lt;&gt;"",K331&lt;&gt;"",OR(L331="PASS",L331="FAIL"),M331&lt;&gt;"",P331="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM331" s="9" t="str">
         <x:f>IF(A331="","",IF(AND(AK331="OK",J331="READY",F331&lt;&gt;"",G331&lt;&gt;"",K331&lt;&gt;"",S331="OK",OR(R331="PASS",R331="FAIL")),"YES","NO"))</x:f>
@@ -18193,7 +18193,7 @@
         <x:f>IF(A332="",IF(B332="","","MISSING_TEST_ID"),IF(B332="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A332,$B$2:$B$501,B332)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL332" s="9" t="str">
-        <x:f>IF(A332="","",IF(AND(AK332="OK",J332="READY",F332&lt;&gt;"",G332&lt;&gt;"",K332&lt;&gt;"",OR(L332="PASS",L332="FAIL"),M332&lt;&gt;"",O332&lt;&gt;"",P332="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A332="","",IF(AND(AK332="OK",J332="READY",F332&lt;&gt;"",G332&lt;&gt;"",K332&lt;&gt;"",OR(L332="PASS",L332="FAIL"),M332&lt;&gt;"",P332="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM332" s="9" t="str">
         <x:f>IF(A332="","",IF(AND(AK332="OK",J332="READY",F332&lt;&gt;"",G332&lt;&gt;"",K332&lt;&gt;"",S332="OK",OR(R332="PASS",R332="FAIL")),"YES","NO"))</x:f>
@@ -18245,7 +18245,7 @@
         <x:f>IF(A333="",IF(B333="","","MISSING_TEST_ID"),IF(B333="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A333,$B$2:$B$501,B333)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL333" s="9" t="str">
-        <x:f>IF(A333="","",IF(AND(AK333="OK",J333="READY",F333&lt;&gt;"",G333&lt;&gt;"",K333&lt;&gt;"",OR(L333="PASS",L333="FAIL"),M333&lt;&gt;"",O333&lt;&gt;"",P333="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A333="","",IF(AND(AK333="OK",J333="READY",F333&lt;&gt;"",G333&lt;&gt;"",K333&lt;&gt;"",OR(L333="PASS",L333="FAIL"),M333&lt;&gt;"",P333="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM333" s="9" t="str">
         <x:f>IF(A333="","",IF(AND(AK333="OK",J333="READY",F333&lt;&gt;"",G333&lt;&gt;"",K333&lt;&gt;"",S333="OK",OR(R333="PASS",R333="FAIL")),"YES","NO"))</x:f>
@@ -18297,7 +18297,7 @@
         <x:f>IF(A334="",IF(B334="","","MISSING_TEST_ID"),IF(B334="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A334,$B$2:$B$501,B334)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL334" s="9" t="str">
-        <x:f>IF(A334="","",IF(AND(AK334="OK",J334="READY",F334&lt;&gt;"",G334&lt;&gt;"",K334&lt;&gt;"",OR(L334="PASS",L334="FAIL"),M334&lt;&gt;"",O334&lt;&gt;"",P334="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A334="","",IF(AND(AK334="OK",J334="READY",F334&lt;&gt;"",G334&lt;&gt;"",K334&lt;&gt;"",OR(L334="PASS",L334="FAIL"),M334&lt;&gt;"",P334="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM334" s="9" t="str">
         <x:f>IF(A334="","",IF(AND(AK334="OK",J334="READY",F334&lt;&gt;"",G334&lt;&gt;"",K334&lt;&gt;"",S334="OK",OR(R334="PASS",R334="FAIL")),"YES","NO"))</x:f>
@@ -18349,7 +18349,7 @@
         <x:f>IF(A335="",IF(B335="","","MISSING_TEST_ID"),IF(B335="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A335,$B$2:$B$501,B335)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL335" s="9" t="str">
-        <x:f>IF(A335="","",IF(AND(AK335="OK",J335="READY",F335&lt;&gt;"",G335&lt;&gt;"",K335&lt;&gt;"",OR(L335="PASS",L335="FAIL"),M335&lt;&gt;"",O335&lt;&gt;"",P335="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A335="","",IF(AND(AK335="OK",J335="READY",F335&lt;&gt;"",G335&lt;&gt;"",K335&lt;&gt;"",OR(L335="PASS",L335="FAIL"),M335&lt;&gt;"",P335="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM335" s="9" t="str">
         <x:f>IF(A335="","",IF(AND(AK335="OK",J335="READY",F335&lt;&gt;"",G335&lt;&gt;"",K335&lt;&gt;"",S335="OK",OR(R335="PASS",R335="FAIL")),"YES","NO"))</x:f>
@@ -18401,7 +18401,7 @@
         <x:f>IF(A336="",IF(B336="","","MISSING_TEST_ID"),IF(B336="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A336,$B$2:$B$501,B336)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL336" s="9" t="str">
-        <x:f>IF(A336="","",IF(AND(AK336="OK",J336="READY",F336&lt;&gt;"",G336&lt;&gt;"",K336&lt;&gt;"",OR(L336="PASS",L336="FAIL"),M336&lt;&gt;"",O336&lt;&gt;"",P336="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A336="","",IF(AND(AK336="OK",J336="READY",F336&lt;&gt;"",G336&lt;&gt;"",K336&lt;&gt;"",OR(L336="PASS",L336="FAIL"),M336&lt;&gt;"",P336="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM336" s="9" t="str">
         <x:f>IF(A336="","",IF(AND(AK336="OK",J336="READY",F336&lt;&gt;"",G336&lt;&gt;"",K336&lt;&gt;"",S336="OK",OR(R336="PASS",R336="FAIL")),"YES","NO"))</x:f>
@@ -18453,7 +18453,7 @@
         <x:f>IF(A337="",IF(B337="","","MISSING_TEST_ID"),IF(B337="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A337,$B$2:$B$501,B337)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL337" s="9" t="str">
-        <x:f>IF(A337="","",IF(AND(AK337="OK",J337="READY",F337&lt;&gt;"",G337&lt;&gt;"",K337&lt;&gt;"",OR(L337="PASS",L337="FAIL"),M337&lt;&gt;"",O337&lt;&gt;"",P337="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A337="","",IF(AND(AK337="OK",J337="READY",F337&lt;&gt;"",G337&lt;&gt;"",K337&lt;&gt;"",OR(L337="PASS",L337="FAIL"),M337&lt;&gt;"",P337="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM337" s="9" t="str">
         <x:f>IF(A337="","",IF(AND(AK337="OK",J337="READY",F337&lt;&gt;"",G337&lt;&gt;"",K337&lt;&gt;"",S337="OK",OR(R337="PASS",R337="FAIL")),"YES","NO"))</x:f>
@@ -18505,7 +18505,7 @@
         <x:f>IF(A338="",IF(B338="","","MISSING_TEST_ID"),IF(B338="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A338,$B$2:$B$501,B338)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL338" s="9" t="str">
-        <x:f>IF(A338="","",IF(AND(AK338="OK",J338="READY",F338&lt;&gt;"",G338&lt;&gt;"",K338&lt;&gt;"",OR(L338="PASS",L338="FAIL"),M338&lt;&gt;"",O338&lt;&gt;"",P338="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A338="","",IF(AND(AK338="OK",J338="READY",F338&lt;&gt;"",G338&lt;&gt;"",K338&lt;&gt;"",OR(L338="PASS",L338="FAIL"),M338&lt;&gt;"",P338="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM338" s="9" t="str">
         <x:f>IF(A338="","",IF(AND(AK338="OK",J338="READY",F338&lt;&gt;"",G338&lt;&gt;"",K338&lt;&gt;"",S338="OK",OR(R338="PASS",R338="FAIL")),"YES","NO"))</x:f>
@@ -18557,7 +18557,7 @@
         <x:f>IF(A339="",IF(B339="","","MISSING_TEST_ID"),IF(B339="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A339,$B$2:$B$501,B339)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL339" s="9" t="str">
-        <x:f>IF(A339="","",IF(AND(AK339="OK",J339="READY",F339&lt;&gt;"",G339&lt;&gt;"",K339&lt;&gt;"",OR(L339="PASS",L339="FAIL"),M339&lt;&gt;"",O339&lt;&gt;"",P339="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A339="","",IF(AND(AK339="OK",J339="READY",F339&lt;&gt;"",G339&lt;&gt;"",K339&lt;&gt;"",OR(L339="PASS",L339="FAIL"),M339&lt;&gt;"",P339="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM339" s="9" t="str">
         <x:f>IF(A339="","",IF(AND(AK339="OK",J339="READY",F339&lt;&gt;"",G339&lt;&gt;"",K339&lt;&gt;"",S339="OK",OR(R339="PASS",R339="FAIL")),"YES","NO"))</x:f>
@@ -18609,7 +18609,7 @@
         <x:f>IF(A340="",IF(B340="","","MISSING_TEST_ID"),IF(B340="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A340,$B$2:$B$501,B340)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL340" s="9" t="str">
-        <x:f>IF(A340="","",IF(AND(AK340="OK",J340="READY",F340&lt;&gt;"",G340&lt;&gt;"",K340&lt;&gt;"",OR(L340="PASS",L340="FAIL"),M340&lt;&gt;"",O340&lt;&gt;"",P340="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A340="","",IF(AND(AK340="OK",J340="READY",F340&lt;&gt;"",G340&lt;&gt;"",K340&lt;&gt;"",OR(L340="PASS",L340="FAIL"),M340&lt;&gt;"",P340="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM340" s="9" t="str">
         <x:f>IF(A340="","",IF(AND(AK340="OK",J340="READY",F340&lt;&gt;"",G340&lt;&gt;"",K340&lt;&gt;"",S340="OK",OR(R340="PASS",R340="FAIL")),"YES","NO"))</x:f>
@@ -18661,7 +18661,7 @@
         <x:f>IF(A341="",IF(B341="","","MISSING_TEST_ID"),IF(B341="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A341,$B$2:$B$501,B341)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL341" s="9" t="str">
-        <x:f>IF(A341="","",IF(AND(AK341="OK",J341="READY",F341&lt;&gt;"",G341&lt;&gt;"",K341&lt;&gt;"",OR(L341="PASS",L341="FAIL"),M341&lt;&gt;"",O341&lt;&gt;"",P341="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A341="","",IF(AND(AK341="OK",J341="READY",F341&lt;&gt;"",G341&lt;&gt;"",K341&lt;&gt;"",OR(L341="PASS",L341="FAIL"),M341&lt;&gt;"",P341="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM341" s="9" t="str">
         <x:f>IF(A341="","",IF(AND(AK341="OK",J341="READY",F341&lt;&gt;"",G341&lt;&gt;"",K341&lt;&gt;"",S341="OK",OR(R341="PASS",R341="FAIL")),"YES","NO"))</x:f>
@@ -18713,7 +18713,7 @@
         <x:f>IF(A342="",IF(B342="","","MISSING_TEST_ID"),IF(B342="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A342,$B$2:$B$501,B342)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL342" s="9" t="str">
-        <x:f>IF(A342="","",IF(AND(AK342="OK",J342="READY",F342&lt;&gt;"",G342&lt;&gt;"",K342&lt;&gt;"",OR(L342="PASS",L342="FAIL"),M342&lt;&gt;"",O342&lt;&gt;"",P342="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A342="","",IF(AND(AK342="OK",J342="READY",F342&lt;&gt;"",G342&lt;&gt;"",K342&lt;&gt;"",OR(L342="PASS",L342="FAIL"),M342&lt;&gt;"",P342="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM342" s="9" t="str">
         <x:f>IF(A342="","",IF(AND(AK342="OK",J342="READY",F342&lt;&gt;"",G342&lt;&gt;"",K342&lt;&gt;"",S342="OK",OR(R342="PASS",R342="FAIL")),"YES","NO"))</x:f>
@@ -18765,7 +18765,7 @@
         <x:f>IF(A343="",IF(B343="","","MISSING_TEST_ID"),IF(B343="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A343,$B$2:$B$501,B343)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL343" s="9" t="str">
-        <x:f>IF(A343="","",IF(AND(AK343="OK",J343="READY",F343&lt;&gt;"",G343&lt;&gt;"",K343&lt;&gt;"",OR(L343="PASS",L343="FAIL"),M343&lt;&gt;"",O343&lt;&gt;"",P343="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A343="","",IF(AND(AK343="OK",J343="READY",F343&lt;&gt;"",G343&lt;&gt;"",K343&lt;&gt;"",OR(L343="PASS",L343="FAIL"),M343&lt;&gt;"",P343="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM343" s="9" t="str">
         <x:f>IF(A343="","",IF(AND(AK343="OK",J343="READY",F343&lt;&gt;"",G343&lt;&gt;"",K343&lt;&gt;"",S343="OK",OR(R343="PASS",R343="FAIL")),"YES","NO"))</x:f>
@@ -18817,7 +18817,7 @@
         <x:f>IF(A344="",IF(B344="","","MISSING_TEST_ID"),IF(B344="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A344,$B$2:$B$501,B344)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL344" s="9" t="str">
-        <x:f>IF(A344="","",IF(AND(AK344="OK",J344="READY",F344&lt;&gt;"",G344&lt;&gt;"",K344&lt;&gt;"",OR(L344="PASS",L344="FAIL"),M344&lt;&gt;"",O344&lt;&gt;"",P344="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A344="","",IF(AND(AK344="OK",J344="READY",F344&lt;&gt;"",G344&lt;&gt;"",K344&lt;&gt;"",OR(L344="PASS",L344="FAIL"),M344&lt;&gt;"",P344="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM344" s="9" t="str">
         <x:f>IF(A344="","",IF(AND(AK344="OK",J344="READY",F344&lt;&gt;"",G344&lt;&gt;"",K344&lt;&gt;"",S344="OK",OR(R344="PASS",R344="FAIL")),"YES","NO"))</x:f>
@@ -18869,7 +18869,7 @@
         <x:f>IF(A345="",IF(B345="","","MISSING_TEST_ID"),IF(B345="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A345,$B$2:$B$501,B345)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL345" s="9" t="str">
-        <x:f>IF(A345="","",IF(AND(AK345="OK",J345="READY",F345&lt;&gt;"",G345&lt;&gt;"",K345&lt;&gt;"",OR(L345="PASS",L345="FAIL"),M345&lt;&gt;"",O345&lt;&gt;"",P345="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A345="","",IF(AND(AK345="OK",J345="READY",F345&lt;&gt;"",G345&lt;&gt;"",K345&lt;&gt;"",OR(L345="PASS",L345="FAIL"),M345&lt;&gt;"",P345="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM345" s="9" t="str">
         <x:f>IF(A345="","",IF(AND(AK345="OK",J345="READY",F345&lt;&gt;"",G345&lt;&gt;"",K345&lt;&gt;"",S345="OK",OR(R345="PASS",R345="FAIL")),"YES","NO"))</x:f>
@@ -18921,7 +18921,7 @@
         <x:f>IF(A346="",IF(B346="","","MISSING_TEST_ID"),IF(B346="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A346,$B$2:$B$501,B346)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL346" s="9" t="str">
-        <x:f>IF(A346="","",IF(AND(AK346="OK",J346="READY",F346&lt;&gt;"",G346&lt;&gt;"",K346&lt;&gt;"",OR(L346="PASS",L346="FAIL"),M346&lt;&gt;"",O346&lt;&gt;"",P346="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A346="","",IF(AND(AK346="OK",J346="READY",F346&lt;&gt;"",G346&lt;&gt;"",K346&lt;&gt;"",OR(L346="PASS",L346="FAIL"),M346&lt;&gt;"",P346="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM346" s="9" t="str">
         <x:f>IF(A346="","",IF(AND(AK346="OK",J346="READY",F346&lt;&gt;"",G346&lt;&gt;"",K346&lt;&gt;"",S346="OK",OR(R346="PASS",R346="FAIL")),"YES","NO"))</x:f>
@@ -18973,7 +18973,7 @@
         <x:f>IF(A347="",IF(B347="","","MISSING_TEST_ID"),IF(B347="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A347,$B$2:$B$501,B347)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL347" s="9" t="str">
-        <x:f>IF(A347="","",IF(AND(AK347="OK",J347="READY",F347&lt;&gt;"",G347&lt;&gt;"",K347&lt;&gt;"",OR(L347="PASS",L347="FAIL"),M347&lt;&gt;"",O347&lt;&gt;"",P347="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A347="","",IF(AND(AK347="OK",J347="READY",F347&lt;&gt;"",G347&lt;&gt;"",K347&lt;&gt;"",OR(L347="PASS",L347="FAIL"),M347&lt;&gt;"",P347="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM347" s="9" t="str">
         <x:f>IF(A347="","",IF(AND(AK347="OK",J347="READY",F347&lt;&gt;"",G347&lt;&gt;"",K347&lt;&gt;"",S347="OK",OR(R347="PASS",R347="FAIL")),"YES","NO"))</x:f>
@@ -19025,7 +19025,7 @@
         <x:f>IF(A348="",IF(B348="","","MISSING_TEST_ID"),IF(B348="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A348,$B$2:$B$501,B348)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL348" s="9" t="str">
-        <x:f>IF(A348="","",IF(AND(AK348="OK",J348="READY",F348&lt;&gt;"",G348&lt;&gt;"",K348&lt;&gt;"",OR(L348="PASS",L348="FAIL"),M348&lt;&gt;"",O348&lt;&gt;"",P348="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A348="","",IF(AND(AK348="OK",J348="READY",F348&lt;&gt;"",G348&lt;&gt;"",K348&lt;&gt;"",OR(L348="PASS",L348="FAIL"),M348&lt;&gt;"",P348="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM348" s="9" t="str">
         <x:f>IF(A348="","",IF(AND(AK348="OK",J348="READY",F348&lt;&gt;"",G348&lt;&gt;"",K348&lt;&gt;"",S348="OK",OR(R348="PASS",R348="FAIL")),"YES","NO"))</x:f>
@@ -19077,7 +19077,7 @@
         <x:f>IF(A349="",IF(B349="","","MISSING_TEST_ID"),IF(B349="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A349,$B$2:$B$501,B349)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL349" s="9" t="str">
-        <x:f>IF(A349="","",IF(AND(AK349="OK",J349="READY",F349&lt;&gt;"",G349&lt;&gt;"",K349&lt;&gt;"",OR(L349="PASS",L349="FAIL"),M349&lt;&gt;"",O349&lt;&gt;"",P349="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A349="","",IF(AND(AK349="OK",J349="READY",F349&lt;&gt;"",G349&lt;&gt;"",K349&lt;&gt;"",OR(L349="PASS",L349="FAIL"),M349&lt;&gt;"",P349="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM349" s="9" t="str">
         <x:f>IF(A349="","",IF(AND(AK349="OK",J349="READY",F349&lt;&gt;"",G349&lt;&gt;"",K349&lt;&gt;"",S349="OK",OR(R349="PASS",R349="FAIL")),"YES","NO"))</x:f>
@@ -19129,7 +19129,7 @@
         <x:f>IF(A350="",IF(B350="","","MISSING_TEST_ID"),IF(B350="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A350,$B$2:$B$501,B350)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL350" s="9" t="str">
-        <x:f>IF(A350="","",IF(AND(AK350="OK",J350="READY",F350&lt;&gt;"",G350&lt;&gt;"",K350&lt;&gt;"",OR(L350="PASS",L350="FAIL"),M350&lt;&gt;"",O350&lt;&gt;"",P350="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A350="","",IF(AND(AK350="OK",J350="READY",F350&lt;&gt;"",G350&lt;&gt;"",K350&lt;&gt;"",OR(L350="PASS",L350="FAIL"),M350&lt;&gt;"",P350="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM350" s="9" t="str">
         <x:f>IF(A350="","",IF(AND(AK350="OK",J350="READY",F350&lt;&gt;"",G350&lt;&gt;"",K350&lt;&gt;"",S350="OK",OR(R350="PASS",R350="FAIL")),"YES","NO"))</x:f>
@@ -19181,7 +19181,7 @@
         <x:f>IF(A351="",IF(B351="","","MISSING_TEST_ID"),IF(B351="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A351,$B$2:$B$501,B351)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL351" s="9" t="str">
-        <x:f>IF(A351="","",IF(AND(AK351="OK",J351="READY",F351&lt;&gt;"",G351&lt;&gt;"",K351&lt;&gt;"",OR(L351="PASS",L351="FAIL"),M351&lt;&gt;"",O351&lt;&gt;"",P351="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A351="","",IF(AND(AK351="OK",J351="READY",F351&lt;&gt;"",G351&lt;&gt;"",K351&lt;&gt;"",OR(L351="PASS",L351="FAIL"),M351&lt;&gt;"",P351="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM351" s="9" t="str">
         <x:f>IF(A351="","",IF(AND(AK351="OK",J351="READY",F351&lt;&gt;"",G351&lt;&gt;"",K351&lt;&gt;"",S351="OK",OR(R351="PASS",R351="FAIL")),"YES","NO"))</x:f>
@@ -19233,7 +19233,7 @@
         <x:f>IF(A352="",IF(B352="","","MISSING_TEST_ID"),IF(B352="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A352,$B$2:$B$501,B352)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL352" s="9" t="str">
-        <x:f>IF(A352="","",IF(AND(AK352="OK",J352="READY",F352&lt;&gt;"",G352&lt;&gt;"",K352&lt;&gt;"",OR(L352="PASS",L352="FAIL"),M352&lt;&gt;"",O352&lt;&gt;"",P352="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A352="","",IF(AND(AK352="OK",J352="READY",F352&lt;&gt;"",G352&lt;&gt;"",K352&lt;&gt;"",OR(L352="PASS",L352="FAIL"),M352&lt;&gt;"",P352="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM352" s="9" t="str">
         <x:f>IF(A352="","",IF(AND(AK352="OK",J352="READY",F352&lt;&gt;"",G352&lt;&gt;"",K352&lt;&gt;"",S352="OK",OR(R352="PASS",R352="FAIL")),"YES","NO"))</x:f>
@@ -19285,7 +19285,7 @@
         <x:f>IF(A353="",IF(B353="","","MISSING_TEST_ID"),IF(B353="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A353,$B$2:$B$501,B353)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL353" s="9" t="str">
-        <x:f>IF(A353="","",IF(AND(AK353="OK",J353="READY",F353&lt;&gt;"",G353&lt;&gt;"",K353&lt;&gt;"",OR(L353="PASS",L353="FAIL"),M353&lt;&gt;"",O353&lt;&gt;"",P353="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A353="","",IF(AND(AK353="OK",J353="READY",F353&lt;&gt;"",G353&lt;&gt;"",K353&lt;&gt;"",OR(L353="PASS",L353="FAIL"),M353&lt;&gt;"",P353="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM353" s="9" t="str">
         <x:f>IF(A353="","",IF(AND(AK353="OK",J353="READY",F353&lt;&gt;"",G353&lt;&gt;"",K353&lt;&gt;"",S353="OK",OR(R353="PASS",R353="FAIL")),"YES","NO"))</x:f>
@@ -19337,7 +19337,7 @@
         <x:f>IF(A354="",IF(B354="","","MISSING_TEST_ID"),IF(B354="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A354,$B$2:$B$501,B354)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL354" s="9" t="str">
-        <x:f>IF(A354="","",IF(AND(AK354="OK",J354="READY",F354&lt;&gt;"",G354&lt;&gt;"",K354&lt;&gt;"",OR(L354="PASS",L354="FAIL"),M354&lt;&gt;"",O354&lt;&gt;"",P354="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A354="","",IF(AND(AK354="OK",J354="READY",F354&lt;&gt;"",G354&lt;&gt;"",K354&lt;&gt;"",OR(L354="PASS",L354="FAIL"),M354&lt;&gt;"",P354="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM354" s="9" t="str">
         <x:f>IF(A354="","",IF(AND(AK354="OK",J354="READY",F354&lt;&gt;"",G354&lt;&gt;"",K354&lt;&gt;"",S354="OK",OR(R354="PASS",R354="FAIL")),"YES","NO"))</x:f>
@@ -19389,7 +19389,7 @@
         <x:f>IF(A355="",IF(B355="","","MISSING_TEST_ID"),IF(B355="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A355,$B$2:$B$501,B355)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL355" s="9" t="str">
-        <x:f>IF(A355="","",IF(AND(AK355="OK",J355="READY",F355&lt;&gt;"",G355&lt;&gt;"",K355&lt;&gt;"",OR(L355="PASS",L355="FAIL"),M355&lt;&gt;"",O355&lt;&gt;"",P355="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A355="","",IF(AND(AK355="OK",J355="READY",F355&lt;&gt;"",G355&lt;&gt;"",K355&lt;&gt;"",OR(L355="PASS",L355="FAIL"),M355&lt;&gt;"",P355="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM355" s="9" t="str">
         <x:f>IF(A355="","",IF(AND(AK355="OK",J355="READY",F355&lt;&gt;"",G355&lt;&gt;"",K355&lt;&gt;"",S355="OK",OR(R355="PASS",R355="FAIL")),"YES","NO"))</x:f>
@@ -19441,7 +19441,7 @@
         <x:f>IF(A356="",IF(B356="","","MISSING_TEST_ID"),IF(B356="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A356,$B$2:$B$501,B356)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL356" s="9" t="str">
-        <x:f>IF(A356="","",IF(AND(AK356="OK",J356="READY",F356&lt;&gt;"",G356&lt;&gt;"",K356&lt;&gt;"",OR(L356="PASS",L356="FAIL"),M356&lt;&gt;"",O356&lt;&gt;"",P356="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A356="","",IF(AND(AK356="OK",J356="READY",F356&lt;&gt;"",G356&lt;&gt;"",K356&lt;&gt;"",OR(L356="PASS",L356="FAIL"),M356&lt;&gt;"",P356="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM356" s="9" t="str">
         <x:f>IF(A356="","",IF(AND(AK356="OK",J356="READY",F356&lt;&gt;"",G356&lt;&gt;"",K356&lt;&gt;"",S356="OK",OR(R356="PASS",R356="FAIL")),"YES","NO"))</x:f>
@@ -19493,7 +19493,7 @@
         <x:f>IF(A357="",IF(B357="","","MISSING_TEST_ID"),IF(B357="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A357,$B$2:$B$501,B357)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL357" s="9" t="str">
-        <x:f>IF(A357="","",IF(AND(AK357="OK",J357="READY",F357&lt;&gt;"",G357&lt;&gt;"",K357&lt;&gt;"",OR(L357="PASS",L357="FAIL"),M357&lt;&gt;"",O357&lt;&gt;"",P357="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A357="","",IF(AND(AK357="OK",J357="READY",F357&lt;&gt;"",G357&lt;&gt;"",K357&lt;&gt;"",OR(L357="PASS",L357="FAIL"),M357&lt;&gt;"",P357="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM357" s="9" t="str">
         <x:f>IF(A357="","",IF(AND(AK357="OK",J357="READY",F357&lt;&gt;"",G357&lt;&gt;"",K357&lt;&gt;"",S357="OK",OR(R357="PASS",R357="FAIL")),"YES","NO"))</x:f>
@@ -19545,7 +19545,7 @@
         <x:f>IF(A358="",IF(B358="","","MISSING_TEST_ID"),IF(B358="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A358,$B$2:$B$501,B358)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL358" s="9" t="str">
-        <x:f>IF(A358="","",IF(AND(AK358="OK",J358="READY",F358&lt;&gt;"",G358&lt;&gt;"",K358&lt;&gt;"",OR(L358="PASS",L358="FAIL"),M358&lt;&gt;"",O358&lt;&gt;"",P358="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A358="","",IF(AND(AK358="OK",J358="READY",F358&lt;&gt;"",G358&lt;&gt;"",K358&lt;&gt;"",OR(L358="PASS",L358="FAIL"),M358&lt;&gt;"",P358="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM358" s="9" t="str">
         <x:f>IF(A358="","",IF(AND(AK358="OK",J358="READY",F358&lt;&gt;"",G358&lt;&gt;"",K358&lt;&gt;"",S358="OK",OR(R358="PASS",R358="FAIL")),"YES","NO"))</x:f>
@@ -19597,7 +19597,7 @@
         <x:f>IF(A359="",IF(B359="","","MISSING_TEST_ID"),IF(B359="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A359,$B$2:$B$501,B359)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL359" s="9" t="str">
-        <x:f>IF(A359="","",IF(AND(AK359="OK",J359="READY",F359&lt;&gt;"",G359&lt;&gt;"",K359&lt;&gt;"",OR(L359="PASS",L359="FAIL"),M359&lt;&gt;"",O359&lt;&gt;"",P359="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A359="","",IF(AND(AK359="OK",J359="READY",F359&lt;&gt;"",G359&lt;&gt;"",K359&lt;&gt;"",OR(L359="PASS",L359="FAIL"),M359&lt;&gt;"",P359="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM359" s="9" t="str">
         <x:f>IF(A359="","",IF(AND(AK359="OK",J359="READY",F359&lt;&gt;"",G359&lt;&gt;"",K359&lt;&gt;"",S359="OK",OR(R359="PASS",R359="FAIL")),"YES","NO"))</x:f>
@@ -19649,7 +19649,7 @@
         <x:f>IF(A360="",IF(B360="","","MISSING_TEST_ID"),IF(B360="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A360,$B$2:$B$501,B360)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL360" s="9" t="str">
-        <x:f>IF(A360="","",IF(AND(AK360="OK",J360="READY",F360&lt;&gt;"",G360&lt;&gt;"",K360&lt;&gt;"",OR(L360="PASS",L360="FAIL"),M360&lt;&gt;"",O360&lt;&gt;"",P360="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A360="","",IF(AND(AK360="OK",J360="READY",F360&lt;&gt;"",G360&lt;&gt;"",K360&lt;&gt;"",OR(L360="PASS",L360="FAIL"),M360&lt;&gt;"",P360="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM360" s="9" t="str">
         <x:f>IF(A360="","",IF(AND(AK360="OK",J360="READY",F360&lt;&gt;"",G360&lt;&gt;"",K360&lt;&gt;"",S360="OK",OR(R360="PASS",R360="FAIL")),"YES","NO"))</x:f>
@@ -19701,7 +19701,7 @@
         <x:f>IF(A361="",IF(B361="","","MISSING_TEST_ID"),IF(B361="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A361,$B$2:$B$501,B361)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL361" s="9" t="str">
-        <x:f>IF(A361="","",IF(AND(AK361="OK",J361="READY",F361&lt;&gt;"",G361&lt;&gt;"",K361&lt;&gt;"",OR(L361="PASS",L361="FAIL"),M361&lt;&gt;"",O361&lt;&gt;"",P361="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A361="","",IF(AND(AK361="OK",J361="READY",F361&lt;&gt;"",G361&lt;&gt;"",K361&lt;&gt;"",OR(L361="PASS",L361="FAIL"),M361&lt;&gt;"",P361="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM361" s="9" t="str">
         <x:f>IF(A361="","",IF(AND(AK361="OK",J361="READY",F361&lt;&gt;"",G361&lt;&gt;"",K361&lt;&gt;"",S361="OK",OR(R361="PASS",R361="FAIL")),"YES","NO"))</x:f>
@@ -19753,7 +19753,7 @@
         <x:f>IF(A362="",IF(B362="","","MISSING_TEST_ID"),IF(B362="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A362,$B$2:$B$501,B362)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL362" s="9" t="str">
-        <x:f>IF(A362="","",IF(AND(AK362="OK",J362="READY",F362&lt;&gt;"",G362&lt;&gt;"",K362&lt;&gt;"",OR(L362="PASS",L362="FAIL"),M362&lt;&gt;"",O362&lt;&gt;"",P362="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A362="","",IF(AND(AK362="OK",J362="READY",F362&lt;&gt;"",G362&lt;&gt;"",K362&lt;&gt;"",OR(L362="PASS",L362="FAIL"),M362&lt;&gt;"",P362="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM362" s="9" t="str">
         <x:f>IF(A362="","",IF(AND(AK362="OK",J362="READY",F362&lt;&gt;"",G362&lt;&gt;"",K362&lt;&gt;"",S362="OK",OR(R362="PASS",R362="FAIL")),"YES","NO"))</x:f>
@@ -19805,7 +19805,7 @@
         <x:f>IF(A363="",IF(B363="","","MISSING_TEST_ID"),IF(B363="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A363,$B$2:$B$501,B363)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL363" s="9" t="str">
-        <x:f>IF(A363="","",IF(AND(AK363="OK",J363="READY",F363&lt;&gt;"",G363&lt;&gt;"",K363&lt;&gt;"",OR(L363="PASS",L363="FAIL"),M363&lt;&gt;"",O363&lt;&gt;"",P363="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A363="","",IF(AND(AK363="OK",J363="READY",F363&lt;&gt;"",G363&lt;&gt;"",K363&lt;&gt;"",OR(L363="PASS",L363="FAIL"),M363&lt;&gt;"",P363="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM363" s="9" t="str">
         <x:f>IF(A363="","",IF(AND(AK363="OK",J363="READY",F363&lt;&gt;"",G363&lt;&gt;"",K363&lt;&gt;"",S363="OK",OR(R363="PASS",R363="FAIL")),"YES","NO"))</x:f>
@@ -19857,7 +19857,7 @@
         <x:f>IF(A364="",IF(B364="","","MISSING_TEST_ID"),IF(B364="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A364,$B$2:$B$501,B364)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL364" s="9" t="str">
-        <x:f>IF(A364="","",IF(AND(AK364="OK",J364="READY",F364&lt;&gt;"",G364&lt;&gt;"",K364&lt;&gt;"",OR(L364="PASS",L364="FAIL"),M364&lt;&gt;"",O364&lt;&gt;"",P364="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A364="","",IF(AND(AK364="OK",J364="READY",F364&lt;&gt;"",G364&lt;&gt;"",K364&lt;&gt;"",OR(L364="PASS",L364="FAIL"),M364&lt;&gt;"",P364="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM364" s="9" t="str">
         <x:f>IF(A364="","",IF(AND(AK364="OK",J364="READY",F364&lt;&gt;"",G364&lt;&gt;"",K364&lt;&gt;"",S364="OK",OR(R364="PASS",R364="FAIL")),"YES","NO"))</x:f>
@@ -19909,7 +19909,7 @@
         <x:f>IF(A365="",IF(B365="","","MISSING_TEST_ID"),IF(B365="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A365,$B$2:$B$501,B365)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL365" s="9" t="str">
-        <x:f>IF(A365="","",IF(AND(AK365="OK",J365="READY",F365&lt;&gt;"",G365&lt;&gt;"",K365&lt;&gt;"",OR(L365="PASS",L365="FAIL"),M365&lt;&gt;"",O365&lt;&gt;"",P365="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A365="","",IF(AND(AK365="OK",J365="READY",F365&lt;&gt;"",G365&lt;&gt;"",K365&lt;&gt;"",OR(L365="PASS",L365="FAIL"),M365&lt;&gt;"",P365="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM365" s="9" t="str">
         <x:f>IF(A365="","",IF(AND(AK365="OK",J365="READY",F365&lt;&gt;"",G365&lt;&gt;"",K365&lt;&gt;"",S365="OK",OR(R365="PASS",R365="FAIL")),"YES","NO"))</x:f>
@@ -19961,7 +19961,7 @@
         <x:f>IF(A366="",IF(B366="","","MISSING_TEST_ID"),IF(B366="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A366,$B$2:$B$501,B366)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL366" s="9" t="str">
-        <x:f>IF(A366="","",IF(AND(AK366="OK",J366="READY",F366&lt;&gt;"",G366&lt;&gt;"",K366&lt;&gt;"",OR(L366="PASS",L366="FAIL"),M366&lt;&gt;"",O366&lt;&gt;"",P366="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A366="","",IF(AND(AK366="OK",J366="READY",F366&lt;&gt;"",G366&lt;&gt;"",K366&lt;&gt;"",OR(L366="PASS",L366="FAIL"),M366&lt;&gt;"",P366="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM366" s="9" t="str">
         <x:f>IF(A366="","",IF(AND(AK366="OK",J366="READY",F366&lt;&gt;"",G366&lt;&gt;"",K366&lt;&gt;"",S366="OK",OR(R366="PASS",R366="FAIL")),"YES","NO"))</x:f>
@@ -20013,7 +20013,7 @@
         <x:f>IF(A367="",IF(B367="","","MISSING_TEST_ID"),IF(B367="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A367,$B$2:$B$501,B367)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL367" s="9" t="str">
-        <x:f>IF(A367="","",IF(AND(AK367="OK",J367="READY",F367&lt;&gt;"",G367&lt;&gt;"",K367&lt;&gt;"",OR(L367="PASS",L367="FAIL"),M367&lt;&gt;"",O367&lt;&gt;"",P367="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A367="","",IF(AND(AK367="OK",J367="READY",F367&lt;&gt;"",G367&lt;&gt;"",K367&lt;&gt;"",OR(L367="PASS",L367="FAIL"),M367&lt;&gt;"",P367="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM367" s="9" t="str">
         <x:f>IF(A367="","",IF(AND(AK367="OK",J367="READY",F367&lt;&gt;"",G367&lt;&gt;"",K367&lt;&gt;"",S367="OK",OR(R367="PASS",R367="FAIL")),"YES","NO"))</x:f>
@@ -20065,7 +20065,7 @@
         <x:f>IF(A368="",IF(B368="","","MISSING_TEST_ID"),IF(B368="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A368,$B$2:$B$501,B368)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL368" s="9" t="str">
-        <x:f>IF(A368="","",IF(AND(AK368="OK",J368="READY",F368&lt;&gt;"",G368&lt;&gt;"",K368&lt;&gt;"",OR(L368="PASS",L368="FAIL"),M368&lt;&gt;"",O368&lt;&gt;"",P368="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A368="","",IF(AND(AK368="OK",J368="READY",F368&lt;&gt;"",G368&lt;&gt;"",K368&lt;&gt;"",OR(L368="PASS",L368="FAIL"),M368&lt;&gt;"",P368="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM368" s="9" t="str">
         <x:f>IF(A368="","",IF(AND(AK368="OK",J368="READY",F368&lt;&gt;"",G368&lt;&gt;"",K368&lt;&gt;"",S368="OK",OR(R368="PASS",R368="FAIL")),"YES","NO"))</x:f>
@@ -20117,7 +20117,7 @@
         <x:f>IF(A369="",IF(B369="","","MISSING_TEST_ID"),IF(B369="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A369,$B$2:$B$501,B369)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL369" s="9" t="str">
-        <x:f>IF(A369="","",IF(AND(AK369="OK",J369="READY",F369&lt;&gt;"",G369&lt;&gt;"",K369&lt;&gt;"",OR(L369="PASS",L369="FAIL"),M369&lt;&gt;"",O369&lt;&gt;"",P369="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A369="","",IF(AND(AK369="OK",J369="READY",F369&lt;&gt;"",G369&lt;&gt;"",K369&lt;&gt;"",OR(L369="PASS",L369="FAIL"),M369&lt;&gt;"",P369="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM369" s="9" t="str">
         <x:f>IF(A369="","",IF(AND(AK369="OK",J369="READY",F369&lt;&gt;"",G369&lt;&gt;"",K369&lt;&gt;"",S369="OK",OR(R369="PASS",R369="FAIL")),"YES","NO"))</x:f>
@@ -20169,7 +20169,7 @@
         <x:f>IF(A370="",IF(B370="","","MISSING_TEST_ID"),IF(B370="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A370,$B$2:$B$501,B370)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL370" s="9" t="str">
-        <x:f>IF(A370="","",IF(AND(AK370="OK",J370="READY",F370&lt;&gt;"",G370&lt;&gt;"",K370&lt;&gt;"",OR(L370="PASS",L370="FAIL"),M370&lt;&gt;"",O370&lt;&gt;"",P370="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A370="","",IF(AND(AK370="OK",J370="READY",F370&lt;&gt;"",G370&lt;&gt;"",K370&lt;&gt;"",OR(L370="PASS",L370="FAIL"),M370&lt;&gt;"",P370="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM370" s="9" t="str">
         <x:f>IF(A370="","",IF(AND(AK370="OK",J370="READY",F370&lt;&gt;"",G370&lt;&gt;"",K370&lt;&gt;"",S370="OK",OR(R370="PASS",R370="FAIL")),"YES","NO"))</x:f>
@@ -20221,7 +20221,7 @@
         <x:f>IF(A371="",IF(B371="","","MISSING_TEST_ID"),IF(B371="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A371,$B$2:$B$501,B371)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL371" s="9" t="str">
-        <x:f>IF(A371="","",IF(AND(AK371="OK",J371="READY",F371&lt;&gt;"",G371&lt;&gt;"",K371&lt;&gt;"",OR(L371="PASS",L371="FAIL"),M371&lt;&gt;"",O371&lt;&gt;"",P371="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A371="","",IF(AND(AK371="OK",J371="READY",F371&lt;&gt;"",G371&lt;&gt;"",K371&lt;&gt;"",OR(L371="PASS",L371="FAIL"),M371&lt;&gt;"",P371="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM371" s="9" t="str">
         <x:f>IF(A371="","",IF(AND(AK371="OK",J371="READY",F371&lt;&gt;"",G371&lt;&gt;"",K371&lt;&gt;"",S371="OK",OR(R371="PASS",R371="FAIL")),"YES","NO"))</x:f>
@@ -20273,7 +20273,7 @@
         <x:f>IF(A372="",IF(B372="","","MISSING_TEST_ID"),IF(B372="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A372,$B$2:$B$501,B372)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL372" s="9" t="str">
-        <x:f>IF(A372="","",IF(AND(AK372="OK",J372="READY",F372&lt;&gt;"",G372&lt;&gt;"",K372&lt;&gt;"",OR(L372="PASS",L372="FAIL"),M372&lt;&gt;"",O372&lt;&gt;"",P372="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A372="","",IF(AND(AK372="OK",J372="READY",F372&lt;&gt;"",G372&lt;&gt;"",K372&lt;&gt;"",OR(L372="PASS",L372="FAIL"),M372&lt;&gt;"",P372="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM372" s="9" t="str">
         <x:f>IF(A372="","",IF(AND(AK372="OK",J372="READY",F372&lt;&gt;"",G372&lt;&gt;"",K372&lt;&gt;"",S372="OK",OR(R372="PASS",R372="FAIL")),"YES","NO"))</x:f>
@@ -20325,7 +20325,7 @@
         <x:f>IF(A373="",IF(B373="","","MISSING_TEST_ID"),IF(B373="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A373,$B$2:$B$501,B373)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL373" s="9" t="str">
-        <x:f>IF(A373="","",IF(AND(AK373="OK",J373="READY",F373&lt;&gt;"",G373&lt;&gt;"",K373&lt;&gt;"",OR(L373="PASS",L373="FAIL"),M373&lt;&gt;"",O373&lt;&gt;"",P373="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A373="","",IF(AND(AK373="OK",J373="READY",F373&lt;&gt;"",G373&lt;&gt;"",K373&lt;&gt;"",OR(L373="PASS",L373="FAIL"),M373&lt;&gt;"",P373="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM373" s="9" t="str">
         <x:f>IF(A373="","",IF(AND(AK373="OK",J373="READY",F373&lt;&gt;"",G373&lt;&gt;"",K373&lt;&gt;"",S373="OK",OR(R373="PASS",R373="FAIL")),"YES","NO"))</x:f>
@@ -20377,7 +20377,7 @@
         <x:f>IF(A374="",IF(B374="","","MISSING_TEST_ID"),IF(B374="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A374,$B$2:$B$501,B374)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL374" s="9" t="str">
-        <x:f>IF(A374="","",IF(AND(AK374="OK",J374="READY",F374&lt;&gt;"",G374&lt;&gt;"",K374&lt;&gt;"",OR(L374="PASS",L374="FAIL"),M374&lt;&gt;"",O374&lt;&gt;"",P374="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A374="","",IF(AND(AK374="OK",J374="READY",F374&lt;&gt;"",G374&lt;&gt;"",K374&lt;&gt;"",OR(L374="PASS",L374="FAIL"),M374&lt;&gt;"",P374="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM374" s="9" t="str">
         <x:f>IF(A374="","",IF(AND(AK374="OK",J374="READY",F374&lt;&gt;"",G374&lt;&gt;"",K374&lt;&gt;"",S374="OK",OR(R374="PASS",R374="FAIL")),"YES","NO"))</x:f>
@@ -20429,7 +20429,7 @@
         <x:f>IF(A375="",IF(B375="","","MISSING_TEST_ID"),IF(B375="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A375,$B$2:$B$501,B375)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL375" s="9" t="str">
-        <x:f>IF(A375="","",IF(AND(AK375="OK",J375="READY",F375&lt;&gt;"",G375&lt;&gt;"",K375&lt;&gt;"",OR(L375="PASS",L375="FAIL"),M375&lt;&gt;"",O375&lt;&gt;"",P375="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A375="","",IF(AND(AK375="OK",J375="READY",F375&lt;&gt;"",G375&lt;&gt;"",K375&lt;&gt;"",OR(L375="PASS",L375="FAIL"),M375&lt;&gt;"",P375="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM375" s="9" t="str">
         <x:f>IF(A375="","",IF(AND(AK375="OK",J375="READY",F375&lt;&gt;"",G375&lt;&gt;"",K375&lt;&gt;"",S375="OK",OR(R375="PASS",R375="FAIL")),"YES","NO"))</x:f>
@@ -20481,7 +20481,7 @@
         <x:f>IF(A376="",IF(B376="","","MISSING_TEST_ID"),IF(B376="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A376,$B$2:$B$501,B376)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL376" s="9" t="str">
-        <x:f>IF(A376="","",IF(AND(AK376="OK",J376="READY",F376&lt;&gt;"",G376&lt;&gt;"",K376&lt;&gt;"",OR(L376="PASS",L376="FAIL"),M376&lt;&gt;"",O376&lt;&gt;"",P376="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A376="","",IF(AND(AK376="OK",J376="READY",F376&lt;&gt;"",G376&lt;&gt;"",K376&lt;&gt;"",OR(L376="PASS",L376="FAIL"),M376&lt;&gt;"",P376="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM376" s="9" t="str">
         <x:f>IF(A376="","",IF(AND(AK376="OK",J376="READY",F376&lt;&gt;"",G376&lt;&gt;"",K376&lt;&gt;"",S376="OK",OR(R376="PASS",R376="FAIL")),"YES","NO"))</x:f>
@@ -20533,7 +20533,7 @@
         <x:f>IF(A377="",IF(B377="","","MISSING_TEST_ID"),IF(B377="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A377,$B$2:$B$501,B377)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL377" s="9" t="str">
-        <x:f>IF(A377="","",IF(AND(AK377="OK",J377="READY",F377&lt;&gt;"",G377&lt;&gt;"",K377&lt;&gt;"",OR(L377="PASS",L377="FAIL"),M377&lt;&gt;"",O377&lt;&gt;"",P377="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A377="","",IF(AND(AK377="OK",J377="READY",F377&lt;&gt;"",G377&lt;&gt;"",K377&lt;&gt;"",OR(L377="PASS",L377="FAIL"),M377&lt;&gt;"",P377="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM377" s="9" t="str">
         <x:f>IF(A377="","",IF(AND(AK377="OK",J377="READY",F377&lt;&gt;"",G377&lt;&gt;"",K377&lt;&gt;"",S377="OK",OR(R377="PASS",R377="FAIL")),"YES","NO"))</x:f>
@@ -20585,7 +20585,7 @@
         <x:f>IF(A378="",IF(B378="","","MISSING_TEST_ID"),IF(B378="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A378,$B$2:$B$501,B378)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL378" s="9" t="str">
-        <x:f>IF(A378="","",IF(AND(AK378="OK",J378="READY",F378&lt;&gt;"",G378&lt;&gt;"",K378&lt;&gt;"",OR(L378="PASS",L378="FAIL"),M378&lt;&gt;"",O378&lt;&gt;"",P378="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A378="","",IF(AND(AK378="OK",J378="READY",F378&lt;&gt;"",G378&lt;&gt;"",K378&lt;&gt;"",OR(L378="PASS",L378="FAIL"),M378&lt;&gt;"",P378="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM378" s="9" t="str">
         <x:f>IF(A378="","",IF(AND(AK378="OK",J378="READY",F378&lt;&gt;"",G378&lt;&gt;"",K378&lt;&gt;"",S378="OK",OR(R378="PASS",R378="FAIL")),"YES","NO"))</x:f>
@@ -20637,7 +20637,7 @@
         <x:f>IF(A379="",IF(B379="","","MISSING_TEST_ID"),IF(B379="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A379,$B$2:$B$501,B379)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL379" s="9" t="str">
-        <x:f>IF(A379="","",IF(AND(AK379="OK",J379="READY",F379&lt;&gt;"",G379&lt;&gt;"",K379&lt;&gt;"",OR(L379="PASS",L379="FAIL"),M379&lt;&gt;"",O379&lt;&gt;"",P379="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A379="","",IF(AND(AK379="OK",J379="READY",F379&lt;&gt;"",G379&lt;&gt;"",K379&lt;&gt;"",OR(L379="PASS",L379="FAIL"),M379&lt;&gt;"",P379="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM379" s="9" t="str">
         <x:f>IF(A379="","",IF(AND(AK379="OK",J379="READY",F379&lt;&gt;"",G379&lt;&gt;"",K379&lt;&gt;"",S379="OK",OR(R379="PASS",R379="FAIL")),"YES","NO"))</x:f>
@@ -20689,7 +20689,7 @@
         <x:f>IF(A380="",IF(B380="","","MISSING_TEST_ID"),IF(B380="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A380,$B$2:$B$501,B380)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL380" s="9" t="str">
-        <x:f>IF(A380="","",IF(AND(AK380="OK",J380="READY",F380&lt;&gt;"",G380&lt;&gt;"",K380&lt;&gt;"",OR(L380="PASS",L380="FAIL"),M380&lt;&gt;"",O380&lt;&gt;"",P380="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A380="","",IF(AND(AK380="OK",J380="READY",F380&lt;&gt;"",G380&lt;&gt;"",K380&lt;&gt;"",OR(L380="PASS",L380="FAIL"),M380&lt;&gt;"",P380="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM380" s="9" t="str">
         <x:f>IF(A380="","",IF(AND(AK380="OK",J380="READY",F380&lt;&gt;"",G380&lt;&gt;"",K380&lt;&gt;"",S380="OK",OR(R380="PASS",R380="FAIL")),"YES","NO"))</x:f>
@@ -20741,7 +20741,7 @@
         <x:f>IF(A381="",IF(B381="","","MISSING_TEST_ID"),IF(B381="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A381,$B$2:$B$501,B381)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL381" s="9" t="str">
-        <x:f>IF(A381="","",IF(AND(AK381="OK",J381="READY",F381&lt;&gt;"",G381&lt;&gt;"",K381&lt;&gt;"",OR(L381="PASS",L381="FAIL"),M381&lt;&gt;"",O381&lt;&gt;"",P381="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A381="","",IF(AND(AK381="OK",J381="READY",F381&lt;&gt;"",G381&lt;&gt;"",K381&lt;&gt;"",OR(L381="PASS",L381="FAIL"),M381&lt;&gt;"",P381="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM381" s="9" t="str">
         <x:f>IF(A381="","",IF(AND(AK381="OK",J381="READY",F381&lt;&gt;"",G381&lt;&gt;"",K381&lt;&gt;"",S381="OK",OR(R381="PASS",R381="FAIL")),"YES","NO"))</x:f>
@@ -20793,7 +20793,7 @@
         <x:f>IF(A382="",IF(B382="","","MISSING_TEST_ID"),IF(B382="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A382,$B$2:$B$501,B382)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL382" s="9" t="str">
-        <x:f>IF(A382="","",IF(AND(AK382="OK",J382="READY",F382&lt;&gt;"",G382&lt;&gt;"",K382&lt;&gt;"",OR(L382="PASS",L382="FAIL"),M382&lt;&gt;"",O382&lt;&gt;"",P382="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A382="","",IF(AND(AK382="OK",J382="READY",F382&lt;&gt;"",G382&lt;&gt;"",K382&lt;&gt;"",OR(L382="PASS",L382="FAIL"),M382&lt;&gt;"",P382="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM382" s="9" t="str">
         <x:f>IF(A382="","",IF(AND(AK382="OK",J382="READY",F382&lt;&gt;"",G382&lt;&gt;"",K382&lt;&gt;"",S382="OK",OR(R382="PASS",R382="FAIL")),"YES","NO"))</x:f>
@@ -20845,7 +20845,7 @@
         <x:f>IF(A383="",IF(B383="","","MISSING_TEST_ID"),IF(B383="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A383,$B$2:$B$501,B383)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL383" s="9" t="str">
-        <x:f>IF(A383="","",IF(AND(AK383="OK",J383="READY",F383&lt;&gt;"",G383&lt;&gt;"",K383&lt;&gt;"",OR(L383="PASS",L383="FAIL"),M383&lt;&gt;"",O383&lt;&gt;"",P383="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A383="","",IF(AND(AK383="OK",J383="READY",F383&lt;&gt;"",G383&lt;&gt;"",K383&lt;&gt;"",OR(L383="PASS",L383="FAIL"),M383&lt;&gt;"",P383="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM383" s="9" t="str">
         <x:f>IF(A383="","",IF(AND(AK383="OK",J383="READY",F383&lt;&gt;"",G383&lt;&gt;"",K383&lt;&gt;"",S383="OK",OR(R383="PASS",R383="FAIL")),"YES","NO"))</x:f>
@@ -20897,7 +20897,7 @@
         <x:f>IF(A384="",IF(B384="","","MISSING_TEST_ID"),IF(B384="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A384,$B$2:$B$501,B384)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL384" s="9" t="str">
-        <x:f>IF(A384="","",IF(AND(AK384="OK",J384="READY",F384&lt;&gt;"",G384&lt;&gt;"",K384&lt;&gt;"",OR(L384="PASS",L384="FAIL"),M384&lt;&gt;"",O384&lt;&gt;"",P384="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A384="","",IF(AND(AK384="OK",J384="READY",F384&lt;&gt;"",G384&lt;&gt;"",K384&lt;&gt;"",OR(L384="PASS",L384="FAIL"),M384&lt;&gt;"",P384="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM384" s="9" t="str">
         <x:f>IF(A384="","",IF(AND(AK384="OK",J384="READY",F384&lt;&gt;"",G384&lt;&gt;"",K384&lt;&gt;"",S384="OK",OR(R384="PASS",R384="FAIL")),"YES","NO"))</x:f>
@@ -20949,7 +20949,7 @@
         <x:f>IF(A385="",IF(B385="","","MISSING_TEST_ID"),IF(B385="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A385,$B$2:$B$501,B385)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL385" s="9" t="str">
-        <x:f>IF(A385="","",IF(AND(AK385="OK",J385="READY",F385&lt;&gt;"",G385&lt;&gt;"",K385&lt;&gt;"",OR(L385="PASS",L385="FAIL"),M385&lt;&gt;"",O385&lt;&gt;"",P385="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A385="","",IF(AND(AK385="OK",J385="READY",F385&lt;&gt;"",G385&lt;&gt;"",K385&lt;&gt;"",OR(L385="PASS",L385="FAIL"),M385&lt;&gt;"",P385="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM385" s="9" t="str">
         <x:f>IF(A385="","",IF(AND(AK385="OK",J385="READY",F385&lt;&gt;"",G385&lt;&gt;"",K385&lt;&gt;"",S385="OK",OR(R385="PASS",R385="FAIL")),"YES","NO"))</x:f>
@@ -21001,7 +21001,7 @@
         <x:f>IF(A386="",IF(B386="","","MISSING_TEST_ID"),IF(B386="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A386,$B$2:$B$501,B386)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL386" s="9" t="str">
-        <x:f>IF(A386="","",IF(AND(AK386="OK",J386="READY",F386&lt;&gt;"",G386&lt;&gt;"",K386&lt;&gt;"",OR(L386="PASS",L386="FAIL"),M386&lt;&gt;"",O386&lt;&gt;"",P386="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A386="","",IF(AND(AK386="OK",J386="READY",F386&lt;&gt;"",G386&lt;&gt;"",K386&lt;&gt;"",OR(L386="PASS",L386="FAIL"),M386&lt;&gt;"",P386="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM386" s="9" t="str">
         <x:f>IF(A386="","",IF(AND(AK386="OK",J386="READY",F386&lt;&gt;"",G386&lt;&gt;"",K386&lt;&gt;"",S386="OK",OR(R386="PASS",R386="FAIL")),"YES","NO"))</x:f>
@@ -21053,7 +21053,7 @@
         <x:f>IF(A387="",IF(B387="","","MISSING_TEST_ID"),IF(B387="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A387,$B$2:$B$501,B387)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL387" s="9" t="str">
-        <x:f>IF(A387="","",IF(AND(AK387="OK",J387="READY",F387&lt;&gt;"",G387&lt;&gt;"",K387&lt;&gt;"",OR(L387="PASS",L387="FAIL"),M387&lt;&gt;"",O387&lt;&gt;"",P387="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A387="","",IF(AND(AK387="OK",J387="READY",F387&lt;&gt;"",G387&lt;&gt;"",K387&lt;&gt;"",OR(L387="PASS",L387="FAIL"),M387&lt;&gt;"",P387="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM387" s="9" t="str">
         <x:f>IF(A387="","",IF(AND(AK387="OK",J387="READY",F387&lt;&gt;"",G387&lt;&gt;"",K387&lt;&gt;"",S387="OK",OR(R387="PASS",R387="FAIL")),"YES","NO"))</x:f>
@@ -21105,7 +21105,7 @@
         <x:f>IF(A388="",IF(B388="","","MISSING_TEST_ID"),IF(B388="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A388,$B$2:$B$501,B388)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL388" s="9" t="str">
-        <x:f>IF(A388="","",IF(AND(AK388="OK",J388="READY",F388&lt;&gt;"",G388&lt;&gt;"",K388&lt;&gt;"",OR(L388="PASS",L388="FAIL"),M388&lt;&gt;"",O388&lt;&gt;"",P388="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A388="","",IF(AND(AK388="OK",J388="READY",F388&lt;&gt;"",G388&lt;&gt;"",K388&lt;&gt;"",OR(L388="PASS",L388="FAIL"),M388&lt;&gt;"",P388="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM388" s="9" t="str">
         <x:f>IF(A388="","",IF(AND(AK388="OK",J388="READY",F388&lt;&gt;"",G388&lt;&gt;"",K388&lt;&gt;"",S388="OK",OR(R388="PASS",R388="FAIL")),"YES","NO"))</x:f>
@@ -21157,7 +21157,7 @@
         <x:f>IF(A389="",IF(B389="","","MISSING_TEST_ID"),IF(B389="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A389,$B$2:$B$501,B389)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL389" s="9" t="str">
-        <x:f>IF(A389="","",IF(AND(AK389="OK",J389="READY",F389&lt;&gt;"",G389&lt;&gt;"",K389&lt;&gt;"",OR(L389="PASS",L389="FAIL"),M389&lt;&gt;"",O389&lt;&gt;"",P389="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A389="","",IF(AND(AK389="OK",J389="READY",F389&lt;&gt;"",G389&lt;&gt;"",K389&lt;&gt;"",OR(L389="PASS",L389="FAIL"),M389&lt;&gt;"",P389="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM389" s="9" t="str">
         <x:f>IF(A389="","",IF(AND(AK389="OK",J389="READY",F389&lt;&gt;"",G389&lt;&gt;"",K389&lt;&gt;"",S389="OK",OR(R389="PASS",R389="FAIL")),"YES","NO"))</x:f>
@@ -21209,7 +21209,7 @@
         <x:f>IF(A390="",IF(B390="","","MISSING_TEST_ID"),IF(B390="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A390,$B$2:$B$501,B390)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL390" s="9" t="str">
-        <x:f>IF(A390="","",IF(AND(AK390="OK",J390="READY",F390&lt;&gt;"",G390&lt;&gt;"",K390&lt;&gt;"",OR(L390="PASS",L390="FAIL"),M390&lt;&gt;"",O390&lt;&gt;"",P390="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A390="","",IF(AND(AK390="OK",J390="READY",F390&lt;&gt;"",G390&lt;&gt;"",K390&lt;&gt;"",OR(L390="PASS",L390="FAIL"),M390&lt;&gt;"",P390="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM390" s="9" t="str">
         <x:f>IF(A390="","",IF(AND(AK390="OK",J390="READY",F390&lt;&gt;"",G390&lt;&gt;"",K390&lt;&gt;"",S390="OK",OR(R390="PASS",R390="FAIL")),"YES","NO"))</x:f>
@@ -21261,7 +21261,7 @@
         <x:f>IF(A391="",IF(B391="","","MISSING_TEST_ID"),IF(B391="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A391,$B$2:$B$501,B391)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL391" s="9" t="str">
-        <x:f>IF(A391="","",IF(AND(AK391="OK",J391="READY",F391&lt;&gt;"",G391&lt;&gt;"",K391&lt;&gt;"",OR(L391="PASS",L391="FAIL"),M391&lt;&gt;"",O391&lt;&gt;"",P391="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A391="","",IF(AND(AK391="OK",J391="READY",F391&lt;&gt;"",G391&lt;&gt;"",K391&lt;&gt;"",OR(L391="PASS",L391="FAIL"),M391&lt;&gt;"",P391="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM391" s="9" t="str">
         <x:f>IF(A391="","",IF(AND(AK391="OK",J391="READY",F391&lt;&gt;"",G391&lt;&gt;"",K391&lt;&gt;"",S391="OK",OR(R391="PASS",R391="FAIL")),"YES","NO"))</x:f>
@@ -21313,7 +21313,7 @@
         <x:f>IF(A392="",IF(B392="","","MISSING_TEST_ID"),IF(B392="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A392,$B$2:$B$501,B392)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL392" s="9" t="str">
-        <x:f>IF(A392="","",IF(AND(AK392="OK",J392="READY",F392&lt;&gt;"",G392&lt;&gt;"",K392&lt;&gt;"",OR(L392="PASS",L392="FAIL"),M392&lt;&gt;"",O392&lt;&gt;"",P392="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A392="","",IF(AND(AK392="OK",J392="READY",F392&lt;&gt;"",G392&lt;&gt;"",K392&lt;&gt;"",OR(L392="PASS",L392="FAIL"),M392&lt;&gt;"",P392="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM392" s="9" t="str">
         <x:f>IF(A392="","",IF(AND(AK392="OK",J392="READY",F392&lt;&gt;"",G392&lt;&gt;"",K392&lt;&gt;"",S392="OK",OR(R392="PASS",R392="FAIL")),"YES","NO"))</x:f>
@@ -21365,7 +21365,7 @@
         <x:f>IF(A393="",IF(B393="","","MISSING_TEST_ID"),IF(B393="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A393,$B$2:$B$501,B393)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL393" s="9" t="str">
-        <x:f>IF(A393="","",IF(AND(AK393="OK",J393="READY",F393&lt;&gt;"",G393&lt;&gt;"",K393&lt;&gt;"",OR(L393="PASS",L393="FAIL"),M393&lt;&gt;"",O393&lt;&gt;"",P393="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A393="","",IF(AND(AK393="OK",J393="READY",F393&lt;&gt;"",G393&lt;&gt;"",K393&lt;&gt;"",OR(L393="PASS",L393="FAIL"),M393&lt;&gt;"",P393="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM393" s="9" t="str">
         <x:f>IF(A393="","",IF(AND(AK393="OK",J393="READY",F393&lt;&gt;"",G393&lt;&gt;"",K393&lt;&gt;"",S393="OK",OR(R393="PASS",R393="FAIL")),"YES","NO"))</x:f>
@@ -21417,7 +21417,7 @@
         <x:f>IF(A394="",IF(B394="","","MISSING_TEST_ID"),IF(B394="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A394,$B$2:$B$501,B394)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL394" s="9" t="str">
-        <x:f>IF(A394="","",IF(AND(AK394="OK",J394="READY",F394&lt;&gt;"",G394&lt;&gt;"",K394&lt;&gt;"",OR(L394="PASS",L394="FAIL"),M394&lt;&gt;"",O394&lt;&gt;"",P394="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A394="","",IF(AND(AK394="OK",J394="READY",F394&lt;&gt;"",G394&lt;&gt;"",K394&lt;&gt;"",OR(L394="PASS",L394="FAIL"),M394&lt;&gt;"",P394="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM394" s="9" t="str">
         <x:f>IF(A394="","",IF(AND(AK394="OK",J394="READY",F394&lt;&gt;"",G394&lt;&gt;"",K394&lt;&gt;"",S394="OK",OR(R394="PASS",R394="FAIL")),"YES","NO"))</x:f>
@@ -21469,7 +21469,7 @@
         <x:f>IF(A395="",IF(B395="","","MISSING_TEST_ID"),IF(B395="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A395,$B$2:$B$501,B395)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL395" s="9" t="str">
-        <x:f>IF(A395="","",IF(AND(AK395="OK",J395="READY",F395&lt;&gt;"",G395&lt;&gt;"",K395&lt;&gt;"",OR(L395="PASS",L395="FAIL"),M395&lt;&gt;"",O395&lt;&gt;"",P395="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A395="","",IF(AND(AK395="OK",J395="READY",F395&lt;&gt;"",G395&lt;&gt;"",K395&lt;&gt;"",OR(L395="PASS",L395="FAIL"),M395&lt;&gt;"",P395="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM395" s="9" t="str">
         <x:f>IF(A395="","",IF(AND(AK395="OK",J395="READY",F395&lt;&gt;"",G395&lt;&gt;"",K395&lt;&gt;"",S395="OK",OR(R395="PASS",R395="FAIL")),"YES","NO"))</x:f>
@@ -21521,7 +21521,7 @@
         <x:f>IF(A396="",IF(B396="","","MISSING_TEST_ID"),IF(B396="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A396,$B$2:$B$501,B396)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL396" s="9" t="str">
-        <x:f>IF(A396="","",IF(AND(AK396="OK",J396="READY",F396&lt;&gt;"",G396&lt;&gt;"",K396&lt;&gt;"",OR(L396="PASS",L396="FAIL"),M396&lt;&gt;"",O396&lt;&gt;"",P396="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A396="","",IF(AND(AK396="OK",J396="READY",F396&lt;&gt;"",G396&lt;&gt;"",K396&lt;&gt;"",OR(L396="PASS",L396="FAIL"),M396&lt;&gt;"",P396="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM396" s="9" t="str">
         <x:f>IF(A396="","",IF(AND(AK396="OK",J396="READY",F396&lt;&gt;"",G396&lt;&gt;"",K396&lt;&gt;"",S396="OK",OR(R396="PASS",R396="FAIL")),"YES","NO"))</x:f>
@@ -21573,7 +21573,7 @@
         <x:f>IF(A397="",IF(B397="","","MISSING_TEST_ID"),IF(B397="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A397,$B$2:$B$501,B397)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL397" s="9" t="str">
-        <x:f>IF(A397="","",IF(AND(AK397="OK",J397="READY",F397&lt;&gt;"",G397&lt;&gt;"",K397&lt;&gt;"",OR(L397="PASS",L397="FAIL"),M397&lt;&gt;"",O397&lt;&gt;"",P397="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A397="","",IF(AND(AK397="OK",J397="READY",F397&lt;&gt;"",G397&lt;&gt;"",K397&lt;&gt;"",OR(L397="PASS",L397="FAIL"),M397&lt;&gt;"",P397="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM397" s="9" t="str">
         <x:f>IF(A397="","",IF(AND(AK397="OK",J397="READY",F397&lt;&gt;"",G397&lt;&gt;"",K397&lt;&gt;"",S397="OK",OR(R397="PASS",R397="FAIL")),"YES","NO"))</x:f>
@@ -21625,7 +21625,7 @@
         <x:f>IF(A398="",IF(B398="","","MISSING_TEST_ID"),IF(B398="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A398,$B$2:$B$501,B398)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL398" s="9" t="str">
-        <x:f>IF(A398="","",IF(AND(AK398="OK",J398="READY",F398&lt;&gt;"",G398&lt;&gt;"",K398&lt;&gt;"",OR(L398="PASS",L398="FAIL"),M398&lt;&gt;"",O398&lt;&gt;"",P398="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A398="","",IF(AND(AK398="OK",J398="READY",F398&lt;&gt;"",G398&lt;&gt;"",K398&lt;&gt;"",OR(L398="PASS",L398="FAIL"),M398&lt;&gt;"",P398="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM398" s="9" t="str">
         <x:f>IF(A398="","",IF(AND(AK398="OK",J398="READY",F398&lt;&gt;"",G398&lt;&gt;"",K398&lt;&gt;"",S398="OK",OR(R398="PASS",R398="FAIL")),"YES","NO"))</x:f>
@@ -21677,7 +21677,7 @@
         <x:f>IF(A399="",IF(B399="","","MISSING_TEST_ID"),IF(B399="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A399,$B$2:$B$501,B399)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL399" s="9" t="str">
-        <x:f>IF(A399="","",IF(AND(AK399="OK",J399="READY",F399&lt;&gt;"",G399&lt;&gt;"",K399&lt;&gt;"",OR(L399="PASS",L399="FAIL"),M399&lt;&gt;"",O399&lt;&gt;"",P399="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A399="","",IF(AND(AK399="OK",J399="READY",F399&lt;&gt;"",G399&lt;&gt;"",K399&lt;&gt;"",OR(L399="PASS",L399="FAIL"),M399&lt;&gt;"",P399="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM399" s="9" t="str">
         <x:f>IF(A399="","",IF(AND(AK399="OK",J399="READY",F399&lt;&gt;"",G399&lt;&gt;"",K399&lt;&gt;"",S399="OK",OR(R399="PASS",R399="FAIL")),"YES","NO"))</x:f>
@@ -21729,7 +21729,7 @@
         <x:f>IF(A400="",IF(B400="","","MISSING_TEST_ID"),IF(B400="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A400,$B$2:$B$501,B400)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL400" s="9" t="str">
-        <x:f>IF(A400="","",IF(AND(AK400="OK",J400="READY",F400&lt;&gt;"",G400&lt;&gt;"",K400&lt;&gt;"",OR(L400="PASS",L400="FAIL"),M400&lt;&gt;"",O400&lt;&gt;"",P400="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A400="","",IF(AND(AK400="OK",J400="READY",F400&lt;&gt;"",G400&lt;&gt;"",K400&lt;&gt;"",OR(L400="PASS",L400="FAIL"),M400&lt;&gt;"",P400="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM400" s="9" t="str">
         <x:f>IF(A400="","",IF(AND(AK400="OK",J400="READY",F400&lt;&gt;"",G400&lt;&gt;"",K400&lt;&gt;"",S400="OK",OR(R400="PASS",R400="FAIL")),"YES","NO"))</x:f>
@@ -21781,7 +21781,7 @@
         <x:f>IF(A401="",IF(B401="","","MISSING_TEST_ID"),IF(B401="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A401,$B$2:$B$501,B401)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL401" s="9" t="str">
-        <x:f>IF(A401="","",IF(AND(AK401="OK",J401="READY",F401&lt;&gt;"",G401&lt;&gt;"",K401&lt;&gt;"",OR(L401="PASS",L401="FAIL"),M401&lt;&gt;"",O401&lt;&gt;"",P401="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A401="","",IF(AND(AK401="OK",J401="READY",F401&lt;&gt;"",G401&lt;&gt;"",K401&lt;&gt;"",OR(L401="PASS",L401="FAIL"),M401&lt;&gt;"",P401="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM401" s="9" t="str">
         <x:f>IF(A401="","",IF(AND(AK401="OK",J401="READY",F401&lt;&gt;"",G401&lt;&gt;"",K401&lt;&gt;"",S401="OK",OR(R401="PASS",R401="FAIL")),"YES","NO"))</x:f>
@@ -21833,7 +21833,7 @@
         <x:f>IF(A402="",IF(B402="","","MISSING_TEST_ID"),IF(B402="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A402,$B$2:$B$501,B402)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL402" s="9" t="str">
-        <x:f>IF(A402="","",IF(AND(AK402="OK",J402="READY",F402&lt;&gt;"",G402&lt;&gt;"",K402&lt;&gt;"",OR(L402="PASS",L402="FAIL"),M402&lt;&gt;"",O402&lt;&gt;"",P402="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A402="","",IF(AND(AK402="OK",J402="READY",F402&lt;&gt;"",G402&lt;&gt;"",K402&lt;&gt;"",OR(L402="PASS",L402="FAIL"),M402&lt;&gt;"",P402="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM402" s="9" t="str">
         <x:f>IF(A402="","",IF(AND(AK402="OK",J402="READY",F402&lt;&gt;"",G402&lt;&gt;"",K402&lt;&gt;"",S402="OK",OR(R402="PASS",R402="FAIL")),"YES","NO"))</x:f>
@@ -21885,7 +21885,7 @@
         <x:f>IF(A403="",IF(B403="","","MISSING_TEST_ID"),IF(B403="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A403,$B$2:$B$501,B403)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL403" s="9" t="str">
-        <x:f>IF(A403="","",IF(AND(AK403="OK",J403="READY",F403&lt;&gt;"",G403&lt;&gt;"",K403&lt;&gt;"",OR(L403="PASS",L403="FAIL"),M403&lt;&gt;"",O403&lt;&gt;"",P403="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A403="","",IF(AND(AK403="OK",J403="READY",F403&lt;&gt;"",G403&lt;&gt;"",K403&lt;&gt;"",OR(L403="PASS",L403="FAIL"),M403&lt;&gt;"",P403="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM403" s="9" t="str">
         <x:f>IF(A403="","",IF(AND(AK403="OK",J403="READY",F403&lt;&gt;"",G403&lt;&gt;"",K403&lt;&gt;"",S403="OK",OR(R403="PASS",R403="FAIL")),"YES","NO"))</x:f>
@@ -21937,7 +21937,7 @@
         <x:f>IF(A404="",IF(B404="","","MISSING_TEST_ID"),IF(B404="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A404,$B$2:$B$501,B404)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL404" s="9" t="str">
-        <x:f>IF(A404="","",IF(AND(AK404="OK",J404="READY",F404&lt;&gt;"",G404&lt;&gt;"",K404&lt;&gt;"",OR(L404="PASS",L404="FAIL"),M404&lt;&gt;"",O404&lt;&gt;"",P404="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A404="","",IF(AND(AK404="OK",J404="READY",F404&lt;&gt;"",G404&lt;&gt;"",K404&lt;&gt;"",OR(L404="PASS",L404="FAIL"),M404&lt;&gt;"",P404="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM404" s="9" t="str">
         <x:f>IF(A404="","",IF(AND(AK404="OK",J404="READY",F404&lt;&gt;"",G404&lt;&gt;"",K404&lt;&gt;"",S404="OK",OR(R404="PASS",R404="FAIL")),"YES","NO"))</x:f>
@@ -21989,7 +21989,7 @@
         <x:f>IF(A405="",IF(B405="","","MISSING_TEST_ID"),IF(B405="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A405,$B$2:$B$501,B405)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL405" s="9" t="str">
-        <x:f>IF(A405="","",IF(AND(AK405="OK",J405="READY",F405&lt;&gt;"",G405&lt;&gt;"",K405&lt;&gt;"",OR(L405="PASS",L405="FAIL"),M405&lt;&gt;"",O405&lt;&gt;"",P405="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A405="","",IF(AND(AK405="OK",J405="READY",F405&lt;&gt;"",G405&lt;&gt;"",K405&lt;&gt;"",OR(L405="PASS",L405="FAIL"),M405&lt;&gt;"",P405="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM405" s="9" t="str">
         <x:f>IF(A405="","",IF(AND(AK405="OK",J405="READY",F405&lt;&gt;"",G405&lt;&gt;"",K405&lt;&gt;"",S405="OK",OR(R405="PASS",R405="FAIL")),"YES","NO"))</x:f>
@@ -22041,7 +22041,7 @@
         <x:f>IF(A406="",IF(B406="","","MISSING_TEST_ID"),IF(B406="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A406,$B$2:$B$501,B406)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL406" s="9" t="str">
-        <x:f>IF(A406="","",IF(AND(AK406="OK",J406="READY",F406&lt;&gt;"",G406&lt;&gt;"",K406&lt;&gt;"",OR(L406="PASS",L406="FAIL"),M406&lt;&gt;"",O406&lt;&gt;"",P406="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A406="","",IF(AND(AK406="OK",J406="READY",F406&lt;&gt;"",G406&lt;&gt;"",K406&lt;&gt;"",OR(L406="PASS",L406="FAIL"),M406&lt;&gt;"",P406="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM406" s="9" t="str">
         <x:f>IF(A406="","",IF(AND(AK406="OK",J406="READY",F406&lt;&gt;"",G406&lt;&gt;"",K406&lt;&gt;"",S406="OK",OR(R406="PASS",R406="FAIL")),"YES","NO"))</x:f>
@@ -22093,7 +22093,7 @@
         <x:f>IF(A407="",IF(B407="","","MISSING_TEST_ID"),IF(B407="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A407,$B$2:$B$501,B407)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL407" s="9" t="str">
-        <x:f>IF(A407="","",IF(AND(AK407="OK",J407="READY",F407&lt;&gt;"",G407&lt;&gt;"",K407&lt;&gt;"",OR(L407="PASS",L407="FAIL"),M407&lt;&gt;"",O407&lt;&gt;"",P407="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A407="","",IF(AND(AK407="OK",J407="READY",F407&lt;&gt;"",G407&lt;&gt;"",K407&lt;&gt;"",OR(L407="PASS",L407="FAIL"),M407&lt;&gt;"",P407="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM407" s="9" t="str">
         <x:f>IF(A407="","",IF(AND(AK407="OK",J407="READY",F407&lt;&gt;"",G407&lt;&gt;"",K407&lt;&gt;"",S407="OK",OR(R407="PASS",R407="FAIL")),"YES","NO"))</x:f>
@@ -22145,7 +22145,7 @@
         <x:f>IF(A408="",IF(B408="","","MISSING_TEST_ID"),IF(B408="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A408,$B$2:$B$501,B408)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL408" s="9" t="str">
-        <x:f>IF(A408="","",IF(AND(AK408="OK",J408="READY",F408&lt;&gt;"",G408&lt;&gt;"",K408&lt;&gt;"",OR(L408="PASS",L408="FAIL"),M408&lt;&gt;"",O408&lt;&gt;"",P408="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A408="","",IF(AND(AK408="OK",J408="READY",F408&lt;&gt;"",G408&lt;&gt;"",K408&lt;&gt;"",OR(L408="PASS",L408="FAIL"),M408&lt;&gt;"",P408="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM408" s="9" t="str">
         <x:f>IF(A408="","",IF(AND(AK408="OK",J408="READY",F408&lt;&gt;"",G408&lt;&gt;"",K408&lt;&gt;"",S408="OK",OR(R408="PASS",R408="FAIL")),"YES","NO"))</x:f>
@@ -22197,7 +22197,7 @@
         <x:f>IF(A409="",IF(B409="","","MISSING_TEST_ID"),IF(B409="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A409,$B$2:$B$501,B409)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL409" s="9" t="str">
-        <x:f>IF(A409="","",IF(AND(AK409="OK",J409="READY",F409&lt;&gt;"",G409&lt;&gt;"",K409&lt;&gt;"",OR(L409="PASS",L409="FAIL"),M409&lt;&gt;"",O409&lt;&gt;"",P409="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A409="","",IF(AND(AK409="OK",J409="READY",F409&lt;&gt;"",G409&lt;&gt;"",K409&lt;&gt;"",OR(L409="PASS",L409="FAIL"),M409&lt;&gt;"",P409="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM409" s="9" t="str">
         <x:f>IF(A409="","",IF(AND(AK409="OK",J409="READY",F409&lt;&gt;"",G409&lt;&gt;"",K409&lt;&gt;"",S409="OK",OR(R409="PASS",R409="FAIL")),"YES","NO"))</x:f>
@@ -22249,7 +22249,7 @@
         <x:f>IF(A410="",IF(B410="","","MISSING_TEST_ID"),IF(B410="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A410,$B$2:$B$501,B410)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL410" s="9" t="str">
-        <x:f>IF(A410="","",IF(AND(AK410="OK",J410="READY",F410&lt;&gt;"",G410&lt;&gt;"",K410&lt;&gt;"",OR(L410="PASS",L410="FAIL"),M410&lt;&gt;"",O410&lt;&gt;"",P410="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A410="","",IF(AND(AK410="OK",J410="READY",F410&lt;&gt;"",G410&lt;&gt;"",K410&lt;&gt;"",OR(L410="PASS",L410="FAIL"),M410&lt;&gt;"",P410="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM410" s="9" t="str">
         <x:f>IF(A410="","",IF(AND(AK410="OK",J410="READY",F410&lt;&gt;"",G410&lt;&gt;"",K410&lt;&gt;"",S410="OK",OR(R410="PASS",R410="FAIL")),"YES","NO"))</x:f>
@@ -22301,7 +22301,7 @@
         <x:f>IF(A411="",IF(B411="","","MISSING_TEST_ID"),IF(B411="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A411,$B$2:$B$501,B411)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL411" s="9" t="str">
-        <x:f>IF(A411="","",IF(AND(AK411="OK",J411="READY",F411&lt;&gt;"",G411&lt;&gt;"",K411&lt;&gt;"",OR(L411="PASS",L411="FAIL"),M411&lt;&gt;"",O411&lt;&gt;"",P411="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A411="","",IF(AND(AK411="OK",J411="READY",F411&lt;&gt;"",G411&lt;&gt;"",K411&lt;&gt;"",OR(L411="PASS",L411="FAIL"),M411&lt;&gt;"",P411="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM411" s="9" t="str">
         <x:f>IF(A411="","",IF(AND(AK411="OK",J411="READY",F411&lt;&gt;"",G411&lt;&gt;"",K411&lt;&gt;"",S411="OK",OR(R411="PASS",R411="FAIL")),"YES","NO"))</x:f>
@@ -22353,7 +22353,7 @@
         <x:f>IF(A412="",IF(B412="","","MISSING_TEST_ID"),IF(B412="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A412,$B$2:$B$501,B412)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL412" s="9" t="str">
-        <x:f>IF(A412="","",IF(AND(AK412="OK",J412="READY",F412&lt;&gt;"",G412&lt;&gt;"",K412&lt;&gt;"",OR(L412="PASS",L412="FAIL"),M412&lt;&gt;"",O412&lt;&gt;"",P412="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A412="","",IF(AND(AK412="OK",J412="READY",F412&lt;&gt;"",G412&lt;&gt;"",K412&lt;&gt;"",OR(L412="PASS",L412="FAIL"),M412&lt;&gt;"",P412="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM412" s="9" t="str">
         <x:f>IF(A412="","",IF(AND(AK412="OK",J412="READY",F412&lt;&gt;"",G412&lt;&gt;"",K412&lt;&gt;"",S412="OK",OR(R412="PASS",R412="FAIL")),"YES","NO"))</x:f>
@@ -22405,7 +22405,7 @@
         <x:f>IF(A413="",IF(B413="","","MISSING_TEST_ID"),IF(B413="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A413,$B$2:$B$501,B413)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL413" s="9" t="str">
-        <x:f>IF(A413="","",IF(AND(AK413="OK",J413="READY",F413&lt;&gt;"",G413&lt;&gt;"",K413&lt;&gt;"",OR(L413="PASS",L413="FAIL"),M413&lt;&gt;"",O413&lt;&gt;"",P413="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A413="","",IF(AND(AK413="OK",J413="READY",F413&lt;&gt;"",G413&lt;&gt;"",K413&lt;&gt;"",OR(L413="PASS",L413="FAIL"),M413&lt;&gt;"",P413="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM413" s="9" t="str">
         <x:f>IF(A413="","",IF(AND(AK413="OK",J413="READY",F413&lt;&gt;"",G413&lt;&gt;"",K413&lt;&gt;"",S413="OK",OR(R413="PASS",R413="FAIL")),"YES","NO"))</x:f>
@@ -22457,7 +22457,7 @@
         <x:f>IF(A414="",IF(B414="","","MISSING_TEST_ID"),IF(B414="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A414,$B$2:$B$501,B414)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL414" s="9" t="str">
-        <x:f>IF(A414="","",IF(AND(AK414="OK",J414="READY",F414&lt;&gt;"",G414&lt;&gt;"",K414&lt;&gt;"",OR(L414="PASS",L414="FAIL"),M414&lt;&gt;"",O414&lt;&gt;"",P414="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A414="","",IF(AND(AK414="OK",J414="READY",F414&lt;&gt;"",G414&lt;&gt;"",K414&lt;&gt;"",OR(L414="PASS",L414="FAIL"),M414&lt;&gt;"",P414="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM414" s="9" t="str">
         <x:f>IF(A414="","",IF(AND(AK414="OK",J414="READY",F414&lt;&gt;"",G414&lt;&gt;"",K414&lt;&gt;"",S414="OK",OR(R414="PASS",R414="FAIL")),"YES","NO"))</x:f>
@@ -22509,7 +22509,7 @@
         <x:f>IF(A415="",IF(B415="","","MISSING_TEST_ID"),IF(B415="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A415,$B$2:$B$501,B415)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL415" s="9" t="str">
-        <x:f>IF(A415="","",IF(AND(AK415="OK",J415="READY",F415&lt;&gt;"",G415&lt;&gt;"",K415&lt;&gt;"",OR(L415="PASS",L415="FAIL"),M415&lt;&gt;"",O415&lt;&gt;"",P415="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A415="","",IF(AND(AK415="OK",J415="READY",F415&lt;&gt;"",G415&lt;&gt;"",K415&lt;&gt;"",OR(L415="PASS",L415="FAIL"),M415&lt;&gt;"",P415="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM415" s="9" t="str">
         <x:f>IF(A415="","",IF(AND(AK415="OK",J415="READY",F415&lt;&gt;"",G415&lt;&gt;"",K415&lt;&gt;"",S415="OK",OR(R415="PASS",R415="FAIL")),"YES","NO"))</x:f>
@@ -22561,7 +22561,7 @@
         <x:f>IF(A416="",IF(B416="","","MISSING_TEST_ID"),IF(B416="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A416,$B$2:$B$501,B416)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL416" s="9" t="str">
-        <x:f>IF(A416="","",IF(AND(AK416="OK",J416="READY",F416&lt;&gt;"",G416&lt;&gt;"",K416&lt;&gt;"",OR(L416="PASS",L416="FAIL"),M416&lt;&gt;"",O416&lt;&gt;"",P416="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A416="","",IF(AND(AK416="OK",J416="READY",F416&lt;&gt;"",G416&lt;&gt;"",K416&lt;&gt;"",OR(L416="PASS",L416="FAIL"),M416&lt;&gt;"",P416="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM416" s="9" t="str">
         <x:f>IF(A416="","",IF(AND(AK416="OK",J416="READY",F416&lt;&gt;"",G416&lt;&gt;"",K416&lt;&gt;"",S416="OK",OR(R416="PASS",R416="FAIL")),"YES","NO"))</x:f>
@@ -22613,7 +22613,7 @@
         <x:f>IF(A417="",IF(B417="","","MISSING_TEST_ID"),IF(B417="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A417,$B$2:$B$501,B417)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL417" s="9" t="str">
-        <x:f>IF(A417="","",IF(AND(AK417="OK",J417="READY",F417&lt;&gt;"",G417&lt;&gt;"",K417&lt;&gt;"",OR(L417="PASS",L417="FAIL"),M417&lt;&gt;"",O417&lt;&gt;"",P417="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A417="","",IF(AND(AK417="OK",J417="READY",F417&lt;&gt;"",G417&lt;&gt;"",K417&lt;&gt;"",OR(L417="PASS",L417="FAIL"),M417&lt;&gt;"",P417="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM417" s="9" t="str">
         <x:f>IF(A417="","",IF(AND(AK417="OK",J417="READY",F417&lt;&gt;"",G417&lt;&gt;"",K417&lt;&gt;"",S417="OK",OR(R417="PASS",R417="FAIL")),"YES","NO"))</x:f>
@@ -22665,7 +22665,7 @@
         <x:f>IF(A418="",IF(B418="","","MISSING_TEST_ID"),IF(B418="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A418,$B$2:$B$501,B418)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL418" s="9" t="str">
-        <x:f>IF(A418="","",IF(AND(AK418="OK",J418="READY",F418&lt;&gt;"",G418&lt;&gt;"",K418&lt;&gt;"",OR(L418="PASS",L418="FAIL"),M418&lt;&gt;"",O418&lt;&gt;"",P418="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A418="","",IF(AND(AK418="OK",J418="READY",F418&lt;&gt;"",G418&lt;&gt;"",K418&lt;&gt;"",OR(L418="PASS",L418="FAIL"),M418&lt;&gt;"",P418="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM418" s="9" t="str">
         <x:f>IF(A418="","",IF(AND(AK418="OK",J418="READY",F418&lt;&gt;"",G418&lt;&gt;"",K418&lt;&gt;"",S418="OK",OR(R418="PASS",R418="FAIL")),"YES","NO"))</x:f>
@@ -22717,7 +22717,7 @@
         <x:f>IF(A419="",IF(B419="","","MISSING_TEST_ID"),IF(B419="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A419,$B$2:$B$501,B419)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL419" s="9" t="str">
-        <x:f>IF(A419="","",IF(AND(AK419="OK",J419="READY",F419&lt;&gt;"",G419&lt;&gt;"",K419&lt;&gt;"",OR(L419="PASS",L419="FAIL"),M419&lt;&gt;"",O419&lt;&gt;"",P419="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A419="","",IF(AND(AK419="OK",J419="READY",F419&lt;&gt;"",G419&lt;&gt;"",K419&lt;&gt;"",OR(L419="PASS",L419="FAIL"),M419&lt;&gt;"",P419="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM419" s="9" t="str">
         <x:f>IF(A419="","",IF(AND(AK419="OK",J419="READY",F419&lt;&gt;"",G419&lt;&gt;"",K419&lt;&gt;"",S419="OK",OR(R419="PASS",R419="FAIL")),"YES","NO"))</x:f>
@@ -22769,7 +22769,7 @@
         <x:f>IF(A420="",IF(B420="","","MISSING_TEST_ID"),IF(B420="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A420,$B$2:$B$501,B420)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL420" s="9" t="str">
-        <x:f>IF(A420="","",IF(AND(AK420="OK",J420="READY",F420&lt;&gt;"",G420&lt;&gt;"",K420&lt;&gt;"",OR(L420="PASS",L420="FAIL"),M420&lt;&gt;"",O420&lt;&gt;"",P420="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A420="","",IF(AND(AK420="OK",J420="READY",F420&lt;&gt;"",G420&lt;&gt;"",K420&lt;&gt;"",OR(L420="PASS",L420="FAIL"),M420&lt;&gt;"",P420="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM420" s="9" t="str">
         <x:f>IF(A420="","",IF(AND(AK420="OK",J420="READY",F420&lt;&gt;"",G420&lt;&gt;"",K420&lt;&gt;"",S420="OK",OR(R420="PASS",R420="FAIL")),"YES","NO"))</x:f>
@@ -22821,7 +22821,7 @@
         <x:f>IF(A421="",IF(B421="","","MISSING_TEST_ID"),IF(B421="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A421,$B$2:$B$501,B421)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL421" s="9" t="str">
-        <x:f>IF(A421="","",IF(AND(AK421="OK",J421="READY",F421&lt;&gt;"",G421&lt;&gt;"",K421&lt;&gt;"",OR(L421="PASS",L421="FAIL"),M421&lt;&gt;"",O421&lt;&gt;"",P421="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A421="","",IF(AND(AK421="OK",J421="READY",F421&lt;&gt;"",G421&lt;&gt;"",K421&lt;&gt;"",OR(L421="PASS",L421="FAIL"),M421&lt;&gt;"",P421="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM421" s="9" t="str">
         <x:f>IF(A421="","",IF(AND(AK421="OK",J421="READY",F421&lt;&gt;"",G421&lt;&gt;"",K421&lt;&gt;"",S421="OK",OR(R421="PASS",R421="FAIL")),"YES","NO"))</x:f>
@@ -22873,7 +22873,7 @@
         <x:f>IF(A422="",IF(B422="","","MISSING_TEST_ID"),IF(B422="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A422,$B$2:$B$501,B422)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL422" s="9" t="str">
-        <x:f>IF(A422="","",IF(AND(AK422="OK",J422="READY",F422&lt;&gt;"",G422&lt;&gt;"",K422&lt;&gt;"",OR(L422="PASS",L422="FAIL"),M422&lt;&gt;"",O422&lt;&gt;"",P422="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A422="","",IF(AND(AK422="OK",J422="READY",F422&lt;&gt;"",G422&lt;&gt;"",K422&lt;&gt;"",OR(L422="PASS",L422="FAIL"),M422&lt;&gt;"",P422="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM422" s="9" t="str">
         <x:f>IF(A422="","",IF(AND(AK422="OK",J422="READY",F422&lt;&gt;"",G422&lt;&gt;"",K422&lt;&gt;"",S422="OK",OR(R422="PASS",R422="FAIL")),"YES","NO"))</x:f>
@@ -22925,7 +22925,7 @@
         <x:f>IF(A423="",IF(B423="","","MISSING_TEST_ID"),IF(B423="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A423,$B$2:$B$501,B423)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL423" s="9" t="str">
-        <x:f>IF(A423="","",IF(AND(AK423="OK",J423="READY",F423&lt;&gt;"",G423&lt;&gt;"",K423&lt;&gt;"",OR(L423="PASS",L423="FAIL"),M423&lt;&gt;"",O423&lt;&gt;"",P423="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A423="","",IF(AND(AK423="OK",J423="READY",F423&lt;&gt;"",G423&lt;&gt;"",K423&lt;&gt;"",OR(L423="PASS",L423="FAIL"),M423&lt;&gt;"",P423="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM423" s="9" t="str">
         <x:f>IF(A423="","",IF(AND(AK423="OK",J423="READY",F423&lt;&gt;"",G423&lt;&gt;"",K423&lt;&gt;"",S423="OK",OR(R423="PASS",R423="FAIL")),"YES","NO"))</x:f>
@@ -22977,7 +22977,7 @@
         <x:f>IF(A424="",IF(B424="","","MISSING_TEST_ID"),IF(B424="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A424,$B$2:$B$501,B424)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL424" s="9" t="str">
-        <x:f>IF(A424="","",IF(AND(AK424="OK",J424="READY",F424&lt;&gt;"",G424&lt;&gt;"",K424&lt;&gt;"",OR(L424="PASS",L424="FAIL"),M424&lt;&gt;"",O424&lt;&gt;"",P424="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A424="","",IF(AND(AK424="OK",J424="READY",F424&lt;&gt;"",G424&lt;&gt;"",K424&lt;&gt;"",OR(L424="PASS",L424="FAIL"),M424&lt;&gt;"",P424="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM424" s="9" t="str">
         <x:f>IF(A424="","",IF(AND(AK424="OK",J424="READY",F424&lt;&gt;"",G424&lt;&gt;"",K424&lt;&gt;"",S424="OK",OR(R424="PASS",R424="FAIL")),"YES","NO"))</x:f>
@@ -23029,7 +23029,7 @@
         <x:f>IF(A425="",IF(B425="","","MISSING_TEST_ID"),IF(B425="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A425,$B$2:$B$501,B425)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL425" s="9" t="str">
-        <x:f>IF(A425="","",IF(AND(AK425="OK",J425="READY",F425&lt;&gt;"",G425&lt;&gt;"",K425&lt;&gt;"",OR(L425="PASS",L425="FAIL"),M425&lt;&gt;"",O425&lt;&gt;"",P425="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A425="","",IF(AND(AK425="OK",J425="READY",F425&lt;&gt;"",G425&lt;&gt;"",K425&lt;&gt;"",OR(L425="PASS",L425="FAIL"),M425&lt;&gt;"",P425="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM425" s="9" t="str">
         <x:f>IF(A425="","",IF(AND(AK425="OK",J425="READY",F425&lt;&gt;"",G425&lt;&gt;"",K425&lt;&gt;"",S425="OK",OR(R425="PASS",R425="FAIL")),"YES","NO"))</x:f>
@@ -23081,7 +23081,7 @@
         <x:f>IF(A426="",IF(B426="","","MISSING_TEST_ID"),IF(B426="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A426,$B$2:$B$501,B426)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL426" s="9" t="str">
-        <x:f>IF(A426="","",IF(AND(AK426="OK",J426="READY",F426&lt;&gt;"",G426&lt;&gt;"",K426&lt;&gt;"",OR(L426="PASS",L426="FAIL"),M426&lt;&gt;"",O426&lt;&gt;"",P426="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A426="","",IF(AND(AK426="OK",J426="READY",F426&lt;&gt;"",G426&lt;&gt;"",K426&lt;&gt;"",OR(L426="PASS",L426="FAIL"),M426&lt;&gt;"",P426="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM426" s="9" t="str">
         <x:f>IF(A426="","",IF(AND(AK426="OK",J426="READY",F426&lt;&gt;"",G426&lt;&gt;"",K426&lt;&gt;"",S426="OK",OR(R426="PASS",R426="FAIL")),"YES","NO"))</x:f>
@@ -23133,7 +23133,7 @@
         <x:f>IF(A427="",IF(B427="","","MISSING_TEST_ID"),IF(B427="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A427,$B$2:$B$501,B427)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL427" s="9" t="str">
-        <x:f>IF(A427="","",IF(AND(AK427="OK",J427="READY",F427&lt;&gt;"",G427&lt;&gt;"",K427&lt;&gt;"",OR(L427="PASS",L427="FAIL"),M427&lt;&gt;"",O427&lt;&gt;"",P427="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A427="","",IF(AND(AK427="OK",J427="READY",F427&lt;&gt;"",G427&lt;&gt;"",K427&lt;&gt;"",OR(L427="PASS",L427="FAIL"),M427&lt;&gt;"",P427="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM427" s="9" t="str">
         <x:f>IF(A427="","",IF(AND(AK427="OK",J427="READY",F427&lt;&gt;"",G427&lt;&gt;"",K427&lt;&gt;"",S427="OK",OR(R427="PASS",R427="FAIL")),"YES","NO"))</x:f>
@@ -23185,7 +23185,7 @@
         <x:f>IF(A428="",IF(B428="","","MISSING_TEST_ID"),IF(B428="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A428,$B$2:$B$501,B428)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL428" s="9" t="str">
-        <x:f>IF(A428="","",IF(AND(AK428="OK",J428="READY",F428&lt;&gt;"",G428&lt;&gt;"",K428&lt;&gt;"",OR(L428="PASS",L428="FAIL"),M428&lt;&gt;"",O428&lt;&gt;"",P428="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A428="","",IF(AND(AK428="OK",J428="READY",F428&lt;&gt;"",G428&lt;&gt;"",K428&lt;&gt;"",OR(L428="PASS",L428="FAIL"),M428&lt;&gt;"",P428="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM428" s="9" t="str">
         <x:f>IF(A428="","",IF(AND(AK428="OK",J428="READY",F428&lt;&gt;"",G428&lt;&gt;"",K428&lt;&gt;"",S428="OK",OR(R428="PASS",R428="FAIL")),"YES","NO"))</x:f>
@@ -23237,7 +23237,7 @@
         <x:f>IF(A429="",IF(B429="","","MISSING_TEST_ID"),IF(B429="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A429,$B$2:$B$501,B429)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL429" s="9" t="str">
-        <x:f>IF(A429="","",IF(AND(AK429="OK",J429="READY",F429&lt;&gt;"",G429&lt;&gt;"",K429&lt;&gt;"",OR(L429="PASS",L429="FAIL"),M429&lt;&gt;"",O429&lt;&gt;"",P429="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A429="","",IF(AND(AK429="OK",J429="READY",F429&lt;&gt;"",G429&lt;&gt;"",K429&lt;&gt;"",OR(L429="PASS",L429="FAIL"),M429&lt;&gt;"",P429="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM429" s="9" t="str">
         <x:f>IF(A429="","",IF(AND(AK429="OK",J429="READY",F429&lt;&gt;"",G429&lt;&gt;"",K429&lt;&gt;"",S429="OK",OR(R429="PASS",R429="FAIL")),"YES","NO"))</x:f>
@@ -23289,7 +23289,7 @@
         <x:f>IF(A430="",IF(B430="","","MISSING_TEST_ID"),IF(B430="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A430,$B$2:$B$501,B430)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL430" s="9" t="str">
-        <x:f>IF(A430="","",IF(AND(AK430="OK",J430="READY",F430&lt;&gt;"",G430&lt;&gt;"",K430&lt;&gt;"",OR(L430="PASS",L430="FAIL"),M430&lt;&gt;"",O430&lt;&gt;"",P430="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A430="","",IF(AND(AK430="OK",J430="READY",F430&lt;&gt;"",G430&lt;&gt;"",K430&lt;&gt;"",OR(L430="PASS",L430="FAIL"),M430&lt;&gt;"",P430="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM430" s="9" t="str">
         <x:f>IF(A430="","",IF(AND(AK430="OK",J430="READY",F430&lt;&gt;"",G430&lt;&gt;"",K430&lt;&gt;"",S430="OK",OR(R430="PASS",R430="FAIL")),"YES","NO"))</x:f>
@@ -23341,7 +23341,7 @@
         <x:f>IF(A431="",IF(B431="","","MISSING_TEST_ID"),IF(B431="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A431,$B$2:$B$501,B431)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL431" s="9" t="str">
-        <x:f>IF(A431="","",IF(AND(AK431="OK",J431="READY",F431&lt;&gt;"",G431&lt;&gt;"",K431&lt;&gt;"",OR(L431="PASS",L431="FAIL"),M431&lt;&gt;"",O431&lt;&gt;"",P431="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A431="","",IF(AND(AK431="OK",J431="READY",F431&lt;&gt;"",G431&lt;&gt;"",K431&lt;&gt;"",OR(L431="PASS",L431="FAIL"),M431&lt;&gt;"",P431="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM431" s="9" t="str">
         <x:f>IF(A431="","",IF(AND(AK431="OK",J431="READY",F431&lt;&gt;"",G431&lt;&gt;"",K431&lt;&gt;"",S431="OK",OR(R431="PASS",R431="FAIL")),"YES","NO"))</x:f>
@@ -23393,7 +23393,7 @@
         <x:f>IF(A432="",IF(B432="","","MISSING_TEST_ID"),IF(B432="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A432,$B$2:$B$501,B432)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL432" s="9" t="str">
-        <x:f>IF(A432="","",IF(AND(AK432="OK",J432="READY",F432&lt;&gt;"",G432&lt;&gt;"",K432&lt;&gt;"",OR(L432="PASS",L432="FAIL"),M432&lt;&gt;"",O432&lt;&gt;"",P432="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A432="","",IF(AND(AK432="OK",J432="READY",F432&lt;&gt;"",G432&lt;&gt;"",K432&lt;&gt;"",OR(L432="PASS",L432="FAIL"),M432&lt;&gt;"",P432="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM432" s="9" t="str">
         <x:f>IF(A432="","",IF(AND(AK432="OK",J432="READY",F432&lt;&gt;"",G432&lt;&gt;"",K432&lt;&gt;"",S432="OK",OR(R432="PASS",R432="FAIL")),"YES","NO"))</x:f>
@@ -23445,7 +23445,7 @@
         <x:f>IF(A433="",IF(B433="","","MISSING_TEST_ID"),IF(B433="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A433,$B$2:$B$501,B433)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL433" s="9" t="str">
-        <x:f>IF(A433="","",IF(AND(AK433="OK",J433="READY",F433&lt;&gt;"",G433&lt;&gt;"",K433&lt;&gt;"",OR(L433="PASS",L433="FAIL"),M433&lt;&gt;"",O433&lt;&gt;"",P433="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A433="","",IF(AND(AK433="OK",J433="READY",F433&lt;&gt;"",G433&lt;&gt;"",K433&lt;&gt;"",OR(L433="PASS",L433="FAIL"),M433&lt;&gt;"",P433="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM433" s="9" t="str">
         <x:f>IF(A433="","",IF(AND(AK433="OK",J433="READY",F433&lt;&gt;"",G433&lt;&gt;"",K433&lt;&gt;"",S433="OK",OR(R433="PASS",R433="FAIL")),"YES","NO"))</x:f>
@@ -23497,7 +23497,7 @@
         <x:f>IF(A434="",IF(B434="","","MISSING_TEST_ID"),IF(B434="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A434,$B$2:$B$501,B434)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL434" s="9" t="str">
-        <x:f>IF(A434="","",IF(AND(AK434="OK",J434="READY",F434&lt;&gt;"",G434&lt;&gt;"",K434&lt;&gt;"",OR(L434="PASS",L434="FAIL"),M434&lt;&gt;"",O434&lt;&gt;"",P434="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A434="","",IF(AND(AK434="OK",J434="READY",F434&lt;&gt;"",G434&lt;&gt;"",K434&lt;&gt;"",OR(L434="PASS",L434="FAIL"),M434&lt;&gt;"",P434="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM434" s="9" t="str">
         <x:f>IF(A434="","",IF(AND(AK434="OK",J434="READY",F434&lt;&gt;"",G434&lt;&gt;"",K434&lt;&gt;"",S434="OK",OR(R434="PASS",R434="FAIL")),"YES","NO"))</x:f>
@@ -23549,7 +23549,7 @@
         <x:f>IF(A435="",IF(B435="","","MISSING_TEST_ID"),IF(B435="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A435,$B$2:$B$501,B435)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL435" s="9" t="str">
-        <x:f>IF(A435="","",IF(AND(AK435="OK",J435="READY",F435&lt;&gt;"",G435&lt;&gt;"",K435&lt;&gt;"",OR(L435="PASS",L435="FAIL"),M435&lt;&gt;"",O435&lt;&gt;"",P435="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A435="","",IF(AND(AK435="OK",J435="READY",F435&lt;&gt;"",G435&lt;&gt;"",K435&lt;&gt;"",OR(L435="PASS",L435="FAIL"),M435&lt;&gt;"",P435="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM435" s="9" t="str">
         <x:f>IF(A435="","",IF(AND(AK435="OK",J435="READY",F435&lt;&gt;"",G435&lt;&gt;"",K435&lt;&gt;"",S435="OK",OR(R435="PASS",R435="FAIL")),"YES","NO"))</x:f>
@@ -23601,7 +23601,7 @@
         <x:f>IF(A436="",IF(B436="","","MISSING_TEST_ID"),IF(B436="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A436,$B$2:$B$501,B436)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL436" s="9" t="str">
-        <x:f>IF(A436="","",IF(AND(AK436="OK",J436="READY",F436&lt;&gt;"",G436&lt;&gt;"",K436&lt;&gt;"",OR(L436="PASS",L436="FAIL"),M436&lt;&gt;"",O436&lt;&gt;"",P436="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A436="","",IF(AND(AK436="OK",J436="READY",F436&lt;&gt;"",G436&lt;&gt;"",K436&lt;&gt;"",OR(L436="PASS",L436="FAIL"),M436&lt;&gt;"",P436="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM436" s="9" t="str">
         <x:f>IF(A436="","",IF(AND(AK436="OK",J436="READY",F436&lt;&gt;"",G436&lt;&gt;"",K436&lt;&gt;"",S436="OK",OR(R436="PASS",R436="FAIL")),"YES","NO"))</x:f>
@@ -23653,7 +23653,7 @@
         <x:f>IF(A437="",IF(B437="","","MISSING_TEST_ID"),IF(B437="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A437,$B$2:$B$501,B437)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL437" s="9" t="str">
-        <x:f>IF(A437="","",IF(AND(AK437="OK",J437="READY",F437&lt;&gt;"",G437&lt;&gt;"",K437&lt;&gt;"",OR(L437="PASS",L437="FAIL"),M437&lt;&gt;"",O437&lt;&gt;"",P437="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A437="","",IF(AND(AK437="OK",J437="READY",F437&lt;&gt;"",G437&lt;&gt;"",K437&lt;&gt;"",OR(L437="PASS",L437="FAIL"),M437&lt;&gt;"",P437="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM437" s="9" t="str">
         <x:f>IF(A437="","",IF(AND(AK437="OK",J437="READY",F437&lt;&gt;"",G437&lt;&gt;"",K437&lt;&gt;"",S437="OK",OR(R437="PASS",R437="FAIL")),"YES","NO"))</x:f>
@@ -23705,7 +23705,7 @@
         <x:f>IF(A438="",IF(B438="","","MISSING_TEST_ID"),IF(B438="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A438,$B$2:$B$501,B438)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL438" s="9" t="str">
-        <x:f>IF(A438="","",IF(AND(AK438="OK",J438="READY",F438&lt;&gt;"",G438&lt;&gt;"",K438&lt;&gt;"",OR(L438="PASS",L438="FAIL"),M438&lt;&gt;"",O438&lt;&gt;"",P438="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A438="","",IF(AND(AK438="OK",J438="READY",F438&lt;&gt;"",G438&lt;&gt;"",K438&lt;&gt;"",OR(L438="PASS",L438="FAIL"),M438&lt;&gt;"",P438="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM438" s="9" t="str">
         <x:f>IF(A438="","",IF(AND(AK438="OK",J438="READY",F438&lt;&gt;"",G438&lt;&gt;"",K438&lt;&gt;"",S438="OK",OR(R438="PASS",R438="FAIL")),"YES","NO"))</x:f>
@@ -23757,7 +23757,7 @@
         <x:f>IF(A439="",IF(B439="","","MISSING_TEST_ID"),IF(B439="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A439,$B$2:$B$501,B439)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL439" s="9" t="str">
-        <x:f>IF(A439="","",IF(AND(AK439="OK",J439="READY",F439&lt;&gt;"",G439&lt;&gt;"",K439&lt;&gt;"",OR(L439="PASS",L439="FAIL"),M439&lt;&gt;"",O439&lt;&gt;"",P439="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A439="","",IF(AND(AK439="OK",J439="READY",F439&lt;&gt;"",G439&lt;&gt;"",K439&lt;&gt;"",OR(L439="PASS",L439="FAIL"),M439&lt;&gt;"",P439="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM439" s="9" t="str">
         <x:f>IF(A439="","",IF(AND(AK439="OK",J439="READY",F439&lt;&gt;"",G439&lt;&gt;"",K439&lt;&gt;"",S439="OK",OR(R439="PASS",R439="FAIL")),"YES","NO"))</x:f>
@@ -23809,7 +23809,7 @@
         <x:f>IF(A440="",IF(B440="","","MISSING_TEST_ID"),IF(B440="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A440,$B$2:$B$501,B440)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL440" s="9" t="str">
-        <x:f>IF(A440="","",IF(AND(AK440="OK",J440="READY",F440&lt;&gt;"",G440&lt;&gt;"",K440&lt;&gt;"",OR(L440="PASS",L440="FAIL"),M440&lt;&gt;"",O440&lt;&gt;"",P440="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A440="","",IF(AND(AK440="OK",J440="READY",F440&lt;&gt;"",G440&lt;&gt;"",K440&lt;&gt;"",OR(L440="PASS",L440="FAIL"),M440&lt;&gt;"",P440="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM440" s="9" t="str">
         <x:f>IF(A440="","",IF(AND(AK440="OK",J440="READY",F440&lt;&gt;"",G440&lt;&gt;"",K440&lt;&gt;"",S440="OK",OR(R440="PASS",R440="FAIL")),"YES","NO"))</x:f>
@@ -23861,7 +23861,7 @@
         <x:f>IF(A441="",IF(B441="","","MISSING_TEST_ID"),IF(B441="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A441,$B$2:$B$501,B441)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL441" s="9" t="str">
-        <x:f>IF(A441="","",IF(AND(AK441="OK",J441="READY",F441&lt;&gt;"",G441&lt;&gt;"",K441&lt;&gt;"",OR(L441="PASS",L441="FAIL"),M441&lt;&gt;"",O441&lt;&gt;"",P441="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A441="","",IF(AND(AK441="OK",J441="READY",F441&lt;&gt;"",G441&lt;&gt;"",K441&lt;&gt;"",OR(L441="PASS",L441="FAIL"),M441&lt;&gt;"",P441="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM441" s="9" t="str">
         <x:f>IF(A441="","",IF(AND(AK441="OK",J441="READY",F441&lt;&gt;"",G441&lt;&gt;"",K441&lt;&gt;"",S441="OK",OR(R441="PASS",R441="FAIL")),"YES","NO"))</x:f>
@@ -23913,7 +23913,7 @@
         <x:f>IF(A442="",IF(B442="","","MISSING_TEST_ID"),IF(B442="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A442,$B$2:$B$501,B442)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL442" s="9" t="str">
-        <x:f>IF(A442="","",IF(AND(AK442="OK",J442="READY",F442&lt;&gt;"",G442&lt;&gt;"",K442&lt;&gt;"",OR(L442="PASS",L442="FAIL"),M442&lt;&gt;"",O442&lt;&gt;"",P442="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A442="","",IF(AND(AK442="OK",J442="READY",F442&lt;&gt;"",G442&lt;&gt;"",K442&lt;&gt;"",OR(L442="PASS",L442="FAIL"),M442&lt;&gt;"",P442="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM442" s="9" t="str">
         <x:f>IF(A442="","",IF(AND(AK442="OK",J442="READY",F442&lt;&gt;"",G442&lt;&gt;"",K442&lt;&gt;"",S442="OK",OR(R442="PASS",R442="FAIL")),"YES","NO"))</x:f>
@@ -23965,7 +23965,7 @@
         <x:f>IF(A443="",IF(B443="","","MISSING_TEST_ID"),IF(B443="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A443,$B$2:$B$501,B443)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL443" s="9" t="str">
-        <x:f>IF(A443="","",IF(AND(AK443="OK",J443="READY",F443&lt;&gt;"",G443&lt;&gt;"",K443&lt;&gt;"",OR(L443="PASS",L443="FAIL"),M443&lt;&gt;"",O443&lt;&gt;"",P443="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A443="","",IF(AND(AK443="OK",J443="READY",F443&lt;&gt;"",G443&lt;&gt;"",K443&lt;&gt;"",OR(L443="PASS",L443="FAIL"),M443&lt;&gt;"",P443="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM443" s="9" t="str">
         <x:f>IF(A443="","",IF(AND(AK443="OK",J443="READY",F443&lt;&gt;"",G443&lt;&gt;"",K443&lt;&gt;"",S443="OK",OR(R443="PASS",R443="FAIL")),"YES","NO"))</x:f>
@@ -24017,7 +24017,7 @@
         <x:f>IF(A444="",IF(B444="","","MISSING_TEST_ID"),IF(B444="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A444,$B$2:$B$501,B444)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL444" s="9" t="str">
-        <x:f>IF(A444="","",IF(AND(AK444="OK",J444="READY",F444&lt;&gt;"",G444&lt;&gt;"",K444&lt;&gt;"",OR(L444="PASS",L444="FAIL"),M444&lt;&gt;"",O444&lt;&gt;"",P444="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A444="","",IF(AND(AK444="OK",J444="READY",F444&lt;&gt;"",G444&lt;&gt;"",K444&lt;&gt;"",OR(L444="PASS",L444="FAIL"),M444&lt;&gt;"",P444="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM444" s="9" t="str">
         <x:f>IF(A444="","",IF(AND(AK444="OK",J444="READY",F444&lt;&gt;"",G444&lt;&gt;"",K444&lt;&gt;"",S444="OK",OR(R444="PASS",R444="FAIL")),"YES","NO"))</x:f>
@@ -24069,7 +24069,7 @@
         <x:f>IF(A445="",IF(B445="","","MISSING_TEST_ID"),IF(B445="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A445,$B$2:$B$501,B445)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL445" s="9" t="str">
-        <x:f>IF(A445="","",IF(AND(AK445="OK",J445="READY",F445&lt;&gt;"",G445&lt;&gt;"",K445&lt;&gt;"",OR(L445="PASS",L445="FAIL"),M445&lt;&gt;"",O445&lt;&gt;"",P445="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A445="","",IF(AND(AK445="OK",J445="READY",F445&lt;&gt;"",G445&lt;&gt;"",K445&lt;&gt;"",OR(L445="PASS",L445="FAIL"),M445&lt;&gt;"",P445="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM445" s="9" t="str">
         <x:f>IF(A445="","",IF(AND(AK445="OK",J445="READY",F445&lt;&gt;"",G445&lt;&gt;"",K445&lt;&gt;"",S445="OK",OR(R445="PASS",R445="FAIL")),"YES","NO"))</x:f>
@@ -24121,7 +24121,7 @@
         <x:f>IF(A446="",IF(B446="","","MISSING_TEST_ID"),IF(B446="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A446,$B$2:$B$501,B446)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL446" s="9" t="str">
-        <x:f>IF(A446="","",IF(AND(AK446="OK",J446="READY",F446&lt;&gt;"",G446&lt;&gt;"",K446&lt;&gt;"",OR(L446="PASS",L446="FAIL"),M446&lt;&gt;"",O446&lt;&gt;"",P446="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A446="","",IF(AND(AK446="OK",J446="READY",F446&lt;&gt;"",G446&lt;&gt;"",K446&lt;&gt;"",OR(L446="PASS",L446="FAIL"),M446&lt;&gt;"",P446="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM446" s="9" t="str">
         <x:f>IF(A446="","",IF(AND(AK446="OK",J446="READY",F446&lt;&gt;"",G446&lt;&gt;"",K446&lt;&gt;"",S446="OK",OR(R446="PASS",R446="FAIL")),"YES","NO"))</x:f>
@@ -24173,7 +24173,7 @@
         <x:f>IF(A447="",IF(B447="","","MISSING_TEST_ID"),IF(B447="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A447,$B$2:$B$501,B447)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL447" s="9" t="str">
-        <x:f>IF(A447="","",IF(AND(AK447="OK",J447="READY",F447&lt;&gt;"",G447&lt;&gt;"",K447&lt;&gt;"",OR(L447="PASS",L447="FAIL"),M447&lt;&gt;"",O447&lt;&gt;"",P447="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A447="","",IF(AND(AK447="OK",J447="READY",F447&lt;&gt;"",G447&lt;&gt;"",K447&lt;&gt;"",OR(L447="PASS",L447="FAIL"),M447&lt;&gt;"",P447="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM447" s="9" t="str">
         <x:f>IF(A447="","",IF(AND(AK447="OK",J447="READY",F447&lt;&gt;"",G447&lt;&gt;"",K447&lt;&gt;"",S447="OK",OR(R447="PASS",R447="FAIL")),"YES","NO"))</x:f>
@@ -24225,7 +24225,7 @@
         <x:f>IF(A448="",IF(B448="","","MISSING_TEST_ID"),IF(B448="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A448,$B$2:$B$501,B448)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL448" s="9" t="str">
-        <x:f>IF(A448="","",IF(AND(AK448="OK",J448="READY",F448&lt;&gt;"",G448&lt;&gt;"",K448&lt;&gt;"",OR(L448="PASS",L448="FAIL"),M448&lt;&gt;"",O448&lt;&gt;"",P448="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A448="","",IF(AND(AK448="OK",J448="READY",F448&lt;&gt;"",G448&lt;&gt;"",K448&lt;&gt;"",OR(L448="PASS",L448="FAIL"),M448&lt;&gt;"",P448="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM448" s="9" t="str">
         <x:f>IF(A448="","",IF(AND(AK448="OK",J448="READY",F448&lt;&gt;"",G448&lt;&gt;"",K448&lt;&gt;"",S448="OK",OR(R448="PASS",R448="FAIL")),"YES","NO"))</x:f>
@@ -24277,7 +24277,7 @@
         <x:f>IF(A449="",IF(B449="","","MISSING_TEST_ID"),IF(B449="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A449,$B$2:$B$501,B449)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL449" s="9" t="str">
-        <x:f>IF(A449="","",IF(AND(AK449="OK",J449="READY",F449&lt;&gt;"",G449&lt;&gt;"",K449&lt;&gt;"",OR(L449="PASS",L449="FAIL"),M449&lt;&gt;"",O449&lt;&gt;"",P449="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A449="","",IF(AND(AK449="OK",J449="READY",F449&lt;&gt;"",G449&lt;&gt;"",K449&lt;&gt;"",OR(L449="PASS",L449="FAIL"),M449&lt;&gt;"",P449="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM449" s="9" t="str">
         <x:f>IF(A449="","",IF(AND(AK449="OK",J449="READY",F449&lt;&gt;"",G449&lt;&gt;"",K449&lt;&gt;"",S449="OK",OR(R449="PASS",R449="FAIL")),"YES","NO"))</x:f>
@@ -24329,7 +24329,7 @@
         <x:f>IF(A450="",IF(B450="","","MISSING_TEST_ID"),IF(B450="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A450,$B$2:$B$501,B450)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL450" s="9" t="str">
-        <x:f>IF(A450="","",IF(AND(AK450="OK",J450="READY",F450&lt;&gt;"",G450&lt;&gt;"",K450&lt;&gt;"",OR(L450="PASS",L450="FAIL"),M450&lt;&gt;"",O450&lt;&gt;"",P450="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A450="","",IF(AND(AK450="OK",J450="READY",F450&lt;&gt;"",G450&lt;&gt;"",K450&lt;&gt;"",OR(L450="PASS",L450="FAIL"),M450&lt;&gt;"",P450="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM450" s="9" t="str">
         <x:f>IF(A450="","",IF(AND(AK450="OK",J450="READY",F450&lt;&gt;"",G450&lt;&gt;"",K450&lt;&gt;"",S450="OK",OR(R450="PASS",R450="FAIL")),"YES","NO"))</x:f>
@@ -24381,7 +24381,7 @@
         <x:f>IF(A451="",IF(B451="","","MISSING_TEST_ID"),IF(B451="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A451,$B$2:$B$501,B451)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL451" s="9" t="str">
-        <x:f>IF(A451="","",IF(AND(AK451="OK",J451="READY",F451&lt;&gt;"",G451&lt;&gt;"",K451&lt;&gt;"",OR(L451="PASS",L451="FAIL"),M451&lt;&gt;"",O451&lt;&gt;"",P451="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A451="","",IF(AND(AK451="OK",J451="READY",F451&lt;&gt;"",G451&lt;&gt;"",K451&lt;&gt;"",OR(L451="PASS",L451="FAIL"),M451&lt;&gt;"",P451="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM451" s="9" t="str">
         <x:f>IF(A451="","",IF(AND(AK451="OK",J451="READY",F451&lt;&gt;"",G451&lt;&gt;"",K451&lt;&gt;"",S451="OK",OR(R451="PASS",R451="FAIL")),"YES","NO"))</x:f>
@@ -24433,7 +24433,7 @@
         <x:f>IF(A452="",IF(B452="","","MISSING_TEST_ID"),IF(B452="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A452,$B$2:$B$501,B452)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL452" s="9" t="str">
-        <x:f>IF(A452="","",IF(AND(AK452="OK",J452="READY",F452&lt;&gt;"",G452&lt;&gt;"",K452&lt;&gt;"",OR(L452="PASS",L452="FAIL"),M452&lt;&gt;"",O452&lt;&gt;"",P452="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A452="","",IF(AND(AK452="OK",J452="READY",F452&lt;&gt;"",G452&lt;&gt;"",K452&lt;&gt;"",OR(L452="PASS",L452="FAIL"),M452&lt;&gt;"",P452="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM452" s="9" t="str">
         <x:f>IF(A452="","",IF(AND(AK452="OK",J452="READY",F452&lt;&gt;"",G452&lt;&gt;"",K452&lt;&gt;"",S452="OK",OR(R452="PASS",R452="FAIL")),"YES","NO"))</x:f>
@@ -24485,7 +24485,7 @@
         <x:f>IF(A453="",IF(B453="","","MISSING_TEST_ID"),IF(B453="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A453,$B$2:$B$501,B453)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL453" s="9" t="str">
-        <x:f>IF(A453="","",IF(AND(AK453="OK",J453="READY",F453&lt;&gt;"",G453&lt;&gt;"",K453&lt;&gt;"",OR(L453="PASS",L453="FAIL"),M453&lt;&gt;"",O453&lt;&gt;"",P453="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A453="","",IF(AND(AK453="OK",J453="READY",F453&lt;&gt;"",G453&lt;&gt;"",K453&lt;&gt;"",OR(L453="PASS",L453="FAIL"),M453&lt;&gt;"",P453="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM453" s="9" t="str">
         <x:f>IF(A453="","",IF(AND(AK453="OK",J453="READY",F453&lt;&gt;"",G453&lt;&gt;"",K453&lt;&gt;"",S453="OK",OR(R453="PASS",R453="FAIL")),"YES","NO"))</x:f>
@@ -24537,7 +24537,7 @@
         <x:f>IF(A454="",IF(B454="","","MISSING_TEST_ID"),IF(B454="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A454,$B$2:$B$501,B454)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL454" s="9" t="str">
-        <x:f>IF(A454="","",IF(AND(AK454="OK",J454="READY",F454&lt;&gt;"",G454&lt;&gt;"",K454&lt;&gt;"",OR(L454="PASS",L454="FAIL"),M454&lt;&gt;"",O454&lt;&gt;"",P454="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A454="","",IF(AND(AK454="OK",J454="READY",F454&lt;&gt;"",G454&lt;&gt;"",K454&lt;&gt;"",OR(L454="PASS",L454="FAIL"),M454&lt;&gt;"",P454="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM454" s="9" t="str">
         <x:f>IF(A454="","",IF(AND(AK454="OK",J454="READY",F454&lt;&gt;"",G454&lt;&gt;"",K454&lt;&gt;"",S454="OK",OR(R454="PASS",R454="FAIL")),"YES","NO"))</x:f>
@@ -24589,7 +24589,7 @@
         <x:f>IF(A455="",IF(B455="","","MISSING_TEST_ID"),IF(B455="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A455,$B$2:$B$501,B455)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL455" s="9" t="str">
-        <x:f>IF(A455="","",IF(AND(AK455="OK",J455="READY",F455&lt;&gt;"",G455&lt;&gt;"",K455&lt;&gt;"",OR(L455="PASS",L455="FAIL"),M455&lt;&gt;"",O455&lt;&gt;"",P455="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A455="","",IF(AND(AK455="OK",J455="READY",F455&lt;&gt;"",G455&lt;&gt;"",K455&lt;&gt;"",OR(L455="PASS",L455="FAIL"),M455&lt;&gt;"",P455="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM455" s="9" t="str">
         <x:f>IF(A455="","",IF(AND(AK455="OK",J455="READY",F455&lt;&gt;"",G455&lt;&gt;"",K455&lt;&gt;"",S455="OK",OR(R455="PASS",R455="FAIL")),"YES","NO"))</x:f>
@@ -24641,7 +24641,7 @@
         <x:f>IF(A456="",IF(B456="","","MISSING_TEST_ID"),IF(B456="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A456,$B$2:$B$501,B456)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL456" s="9" t="str">
-        <x:f>IF(A456="","",IF(AND(AK456="OK",J456="READY",F456&lt;&gt;"",G456&lt;&gt;"",K456&lt;&gt;"",OR(L456="PASS",L456="FAIL"),M456&lt;&gt;"",O456&lt;&gt;"",P456="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A456="","",IF(AND(AK456="OK",J456="READY",F456&lt;&gt;"",G456&lt;&gt;"",K456&lt;&gt;"",OR(L456="PASS",L456="FAIL"),M456&lt;&gt;"",P456="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM456" s="9" t="str">
         <x:f>IF(A456="","",IF(AND(AK456="OK",J456="READY",F456&lt;&gt;"",G456&lt;&gt;"",K456&lt;&gt;"",S456="OK",OR(R456="PASS",R456="FAIL")),"YES","NO"))</x:f>
@@ -24693,7 +24693,7 @@
         <x:f>IF(A457="",IF(B457="","","MISSING_TEST_ID"),IF(B457="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A457,$B$2:$B$501,B457)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL457" s="9" t="str">
-        <x:f>IF(A457="","",IF(AND(AK457="OK",J457="READY",F457&lt;&gt;"",G457&lt;&gt;"",K457&lt;&gt;"",OR(L457="PASS",L457="FAIL"),M457&lt;&gt;"",O457&lt;&gt;"",P457="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A457="","",IF(AND(AK457="OK",J457="READY",F457&lt;&gt;"",G457&lt;&gt;"",K457&lt;&gt;"",OR(L457="PASS",L457="FAIL"),M457&lt;&gt;"",P457="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM457" s="9" t="str">
         <x:f>IF(A457="","",IF(AND(AK457="OK",J457="READY",F457&lt;&gt;"",G457&lt;&gt;"",K457&lt;&gt;"",S457="OK",OR(R457="PASS",R457="FAIL")),"YES","NO"))</x:f>
@@ -24745,7 +24745,7 @@
         <x:f>IF(A458="",IF(B458="","","MISSING_TEST_ID"),IF(B458="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A458,$B$2:$B$501,B458)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL458" s="9" t="str">
-        <x:f>IF(A458="","",IF(AND(AK458="OK",J458="READY",F458&lt;&gt;"",G458&lt;&gt;"",K458&lt;&gt;"",OR(L458="PASS",L458="FAIL"),M458&lt;&gt;"",O458&lt;&gt;"",P458="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A458="","",IF(AND(AK458="OK",J458="READY",F458&lt;&gt;"",G458&lt;&gt;"",K458&lt;&gt;"",OR(L458="PASS",L458="FAIL"),M458&lt;&gt;"",P458="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM458" s="9" t="str">
         <x:f>IF(A458="","",IF(AND(AK458="OK",J458="READY",F458&lt;&gt;"",G458&lt;&gt;"",K458&lt;&gt;"",S458="OK",OR(R458="PASS",R458="FAIL")),"YES","NO"))</x:f>
@@ -24797,7 +24797,7 @@
         <x:f>IF(A459="",IF(B459="","","MISSING_TEST_ID"),IF(B459="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A459,$B$2:$B$501,B459)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL459" s="9" t="str">
-        <x:f>IF(A459="","",IF(AND(AK459="OK",J459="READY",F459&lt;&gt;"",G459&lt;&gt;"",K459&lt;&gt;"",OR(L459="PASS",L459="FAIL"),M459&lt;&gt;"",O459&lt;&gt;"",P459="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A459="","",IF(AND(AK459="OK",J459="READY",F459&lt;&gt;"",G459&lt;&gt;"",K459&lt;&gt;"",OR(L459="PASS",L459="FAIL"),M459&lt;&gt;"",P459="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM459" s="9" t="str">
         <x:f>IF(A459="","",IF(AND(AK459="OK",J459="READY",F459&lt;&gt;"",G459&lt;&gt;"",K459&lt;&gt;"",S459="OK",OR(R459="PASS",R459="FAIL")),"YES","NO"))</x:f>
@@ -24849,7 +24849,7 @@
         <x:f>IF(A460="",IF(B460="","","MISSING_TEST_ID"),IF(B460="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A460,$B$2:$B$501,B460)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL460" s="9" t="str">
-        <x:f>IF(A460="","",IF(AND(AK460="OK",J460="READY",F460&lt;&gt;"",G460&lt;&gt;"",K460&lt;&gt;"",OR(L460="PASS",L460="FAIL"),M460&lt;&gt;"",O460&lt;&gt;"",P460="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A460="","",IF(AND(AK460="OK",J460="READY",F460&lt;&gt;"",G460&lt;&gt;"",K460&lt;&gt;"",OR(L460="PASS",L460="FAIL"),M460&lt;&gt;"",P460="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM460" s="9" t="str">
         <x:f>IF(A460="","",IF(AND(AK460="OK",J460="READY",F460&lt;&gt;"",G460&lt;&gt;"",K460&lt;&gt;"",S460="OK",OR(R460="PASS",R460="FAIL")),"YES","NO"))</x:f>
@@ -24901,7 +24901,7 @@
         <x:f>IF(A461="",IF(B461="","","MISSING_TEST_ID"),IF(B461="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A461,$B$2:$B$501,B461)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL461" s="9" t="str">
-        <x:f>IF(A461="","",IF(AND(AK461="OK",J461="READY",F461&lt;&gt;"",G461&lt;&gt;"",K461&lt;&gt;"",OR(L461="PASS",L461="FAIL"),M461&lt;&gt;"",O461&lt;&gt;"",P461="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A461="","",IF(AND(AK461="OK",J461="READY",F461&lt;&gt;"",G461&lt;&gt;"",K461&lt;&gt;"",OR(L461="PASS",L461="FAIL"),M461&lt;&gt;"",P461="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM461" s="9" t="str">
         <x:f>IF(A461="","",IF(AND(AK461="OK",J461="READY",F461&lt;&gt;"",G461&lt;&gt;"",K461&lt;&gt;"",S461="OK",OR(R461="PASS",R461="FAIL")),"YES","NO"))</x:f>
@@ -24953,7 +24953,7 @@
         <x:f>IF(A462="",IF(B462="","","MISSING_TEST_ID"),IF(B462="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A462,$B$2:$B$501,B462)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL462" s="9" t="str">
-        <x:f>IF(A462="","",IF(AND(AK462="OK",J462="READY",F462&lt;&gt;"",G462&lt;&gt;"",K462&lt;&gt;"",OR(L462="PASS",L462="FAIL"),M462&lt;&gt;"",O462&lt;&gt;"",P462="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A462="","",IF(AND(AK462="OK",J462="READY",F462&lt;&gt;"",G462&lt;&gt;"",K462&lt;&gt;"",OR(L462="PASS",L462="FAIL"),M462&lt;&gt;"",P462="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM462" s="9" t="str">
         <x:f>IF(A462="","",IF(AND(AK462="OK",J462="READY",F462&lt;&gt;"",G462&lt;&gt;"",K462&lt;&gt;"",S462="OK",OR(R462="PASS",R462="FAIL")),"YES","NO"))</x:f>
@@ -25005,7 +25005,7 @@
         <x:f>IF(A463="",IF(B463="","","MISSING_TEST_ID"),IF(B463="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A463,$B$2:$B$501,B463)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL463" s="9" t="str">
-        <x:f>IF(A463="","",IF(AND(AK463="OK",J463="READY",F463&lt;&gt;"",G463&lt;&gt;"",K463&lt;&gt;"",OR(L463="PASS",L463="FAIL"),M463&lt;&gt;"",O463&lt;&gt;"",P463="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A463="","",IF(AND(AK463="OK",J463="READY",F463&lt;&gt;"",G463&lt;&gt;"",K463&lt;&gt;"",OR(L463="PASS",L463="FAIL"),M463&lt;&gt;"",P463="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM463" s="9" t="str">
         <x:f>IF(A463="","",IF(AND(AK463="OK",J463="READY",F463&lt;&gt;"",G463&lt;&gt;"",K463&lt;&gt;"",S463="OK",OR(R463="PASS",R463="FAIL")),"YES","NO"))</x:f>
@@ -25057,7 +25057,7 @@
         <x:f>IF(A464="",IF(B464="","","MISSING_TEST_ID"),IF(B464="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A464,$B$2:$B$501,B464)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL464" s="9" t="str">
-        <x:f>IF(A464="","",IF(AND(AK464="OK",J464="READY",F464&lt;&gt;"",G464&lt;&gt;"",K464&lt;&gt;"",OR(L464="PASS",L464="FAIL"),M464&lt;&gt;"",O464&lt;&gt;"",P464="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A464="","",IF(AND(AK464="OK",J464="READY",F464&lt;&gt;"",G464&lt;&gt;"",K464&lt;&gt;"",OR(L464="PASS",L464="FAIL"),M464&lt;&gt;"",P464="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM464" s="9" t="str">
         <x:f>IF(A464="","",IF(AND(AK464="OK",J464="READY",F464&lt;&gt;"",G464&lt;&gt;"",K464&lt;&gt;"",S464="OK",OR(R464="PASS",R464="FAIL")),"YES","NO"))</x:f>
@@ -25109,7 +25109,7 @@
         <x:f>IF(A465="",IF(B465="","","MISSING_TEST_ID"),IF(B465="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A465,$B$2:$B$501,B465)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL465" s="9" t="str">
-        <x:f>IF(A465="","",IF(AND(AK465="OK",J465="READY",F465&lt;&gt;"",G465&lt;&gt;"",K465&lt;&gt;"",OR(L465="PASS",L465="FAIL"),M465&lt;&gt;"",O465&lt;&gt;"",P465="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A465="","",IF(AND(AK465="OK",J465="READY",F465&lt;&gt;"",G465&lt;&gt;"",K465&lt;&gt;"",OR(L465="PASS",L465="FAIL"),M465&lt;&gt;"",P465="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM465" s="9" t="str">
         <x:f>IF(A465="","",IF(AND(AK465="OK",J465="READY",F465&lt;&gt;"",G465&lt;&gt;"",K465&lt;&gt;"",S465="OK",OR(R465="PASS",R465="FAIL")),"YES","NO"))</x:f>
@@ -25161,7 +25161,7 @@
         <x:f>IF(A466="",IF(B466="","","MISSING_TEST_ID"),IF(B466="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A466,$B$2:$B$501,B466)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL466" s="9" t="str">
-        <x:f>IF(A466="","",IF(AND(AK466="OK",J466="READY",F466&lt;&gt;"",G466&lt;&gt;"",K466&lt;&gt;"",OR(L466="PASS",L466="FAIL"),M466&lt;&gt;"",O466&lt;&gt;"",P466="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A466="","",IF(AND(AK466="OK",J466="READY",F466&lt;&gt;"",G466&lt;&gt;"",K466&lt;&gt;"",OR(L466="PASS",L466="FAIL"),M466&lt;&gt;"",P466="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM466" s="9" t="str">
         <x:f>IF(A466="","",IF(AND(AK466="OK",J466="READY",F466&lt;&gt;"",G466&lt;&gt;"",K466&lt;&gt;"",S466="OK",OR(R466="PASS",R466="FAIL")),"YES","NO"))</x:f>
@@ -25213,7 +25213,7 @@
         <x:f>IF(A467="",IF(B467="","","MISSING_TEST_ID"),IF(B467="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A467,$B$2:$B$501,B467)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL467" s="9" t="str">
-        <x:f>IF(A467="","",IF(AND(AK467="OK",J467="READY",F467&lt;&gt;"",G467&lt;&gt;"",K467&lt;&gt;"",OR(L467="PASS",L467="FAIL"),M467&lt;&gt;"",O467&lt;&gt;"",P467="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A467="","",IF(AND(AK467="OK",J467="READY",F467&lt;&gt;"",G467&lt;&gt;"",K467&lt;&gt;"",OR(L467="PASS",L467="FAIL"),M467&lt;&gt;"",P467="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM467" s="9" t="str">
         <x:f>IF(A467="","",IF(AND(AK467="OK",J467="READY",F467&lt;&gt;"",G467&lt;&gt;"",K467&lt;&gt;"",S467="OK",OR(R467="PASS",R467="FAIL")),"YES","NO"))</x:f>
@@ -25265,7 +25265,7 @@
         <x:f>IF(A468="",IF(B468="","","MISSING_TEST_ID"),IF(B468="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A468,$B$2:$B$501,B468)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL468" s="9" t="str">
-        <x:f>IF(A468="","",IF(AND(AK468="OK",J468="READY",F468&lt;&gt;"",G468&lt;&gt;"",K468&lt;&gt;"",OR(L468="PASS",L468="FAIL"),M468&lt;&gt;"",O468&lt;&gt;"",P468="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A468="","",IF(AND(AK468="OK",J468="READY",F468&lt;&gt;"",G468&lt;&gt;"",K468&lt;&gt;"",OR(L468="PASS",L468="FAIL"),M468&lt;&gt;"",P468="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM468" s="9" t="str">
         <x:f>IF(A468="","",IF(AND(AK468="OK",J468="READY",F468&lt;&gt;"",G468&lt;&gt;"",K468&lt;&gt;"",S468="OK",OR(R468="PASS",R468="FAIL")),"YES","NO"))</x:f>
@@ -25317,7 +25317,7 @@
         <x:f>IF(A469="",IF(B469="","","MISSING_TEST_ID"),IF(B469="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A469,$B$2:$B$501,B469)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL469" s="9" t="str">
-        <x:f>IF(A469="","",IF(AND(AK469="OK",J469="READY",F469&lt;&gt;"",G469&lt;&gt;"",K469&lt;&gt;"",OR(L469="PASS",L469="FAIL"),M469&lt;&gt;"",O469&lt;&gt;"",P469="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A469="","",IF(AND(AK469="OK",J469="READY",F469&lt;&gt;"",G469&lt;&gt;"",K469&lt;&gt;"",OR(L469="PASS",L469="FAIL"),M469&lt;&gt;"",P469="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM469" s="9" t="str">
         <x:f>IF(A469="","",IF(AND(AK469="OK",J469="READY",F469&lt;&gt;"",G469&lt;&gt;"",K469&lt;&gt;"",S469="OK",OR(R469="PASS",R469="FAIL")),"YES","NO"))</x:f>
@@ -25369,7 +25369,7 @@
         <x:f>IF(A470="",IF(B470="","","MISSING_TEST_ID"),IF(B470="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A470,$B$2:$B$501,B470)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL470" s="9" t="str">
-        <x:f>IF(A470="","",IF(AND(AK470="OK",J470="READY",F470&lt;&gt;"",G470&lt;&gt;"",K470&lt;&gt;"",OR(L470="PASS",L470="FAIL"),M470&lt;&gt;"",O470&lt;&gt;"",P470="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A470="","",IF(AND(AK470="OK",J470="READY",F470&lt;&gt;"",G470&lt;&gt;"",K470&lt;&gt;"",OR(L470="PASS",L470="FAIL"),M470&lt;&gt;"",P470="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM470" s="9" t="str">
         <x:f>IF(A470="","",IF(AND(AK470="OK",J470="READY",F470&lt;&gt;"",G470&lt;&gt;"",K470&lt;&gt;"",S470="OK",OR(R470="PASS",R470="FAIL")),"YES","NO"))</x:f>
@@ -25421,7 +25421,7 @@
         <x:f>IF(A471="",IF(B471="","","MISSING_TEST_ID"),IF(B471="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A471,$B$2:$B$501,B471)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL471" s="9" t="str">
-        <x:f>IF(A471="","",IF(AND(AK471="OK",J471="READY",F471&lt;&gt;"",G471&lt;&gt;"",K471&lt;&gt;"",OR(L471="PASS",L471="FAIL"),M471&lt;&gt;"",O471&lt;&gt;"",P471="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A471="","",IF(AND(AK471="OK",J471="READY",F471&lt;&gt;"",G471&lt;&gt;"",K471&lt;&gt;"",OR(L471="PASS",L471="FAIL"),M471&lt;&gt;"",P471="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM471" s="9" t="str">
         <x:f>IF(A471="","",IF(AND(AK471="OK",J471="READY",F471&lt;&gt;"",G471&lt;&gt;"",K471&lt;&gt;"",S471="OK",OR(R471="PASS",R471="FAIL")),"YES","NO"))</x:f>
@@ -25473,7 +25473,7 @@
         <x:f>IF(A472="",IF(B472="","","MISSING_TEST_ID"),IF(B472="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A472,$B$2:$B$501,B472)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL472" s="9" t="str">
-        <x:f>IF(A472="","",IF(AND(AK472="OK",J472="READY",F472&lt;&gt;"",G472&lt;&gt;"",K472&lt;&gt;"",OR(L472="PASS",L472="FAIL"),M472&lt;&gt;"",O472&lt;&gt;"",P472="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A472="","",IF(AND(AK472="OK",J472="READY",F472&lt;&gt;"",G472&lt;&gt;"",K472&lt;&gt;"",OR(L472="PASS",L472="FAIL"),M472&lt;&gt;"",P472="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM472" s="9" t="str">
         <x:f>IF(A472="","",IF(AND(AK472="OK",J472="READY",F472&lt;&gt;"",G472&lt;&gt;"",K472&lt;&gt;"",S472="OK",OR(R472="PASS",R472="FAIL")),"YES","NO"))</x:f>
@@ -25525,7 +25525,7 @@
         <x:f>IF(A473="",IF(B473="","","MISSING_TEST_ID"),IF(B473="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A473,$B$2:$B$501,B473)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL473" s="9" t="str">
-        <x:f>IF(A473="","",IF(AND(AK473="OK",J473="READY",F473&lt;&gt;"",G473&lt;&gt;"",K473&lt;&gt;"",OR(L473="PASS",L473="FAIL"),M473&lt;&gt;"",O473&lt;&gt;"",P473="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A473="","",IF(AND(AK473="OK",J473="READY",F473&lt;&gt;"",G473&lt;&gt;"",K473&lt;&gt;"",OR(L473="PASS",L473="FAIL"),M473&lt;&gt;"",P473="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM473" s="9" t="str">
         <x:f>IF(A473="","",IF(AND(AK473="OK",J473="READY",F473&lt;&gt;"",G473&lt;&gt;"",K473&lt;&gt;"",S473="OK",OR(R473="PASS",R473="FAIL")),"YES","NO"))</x:f>
@@ -25577,7 +25577,7 @@
         <x:f>IF(A474="",IF(B474="","","MISSING_TEST_ID"),IF(B474="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A474,$B$2:$B$501,B474)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL474" s="9" t="str">
-        <x:f>IF(A474="","",IF(AND(AK474="OK",J474="READY",F474&lt;&gt;"",G474&lt;&gt;"",K474&lt;&gt;"",OR(L474="PASS",L474="FAIL"),M474&lt;&gt;"",O474&lt;&gt;"",P474="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A474="","",IF(AND(AK474="OK",J474="READY",F474&lt;&gt;"",G474&lt;&gt;"",K474&lt;&gt;"",OR(L474="PASS",L474="FAIL"),M474&lt;&gt;"",P474="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM474" s="9" t="str">
         <x:f>IF(A474="","",IF(AND(AK474="OK",J474="READY",F474&lt;&gt;"",G474&lt;&gt;"",K474&lt;&gt;"",S474="OK",OR(R474="PASS",R474="FAIL")),"YES","NO"))</x:f>
@@ -25629,7 +25629,7 @@
         <x:f>IF(A475="",IF(B475="","","MISSING_TEST_ID"),IF(B475="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A475,$B$2:$B$501,B475)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL475" s="9" t="str">
-        <x:f>IF(A475="","",IF(AND(AK475="OK",J475="READY",F475&lt;&gt;"",G475&lt;&gt;"",K475&lt;&gt;"",OR(L475="PASS",L475="FAIL"),M475&lt;&gt;"",O475&lt;&gt;"",P475="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A475="","",IF(AND(AK475="OK",J475="READY",F475&lt;&gt;"",G475&lt;&gt;"",K475&lt;&gt;"",OR(L475="PASS",L475="FAIL"),M475&lt;&gt;"",P475="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM475" s="9" t="str">
         <x:f>IF(A475="","",IF(AND(AK475="OK",J475="READY",F475&lt;&gt;"",G475&lt;&gt;"",K475&lt;&gt;"",S475="OK",OR(R475="PASS",R475="FAIL")),"YES","NO"))</x:f>
@@ -25681,7 +25681,7 @@
         <x:f>IF(A476="",IF(B476="","","MISSING_TEST_ID"),IF(B476="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A476,$B$2:$B$501,B476)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL476" s="9" t="str">
-        <x:f>IF(A476="","",IF(AND(AK476="OK",J476="READY",F476&lt;&gt;"",G476&lt;&gt;"",K476&lt;&gt;"",OR(L476="PASS",L476="FAIL"),M476&lt;&gt;"",O476&lt;&gt;"",P476="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A476="","",IF(AND(AK476="OK",J476="READY",F476&lt;&gt;"",G476&lt;&gt;"",K476&lt;&gt;"",OR(L476="PASS",L476="FAIL"),M476&lt;&gt;"",P476="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM476" s="9" t="str">
         <x:f>IF(A476="","",IF(AND(AK476="OK",J476="READY",F476&lt;&gt;"",G476&lt;&gt;"",K476&lt;&gt;"",S476="OK",OR(R476="PASS",R476="FAIL")),"YES","NO"))</x:f>
@@ -25733,7 +25733,7 @@
         <x:f>IF(A477="",IF(B477="","","MISSING_TEST_ID"),IF(B477="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A477,$B$2:$B$501,B477)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL477" s="9" t="str">
-        <x:f>IF(A477="","",IF(AND(AK477="OK",J477="READY",F477&lt;&gt;"",G477&lt;&gt;"",K477&lt;&gt;"",OR(L477="PASS",L477="FAIL"),M477&lt;&gt;"",O477&lt;&gt;"",P477="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A477="","",IF(AND(AK477="OK",J477="READY",F477&lt;&gt;"",G477&lt;&gt;"",K477&lt;&gt;"",OR(L477="PASS",L477="FAIL"),M477&lt;&gt;"",P477="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM477" s="9" t="str">
         <x:f>IF(A477="","",IF(AND(AK477="OK",J477="READY",F477&lt;&gt;"",G477&lt;&gt;"",K477&lt;&gt;"",S477="OK",OR(R477="PASS",R477="FAIL")),"YES","NO"))</x:f>
@@ -25785,7 +25785,7 @@
         <x:f>IF(A478="",IF(B478="","","MISSING_TEST_ID"),IF(B478="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A478,$B$2:$B$501,B478)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL478" s="9" t="str">
-        <x:f>IF(A478="","",IF(AND(AK478="OK",J478="READY",F478&lt;&gt;"",G478&lt;&gt;"",K478&lt;&gt;"",OR(L478="PASS",L478="FAIL"),M478&lt;&gt;"",O478&lt;&gt;"",P478="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A478="","",IF(AND(AK478="OK",J478="READY",F478&lt;&gt;"",G478&lt;&gt;"",K478&lt;&gt;"",OR(L478="PASS",L478="FAIL"),M478&lt;&gt;"",P478="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM478" s="9" t="str">
         <x:f>IF(A478="","",IF(AND(AK478="OK",J478="READY",F478&lt;&gt;"",G478&lt;&gt;"",K478&lt;&gt;"",S478="OK",OR(R478="PASS",R478="FAIL")),"YES","NO"))</x:f>
@@ -25837,7 +25837,7 @@
         <x:f>IF(A479="",IF(B479="","","MISSING_TEST_ID"),IF(B479="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A479,$B$2:$B$501,B479)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL479" s="9" t="str">
-        <x:f>IF(A479="","",IF(AND(AK479="OK",J479="READY",F479&lt;&gt;"",G479&lt;&gt;"",K479&lt;&gt;"",OR(L479="PASS",L479="FAIL"),M479&lt;&gt;"",O479&lt;&gt;"",P479="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A479="","",IF(AND(AK479="OK",J479="READY",F479&lt;&gt;"",G479&lt;&gt;"",K479&lt;&gt;"",OR(L479="PASS",L479="FAIL"),M479&lt;&gt;"",P479="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM479" s="9" t="str">
         <x:f>IF(A479="","",IF(AND(AK479="OK",J479="READY",F479&lt;&gt;"",G479&lt;&gt;"",K479&lt;&gt;"",S479="OK",OR(R479="PASS",R479="FAIL")),"YES","NO"))</x:f>
@@ -25889,7 +25889,7 @@
         <x:f>IF(A480="",IF(B480="","","MISSING_TEST_ID"),IF(B480="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A480,$B$2:$B$501,B480)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL480" s="9" t="str">
-        <x:f>IF(A480="","",IF(AND(AK480="OK",J480="READY",F480&lt;&gt;"",G480&lt;&gt;"",K480&lt;&gt;"",OR(L480="PASS",L480="FAIL"),M480&lt;&gt;"",O480&lt;&gt;"",P480="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A480="","",IF(AND(AK480="OK",J480="READY",F480&lt;&gt;"",G480&lt;&gt;"",K480&lt;&gt;"",OR(L480="PASS",L480="FAIL"),M480&lt;&gt;"",P480="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM480" s="9" t="str">
         <x:f>IF(A480="","",IF(AND(AK480="OK",J480="READY",F480&lt;&gt;"",G480&lt;&gt;"",K480&lt;&gt;"",S480="OK",OR(R480="PASS",R480="FAIL")),"YES","NO"))</x:f>
@@ -25941,7 +25941,7 @@
         <x:f>IF(A481="",IF(B481="","","MISSING_TEST_ID"),IF(B481="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A481,$B$2:$B$501,B481)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL481" s="9" t="str">
-        <x:f>IF(A481="","",IF(AND(AK481="OK",J481="READY",F481&lt;&gt;"",G481&lt;&gt;"",K481&lt;&gt;"",OR(L481="PASS",L481="FAIL"),M481&lt;&gt;"",O481&lt;&gt;"",P481="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A481="","",IF(AND(AK481="OK",J481="READY",F481&lt;&gt;"",G481&lt;&gt;"",K481&lt;&gt;"",OR(L481="PASS",L481="FAIL"),M481&lt;&gt;"",P481="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM481" s="9" t="str">
         <x:f>IF(A481="","",IF(AND(AK481="OK",J481="READY",F481&lt;&gt;"",G481&lt;&gt;"",K481&lt;&gt;"",S481="OK",OR(R481="PASS",R481="FAIL")),"YES","NO"))</x:f>
@@ -25993,7 +25993,7 @@
         <x:f>IF(A482="",IF(B482="","","MISSING_TEST_ID"),IF(B482="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A482,$B$2:$B$501,B482)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL482" s="9" t="str">
-        <x:f>IF(A482="","",IF(AND(AK482="OK",J482="READY",F482&lt;&gt;"",G482&lt;&gt;"",K482&lt;&gt;"",OR(L482="PASS",L482="FAIL"),M482&lt;&gt;"",O482&lt;&gt;"",P482="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A482="","",IF(AND(AK482="OK",J482="READY",F482&lt;&gt;"",G482&lt;&gt;"",K482&lt;&gt;"",OR(L482="PASS",L482="FAIL"),M482&lt;&gt;"",P482="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM482" s="9" t="str">
         <x:f>IF(A482="","",IF(AND(AK482="OK",J482="READY",F482&lt;&gt;"",G482&lt;&gt;"",K482&lt;&gt;"",S482="OK",OR(R482="PASS",R482="FAIL")),"YES","NO"))</x:f>
@@ -26045,7 +26045,7 @@
         <x:f>IF(A483="",IF(B483="","","MISSING_TEST_ID"),IF(B483="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A483,$B$2:$B$501,B483)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL483" s="9" t="str">
-        <x:f>IF(A483="","",IF(AND(AK483="OK",J483="READY",F483&lt;&gt;"",G483&lt;&gt;"",K483&lt;&gt;"",OR(L483="PASS",L483="FAIL"),M483&lt;&gt;"",O483&lt;&gt;"",P483="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A483="","",IF(AND(AK483="OK",J483="READY",F483&lt;&gt;"",G483&lt;&gt;"",K483&lt;&gt;"",OR(L483="PASS",L483="FAIL"),M483&lt;&gt;"",P483="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM483" s="9" t="str">
         <x:f>IF(A483="","",IF(AND(AK483="OK",J483="READY",F483&lt;&gt;"",G483&lt;&gt;"",K483&lt;&gt;"",S483="OK",OR(R483="PASS",R483="FAIL")),"YES","NO"))</x:f>
@@ -26097,7 +26097,7 @@
         <x:f>IF(A484="",IF(B484="","","MISSING_TEST_ID"),IF(B484="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A484,$B$2:$B$501,B484)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL484" s="9" t="str">
-        <x:f>IF(A484="","",IF(AND(AK484="OK",J484="READY",F484&lt;&gt;"",G484&lt;&gt;"",K484&lt;&gt;"",OR(L484="PASS",L484="FAIL"),M484&lt;&gt;"",O484&lt;&gt;"",P484="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A484="","",IF(AND(AK484="OK",J484="READY",F484&lt;&gt;"",G484&lt;&gt;"",K484&lt;&gt;"",OR(L484="PASS",L484="FAIL"),M484&lt;&gt;"",P484="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM484" s="9" t="str">
         <x:f>IF(A484="","",IF(AND(AK484="OK",J484="READY",F484&lt;&gt;"",G484&lt;&gt;"",K484&lt;&gt;"",S484="OK",OR(R484="PASS",R484="FAIL")),"YES","NO"))</x:f>
@@ -26149,7 +26149,7 @@
         <x:f>IF(A485="",IF(B485="","","MISSING_TEST_ID"),IF(B485="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A485,$B$2:$B$501,B485)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL485" s="9" t="str">
-        <x:f>IF(A485="","",IF(AND(AK485="OK",J485="READY",F485&lt;&gt;"",G485&lt;&gt;"",K485&lt;&gt;"",OR(L485="PASS",L485="FAIL"),M485&lt;&gt;"",O485&lt;&gt;"",P485="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A485="","",IF(AND(AK485="OK",J485="READY",F485&lt;&gt;"",G485&lt;&gt;"",K485&lt;&gt;"",OR(L485="PASS",L485="FAIL"),M485&lt;&gt;"",P485="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM485" s="9" t="str">
         <x:f>IF(A485="","",IF(AND(AK485="OK",J485="READY",F485&lt;&gt;"",G485&lt;&gt;"",K485&lt;&gt;"",S485="OK",OR(R485="PASS",R485="FAIL")),"YES","NO"))</x:f>
@@ -26201,7 +26201,7 @@
         <x:f>IF(A486="",IF(B486="","","MISSING_TEST_ID"),IF(B486="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A486,$B$2:$B$501,B486)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL486" s="9" t="str">
-        <x:f>IF(A486="","",IF(AND(AK486="OK",J486="READY",F486&lt;&gt;"",G486&lt;&gt;"",K486&lt;&gt;"",OR(L486="PASS",L486="FAIL"),M486&lt;&gt;"",O486&lt;&gt;"",P486="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A486="","",IF(AND(AK486="OK",J486="READY",F486&lt;&gt;"",G486&lt;&gt;"",K486&lt;&gt;"",OR(L486="PASS",L486="FAIL"),M486&lt;&gt;"",P486="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM486" s="9" t="str">
         <x:f>IF(A486="","",IF(AND(AK486="OK",J486="READY",F486&lt;&gt;"",G486&lt;&gt;"",K486&lt;&gt;"",S486="OK",OR(R486="PASS",R486="FAIL")),"YES","NO"))</x:f>
@@ -26253,7 +26253,7 @@
         <x:f>IF(A487="",IF(B487="","","MISSING_TEST_ID"),IF(B487="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A487,$B$2:$B$501,B487)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL487" s="9" t="str">
-        <x:f>IF(A487="","",IF(AND(AK487="OK",J487="READY",F487&lt;&gt;"",G487&lt;&gt;"",K487&lt;&gt;"",OR(L487="PASS",L487="FAIL"),M487&lt;&gt;"",O487&lt;&gt;"",P487="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A487="","",IF(AND(AK487="OK",J487="READY",F487&lt;&gt;"",G487&lt;&gt;"",K487&lt;&gt;"",OR(L487="PASS",L487="FAIL"),M487&lt;&gt;"",P487="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM487" s="9" t="str">
         <x:f>IF(A487="","",IF(AND(AK487="OK",J487="READY",F487&lt;&gt;"",G487&lt;&gt;"",K487&lt;&gt;"",S487="OK",OR(R487="PASS",R487="FAIL")),"YES","NO"))</x:f>
@@ -26305,7 +26305,7 @@
         <x:f>IF(A488="",IF(B488="","","MISSING_TEST_ID"),IF(B488="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A488,$B$2:$B$501,B488)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL488" s="9" t="str">
-        <x:f>IF(A488="","",IF(AND(AK488="OK",J488="READY",F488&lt;&gt;"",G488&lt;&gt;"",K488&lt;&gt;"",OR(L488="PASS",L488="FAIL"),M488&lt;&gt;"",O488&lt;&gt;"",P488="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A488="","",IF(AND(AK488="OK",J488="READY",F488&lt;&gt;"",G488&lt;&gt;"",K488&lt;&gt;"",OR(L488="PASS",L488="FAIL"),M488&lt;&gt;"",P488="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM488" s="9" t="str">
         <x:f>IF(A488="","",IF(AND(AK488="OK",J488="READY",F488&lt;&gt;"",G488&lt;&gt;"",K488&lt;&gt;"",S488="OK",OR(R488="PASS",R488="FAIL")),"YES","NO"))</x:f>
@@ -26357,7 +26357,7 @@
         <x:f>IF(A489="",IF(B489="","","MISSING_TEST_ID"),IF(B489="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A489,$B$2:$B$501,B489)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL489" s="9" t="str">
-        <x:f>IF(A489="","",IF(AND(AK489="OK",J489="READY",F489&lt;&gt;"",G489&lt;&gt;"",K489&lt;&gt;"",OR(L489="PASS",L489="FAIL"),M489&lt;&gt;"",O489&lt;&gt;"",P489="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A489="","",IF(AND(AK489="OK",J489="READY",F489&lt;&gt;"",G489&lt;&gt;"",K489&lt;&gt;"",OR(L489="PASS",L489="FAIL"),M489&lt;&gt;"",P489="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM489" s="9" t="str">
         <x:f>IF(A489="","",IF(AND(AK489="OK",J489="READY",F489&lt;&gt;"",G489&lt;&gt;"",K489&lt;&gt;"",S489="OK",OR(R489="PASS",R489="FAIL")),"YES","NO"))</x:f>
@@ -26409,7 +26409,7 @@
         <x:f>IF(A490="",IF(B490="","","MISSING_TEST_ID"),IF(B490="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A490,$B$2:$B$501,B490)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL490" s="9" t="str">
-        <x:f>IF(A490="","",IF(AND(AK490="OK",J490="READY",F490&lt;&gt;"",G490&lt;&gt;"",K490&lt;&gt;"",OR(L490="PASS",L490="FAIL"),M490&lt;&gt;"",O490&lt;&gt;"",P490="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A490="","",IF(AND(AK490="OK",J490="READY",F490&lt;&gt;"",G490&lt;&gt;"",K490&lt;&gt;"",OR(L490="PASS",L490="FAIL"),M490&lt;&gt;"",P490="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM490" s="9" t="str">
         <x:f>IF(A490="","",IF(AND(AK490="OK",J490="READY",F490&lt;&gt;"",G490&lt;&gt;"",K490&lt;&gt;"",S490="OK",OR(R490="PASS",R490="FAIL")),"YES","NO"))</x:f>
@@ -26461,7 +26461,7 @@
         <x:f>IF(A491="",IF(B491="","","MISSING_TEST_ID"),IF(B491="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A491,$B$2:$B$501,B491)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL491" s="9" t="str">
-        <x:f>IF(A491="","",IF(AND(AK491="OK",J491="READY",F491&lt;&gt;"",G491&lt;&gt;"",K491&lt;&gt;"",OR(L491="PASS",L491="FAIL"),M491&lt;&gt;"",O491&lt;&gt;"",P491="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A491="","",IF(AND(AK491="OK",J491="READY",F491&lt;&gt;"",G491&lt;&gt;"",K491&lt;&gt;"",OR(L491="PASS",L491="FAIL"),M491&lt;&gt;"",P491="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM491" s="9" t="str">
         <x:f>IF(A491="","",IF(AND(AK491="OK",J491="READY",F491&lt;&gt;"",G491&lt;&gt;"",K491&lt;&gt;"",S491="OK",OR(R491="PASS",R491="FAIL")),"YES","NO"))</x:f>
@@ -26513,7 +26513,7 @@
         <x:f>IF(A492="",IF(B492="","","MISSING_TEST_ID"),IF(B492="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A492,$B$2:$B$501,B492)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL492" s="9" t="str">
-        <x:f>IF(A492="","",IF(AND(AK492="OK",J492="READY",F492&lt;&gt;"",G492&lt;&gt;"",K492&lt;&gt;"",OR(L492="PASS",L492="FAIL"),M492&lt;&gt;"",O492&lt;&gt;"",P492="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A492="","",IF(AND(AK492="OK",J492="READY",F492&lt;&gt;"",G492&lt;&gt;"",K492&lt;&gt;"",OR(L492="PASS",L492="FAIL"),M492&lt;&gt;"",P492="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM492" s="9" t="str">
         <x:f>IF(A492="","",IF(AND(AK492="OK",J492="READY",F492&lt;&gt;"",G492&lt;&gt;"",K492&lt;&gt;"",S492="OK",OR(R492="PASS",R492="FAIL")),"YES","NO"))</x:f>
@@ -26565,7 +26565,7 @@
         <x:f>IF(A493="",IF(B493="","","MISSING_TEST_ID"),IF(B493="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A493,$B$2:$B$501,B493)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL493" s="9" t="str">
-        <x:f>IF(A493="","",IF(AND(AK493="OK",J493="READY",F493&lt;&gt;"",G493&lt;&gt;"",K493&lt;&gt;"",OR(L493="PASS",L493="FAIL"),M493&lt;&gt;"",O493&lt;&gt;"",P493="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A493="","",IF(AND(AK493="OK",J493="READY",F493&lt;&gt;"",G493&lt;&gt;"",K493&lt;&gt;"",OR(L493="PASS",L493="FAIL"),M493&lt;&gt;"",P493="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM493" s="9" t="str">
         <x:f>IF(A493="","",IF(AND(AK493="OK",J493="READY",F493&lt;&gt;"",G493&lt;&gt;"",K493&lt;&gt;"",S493="OK",OR(R493="PASS",R493="FAIL")),"YES","NO"))</x:f>
@@ -26617,7 +26617,7 @@
         <x:f>IF(A494="",IF(B494="","","MISSING_TEST_ID"),IF(B494="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A494,$B$2:$B$501,B494)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL494" s="9" t="str">
-        <x:f>IF(A494="","",IF(AND(AK494="OK",J494="READY",F494&lt;&gt;"",G494&lt;&gt;"",K494&lt;&gt;"",OR(L494="PASS",L494="FAIL"),M494&lt;&gt;"",O494&lt;&gt;"",P494="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A494="","",IF(AND(AK494="OK",J494="READY",F494&lt;&gt;"",G494&lt;&gt;"",K494&lt;&gt;"",OR(L494="PASS",L494="FAIL"),M494&lt;&gt;"",P494="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM494" s="9" t="str">
         <x:f>IF(A494="","",IF(AND(AK494="OK",J494="READY",F494&lt;&gt;"",G494&lt;&gt;"",K494&lt;&gt;"",S494="OK",OR(R494="PASS",R494="FAIL")),"YES","NO"))</x:f>
@@ -26669,7 +26669,7 @@
         <x:f>IF(A495="",IF(B495="","","MISSING_TEST_ID"),IF(B495="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A495,$B$2:$B$501,B495)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL495" s="9" t="str">
-        <x:f>IF(A495="","",IF(AND(AK495="OK",J495="READY",F495&lt;&gt;"",G495&lt;&gt;"",K495&lt;&gt;"",OR(L495="PASS",L495="FAIL"),M495&lt;&gt;"",O495&lt;&gt;"",P495="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A495="","",IF(AND(AK495="OK",J495="READY",F495&lt;&gt;"",G495&lt;&gt;"",K495&lt;&gt;"",OR(L495="PASS",L495="FAIL"),M495&lt;&gt;"",P495="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM495" s="9" t="str">
         <x:f>IF(A495="","",IF(AND(AK495="OK",J495="READY",F495&lt;&gt;"",G495&lt;&gt;"",K495&lt;&gt;"",S495="OK",OR(R495="PASS",R495="FAIL")),"YES","NO"))</x:f>
@@ -26721,7 +26721,7 @@
         <x:f>IF(A496="",IF(B496="","","MISSING_TEST_ID"),IF(B496="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A496,$B$2:$B$501,B496)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL496" s="9" t="str">
-        <x:f>IF(A496="","",IF(AND(AK496="OK",J496="READY",F496&lt;&gt;"",G496&lt;&gt;"",K496&lt;&gt;"",OR(L496="PASS",L496="FAIL"),M496&lt;&gt;"",O496&lt;&gt;"",P496="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A496="","",IF(AND(AK496="OK",J496="READY",F496&lt;&gt;"",G496&lt;&gt;"",K496&lt;&gt;"",OR(L496="PASS",L496="FAIL"),M496&lt;&gt;"",P496="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM496" s="9" t="str">
         <x:f>IF(A496="","",IF(AND(AK496="OK",J496="READY",F496&lt;&gt;"",G496&lt;&gt;"",K496&lt;&gt;"",S496="OK",OR(R496="PASS",R496="FAIL")),"YES","NO"))</x:f>
@@ -26773,7 +26773,7 @@
         <x:f>IF(A497="",IF(B497="","","MISSING_TEST_ID"),IF(B497="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A497,$B$2:$B$501,B497)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL497" s="9" t="str">
-        <x:f>IF(A497="","",IF(AND(AK497="OK",J497="READY",F497&lt;&gt;"",G497&lt;&gt;"",K497&lt;&gt;"",OR(L497="PASS",L497="FAIL"),M497&lt;&gt;"",O497&lt;&gt;"",P497="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A497="","",IF(AND(AK497="OK",J497="READY",F497&lt;&gt;"",G497&lt;&gt;"",K497&lt;&gt;"",OR(L497="PASS",L497="FAIL"),M497&lt;&gt;"",P497="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM497" s="9" t="str">
         <x:f>IF(A497="","",IF(AND(AK497="OK",J497="READY",F497&lt;&gt;"",G497&lt;&gt;"",K497&lt;&gt;"",S497="OK",OR(R497="PASS",R497="FAIL")),"YES","NO"))</x:f>
@@ -26825,7 +26825,7 @@
         <x:f>IF(A498="",IF(B498="","","MISSING_TEST_ID"),IF(B498="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A498,$B$2:$B$501,B498)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL498" s="9" t="str">
-        <x:f>IF(A498="","",IF(AND(AK498="OK",J498="READY",F498&lt;&gt;"",G498&lt;&gt;"",K498&lt;&gt;"",OR(L498="PASS",L498="FAIL"),M498&lt;&gt;"",O498&lt;&gt;"",P498="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A498="","",IF(AND(AK498="OK",J498="READY",F498&lt;&gt;"",G498&lt;&gt;"",K498&lt;&gt;"",OR(L498="PASS",L498="FAIL"),M498&lt;&gt;"",P498="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM498" s="9" t="str">
         <x:f>IF(A498="","",IF(AND(AK498="OK",J498="READY",F498&lt;&gt;"",G498&lt;&gt;"",K498&lt;&gt;"",S498="OK",OR(R498="PASS",R498="FAIL")),"YES","NO"))</x:f>
@@ -26877,7 +26877,7 @@
         <x:f>IF(A499="",IF(B499="","","MISSING_TEST_ID"),IF(B499="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A499,$B$2:$B$501,B499)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL499" s="9" t="str">
-        <x:f>IF(A499="","",IF(AND(AK499="OK",J499="READY",F499&lt;&gt;"",G499&lt;&gt;"",K499&lt;&gt;"",OR(L499="PASS",L499="FAIL"),M499&lt;&gt;"",O499&lt;&gt;"",P499="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A499="","",IF(AND(AK499="OK",J499="READY",F499&lt;&gt;"",G499&lt;&gt;"",K499&lt;&gt;"",OR(L499="PASS",L499="FAIL"),M499&lt;&gt;"",P499="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM499" s="9" t="str">
         <x:f>IF(A499="","",IF(AND(AK499="OK",J499="READY",F499&lt;&gt;"",G499&lt;&gt;"",K499&lt;&gt;"",S499="OK",OR(R499="PASS",R499="FAIL")),"YES","NO"))</x:f>
@@ -26929,7 +26929,7 @@
         <x:f>IF(A500="",IF(B500="","","MISSING_TEST_ID"),IF(B500="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A500,$B$2:$B$501,B500)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL500" s="9" t="str">
-        <x:f>IF(A500="","",IF(AND(AK500="OK",J500="READY",F500&lt;&gt;"",G500&lt;&gt;"",K500&lt;&gt;"",OR(L500="PASS",L500="FAIL"),M500&lt;&gt;"",O500&lt;&gt;"",P500="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A500="","",IF(AND(AK500="OK",J500="READY",F500&lt;&gt;"",G500&lt;&gt;"",K500&lt;&gt;"",OR(L500="PASS",L500="FAIL"),M500&lt;&gt;"",P500="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM500" s="9" t="str">
         <x:f>IF(A500="","",IF(AND(AK500="OK",J500="READY",F500&lt;&gt;"",G500&lt;&gt;"",K500&lt;&gt;"",S500="OK",OR(R500="PASS",R500="FAIL")),"YES","NO"))</x:f>
@@ -26981,7 +26981,7 @@
         <x:f>IF(A501="",IF(B501="","","MISSING_TEST_ID"),IF(B501="","MISSING_RUN_ID",IF(COUNTIFS($A$2:$A$501,A501,$B$2:$B$501,B501)&lt;&gt;1,"DUPLICATE_ID","OK")))</x:f>
       </x:c>
       <x:c r="AL501" s="9" t="str">
-        <x:f>IF(A501="","",IF(AND(AK501="OK",J501="READY",F501&lt;&gt;"",G501&lt;&gt;"",K501&lt;&gt;"",OR(L501="PASS",L501="FAIL"),M501&lt;&gt;"",O501&lt;&gt;"",P501="social-publication-v2"),"YES","NO"))</x:f>
+        <x:f>IF(A501="","",IF(AND(AK501="OK",J501="READY",F501&lt;&gt;"",G501&lt;&gt;"",K501&lt;&gt;"",OR(L501="PASS",L501="FAIL"),M501&lt;&gt;"",P501="social-publication-v2"),"YES","NO"))</x:f>
       </x:c>
       <x:c r="AM501" s="9" t="str">
         <x:f>IF(A501="","",IF(AND(AK501="OK",J501="READY",F501&lt;&gt;"",G501&lt;&gt;"",K501&lt;&gt;"",S501="OK",OR(R501="PASS",R501="FAIL")),"YES","NO"))</x:f>
@@ -27155,7 +27155,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C11" s="3" t="str">
-        <x:v>Unique IDs, complete context, post, critique, reviewer and matching policy.</x:v>
+        <x:v>Unique IDs, complete context, post, decision, critique and matching policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Ground failure categories in the twelve worked reviews
</commit_message>
<xml_diff>
--- a/Social Media Post Evaluation.xlsx
+++ b/Social Media Post Evaluation.xlsx
@@ -18,11 +18,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="138">
   <si>
     <t>Test_ID</t>
   </si>
   <si>
+    <t>Dimension</t>
+  </si>
+  <si>
     <t>User_Input</t>
   </si>
   <si>
@@ -53,13 +56,34 @@
     <t>Failure_Category</t>
   </si>
   <si>
+    <t>P01</t>
+  </si>
+  <si>
+    <t>PASS when…</t>
+  </si>
+  <si>
+    <t>FAIL when…</t>
+  </si>
+  <si>
     <t>POST_004</t>
   </si>
   <si>
+    <t>Factual Correctness</t>
+  </si>
+  <si>
+    <t>Every concrete claim agrees with the approved facts. No invented numbers, dates, quotes, capabilities, links or outcomes.</t>
+  </si>
+  <si>
+    <t>A concrete claim contradicts the approved facts or adds unsupported information.</t>
+  </si>
+  <si>
     <t>LLM Evaluation Resources Everyone Should Know</t>
   </si>
   <si>
-    <t>Dimension</t>
+    <t>The main point is easy to understand. The writing is coherent, concise and readable without a substantive rewrite.</t>
+  </si>
+  <si>
+    <t>Confusing wording, repetition or poor structure obscures the main point.</t>
   </si>
   <si>
     <t>If you’re working with LLMs in 2026, evaluation can’t be an afterthought.
@@ -77,136 +101,172 @@
 If you’re serious about shipping reliable AI, start by learning how others evaluate what they build.</t>
   </si>
   <si>
-    <t>PASS when…</t>
-  </si>
-  <si>
-    <t>FAIL when…</t>
-  </si>
-  <si>
-    <t>Factual Correctness</t>
+    <t>Value / Insight</t>
+  </si>
+  <si>
+    <t>The post delivers the requested information, example, resource or practical takeaway. Its substance is specific and useful for the stated audience.</t>
+  </si>
+  <si>
+    <t>The post is generic filler, omits requested substance, or promises resources or practical content that are not actually provided.</t>
+  </si>
+  <si>
+    <t>The opening gives the audience a clear reason to read, and the post ends with a relevant, clear call to action or question. If the brief explicitly prohibits a call to action or question, a relevant closing takeaway is sufficient.</t>
+  </si>
+  <si>
+    <t>The opening gives no clear reason to read, or the ending lacks a relevant action or question when one is permitted. Clickbait or an unsupported promise is not a valid hook.</t>
+  </si>
+  <si>
+    <t>Tone Fit</t>
+  </si>
+  <si>
+    <t>The language is professional, accessible and suitable for the stated audience and requested voice.</t>
   </si>
   <si>
     <t>PASS</t>
   </si>
   <si>
+    <t>The language is inappropriate for the audience, unnecessarily difficult, condescending or inconsistent with the requested voice.</t>
+  </si>
+  <si>
     <t>FAIL</t>
   </si>
   <si>
-    <t>Every concrete claim agrees with the approved facts. No invented numbers, dates, quotes, capabilities, links or outcomes.</t>
-  </si>
-  <si>
-    <t>A concrete claim contradicts the approved facts or adds unsupported information.</t>
-  </si>
-  <si>
-    <t>The main point is easy to understand. The writing is coherent, concise and readable without a substantive rewrite.</t>
-  </si>
-  <si>
-    <t>Confusing wording, repetition or poor structure obscures the main point.</t>
-  </si>
-  <si>
-    <t>Value / Insight</t>
-  </si>
-  <si>
-    <t>The post delivers the requested information, example, resource or practical takeaway. Its substance is specific and useful for the stated audience.</t>
-  </si>
-  <si>
-    <t>The post is generic filler, omits requested substance, or promises resources or practical content that are not actually provided.</t>
-  </si>
-  <si>
-    <t>The opening gives the audience a clear reason to read, and the post ends with a relevant, clear call to action or question. If the brief explicitly prohibits a call to action or question, a relevant closing takeaway is sufficient.</t>
-  </si>
-  <si>
-    <t>The opening gives no clear reason to read, or the ending lacks a relevant action or question when one is permitted. Clickbait or an unsupported promise is not a valid hook.</t>
-  </si>
-  <si>
-    <t>Tone Fit</t>
-  </si>
-  <si>
-    <t>The language is professional, accessible and suitable for the stated audience and requested voice.</t>
-  </si>
-  <si>
-    <t>The language is inappropriate for the audience, unnecessarily difficult, condescending or inconsistent with the requested voice.</t>
-  </si>
-  <si>
     <t>Overall rule</t>
   </si>
   <si>
     <t>All five dimensions PASS = overall PASS. Any FAIL = overall FAIL.</t>
   </si>
   <si>
-    <t>A generated post with unfinished reviews shows PENDING. Still review all five dimensions.</t>
-  </si>
-  <si>
     <t>10-post exercise</t>
   </si>
   <si>
     <t>Invent 10 inputs of your own in Evaluation Log. Include the audience, purpose, requirements and approved facts. Then export that tab as CSV and run the generation workflow.</t>
   </si>
   <si>
+    <t>Keep IDs P01–P10. Add an Approved facts: section to each input. Define fictional facts yourself or use verified facts; do not ask the generator to invent them.</t>
+  </si>
+  <si>
+    <t>Your review</t>
+  </si>
+  <si>
+    <t>Choose PASS or FAIL for each dimension. Explain failures in Human_Feedback.</t>
+  </si>
+  <si>
+    <t>If source context is missing, leave the affected dimension blank and explain what is needed.</t>
+  </si>
+  <si>
+    <t>Explicit requirements</t>
+  </si>
+  <si>
+    <t>Missing requested content, a required link, word limit or format fails Value / Insight.</t>
+  </si>
+  <si>
+    <t>An unsupported claim fails Factual Correctness. Style cannot offset another dimension’s failure.</t>
+  </si>
+  <si>
+    <t>Rerun</t>
+  </si>
+  <si>
+    <t>Preserve Evaluation Log. Save revised outputs and fresh reviews in Revised Posts.</t>
+  </si>
+  <si>
+    <t>Comparison matches Test_ID automatically. Rerun failed posts and at least one previously passing post.</t>
+  </si>
+  <si>
+    <t>Existing examples</t>
+  </si>
+  <si>
+    <t>Start with the 12 worked reviews in Existing Examples. Read the post, feedback, five dimension decisions, overall result and main failure category.</t>
+  </si>
+  <si>
+    <t>Decisions interpret the supplied feedback; original posts and comments are unchanged. A blank factual check means the saved evidence is insufficient. Any known FAIL still makes the post FAIL.</t>
+  </si>
+  <si>
+    <t>Failure category</t>
+  </si>
+  <si>
+    <t>Use when…</t>
+  </si>
+  <si>
+    <t>Worked example</t>
+  </si>
+  <si>
+    <t>False or Unsupported Claims</t>
+  </si>
+  <si>
+    <t>A claim is false, unsupported or invented, including dates, capabilities, statistics or testimonials.</t>
+  </si>
+  <si>
+    <t>POST_012: made-up participant testimonials.</t>
+  </si>
+  <si>
+    <t>Missing Useful Content</t>
+  </si>
+  <si>
     <t>The post content is great if we are supplementing it with an actual list of resources. This seems like good content if we already have the infographic ready. As a standalone post, though, it promises resources but only lists types of resources, without naming any evaluation frameworks, repositories or tutorials. Would have added much more value if it included a few useful names and explained what each is for. The ending is vague; would ideally want people to share resources in the comments.</t>
   </si>
   <si>
-    <t>Keep IDs P01–P10. Add an Approved facts: section to each input. Define fictional facts yourself or use verified facts; do not ask the generator to invent them.</t>
-  </si>
-  <si>
-    <t>Low Informational Value</t>
+    <t>The post promises resources, examples or practical guidance but does not deliver useful substance.</t>
+  </si>
+  <si>
+    <t>P02</t>
+  </si>
+  <si>
+    <t>POST_004: names no resources. POST_008: promotes a cheat sheet but supplies no useful checks.</t>
+  </si>
+  <si>
+    <t>Missing Essential Details</t>
+  </si>
+  <si>
+    <t>Information readers need to act is missing, such as workshop date, time or delivery mode. Check whether the brief supplied it.</t>
+  </si>
+  <si>
+    <t>POST_001 and POST_003: missing workshop details. If facts were absent from the brief, fix the input; do not invent them.</t>
+  </si>
+  <si>
+    <t>Missing Closing Action</t>
+  </si>
+  <si>
+    <t>The ending lacks a relevant action or question required by the Engagement rule. A useful takeaway is enough if the request prohibits a CTA.</t>
+  </si>
+  <si>
+    <t>POST_009 and POST_010: useful content, but no closing action or question.</t>
+  </si>
+  <si>
+    <t>Choose one main category</t>
+  </si>
+  <si>
+    <t>These four patterns come from the 12 saved posts and your instructor’s feedback. Pick the main problem; explain all failed dimensions in your feedback.</t>
+  </si>
+  <si>
+    <t>Failure Analysis counts your ten new posts. POST_008’s brief is ambiguous, so it does not prove an explicit instruction was ignored.</t>
+  </si>
+  <si>
+    <t>P03</t>
   </si>
   <si>
     <t>POST_001</t>
   </si>
   <si>
-    <t>Your review</t>
-  </si>
-  <si>
     <t>AI Evaluations Workshop Announcement</t>
   </si>
   <si>
-    <t>Choose PASS or FAIL for each dimension. Explain failures in Human_Feedback.</t>
-  </si>
-  <si>
-    <t>If source context is missing, leave the affected dimension blank and explain what is needed.</t>
-  </si>
-  <si>
-    <t>Explicit requirements</t>
-  </si>
-  <si>
     <t>Building AI systems is one thing. Knowing whether they actually work in production is another. At The Gen Academy, we’re hosting an AI Evaluations Workshop focused on the practical side of evaluating LLMs, RAG pipelines, and AI agents—the part most teams struggle with once prototypes meet reality. In this workshop, we’ll cover: How to think about LLM evaluation beyond accuracy Evaluating RAG pipelines and retrieval quality When and how to use LLMs as judges Designing evals that scale from experiments to production Common evaluation pitfalls (and how to avoid them) Whether you’re: Shipping AI features, Building agentic systems, Or setting up evals for the first time, this session is designed to give you clear frameworks and practical approaches, not just theory. 📅 Seats are limited. 👉 Register now and start building AI systems you can actually trust.</t>
   </si>
   <si>
-    <t>Missing requested content, a required link, word limit or format fails Value / Insight.</t>
-  </si>
-  <si>
-    <t>An unsupported claim fails Factual Correctness. Style cannot offset another dimension’s failure.</t>
-  </si>
-  <si>
-    <t>Rerun</t>
-  </si>
-  <si>
-    <t>P01</t>
-  </si>
-  <si>
-    <t>Preserve Evaluation Log. Save revised outputs and fresh reviews in Revised Posts.</t>
-  </si>
-  <si>
-    <t>Comparison matches Test_ID automatically. Rerun failed posts and at least one previously passing post.</t>
-  </si>
-  <si>
-    <t>Existing examples</t>
-  </si>
-  <si>
-    <t>Start with the 12 worked reviews in Existing Examples. Read the post, feedback, five dimension decisions, overall result and main failure category.</t>
-  </si>
-  <si>
-    <t>Decisions interpret the supplied feedback; original posts and comments are unchanged. A blank factual check means the saved evidence is insufficient. Any known FAIL still makes the post FAIL.</t>
+    <t>P04</t>
+  </si>
+  <si>
+    <t>P05</t>
+  </si>
+  <si>
+    <t>P06</t>
   </si>
   <si>
     <t>The workshop date and time are not mentioned, so readers don't have the basic details they need to decide whether to attend. It is also a bit too wordy for this type of promotional post. I feel like people would not read through the entire thing before getting to the point. Would make the announcement shorter and bring the workshop details and main benefit up front. There is already a CTA to register; a question inviting discussion in the comments could help too, but the missing details and wordy framing are the main problems.</t>
   </si>
   <si>
-    <t>Failure category</t>
-  </si>
-  <si>
-    <t>Poor Framing</t>
+    <t>P07</t>
   </si>
   <si>
     <t>POST_002</t>
@@ -215,13 +275,7 @@
     <t>Evaluating RAG Pipelines: A Framework for Production-Ready Retrieval Systems</t>
   </si>
   <si>
-    <t>Use when…</t>
-  </si>
-  <si>
-    <t>Worked example</t>
-  </si>
-  <si>
-    <t>Incorrect or Hallucinated Content</t>
+    <t>P08</t>
   </si>
   <si>
     <t>RAG systems don’t fail because of the LLM.
@@ -239,25 +293,10 @@
 If you’re serious about shipping reliable RAG systems, your eval strategy needs to mature before your system does.</t>
   </si>
   <si>
-    <t>A claim is false, unsupported or invented, including dates, capabilities, statistics or testimonials.</t>
-  </si>
-  <si>
-    <t>POST_012: made-up participant testimonials.</t>
-  </si>
-  <si>
-    <t>The post is generic or lacks the useful examples, resources or practical substance it promises.</t>
-  </si>
-  <si>
-    <t>POST_004: promises evaluation resources but names none.</t>
-  </si>
-  <si>
-    <t>Instruction Non-Compliance</t>
-  </si>
-  <si>
-    <t>The output does a different task or misses an explicit requirement, such as format, required content or a word limit.</t>
-  </si>
-  <si>
-    <t>POST_008: promotional copy instead of the intended cheat sheet.</t>
+    <t>P09</t>
+  </si>
+  <si>
+    <t>P10</t>
   </si>
   <si>
     <t>The opening claim is too absolute. There are more reasons why RAG systems fail, so saying they don't fail because of the LLM and only pointing to retrieval is misleading. Would qualify that claim. Could add more value if the actual breakdown of evaluating a RAG system, with example metrics for each part, was included instead of just saying we need a framework. There is no clear call to action. Ideally, we would want to invite people to discuss their RAG failures in production.</t>
@@ -267,15 +306,6 @@
   </si>
   <si>
     <t>Register for our AI Evaluations Workshop Now!</t>
-  </si>
-  <si>
-    <t>The presentation gets in the way: wordy or unclear writing, unsuitable tone, or a weak opening or closing.</t>
-  </si>
-  <si>
-    <t>POST_009: useful content, but no clear closing action or question.</t>
-  </si>
-  <si>
-    <t>Choose one main category</t>
   </si>
   <si>
     <t>You can build powerful AI systems.
@@ -291,12 +321,6 @@
 This workshop is built for practitioners who want **practical frameworks, clear mental models, and real-world evaluation strategies** — not just theory.
 📅 Seats are limited.
 👉 Register now and start building AI systems you can trust.</t>
-  </si>
-  <si>
-    <t>Use these categories for your ten new posts. Pick the main problem for each failed post; keep all failed dimension decisions and explain them in your feedback.</t>
-  </si>
-  <si>
-    <t>Failure Analysis counts your own new posts. The worked examples are separate.</t>
   </si>
   <si>
     <t>The date, time and mode of the workshop are missing. For a registration post, I would want those details clearly mentioned. Would also make the intended audience more specific; 'practitioners' is quite broad. The content feels a bit rambly for this category and could get to the point faster. There is already a CTA to register. Encouraging comments or shares could help engagement too, but that is an optional improvement rather than the main issue.</t>
@@ -402,9 +426,6 @@
     <t>Four Questions Your RAG Eval Must Answer</t>
   </si>
   <si>
-    <t>P02</t>
-  </si>
-  <si>
     <t xml:space="preserve">🔍 Evaluating your RAG system? Ask the Right Questions!
 A solid RAG (Retrieval-Augmented Generation) evaluation isn’t complete without answering these four critical questions:
 1️⃣ **Relevance:** Are the retrieved documents actually answering the query?
@@ -435,9 +456,6 @@
 #AI #LLM #AIEvaluation #GenAcademy #MachineLearning #AIWorkflow</t>
   </si>
   <si>
-    <t>P03</t>
-  </si>
-  <si>
     <t>Great content with clear steps that readers can follow when building an LLM-as-a-Judge pipeline. Would add value to someone implementing LLM-J, and the tone is appropriate. The main thing missing is a clear CTA or closing question. It finishes with a general statement about the benefits and then hashtags, without giving readers a next step or inviting them to discuss how they check their own judges.</t>
   </si>
   <si>
@@ -456,9 +474,6 @@
 🔹 **Day 7:** Deploy and monitor production evaluations
 Speed doesn’t mean cutting corners—it means working smarter, automating where possible, and focusing on what truly matters. Ready to accelerate your AI evaluation journey? Let’s make it happen! 💡
 #AI #AIEvaluation #MachineLearning #GenAcademy #ProductionReady #AIWorkflow</t>
-  </si>
-  <si>
-    <t>P04</t>
   </si>
   <si>
     <t>Provides clear steps to build an eval pipeline, although I'm not sure these steps are realistically possible in seven days. The post presents production readiness in a week as something readers can expect, without any evidence for that timeline. Evaluation can be more nuanced and require iteration. Would present this as an example one-week starting plan rather than promising a production-ready system. The CTA works, and the outline would add value to someone learning the steps involved once that claim is qualified.</t>
@@ -483,25 +498,7 @@
 #AIEvals #LLM #GenerativeAI #TheGenAcademy #AITesting #EngineeringExcellence</t>
   </si>
   <si>
-    <t>P05</t>
-  </si>
-  <si>
     <t>The LLM made up testimonials, which is not acceptable. The quotes and the claim that a participant deployed an eval pipeline the next day need to come from actual participant feedback; we shouldn't invent them to make the workshop sound good. Tone is otherwise appropriate, although I would prefer no hashtags or emojis for this type of post. The CTA at the end is clear. The invented testimonials are the main problem here.</t>
-  </si>
-  <si>
-    <t>P06</t>
-  </si>
-  <si>
-    <t>P07</t>
-  </si>
-  <si>
-    <t>P08</t>
-  </si>
-  <si>
-    <t>P09</t>
-  </si>
-  <si>
-    <t>P10</t>
   </si>
   <si>
     <t>Original_Status</t>
@@ -633,21 +630,21 @@
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
     <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -930,210 +927,208 @@
   <sheetData>
     <row r="1" ht="33.75" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" ht="105.0" customHeight="1">
+      <c r="A2" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" ht="105.0" customHeight="1">
-      <c r="A2" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" ht="105.0" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C3" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" ht="105.0" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="4" t="s">
+    <row r="4" ht="105.0" customHeight="1">
+      <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="4" ht="105.0" customHeight="1">
-      <c r="A4" s="4" t="s">
+      <c r="B4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="4" t="s">
+    </row>
+    <row r="5" ht="105.0" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="5" ht="105.0" customHeight="1">
-      <c r="A5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="4" t="s">
+    </row>
+    <row r="6" ht="105.0" customHeight="1">
+      <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="6" ht="105.0" customHeight="1">
-      <c r="A6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" ht="64.5" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="5" t="s">
         <v>34</v>
       </c>
+      <c r="C8" s="5"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="s">
+      <c r="B10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="4" t="s">
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="s">
+      <c r="B12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C12" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>55</v>
-      </c>
     </row>
     <row r="14">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="B15" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="B18" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="s">
+      <c r="C18" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="2" t="s">
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B17" s="2" t="s">
+    <row r="20">
+      <c r="A20" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="s">
+      <c r="C20" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -2145,454 +2140,454 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" ht="600.0" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="A2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" s="6" t="str">
+      <c r="C2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="7" t="str">
         <f t="shared" ref="I2:I13" si="1">IF(C2="","",IF(COUNTIF(D2:H2,"FAIL")&gt;0,"FAIL",IF(COUNTIF(D2:H2,"PASS")=5,"PASS","PENDING")))</f>
         <v>FAIL</v>
       </c>
-      <c r="J2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>39</v>
+      <c r="J2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="3" ht="600.0" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" s="6" t="str">
+      <c r="A3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3" s="6"/>
+      <c r="E3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" s="7" t="str">
         <f t="shared" si="1"/>
         <v>FAIL</v>
       </c>
-      <c r="J3" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>58</v>
+      <c r="J3" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="4" ht="600.0" customHeight="1">
-      <c r="A4" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" s="6" t="str">
+      <c r="A4" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="7" t="str">
         <f t="shared" si="1"/>
         <v>FAIL</v>
       </c>
-      <c r="J4" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>63</v>
+      <c r="J4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="5" ht="600.0" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I5" s="6" t="str">
+      <c r="A5" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D5" s="6"/>
+      <c r="E5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="7" t="str">
         <f t="shared" si="1"/>
         <v>FAIL</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>58</v>
+      <c r="J5" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="6" ht="600.0" customHeight="1">
-      <c r="A6" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I6" s="6" t="str">
+      <c r="A6" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="6"/>
+      <c r="E6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="7" t="str">
         <f t="shared" si="1"/>
         <v>FAIL</v>
       </c>
-      <c r="J6" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>39</v>
+      <c r="J6" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="7" ht="600.0" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I7" s="6" t="str">
+      <c r="A7" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I7" s="7" t="str">
         <f t="shared" si="1"/>
         <v>FAIL</v>
       </c>
-      <c r="J7" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>63</v>
+      <c r="J7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="8" ht="600.0" customHeight="1">
-      <c r="A8" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="6" t="str">
+      <c r="A8" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D8" s="6"/>
+      <c r="E8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I8" s="7" t="str">
         <f t="shared" si="1"/>
         <v>FAIL</v>
       </c>
-      <c r="J8" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>39</v>
+      <c r="J8" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="9" ht="600.0" customHeight="1">
-      <c r="A9" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I9" s="6" t="str">
+      <c r="A9" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" s="7" t="str">
         <f t="shared" si="1"/>
         <v>FAIL</v>
       </c>
-      <c r="J9" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>69</v>
+      <c r="J9" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="10" ht="600.0" customHeight="1">
-      <c r="A10" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I10" s="6" t="str">
+      <c r="A10" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="7" t="str">
         <f t="shared" si="1"/>
         <v>FAIL</v>
       </c>
-      <c r="J10" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>58</v>
+      <c r="J10" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="11" ht="600.0" customHeight="1">
-      <c r="A11" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I11" s="6" t="str">
+      <c r="A11" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I11" s="7" t="str">
         <f t="shared" si="1"/>
         <v>FAIL</v>
       </c>
-      <c r="J11" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>58</v>
+      <c r="J11" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="12" ht="600.0" customHeight="1">
-      <c r="A12" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I12" s="6" t="str">
+      <c r="A12" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I12" s="7" t="str">
         <f t="shared" si="1"/>
         <v>FAIL</v>
       </c>
-      <c r="J12" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>63</v>
+      <c r="J12" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="13" ht="600.0" customHeight="1">
-      <c r="A13" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I13" s="6" t="str">
+      <c r="A13" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I13" s="7" t="str">
         <f t="shared" si="1"/>
         <v>FAIL</v>
       </c>
-      <c r="J13" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>63</v>
+      <c r="J13" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -3588,7 +3583,7 @@
   </conditionalFormatting>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" sqref="K2:K13">
-      <formula1>"Incorrect or Hallucinated Content,Low Informational Value,Instruction Non-Compliance,Poor Framing"</formula1>
+      <formula1>"False or Unsupported Claims,Missing Useful Content,Missing Essential Details,Missing Closing Action"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D2:H13">
       <formula1>"PASS,FAIL"</formula1>
@@ -3626,215 +3621,215 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" ht="159.75" customHeight="1">
-      <c r="A2" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="6" t="str">
+      <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="7" t="str">
         <f t="shared" ref="I2:I11" si="1">IF(C2="","",IF(COUNTIF(D2:H2,"FAIL")&gt;0,"FAIL",IF(COUNTIF(D2:H2,"PASS")=5,"PASS","PENDING")))</f>
         <v/>
       </c>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
     </row>
     <row r="3" ht="159.75" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="6" t="str">
+      <c r="A3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
     </row>
     <row r="4" ht="159.75" customHeight="1">
-      <c r="A4" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="6" t="str">
+      <c r="A4" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
     </row>
     <row r="5" ht="159.75" customHeight="1">
-      <c r="A5" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="6" t="str">
+      <c r="A5" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
     </row>
     <row r="6" ht="159.75" customHeight="1">
-      <c r="A6" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="6" t="str">
+      <c r="A6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
     </row>
     <row r="7" ht="159.75" customHeight="1">
-      <c r="A7" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="6" t="str">
+      <c r="A7" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
     </row>
     <row r="8" ht="159.75" customHeight="1">
-      <c r="A8" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="6" t="str">
+      <c r="A8" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
     </row>
     <row r="9" ht="159.75" customHeight="1">
-      <c r="A9" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="6" t="str">
+      <c r="A9" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
     </row>
     <row r="10" ht="159.75" customHeight="1">
-      <c r="A10" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="6" t="str">
+      <c r="A10" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
     </row>
     <row r="11" ht="159.75" customHeight="1">
-      <c r="A11" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="6" t="str">
+      <c r="A11" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -4829,7 +4824,7 @@
   </conditionalFormatting>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" sqref="K2:K11">
-      <formula1>"Incorrect or Hallucinated Content,Low Informational Value,Instruction Non-Compliance,Poor Framing"</formula1>
+      <formula1>"False or Unsupported Claims,Missing Useful Content,Missing Essential Details,Missing Closing Action"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D2:H11">
       <formula1>"PASS,FAIL"</formula1>
@@ -4867,195 +4862,195 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" ht="159.75" customHeight="1">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="6" t="str">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="7" t="str">
         <f t="shared" ref="I2:I11" si="1">IF(C2="","",IF(COUNTIF(D2:H2,"FAIL")&gt;0,"FAIL",IF(COUNTIF(D2:H2,"PASS")=5,"PASS","PENDING")))</f>
         <v/>
       </c>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
     </row>
     <row r="3" ht="159.75" customHeight="1">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="6" t="str">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
     </row>
     <row r="4" ht="159.75" customHeight="1">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="6" t="str">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
     </row>
     <row r="5" ht="159.75" customHeight="1">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="6" t="str">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
     </row>
     <row r="6" ht="159.75" customHeight="1">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="6" t="str">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
     </row>
     <row r="7" ht="159.75" customHeight="1">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="6" t="str">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
     </row>
     <row r="8" ht="159.75" customHeight="1">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="6" t="str">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
     </row>
     <row r="9" ht="159.75" customHeight="1">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="6" t="str">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
     </row>
     <row r="10" ht="159.75" customHeight="1">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="6" t="str">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
     </row>
     <row r="11" ht="159.75" customHeight="1">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="6" t="str">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -6050,7 +6045,7 @@
   </conditionalFormatting>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" sqref="K2:K11">
-      <formula1>"Incorrect or Hallucinated Content,Low Informational Value,Instruction Non-Compliance,Poor Framing"</formula1>
+      <formula1>"False or Unsupported Claims,Missing Useful Content,Missing Essential Details,Missing Closing Action"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D2:H11">
       <formula1>"PASS,FAIL"</formula1>
@@ -6081,181 +6076,181 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>125</v>
-      </c>
     </row>
     <row r="2" ht="30.0" customHeight="1">
-      <c r="A2" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B2" s="4" t="str">
+      <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2" t="str">
         <f t="array" ref="B2">IF(COUNTIF('Evaluation Log'!$A$2:$A$11,A2)=0,"",IF(INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A2,'Evaluation Log'!$A$2:$A$11,0))="","",INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A2,'Evaluation Log'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="2" t="str">
         <f t="array" ref="C2">IF(COUNTIF('Revised Posts'!$A$2:$A$11,A2)=0,"",IF(INDEX('Revised Posts'!$I$2:$I$11,MATCH(A2,'Revised Posts'!$A$2:$A$11,0))="","",INDEX('Revised Posts'!$I$2:$I$11,MATCH(A2,'Revised Posts'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="D2" s="4" t="str">
+      <c r="D2" s="2" t="str">
         <f t="shared" ref="D2:D11" si="1">IF(OR(B2="",C2=""),"",IF(OR(B2="PENDING",C2="PENDING"),"Awaiting review",IF(B2="FAIL",IF(C2="PASS","Fixed","Still fails"),IF(C2="FAIL","Got worse","Still passes"))))</f>
         <v/>
       </c>
     </row>
     <row r="3" ht="30.0" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B3" s="4" t="str">
+      <c r="A3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="2" t="str">
         <f t="array" ref="B3">IF(COUNTIF('Evaluation Log'!$A$2:$A$11,A3)=0,"",IF(INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A3,'Evaluation Log'!$A$2:$A$11,0))="","",INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A3,'Evaluation Log'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="C3" s="4" t="str">
+      <c r="C3" s="2" t="str">
         <f t="array" ref="C3">IF(COUNTIF('Revised Posts'!$A$2:$A$11,A3)=0,"",IF(INDEX('Revised Posts'!$I$2:$I$11,MATCH(A3,'Revised Posts'!$A$2:$A$11,0))="","",INDEX('Revised Posts'!$I$2:$I$11,MATCH(A3,'Revised Posts'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="D3" s="4" t="str">
+      <c r="D3" s="2" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="4" ht="30.0" customHeight="1">
-      <c r="A4" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B4" s="4" t="str">
+      <c r="A4" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="2" t="str">
         <f t="array" ref="B4">IF(COUNTIF('Evaluation Log'!$A$2:$A$11,A4)=0,"",IF(INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A4,'Evaluation Log'!$A$2:$A$11,0))="","",INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A4,'Evaluation Log'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="C4" s="4" t="str">
+      <c r="C4" s="2" t="str">
         <f t="array" ref="C4">IF(COUNTIF('Revised Posts'!$A$2:$A$11,A4)=0,"",IF(INDEX('Revised Posts'!$I$2:$I$11,MATCH(A4,'Revised Posts'!$A$2:$A$11,0))="","",INDEX('Revised Posts'!$I$2:$I$11,MATCH(A4,'Revised Posts'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="D4" s="4" t="str">
+      <c r="D4" s="2" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="5" ht="30.0" customHeight="1">
-      <c r="A5" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B5" s="4" t="str">
+      <c r="A5" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="2" t="str">
         <f t="array" ref="B5">IF(COUNTIF('Evaluation Log'!$A$2:$A$11,A5)=0,"",IF(INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A5,'Evaluation Log'!$A$2:$A$11,0))="","",INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A5,'Evaluation Log'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="2" t="str">
         <f t="array" ref="C5">IF(COUNTIF('Revised Posts'!$A$2:$A$11,A5)=0,"",IF(INDEX('Revised Posts'!$I$2:$I$11,MATCH(A5,'Revised Posts'!$A$2:$A$11,0))="","",INDEX('Revised Posts'!$I$2:$I$11,MATCH(A5,'Revised Posts'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="D5" s="4" t="str">
+      <c r="D5" s="2" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="6" ht="30.0" customHeight="1">
-      <c r="A6" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B6" s="4" t="str">
+      <c r="A6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="2" t="str">
         <f t="array" ref="B6">IF(COUNTIF('Evaluation Log'!$A$2:$A$11,A6)=0,"",IF(INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A6,'Evaluation Log'!$A$2:$A$11,0))="","",INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A6,'Evaluation Log'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="C6" s="4" t="str">
+      <c r="C6" s="2" t="str">
         <f t="array" ref="C6">IF(COUNTIF('Revised Posts'!$A$2:$A$11,A6)=0,"",IF(INDEX('Revised Posts'!$I$2:$I$11,MATCH(A6,'Revised Posts'!$A$2:$A$11,0))="","",INDEX('Revised Posts'!$I$2:$I$11,MATCH(A6,'Revised Posts'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="D6" s="4" t="str">
+      <c r="D6" s="2" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="7" ht="30.0" customHeight="1">
-      <c r="A7" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B7" s="4" t="str">
+      <c r="A7" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="2" t="str">
         <f t="array" ref="B7">IF(COUNTIF('Evaluation Log'!$A$2:$A$11,A7)=0,"",IF(INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A7,'Evaluation Log'!$A$2:$A$11,0))="","",INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A7,'Evaluation Log'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="C7" s="4" t="str">
+      <c r="C7" s="2" t="str">
         <f t="array" ref="C7">IF(COUNTIF('Revised Posts'!$A$2:$A$11,A7)=0,"",IF(INDEX('Revised Posts'!$I$2:$I$11,MATCH(A7,'Revised Posts'!$A$2:$A$11,0))="","",INDEX('Revised Posts'!$I$2:$I$11,MATCH(A7,'Revised Posts'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="D7" s="4" t="str">
+      <c r="D7" s="2" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="8" ht="30.0" customHeight="1">
-      <c r="A8" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="B8" s="4" t="str">
+      <c r="A8" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="2" t="str">
         <f t="array" ref="B8">IF(COUNTIF('Evaluation Log'!$A$2:$A$11,A8)=0,"",IF(INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A8,'Evaluation Log'!$A$2:$A$11,0))="","",INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A8,'Evaluation Log'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="C8" s="4" t="str">
+      <c r="C8" s="2" t="str">
         <f t="array" ref="C8">IF(COUNTIF('Revised Posts'!$A$2:$A$11,A8)=0,"",IF(INDEX('Revised Posts'!$I$2:$I$11,MATCH(A8,'Revised Posts'!$A$2:$A$11,0))="","",INDEX('Revised Posts'!$I$2:$I$11,MATCH(A8,'Revised Posts'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="D8" s="4" t="str">
+      <c r="D8" s="2" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="9" ht="30.0" customHeight="1">
-      <c r="A9" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="B9" s="4" t="str">
+      <c r="A9" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="2" t="str">
         <f t="array" ref="B9">IF(COUNTIF('Evaluation Log'!$A$2:$A$11,A9)=0,"",IF(INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A9,'Evaluation Log'!$A$2:$A$11,0))="","",INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A9,'Evaluation Log'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="C9" s="4" t="str">
+      <c r="C9" s="2" t="str">
         <f t="array" ref="C9">IF(COUNTIF('Revised Posts'!$A$2:$A$11,A9)=0,"",IF(INDEX('Revised Posts'!$I$2:$I$11,MATCH(A9,'Revised Posts'!$A$2:$A$11,0))="","",INDEX('Revised Posts'!$I$2:$I$11,MATCH(A9,'Revised Posts'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="D9" s="4" t="str">
+      <c r="D9" s="2" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="10" ht="30.0" customHeight="1">
-      <c r="A10" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B10" s="4" t="str">
+      <c r="A10" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="2" t="str">
         <f t="array" ref="B10">IF(COUNTIF('Evaluation Log'!$A$2:$A$11,A10)=0,"",IF(INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A10,'Evaluation Log'!$A$2:$A$11,0))="","",INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A10,'Evaluation Log'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="C10" s="4" t="str">
+      <c r="C10" s="2" t="str">
         <f t="array" ref="C10">IF(COUNTIF('Revised Posts'!$A$2:$A$11,A10)=0,"",IF(INDEX('Revised Posts'!$I$2:$I$11,MATCH(A10,'Revised Posts'!$A$2:$A$11,0))="","",INDEX('Revised Posts'!$I$2:$I$11,MATCH(A10,'Revised Posts'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="D10" s="4" t="str">
+      <c r="D10" s="2" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="11" ht="30.0" customHeight="1">
-      <c r="A11" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="B11" s="4" t="str">
+      <c r="A11" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="2" t="str">
         <f t="array" ref="B11">IF(COUNTIF('Evaluation Log'!$A$2:$A$11,A11)=0,"",IF(INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A11,'Evaluation Log'!$A$2:$A$11,0))="","",INDEX('Evaluation Log'!$I$2:$I$11,MATCH(A11,'Evaluation Log'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="C11" s="4" t="str">
+      <c r="C11" s="2" t="str">
         <f t="array" ref="C11">IF(COUNTIF('Revised Posts'!$A$2:$A$11,A11)=0,"",IF(INDEX('Revised Posts'!$I$2:$I$11,MATCH(A11,'Revised Posts'!$A$2:$A$11,0))="","",INDEX('Revised Posts'!$I$2:$I$11,MATCH(A11,'Revised Posts'!$A$2:$A$11,0))))</f>
         <v/>
       </c>
-      <c r="D11" s="4" t="str">
+      <c r="D11" s="2" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -7273,54 +7268,54 @@
   <sheetData>
     <row r="1" ht="33.75" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>128</v>
-      </c>
     </row>
     <row r="2" ht="54.75" customHeight="1">
-      <c r="A2" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B2" s="4">
+      <c r="A2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="2">
         <f>COUNTIFS('Evaluation Log'!$K$2:$K$11,A2,'Evaluation Log'!$I$2:$I$11,"FAIL")</f>
         <v>0</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" ht="54.75" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3" s="4">
+      <c r="A3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="2">
         <f>COUNTIFS('Evaluation Log'!$K$2:$K$11,A3,'Evaluation Log'!$I$2:$I$11,"FAIL")</f>
         <v>0</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" ht="54.75" customHeight="1">
-      <c r="A4" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B4" s="4">
+      <c r="A4" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="2">
         <f>COUNTIFS('Evaluation Log'!$K$2:$K$11,A4,'Evaluation Log'!$I$2:$I$11,"FAIL")</f>
         <v>0</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" ht="54.75" customHeight="1">
-      <c r="A5" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B5" s="4">
+      <c r="A5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="2">
         <f>COUNTIFS('Evaluation Log'!$K$2:$K$11,A5,'Evaluation Log'!$I$2:$I$11,"FAIL")</f>
         <v>0</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="2"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -8328,84 +8323,84 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" ht="139.5" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="2" ht="139.5" customHeight="1">
-      <c r="A2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -9417,626 +9412,626 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>138</v>
-      </c>
     </row>
     <row r="2" ht="54.75" customHeight="1">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="3" ht="54.75" customHeight="1">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
     <row r="4" ht="54.75" customHeight="1">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
     </row>
     <row r="5" ht="54.75" customHeight="1">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
     </row>
     <row r="6" ht="54.75" customHeight="1">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
     </row>
     <row r="7" ht="54.75" customHeight="1">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
     </row>
     <row r="8" ht="54.75" customHeight="1">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
     </row>
     <row r="9" ht="54.75" customHeight="1">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
     </row>
     <row r="10" ht="54.75" customHeight="1">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
     </row>
     <row r="11" ht="54.75" customHeight="1">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
     </row>
     <row r="12" ht="54.75" customHeight="1">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
     </row>
     <row r="13" ht="54.75" customHeight="1">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
     </row>
     <row r="14" ht="54.75" customHeight="1">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
     </row>
     <row r="15" ht="54.75" customHeight="1">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
     </row>
     <row r="16" ht="54.75" customHeight="1">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
     <row r="17" ht="54.75" customHeight="1">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
     </row>
     <row r="18" ht="54.75" customHeight="1">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
     </row>
     <row r="19" ht="54.75" customHeight="1">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
     </row>
     <row r="20" ht="54.75" customHeight="1">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
     </row>
     <row r="21" ht="54.75" customHeight="1">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
     </row>
     <row r="22" ht="54.75" customHeight="1">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
     </row>
     <row r="23" ht="54.75" customHeight="1">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
     </row>
     <row r="24" ht="54.75" customHeight="1">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
     </row>
     <row r="25" ht="54.75" customHeight="1">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
     </row>
     <row r="26" ht="54.75" customHeight="1">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
     </row>
     <row r="27" ht="54.75" customHeight="1">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
     </row>
     <row r="28" ht="54.75" customHeight="1">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
     </row>
     <row r="29" ht="54.75" customHeight="1">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
     </row>
     <row r="30" ht="54.75" customHeight="1">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
     </row>
     <row r="31" ht="54.75" customHeight="1">
-      <c r="A31" s="4"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
     </row>
     <row r="32" ht="54.75" customHeight="1">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
     </row>
     <row r="33" ht="54.75" customHeight="1">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
     </row>
     <row r="34" ht="54.75" customHeight="1">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
     </row>
     <row r="35" ht="54.75" customHeight="1">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
     </row>
     <row r="36" ht="54.75" customHeight="1">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
     </row>
     <row r="37" ht="54.75" customHeight="1">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
     </row>
     <row r="38" ht="54.75" customHeight="1">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
     </row>
     <row r="39" ht="54.75" customHeight="1">
-      <c r="A39" s="4"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
     </row>
     <row r="40" ht="54.75" customHeight="1">
-      <c r="A40" s="4"/>
-      <c r="B40" s="4"/>
-      <c r="C40" s="4"/>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
     </row>
     <row r="41" ht="54.75" customHeight="1">
-      <c r="A41" s="4"/>
-      <c r="B41" s="4"/>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
     </row>
     <row r="42" ht="54.75" customHeight="1">
-      <c r="A42" s="4"/>
-      <c r="B42" s="4"/>
-      <c r="C42" s="4"/>
-      <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
-      <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4"/>
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
     </row>
     <row r="43" ht="54.75" customHeight="1">
-      <c r="A43" s="4"/>
-      <c r="B43" s="4"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
     </row>
     <row r="44" ht="54.75" customHeight="1">
-      <c r="A44" s="4"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
     </row>
     <row r="45" ht="54.75" customHeight="1">
-      <c r="A45" s="4"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
+      <c r="A45" s="2"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
     </row>
     <row r="46" ht="54.75" customHeight="1">
-      <c r="A46" s="4"/>
-      <c r="B46" s="4"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
     </row>
     <row r="47" ht="54.75" customHeight="1">
-      <c r="A47" s="4"/>
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
     </row>
     <row r="48" ht="54.75" customHeight="1">
-      <c r="A48" s="4"/>
-      <c r="B48" s="4"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
     </row>
     <row r="49" ht="54.75" customHeight="1">
-      <c r="A49" s="4"/>
-      <c r="B49" s="4"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
+      <c r="A49" s="2"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
     </row>
     <row r="50" ht="54.75" customHeight="1">
-      <c r="A50" s="4"/>
-      <c r="B50" s="4"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="4"/>
-      <c r="E50" s="4"/>
-      <c r="F50" s="4"/>
-      <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
+      <c r="F50" s="2"/>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
     </row>
     <row r="51" ht="54.75" customHeight="1">
-      <c r="A51" s="4"/>
-      <c r="B51" s="4"/>
-      <c r="C51" s="4"/>
-      <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
+      <c r="A51" s="2"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
     </row>
     <row r="52" ht="54.75" customHeight="1">
-      <c r="A52" s="4"/>
-      <c r="B52" s="4"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
-      <c r="F52" s="4"/>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
     </row>
     <row r="53" ht="54.75" customHeight="1">
-      <c r="A53" s="4"/>
-      <c r="B53" s="4"/>
-      <c r="C53" s="4"/>
-      <c r="D53" s="4"/>
-      <c r="E53" s="4"/>
-      <c r="F53" s="4"/>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
+      <c r="A53" s="2"/>
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="H53" s="2"/>
     </row>
     <row r="54" ht="54.75" customHeight="1">
-      <c r="A54" s="4"/>
-      <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
-      <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2"/>
+      <c r="G54" s="2"/>
+      <c r="H54" s="2"/>
     </row>
     <row r="55" ht="54.75" customHeight="1">
-      <c r="A55" s="4"/>
-      <c r="B55" s="4"/>
-      <c r="C55" s="4"/>
-      <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
     </row>
     <row r="56" ht="54.75" customHeight="1">
-      <c r="A56" s="4"/>
-      <c r="B56" s="4"/>
-      <c r="C56" s="4"/>
-      <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
-      <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
     </row>
     <row r="57" ht="54.75" customHeight="1">
-      <c r="A57" s="4"/>
-      <c r="B57" s="4"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
-      <c r="F57" s="4"/>
-      <c r="G57" s="4"/>
-      <c r="H57" s="4"/>
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
     </row>
     <row r="58" ht="54.75" customHeight="1">
-      <c r="A58" s="4"/>
-      <c r="B58" s="4"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
     </row>
     <row r="59" ht="54.75" customHeight="1">
-      <c r="A59" s="4"/>
-      <c r="B59" s="4"/>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4"/>
-      <c r="E59" s="4"/>
-      <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4"/>
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
     </row>
     <row r="60" ht="54.75" customHeight="1">
-      <c r="A60" s="4"/>
-      <c r="B60" s="4"/>
-      <c r="C60" s="4"/>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2"/>
+      <c r="G60" s="2"/>
+      <c r="H60" s="2"/>
     </row>
     <row r="61" ht="54.75" customHeight="1">
-      <c r="A61" s="4"/>
-      <c r="B61" s="4"/>
-      <c r="C61" s="4"/>
-      <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
-      <c r="F61" s="4"/>
-      <c r="G61" s="4"/>
-      <c r="H61" s="4"/>
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
     </row>
     <row r="62" ht="15.75" customHeight="1"/>
     <row r="63" ht="15.75" customHeight="1"/>

</xml_diff>